<commit_message>
Added 7th recruit method after technical presentation, poster, etc to IRB protocol
</commit_message>
<xml_diff>
--- a/LakeMeadWaterBankDivideInflow.xlsx
+++ b/LakeMeadWaterBankDivideInflow.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Box\ColoradoRiver\LakeMeadInflow-ImmersiveModel\LakeMeadDivideInflow\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2098394058039/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD78D97-C7E9-4C27-BF8C-60CA00335947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
+    <workbookView xWindow="28680" yWindow="-1200" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe-Directions" sheetId="62" r:id="rId1"/>
@@ -4135,67 +4135,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -4258,6 +4198,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4290,6 +4233,63 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4351,12 +4351,6 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4365,15 +4359,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4405,6 +4390,9 @@
     <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4414,11 +4402,23 @@
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -15861,20 +15861,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="368" t="s">
+      <c r="A1" s="348" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="368"/>
-      <c r="C1" s="368"/>
-      <c r="D1" s="368"/>
-      <c r="E1" s="368"/>
-      <c r="F1" s="368"/>
-      <c r="G1" s="368"/>
-      <c r="H1" s="368"/>
-      <c r="I1" s="368"/>
-      <c r="J1" s="368"/>
-      <c r="K1" s="368"/>
-      <c r="L1" s="368"/>
+      <c r="B1" s="348"/>
+      <c r="C1" s="348"/>
+      <c r="D1" s="348"/>
+      <c r="E1" s="348"/>
+      <c r="F1" s="348"/>
+      <c r="G1" s="348"/>
+      <c r="H1" s="348"/>
+      <c r="I1" s="348"/>
+      <c r="J1" s="348"/>
+      <c r="K1" s="348"/>
+      <c r="L1" s="348"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -15900,41 +15900,41 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:18" s="52" customFormat="1" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="369" t="s">
+      <c r="A4" s="349" t="s">
         <v>296</v>
       </c>
-      <c r="B4" s="370"/>
-      <c r="C4" s="370"/>
-      <c r="D4" s="370"/>
-      <c r="E4" s="370"/>
-      <c r="F4" s="370"/>
-      <c r="G4" s="370"/>
-      <c r="H4" s="370"/>
-      <c r="I4" s="370"/>
-      <c r="J4" s="370"/>
-      <c r="K4" s="370"/>
-      <c r="L4" s="371"/>
-      <c r="N4" s="372"/>
-      <c r="O4" s="372"/>
-      <c r="P4" s="372"/>
-      <c r="Q4" s="372"/>
-      <c r="R4" s="372"/>
+      <c r="B4" s="350"/>
+      <c r="C4" s="350"/>
+      <c r="D4" s="350"/>
+      <c r="E4" s="350"/>
+      <c r="F4" s="350"/>
+      <c r="G4" s="350"/>
+      <c r="H4" s="350"/>
+      <c r="I4" s="350"/>
+      <c r="J4" s="350"/>
+      <c r="K4" s="350"/>
+      <c r="L4" s="351"/>
+      <c r="N4" s="352"/>
+      <c r="O4" s="352"/>
+      <c r="P4" s="352"/>
+      <c r="Q4" s="352"/>
+      <c r="R4" s="352"/>
     </row>
     <row r="5" spans="1:18" s="52" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="373" t="s">
+      <c r="A5" s="353" t="s">
         <v>280</v>
       </c>
-      <c r="B5" s="374"/>
-      <c r="C5" s="374"/>
-      <c r="D5" s="374"/>
-      <c r="E5" s="374"/>
-      <c r="F5" s="374"/>
-      <c r="G5" s="374"/>
-      <c r="H5" s="374"/>
-      <c r="I5" s="374"/>
-      <c r="J5" s="374"/>
-      <c r="K5" s="374"/>
-      <c r="L5" s="375"/>
+      <c r="B5" s="354"/>
+      <c r="C5" s="354"/>
+      <c r="D5" s="354"/>
+      <c r="E5" s="354"/>
+      <c r="F5" s="354"/>
+      <c r="G5" s="354"/>
+      <c r="H5" s="354"/>
+      <c r="I5" s="354"/>
+      <c r="J5" s="354"/>
+      <c r="K5" s="354"/>
+      <c r="L5" s="355"/>
       <c r="N5" s="110"/>
       <c r="O5" s="110"/>
       <c r="P5" s="110"/>
@@ -15942,20 +15942,20 @@
       <c r="R5" s="110"/>
     </row>
     <row r="6" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="373" t="s">
+      <c r="A6" s="353" t="s">
         <v>297</v>
       </c>
-      <c r="B6" s="374"/>
-      <c r="C6" s="374"/>
-      <c r="D6" s="374"/>
-      <c r="E6" s="374"/>
-      <c r="F6" s="374"/>
-      <c r="G6" s="374"/>
-      <c r="H6" s="374"/>
-      <c r="I6" s="374"/>
-      <c r="J6" s="374"/>
-      <c r="K6" s="374"/>
-      <c r="L6" s="375"/>
+      <c r="B6" s="354"/>
+      <c r="C6" s="354"/>
+      <c r="D6" s="354"/>
+      <c r="E6" s="354"/>
+      <c r="F6" s="354"/>
+      <c r="G6" s="354"/>
+      <c r="H6" s="354"/>
+      <c r="I6" s="354"/>
+      <c r="J6" s="354"/>
+      <c r="K6" s="354"/>
+      <c r="L6" s="355"/>
       <c r="N6" s="110"/>
       <c r="O6" s="110"/>
       <c r="P6" s="110"/>
@@ -15964,19 +15964,19 @@
     </row>
     <row r="7" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="214"/>
-      <c r="B7" s="374" t="s">
+      <c r="B7" s="354" t="s">
         <v>298</v>
       </c>
-      <c r="C7" s="374"/>
-      <c r="D7" s="374"/>
-      <c r="E7" s="374"/>
-      <c r="F7" s="374"/>
-      <c r="G7" s="374"/>
-      <c r="H7" s="374"/>
-      <c r="I7" s="374"/>
-      <c r="J7" s="374"/>
-      <c r="K7" s="374"/>
-      <c r="L7" s="375"/>
+      <c r="C7" s="354"/>
+      <c r="D7" s="354"/>
+      <c r="E7" s="354"/>
+      <c r="F7" s="354"/>
+      <c r="G7" s="354"/>
+      <c r="H7" s="354"/>
+      <c r="I7" s="354"/>
+      <c r="J7" s="354"/>
+      <c r="K7" s="354"/>
+      <c r="L7" s="355"/>
       <c r="N7" s="110"/>
       <c r="O7" s="110"/>
       <c r="P7" s="110"/>
@@ -15985,19 +15985,19 @@
     </row>
     <row r="8" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="215"/>
-      <c r="B8" s="389" t="s">
+      <c r="B8" s="370" t="s">
         <v>299</v>
       </c>
-      <c r="C8" s="389"/>
-      <c r="D8" s="389"/>
-      <c r="E8" s="389"/>
-      <c r="F8" s="389"/>
-      <c r="G8" s="389"/>
-      <c r="H8" s="389"/>
-      <c r="I8" s="389"/>
-      <c r="J8" s="389"/>
-      <c r="K8" s="389"/>
-      <c r="L8" s="390"/>
+      <c r="C8" s="370"/>
+      <c r="D8" s="370"/>
+      <c r="E8" s="370"/>
+      <c r="F8" s="370"/>
+      <c r="G8" s="370"/>
+      <c r="H8" s="370"/>
+      <c r="I8" s="370"/>
+      <c r="J8" s="370"/>
+      <c r="K8" s="370"/>
+      <c r="L8" s="371"/>
       <c r="N8" s="110"/>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
@@ -16019,38 +16019,38 @@
       <c r="L9" s="110"/>
     </row>
     <row r="10" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="391" t="s">
+      <c r="A10" s="372" t="s">
         <v>334</v>
       </c>
-      <c r="B10" s="392"/>
-      <c r="C10" s="392"/>
-      <c r="D10" s="392"/>
-      <c r="E10" s="392"/>
-      <c r="F10" s="392"/>
-      <c r="G10" s="392"/>
-      <c r="H10" s="392"/>
-      <c r="I10" s="392"/>
-      <c r="J10" s="392"/>
-      <c r="K10" s="392"/>
-      <c r="L10" s="393"/>
+      <c r="B10" s="373"/>
+      <c r="C10" s="373"/>
+      <c r="D10" s="373"/>
+      <c r="E10" s="373"/>
+      <c r="F10" s="373"/>
+      <c r="G10" s="373"/>
+      <c r="H10" s="373"/>
+      <c r="I10" s="373"/>
+      <c r="J10" s="373"/>
+      <c r="K10" s="373"/>
+      <c r="L10" s="374"/>
     </row>
     <row r="11" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="235" t="s">
         <v>335</v>
       </c>
-      <c r="B11" s="344" t="s">
+      <c r="B11" s="375" t="s">
         <v>338</v>
       </c>
-      <c r="C11" s="344"/>
-      <c r="D11" s="344"/>
-      <c r="E11" s="344"/>
-      <c r="F11" s="344"/>
-      <c r="G11" s="344"/>
-      <c r="H11" s="344"/>
-      <c r="I11" s="344"/>
-      <c r="J11" s="344"/>
-      <c r="K11" s="344"/>
-      <c r="L11" s="345"/>
+      <c r="C11" s="375"/>
+      <c r="D11" s="375"/>
+      <c r="E11" s="375"/>
+      <c r="F11" s="375"/>
+      <c r="G11" s="375"/>
+      <c r="H11" s="375"/>
+      <c r="I11" s="375"/>
+      <c r="J11" s="375"/>
+      <c r="K11" s="375"/>
+      <c r="L11" s="376"/>
     </row>
     <row r="12" spans="1:18" s="57" customFormat="1" ht="161.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="227"/>
@@ -16070,51 +16070,51 @@
       <c r="A13" s="235" t="s">
         <v>336</v>
       </c>
-      <c r="B13" s="344" t="s">
+      <c r="B13" s="375" t="s">
         <v>339</v>
       </c>
-      <c r="C13" s="344"/>
-      <c r="D13" s="344"/>
-      <c r="E13" s="344"/>
-      <c r="F13" s="344"/>
-      <c r="G13" s="344"/>
-      <c r="H13" s="344"/>
-      <c r="I13" s="344"/>
-      <c r="J13" s="344"/>
-      <c r="K13" s="344"/>
-      <c r="L13" s="345"/>
+      <c r="C13" s="375"/>
+      <c r="D13" s="375"/>
+      <c r="E13" s="375"/>
+      <c r="F13" s="375"/>
+      <c r="G13" s="375"/>
+      <c r="H13" s="375"/>
+      <c r="I13" s="375"/>
+      <c r="J13" s="375"/>
+      <c r="K13" s="375"/>
+      <c r="L13" s="376"/>
     </row>
     <row r="14" spans="1:18" s="57" customFormat="1" ht="90.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="227"/>
-      <c r="B14" s="346"/>
-      <c r="C14" s="346"/>
-      <c r="D14" s="346"/>
-      <c r="E14" s="346"/>
-      <c r="F14" s="346"/>
-      <c r="G14" s="346"/>
-      <c r="H14" s="346"/>
-      <c r="I14" s="346"/>
-      <c r="J14" s="346"/>
-      <c r="K14" s="346"/>
-      <c r="L14" s="347"/>
+      <c r="B14" s="386"/>
+      <c r="C14" s="386"/>
+      <c r="D14" s="386"/>
+      <c r="E14" s="386"/>
+      <c r="F14" s="386"/>
+      <c r="G14" s="386"/>
+      <c r="H14" s="386"/>
+      <c r="I14" s="386"/>
+      <c r="J14" s="386"/>
+      <c r="K14" s="386"/>
+      <c r="L14" s="387"/>
     </row>
     <row r="15" spans="1:18" s="56" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="235" t="s">
         <v>337</v>
       </c>
-      <c r="B15" s="344" t="s">
+      <c r="B15" s="375" t="s">
         <v>465</v>
       </c>
-      <c r="C15" s="344"/>
-      <c r="D15" s="344"/>
-      <c r="E15" s="344"/>
-      <c r="F15" s="344"/>
-      <c r="G15" s="344"/>
-      <c r="H15" s="344"/>
-      <c r="I15" s="344"/>
-      <c r="J15" s="344"/>
-      <c r="K15" s="344"/>
-      <c r="L15" s="345"/>
+      <c r="C15" s="375"/>
+      <c r="D15" s="375"/>
+      <c r="E15" s="375"/>
+      <c r="F15" s="375"/>
+      <c r="G15" s="375"/>
+      <c r="H15" s="375"/>
+      <c r="I15" s="375"/>
+      <c r="J15" s="375"/>
+      <c r="K15" s="375"/>
+      <c r="L15" s="376"/>
     </row>
     <row r="16" spans="1:18" s="57" customFormat="1" ht="269" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="227"/>
@@ -16131,12 +16131,12 @@
       <c r="L16" s="234"/>
     </row>
     <row r="17" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="342" t="s">
+      <c r="A17" s="384" t="s">
         <v>343</v>
       </c>
-      <c r="B17" s="343"/>
-      <c r="C17" s="343"/>
-      <c r="D17" s="343"/>
+      <c r="B17" s="385"/>
+      <c r="C17" s="385"/>
+      <c r="D17" s="385"/>
       <c r="E17" s="232" t="s">
         <v>344</v>
       </c>
@@ -16163,84 +16163,84 @@
       <c r="L18" s="110"/>
     </row>
     <row r="19" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="376" t="s">
+      <c r="A19" s="356" t="s">
         <v>165</v>
       </c>
-      <c r="B19" s="377"/>
-      <c r="C19" s="377"/>
-      <c r="D19" s="377"/>
-      <c r="E19" s="377"/>
-      <c r="F19" s="377"/>
-      <c r="G19" s="377"/>
-      <c r="H19" s="377"/>
-      <c r="I19" s="377"/>
-      <c r="J19" s="377"/>
-      <c r="K19" s="377"/>
-      <c r="L19" s="378"/>
+      <c r="B19" s="357"/>
+      <c r="C19" s="357"/>
+      <c r="D19" s="357"/>
+      <c r="E19" s="357"/>
+      <c r="F19" s="357"/>
+      <c r="G19" s="357"/>
+      <c r="H19" s="357"/>
+      <c r="I19" s="357"/>
+      <c r="J19" s="357"/>
+      <c r="K19" s="357"/>
+      <c r="L19" s="358"/>
     </row>
     <row r="20" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="379" t="s">
+      <c r="A20" s="359" t="s">
         <v>281</v>
       </c>
-      <c r="B20" s="380"/>
-      <c r="C20" s="380"/>
-      <c r="D20" s="380"/>
-      <c r="E20" s="380"/>
-      <c r="F20" s="380"/>
-      <c r="G20" s="380"/>
-      <c r="H20" s="380"/>
-      <c r="I20" s="380"/>
-      <c r="J20" s="380"/>
-      <c r="K20" s="380"/>
-      <c r="L20" s="381"/>
+      <c r="B20" s="360"/>
+      <c r="C20" s="360"/>
+      <c r="D20" s="360"/>
+      <c r="E20" s="360"/>
+      <c r="F20" s="360"/>
+      <c r="G20" s="360"/>
+      <c r="H20" s="360"/>
+      <c r="I20" s="360"/>
+      <c r="J20" s="360"/>
+      <c r="K20" s="360"/>
+      <c r="L20" s="361"/>
     </row>
     <row r="21" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="382" t="s">
+      <c r="A21" s="362" t="s">
         <v>282</v>
       </c>
-      <c r="B21" s="358"/>
-      <c r="C21" s="358"/>
-      <c r="D21" s="358"/>
-      <c r="E21" s="358"/>
-      <c r="F21" s="358"/>
-      <c r="G21" s="358"/>
-      <c r="H21" s="358"/>
-      <c r="I21" s="358"/>
-      <c r="J21" s="358"/>
-      <c r="K21" s="358"/>
-      <c r="L21" s="359"/>
+      <c r="B21" s="342"/>
+      <c r="C21" s="342"/>
+      <c r="D21" s="342"/>
+      <c r="E21" s="342"/>
+      <c r="F21" s="342"/>
+      <c r="G21" s="342"/>
+      <c r="H21" s="342"/>
+      <c r="I21" s="342"/>
+      <c r="J21" s="342"/>
+      <c r="K21" s="342"/>
+      <c r="L21" s="363"/>
     </row>
     <row r="22" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="382" t="s">
+      <c r="A22" s="362" t="s">
         <v>166</v>
       </c>
-      <c r="B22" s="358"/>
-      <c r="C22" s="358"/>
-      <c r="D22" s="358"/>
-      <c r="E22" s="358"/>
-      <c r="F22" s="358"/>
-      <c r="G22" s="358"/>
-      <c r="H22" s="358"/>
-      <c r="I22" s="358"/>
-      <c r="J22" s="358"/>
-      <c r="K22" s="358"/>
-      <c r="L22" s="359"/>
+      <c r="B22" s="342"/>
+      <c r="C22" s="342"/>
+      <c r="D22" s="342"/>
+      <c r="E22" s="342"/>
+      <c r="F22" s="342"/>
+      <c r="G22" s="342"/>
+      <c r="H22" s="342"/>
+      <c r="I22" s="342"/>
+      <c r="J22" s="342"/>
+      <c r="K22" s="342"/>
+      <c r="L22" s="363"/>
     </row>
     <row r="23" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="383" t="s">
+      <c r="A23" s="364" t="s">
         <v>283</v>
       </c>
-      <c r="B23" s="384"/>
-      <c r="C23" s="384"/>
-      <c r="D23" s="384"/>
-      <c r="E23" s="384"/>
-      <c r="F23" s="384"/>
-      <c r="G23" s="384"/>
-      <c r="H23" s="384"/>
-      <c r="I23" s="384"/>
-      <c r="J23" s="384"/>
-      <c r="K23" s="384"/>
-      <c r="L23" s="385"/>
+      <c r="B23" s="365"/>
+      <c r="C23" s="365"/>
+      <c r="D23" s="365"/>
+      <c r="E23" s="365"/>
+      <c r="F23" s="365"/>
+      <c r="G23" s="365"/>
+      <c r="H23" s="365"/>
+      <c r="I23" s="365"/>
+      <c r="J23" s="365"/>
+      <c r="K23" s="365"/>
+      <c r="L23" s="366"/>
     </row>
     <row r="24" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="110"/>
@@ -16257,332 +16257,332 @@
       <c r="L24" s="110"/>
     </row>
     <row r="25" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="386" t="s">
+      <c r="A25" s="367" t="s">
         <v>279</v>
       </c>
-      <c r="B25" s="387"/>
-      <c r="C25" s="387"/>
-      <c r="D25" s="387"/>
-      <c r="E25" s="387"/>
-      <c r="F25" s="387"/>
-      <c r="G25" s="387"/>
-      <c r="H25" s="387"/>
-      <c r="I25" s="387"/>
-      <c r="J25" s="387"/>
-      <c r="K25" s="387"/>
-      <c r="L25" s="388"/>
+      <c r="B25" s="368"/>
+      <c r="C25" s="368"/>
+      <c r="D25" s="368"/>
+      <c r="E25" s="368"/>
+      <c r="F25" s="368"/>
+      <c r="G25" s="368"/>
+      <c r="H25" s="368"/>
+      <c r="I25" s="368"/>
+      <c r="J25" s="368"/>
+      <c r="K25" s="368"/>
+      <c r="L25" s="369"/>
       <c r="N25" s="1"/>
     </row>
     <row r="26" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="365" t="s">
+      <c r="A26" s="345" t="s">
         <v>175</v>
       </c>
-      <c r="B26" s="366"/>
-      <c r="C26" s="366"/>
-      <c r="D26" s="366"/>
-      <c r="E26" s="366"/>
-      <c r="F26" s="366"/>
-      <c r="G26" s="366"/>
-      <c r="H26" s="366"/>
-      <c r="I26" s="366"/>
-      <c r="J26" s="366"/>
-      <c r="K26" s="366"/>
-      <c r="L26" s="367"/>
+      <c r="B26" s="346"/>
+      <c r="C26" s="346"/>
+      <c r="D26" s="346"/>
+      <c r="E26" s="346"/>
+      <c r="F26" s="346"/>
+      <c r="G26" s="346"/>
+      <c r="H26" s="346"/>
+      <c r="I26" s="346"/>
+      <c r="J26" s="346"/>
+      <c r="K26" s="346"/>
+      <c r="L26" s="347"/>
       <c r="N26" s="1"/>
     </row>
     <row r="27" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="209">
         <v>1</v>
       </c>
-      <c r="B27" s="351" t="s">
+      <c r="B27" s="379" t="s">
         <v>174</v>
       </c>
-      <c r="C27" s="351"/>
-      <c r="D27" s="351"/>
-      <c r="E27" s="351"/>
-      <c r="F27" s="351"/>
-      <c r="G27" s="351"/>
-      <c r="H27" s="351"/>
-      <c r="I27" s="351"/>
-      <c r="J27" s="351"/>
-      <c r="K27" s="351"/>
-      <c r="L27" s="352"/>
+      <c r="C27" s="379"/>
+      <c r="D27" s="379"/>
+      <c r="E27" s="379"/>
+      <c r="F27" s="379"/>
+      <c r="G27" s="379"/>
+      <c r="H27" s="379"/>
+      <c r="I27" s="379"/>
+      <c r="J27" s="379"/>
+      <c r="K27" s="379"/>
+      <c r="L27" s="380"/>
     </row>
     <row r="28" spans="1:14" s="57" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="209">
         <v>2</v>
       </c>
-      <c r="B28" s="351" t="s">
+      <c r="B28" s="379" t="s">
         <v>275</v>
       </c>
-      <c r="C28" s="351"/>
-      <c r="D28" s="351"/>
-      <c r="E28" s="351"/>
-      <c r="F28" s="351"/>
-      <c r="G28" s="351"/>
-      <c r="H28" s="351"/>
-      <c r="I28" s="351"/>
-      <c r="J28" s="351"/>
-      <c r="K28" s="351"/>
-      <c r="L28" s="352"/>
+      <c r="C28" s="379"/>
+      <c r="D28" s="379"/>
+      <c r="E28" s="379"/>
+      <c r="F28" s="379"/>
+      <c r="G28" s="379"/>
+      <c r="H28" s="379"/>
+      <c r="I28" s="379"/>
+      <c r="J28" s="379"/>
+      <c r="K28" s="379"/>
+      <c r="L28" s="380"/>
       <c r="N28" s="104"/>
     </row>
     <row r="29" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="209">
         <v>3</v>
       </c>
-      <c r="B29" s="351" t="s">
+      <c r="B29" s="379" t="s">
         <v>167</v>
       </c>
-      <c r="C29" s="351"/>
-      <c r="D29" s="351"/>
-      <c r="E29" s="351"/>
-      <c r="F29" s="351"/>
-      <c r="G29" s="351"/>
-      <c r="H29" s="351"/>
-      <c r="I29" s="351"/>
-      <c r="J29" s="351"/>
-      <c r="K29" s="351"/>
-      <c r="L29" s="352"/>
+      <c r="C29" s="379"/>
+      <c r="D29" s="379"/>
+      <c r="E29" s="379"/>
+      <c r="F29" s="379"/>
+      <c r="G29" s="379"/>
+      <c r="H29" s="379"/>
+      <c r="I29" s="379"/>
+      <c r="J29" s="379"/>
+      <c r="K29" s="379"/>
+      <c r="L29" s="380"/>
       <c r="N29" s="104"/>
     </row>
     <row r="30" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="209">
         <v>4</v>
       </c>
-      <c r="B30" s="351" t="s">
+      <c r="B30" s="379" t="s">
         <v>284</v>
       </c>
-      <c r="C30" s="351"/>
-      <c r="D30" s="351"/>
-      <c r="E30" s="351"/>
-      <c r="F30" s="351"/>
-      <c r="G30" s="351"/>
-      <c r="H30" s="351"/>
-      <c r="I30" s="351"/>
-      <c r="J30" s="351"/>
-      <c r="K30" s="351"/>
-      <c r="L30" s="352"/>
+      <c r="C30" s="379"/>
+      <c r="D30" s="379"/>
+      <c r="E30" s="379"/>
+      <c r="F30" s="379"/>
+      <c r="G30" s="379"/>
+      <c r="H30" s="379"/>
+      <c r="I30" s="379"/>
+      <c r="J30" s="379"/>
+      <c r="K30" s="379"/>
+      <c r="L30" s="380"/>
       <c r="N30" s="104"/>
     </row>
     <row r="31" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="209">
         <v>5</v>
       </c>
-      <c r="B31" s="351" t="s">
+      <c r="B31" s="379" t="s">
         <v>168</v>
       </c>
-      <c r="C31" s="351"/>
-      <c r="D31" s="351"/>
-      <c r="E31" s="351"/>
-      <c r="F31" s="351"/>
-      <c r="G31" s="351"/>
-      <c r="H31" s="351"/>
-      <c r="I31" s="351"/>
-      <c r="J31" s="351"/>
-      <c r="K31" s="351"/>
-      <c r="L31" s="352"/>
+      <c r="C31" s="379"/>
+      <c r="D31" s="379"/>
+      <c r="E31" s="379"/>
+      <c r="F31" s="379"/>
+      <c r="G31" s="379"/>
+      <c r="H31" s="379"/>
+      <c r="I31" s="379"/>
+      <c r="J31" s="379"/>
+      <c r="K31" s="379"/>
+      <c r="L31" s="380"/>
       <c r="N31" s="104"/>
     </row>
     <row r="32" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="209"/>
-      <c r="B32" s="351" t="s">
+      <c r="B32" s="379" t="s">
         <v>169</v>
       </c>
-      <c r="C32" s="351"/>
-      <c r="D32" s="351"/>
-      <c r="E32" s="351"/>
-      <c r="F32" s="351"/>
-      <c r="G32" s="351"/>
-      <c r="H32" s="351"/>
-      <c r="I32" s="351"/>
-      <c r="J32" s="351"/>
-      <c r="K32" s="351"/>
-      <c r="L32" s="352"/>
+      <c r="C32" s="379"/>
+      <c r="D32" s="379"/>
+      <c r="E32" s="379"/>
+      <c r="F32" s="379"/>
+      <c r="G32" s="379"/>
+      <c r="H32" s="379"/>
+      <c r="I32" s="379"/>
+      <c r="J32" s="379"/>
+      <c r="K32" s="379"/>
+      <c r="L32" s="380"/>
       <c r="N32" s="104"/>
     </row>
     <row r="33" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="209"/>
-      <c r="B33" s="351" t="s">
+      <c r="B33" s="379" t="s">
         <v>170</v>
       </c>
-      <c r="C33" s="351"/>
-      <c r="D33" s="351"/>
-      <c r="E33" s="351"/>
-      <c r="F33" s="351"/>
-      <c r="G33" s="351"/>
-      <c r="H33" s="351"/>
-      <c r="I33" s="351"/>
-      <c r="J33" s="351"/>
-      <c r="K33" s="351"/>
-      <c r="L33" s="352"/>
+      <c r="C33" s="379"/>
+      <c r="D33" s="379"/>
+      <c r="E33" s="379"/>
+      <c r="F33" s="379"/>
+      <c r="G33" s="379"/>
+      <c r="H33" s="379"/>
+      <c r="I33" s="379"/>
+      <c r="J33" s="379"/>
+      <c r="K33" s="379"/>
+      <c r="L33" s="380"/>
       <c r="N33" s="104"/>
     </row>
     <row r="34" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="360" t="s">
+      <c r="A34" s="381" t="s">
         <v>176</v>
       </c>
-      <c r="B34" s="361"/>
-      <c r="C34" s="361"/>
-      <c r="D34" s="361"/>
-      <c r="E34" s="361"/>
-      <c r="F34" s="361"/>
-      <c r="G34" s="361"/>
-      <c r="H34" s="361"/>
-      <c r="I34" s="361"/>
-      <c r="J34" s="361"/>
-      <c r="K34" s="361"/>
-      <c r="L34" s="362"/>
+      <c r="B34" s="382"/>
+      <c r="C34" s="382"/>
+      <c r="D34" s="382"/>
+      <c r="E34" s="382"/>
+      <c r="F34" s="382"/>
+      <c r="G34" s="382"/>
+      <c r="H34" s="382"/>
+      <c r="I34" s="382"/>
+      <c r="J34" s="382"/>
+      <c r="K34" s="382"/>
+      <c r="L34" s="383"/>
       <c r="N34" s="104"/>
     </row>
     <row r="35" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="209">
         <v>1</v>
       </c>
-      <c r="B35" s="351" t="s">
+      <c r="B35" s="379" t="s">
         <v>171</v>
       </c>
-      <c r="C35" s="351"/>
-      <c r="D35" s="351"/>
-      <c r="E35" s="351"/>
-      <c r="F35" s="351"/>
-      <c r="G35" s="351"/>
-      <c r="H35" s="351"/>
-      <c r="I35" s="351"/>
-      <c r="J35" s="351"/>
-      <c r="K35" s="351"/>
-      <c r="L35" s="352"/>
+      <c r="C35" s="379"/>
+      <c r="D35" s="379"/>
+      <c r="E35" s="379"/>
+      <c r="F35" s="379"/>
+      <c r="G35" s="379"/>
+      <c r="H35" s="379"/>
+      <c r="I35" s="379"/>
+      <c r="J35" s="379"/>
+      <c r="K35" s="379"/>
+      <c r="L35" s="380"/>
       <c r="N35" s="104"/>
     </row>
     <row r="36" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="209"/>
-      <c r="B36" s="349" t="s">
+      <c r="B36" s="377" t="s">
         <v>426</v>
       </c>
-      <c r="C36" s="349"/>
-      <c r="D36" s="349"/>
-      <c r="E36" s="349"/>
-      <c r="F36" s="349"/>
-      <c r="G36" s="349"/>
-      <c r="H36" s="349"/>
-      <c r="I36" s="349"/>
-      <c r="J36" s="349"/>
-      <c r="K36" s="349"/>
-      <c r="L36" s="350"/>
+      <c r="C36" s="377"/>
+      <c r="D36" s="377"/>
+      <c r="E36" s="377"/>
+      <c r="F36" s="377"/>
+      <c r="G36" s="377"/>
+      <c r="H36" s="377"/>
+      <c r="I36" s="377"/>
+      <c r="J36" s="377"/>
+      <c r="K36" s="377"/>
+      <c r="L36" s="378"/>
       <c r="N36" s="104"/>
     </row>
     <row r="37" spans="1:14" s="57" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="209">
         <v>2</v>
       </c>
-      <c r="B37" s="351" t="s">
+      <c r="B37" s="379" t="s">
         <v>278</v>
       </c>
-      <c r="C37" s="351"/>
-      <c r="D37" s="351"/>
-      <c r="E37" s="351"/>
-      <c r="F37" s="351"/>
-      <c r="G37" s="351"/>
-      <c r="H37" s="351"/>
-      <c r="I37" s="351"/>
-      <c r="J37" s="351"/>
-      <c r="K37" s="351"/>
-      <c r="L37" s="352"/>
+      <c r="C37" s="379"/>
+      <c r="D37" s="379"/>
+      <c r="E37" s="379"/>
+      <c r="F37" s="379"/>
+      <c r="G37" s="379"/>
+      <c r="H37" s="379"/>
+      <c r="I37" s="379"/>
+      <c r="J37" s="379"/>
+      <c r="K37" s="379"/>
+      <c r="L37" s="380"/>
       <c r="N37" s="104"/>
     </row>
     <row r="38" spans="1:14" s="57" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="209">
         <v>3</v>
       </c>
-      <c r="B38" s="351" t="s">
+      <c r="B38" s="379" t="s">
         <v>475</v>
       </c>
-      <c r="C38" s="351"/>
-      <c r="D38" s="351"/>
-      <c r="E38" s="351"/>
-      <c r="F38" s="351"/>
-      <c r="G38" s="351"/>
-      <c r="H38" s="351"/>
-      <c r="I38" s="351"/>
-      <c r="J38" s="351"/>
-      <c r="K38" s="351"/>
-      <c r="L38" s="352"/>
+      <c r="C38" s="379"/>
+      <c r="D38" s="379"/>
+      <c r="E38" s="379"/>
+      <c r="F38" s="379"/>
+      <c r="G38" s="379"/>
+      <c r="H38" s="379"/>
+      <c r="I38" s="379"/>
+      <c r="J38" s="379"/>
+      <c r="K38" s="379"/>
+      <c r="L38" s="380"/>
       <c r="N38" s="104"/>
     </row>
     <row r="39" spans="1:14" s="57" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="209">
         <v>4</v>
       </c>
-      <c r="B39" s="351" t="s">
+      <c r="B39" s="379" t="s">
         <v>285</v>
       </c>
-      <c r="C39" s="351"/>
-      <c r="D39" s="351"/>
-      <c r="E39" s="351"/>
-      <c r="F39" s="351"/>
-      <c r="G39" s="351"/>
-      <c r="H39" s="351"/>
-      <c r="I39" s="351"/>
-      <c r="J39" s="351"/>
-      <c r="K39" s="351"/>
-      <c r="L39" s="352"/>
+      <c r="C39" s="379"/>
+      <c r="D39" s="379"/>
+      <c r="E39" s="379"/>
+      <c r="F39" s="379"/>
+      <c r="G39" s="379"/>
+      <c r="H39" s="379"/>
+      <c r="I39" s="379"/>
+      <c r="J39" s="379"/>
+      <c r="K39" s="379"/>
+      <c r="L39" s="380"/>
       <c r="N39" s="104"/>
     </row>
     <row r="40" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="209">
         <v>5</v>
       </c>
-      <c r="B40" s="349" t="s">
+      <c r="B40" s="377" t="s">
         <v>269</v>
       </c>
-      <c r="C40" s="349"/>
-      <c r="D40" s="349"/>
-      <c r="E40" s="349"/>
-      <c r="F40" s="349"/>
-      <c r="G40" s="349"/>
-      <c r="H40" s="349"/>
-      <c r="I40" s="349"/>
-      <c r="J40" s="349"/>
-      <c r="K40" s="349"/>
-      <c r="L40" s="350"/>
+      <c r="C40" s="377"/>
+      <c r="D40" s="377"/>
+      <c r="E40" s="377"/>
+      <c r="F40" s="377"/>
+      <c r="G40" s="377"/>
+      <c r="H40" s="377"/>
+      <c r="I40" s="377"/>
+      <c r="J40" s="377"/>
+      <c r="K40" s="377"/>
+      <c r="L40" s="378"/>
       <c r="N40" s="104"/>
     </row>
     <row r="41" spans="1:14" s="57" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="209">
         <v>6</v>
       </c>
-      <c r="B41" s="349" t="s">
+      <c r="B41" s="377" t="s">
         <v>476</v>
       </c>
-      <c r="C41" s="349"/>
-      <c r="D41" s="349"/>
-      <c r="E41" s="349"/>
-      <c r="F41" s="349"/>
-      <c r="G41" s="349"/>
-      <c r="H41" s="349"/>
-      <c r="I41" s="349"/>
-      <c r="J41" s="349"/>
-      <c r="K41" s="349"/>
-      <c r="L41" s="350"/>
+      <c r="C41" s="377"/>
+      <c r="D41" s="377"/>
+      <c r="E41" s="377"/>
+      <c r="F41" s="377"/>
+      <c r="G41" s="377"/>
+      <c r="H41" s="377"/>
+      <c r="I41" s="377"/>
+      <c r="J41" s="377"/>
+      <c r="K41" s="377"/>
+      <c r="L41" s="378"/>
       <c r="N41" s="104"/>
     </row>
     <row r="42" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="209">
         <v>7</v>
       </c>
-      <c r="B42" s="351" t="s">
+      <c r="B42" s="379" t="s">
         <v>270</v>
       </c>
-      <c r="C42" s="351"/>
-      <c r="D42" s="351"/>
-      <c r="E42" s="351"/>
-      <c r="F42" s="351"/>
-      <c r="G42" s="351"/>
-      <c r="H42" s="351"/>
-      <c r="I42" s="351"/>
-      <c r="J42" s="351"/>
-      <c r="K42" s="351"/>
-      <c r="L42" s="352"/>
+      <c r="C42" s="379"/>
+      <c r="D42" s="379"/>
+      <c r="E42" s="379"/>
+      <c r="F42" s="379"/>
+      <c r="G42" s="379"/>
+      <c r="H42" s="379"/>
+      <c r="I42" s="379"/>
+      <c r="J42" s="379"/>
+      <c r="K42" s="379"/>
+      <c r="L42" s="380"/>
     </row>
     <row r="43" spans="1:14" s="57" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="209"/>
@@ -16599,56 +16599,56 @@
       <c r="L43" s="211"/>
     </row>
     <row r="44" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="360" t="s">
+      <c r="A44" s="381" t="s">
         <v>273</v>
       </c>
-      <c r="B44" s="361"/>
-      <c r="C44" s="361"/>
-      <c r="D44" s="361"/>
-      <c r="E44" s="361"/>
-      <c r="F44" s="361"/>
-      <c r="G44" s="361"/>
-      <c r="H44" s="361"/>
-      <c r="I44" s="361"/>
-      <c r="J44" s="361"/>
-      <c r="K44" s="361"/>
-      <c r="L44" s="362"/>
+      <c r="B44" s="382"/>
+      <c r="C44" s="382"/>
+      <c r="D44" s="382"/>
+      <c r="E44" s="382"/>
+      <c r="F44" s="382"/>
+      <c r="G44" s="382"/>
+      <c r="H44" s="382"/>
+      <c r="I44" s="382"/>
+      <c r="J44" s="382"/>
+      <c r="K44" s="382"/>
+      <c r="L44" s="383"/>
     </row>
     <row r="45" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="212" t="s">
         <v>271</v>
       </c>
-      <c r="B45" s="351" t="s">
+      <c r="B45" s="379" t="s">
         <v>172</v>
       </c>
-      <c r="C45" s="351"/>
-      <c r="D45" s="351"/>
-      <c r="E45" s="351"/>
-      <c r="F45" s="351"/>
-      <c r="G45" s="351"/>
-      <c r="H45" s="351"/>
-      <c r="I45" s="351"/>
-      <c r="J45" s="351"/>
-      <c r="K45" s="351"/>
-      <c r="L45" s="352"/>
+      <c r="C45" s="379"/>
+      <c r="D45" s="379"/>
+      <c r="E45" s="379"/>
+      <c r="F45" s="379"/>
+      <c r="G45" s="379"/>
+      <c r="H45" s="379"/>
+      <c r="I45" s="379"/>
+      <c r="J45" s="379"/>
+      <c r="K45" s="379"/>
+      <c r="L45" s="380"/>
     </row>
     <row r="46" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="213" t="s">
         <v>272</v>
       </c>
-      <c r="B46" s="353" t="s">
+      <c r="B46" s="389" t="s">
         <v>274</v>
       </c>
-      <c r="C46" s="353"/>
-      <c r="D46" s="353"/>
-      <c r="E46" s="353"/>
-      <c r="F46" s="353"/>
-      <c r="G46" s="353"/>
-      <c r="H46" s="353"/>
-      <c r="I46" s="353"/>
-      <c r="J46" s="353"/>
-      <c r="K46" s="353"/>
-      <c r="L46" s="354"/>
+      <c r="C46" s="389"/>
+      <c r="D46" s="389"/>
+      <c r="E46" s="389"/>
+      <c r="F46" s="389"/>
+      <c r="G46" s="389"/>
+      <c r="H46" s="389"/>
+      <c r="I46" s="389"/>
+      <c r="J46" s="389"/>
+      <c r="K46" s="389"/>
+      <c r="L46" s="390"/>
     </row>
     <row r="47" spans="1:14" s="57" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="157"/>
@@ -16665,20 +16665,20 @@
       <c r="L47" s="110"/>
     </row>
     <row r="48" spans="1:14" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="355" t="s">
+      <c r="A48" s="391" t="s">
         <v>200</v>
       </c>
-      <c r="B48" s="356"/>
-      <c r="C48" s="356"/>
-      <c r="D48" s="356"/>
-      <c r="E48" s="356"/>
-      <c r="F48" s="356"/>
-      <c r="G48" s="356"/>
-      <c r="H48" s="356"/>
-      <c r="I48" s="356"/>
-      <c r="J48" s="356"/>
-      <c r="K48" s="356"/>
-      <c r="L48" s="357"/>
+      <c r="B48" s="392"/>
+      <c r="C48" s="392"/>
+      <c r="D48" s="392"/>
+      <c r="E48" s="392"/>
+      <c r="F48" s="392"/>
+      <c r="G48" s="392"/>
+      <c r="H48" s="392"/>
+      <c r="I48" s="392"/>
+      <c r="J48" s="392"/>
+      <c r="K48" s="392"/>
+      <c r="L48" s="393"/>
     </row>
     <row r="49" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="216" t="s">
@@ -16766,126 +16766,126 @@
       <c r="B54" s="165" t="s">
         <v>24</v>
       </c>
-      <c r="C54" s="358" t="s">
+      <c r="C54" s="342" t="s">
         <v>262</v>
       </c>
-      <c r="D54" s="358"/>
-      <c r="E54" s="358"/>
-      <c r="F54" s="358"/>
-      <c r="G54" s="358"/>
-      <c r="H54" s="358"/>
-      <c r="I54" s="358"/>
-      <c r="J54" s="358"/>
-      <c r="K54" s="358"/>
-      <c r="L54" s="359"/>
+      <c r="D54" s="342"/>
+      <c r="E54" s="342"/>
+      <c r="F54" s="342"/>
+      <c r="G54" s="342"/>
+      <c r="H54" s="342"/>
+      <c r="I54" s="342"/>
+      <c r="J54" s="342"/>
+      <c r="K54" s="342"/>
+      <c r="L54" s="363"/>
     </row>
     <row r="55" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="164"/>
       <c r="B55" s="165" t="s">
         <v>263</v>
       </c>
-      <c r="C55" s="358" t="s">
+      <c r="C55" s="342" t="s">
         <v>264</v>
       </c>
-      <c r="D55" s="358"/>
-      <c r="E55" s="358"/>
-      <c r="F55" s="358"/>
-      <c r="G55" s="358"/>
-      <c r="H55" s="358"/>
-      <c r="I55" s="358"/>
-      <c r="J55" s="358"/>
-      <c r="K55" s="358"/>
-      <c r="L55" s="359"/>
+      <c r="D55" s="342"/>
+      <c r="E55" s="342"/>
+      <c r="F55" s="342"/>
+      <c r="G55" s="342"/>
+      <c r="H55" s="342"/>
+      <c r="I55" s="342"/>
+      <c r="J55" s="342"/>
+      <c r="K55" s="342"/>
+      <c r="L55" s="363"/>
     </row>
     <row r="56" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="164"/>
       <c r="B56" s="165" t="s">
         <v>327</v>
       </c>
-      <c r="C56" s="358" t="s">
+      <c r="C56" s="342" t="s">
         <v>328</v>
       </c>
-      <c r="D56" s="358"/>
-      <c r="E56" s="358"/>
-      <c r="F56" s="358"/>
-      <c r="G56" s="358"/>
-      <c r="H56" s="358"/>
-      <c r="I56" s="358"/>
-      <c r="J56" s="358"/>
-      <c r="K56" s="358"/>
-      <c r="L56" s="359"/>
+      <c r="D56" s="342"/>
+      <c r="E56" s="342"/>
+      <c r="F56" s="342"/>
+      <c r="G56" s="342"/>
+      <c r="H56" s="342"/>
+      <c r="I56" s="342"/>
+      <c r="J56" s="342"/>
+      <c r="K56" s="342"/>
+      <c r="L56" s="363"/>
     </row>
     <row r="57" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="164"/>
       <c r="B57" s="165" t="s">
         <v>98</v>
       </c>
-      <c r="C57" s="358" t="s">
+      <c r="C57" s="342" t="s">
         <v>99</v>
       </c>
-      <c r="D57" s="358"/>
-      <c r="E57" s="358"/>
-      <c r="F57" s="358"/>
-      <c r="G57" s="358"/>
-      <c r="H57" s="358"/>
-      <c r="I57" s="358"/>
-      <c r="J57" s="358"/>
-      <c r="K57" s="358"/>
-      <c r="L57" s="359"/>
+      <c r="D57" s="342"/>
+      <c r="E57" s="342"/>
+      <c r="F57" s="342"/>
+      <c r="G57" s="342"/>
+      <c r="H57" s="342"/>
+      <c r="I57" s="342"/>
+      <c r="J57" s="342"/>
+      <c r="K57" s="342"/>
+      <c r="L57" s="363"/>
     </row>
     <row r="58" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="164"/>
       <c r="B58" s="165" t="s">
         <v>198</v>
       </c>
-      <c r="C58" s="358" t="s">
+      <c r="C58" s="342" t="s">
         <v>199</v>
       </c>
-      <c r="D58" s="358"/>
-      <c r="E58" s="358"/>
-      <c r="F58" s="358"/>
-      <c r="G58" s="358"/>
-      <c r="H58" s="358"/>
-      <c r="I58" s="358"/>
-      <c r="J58" s="358"/>
-      <c r="K58" s="358"/>
-      <c r="L58" s="359"/>
+      <c r="D58" s="342"/>
+      <c r="E58" s="342"/>
+      <c r="F58" s="342"/>
+      <c r="G58" s="342"/>
+      <c r="H58" s="342"/>
+      <c r="I58" s="342"/>
+      <c r="J58" s="342"/>
+      <c r="K58" s="342"/>
+      <c r="L58" s="363"/>
     </row>
     <row r="59" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="164"/>
       <c r="B59" s="165" t="s">
         <v>163</v>
       </c>
-      <c r="C59" s="358" t="s">
+      <c r="C59" s="342" t="s">
         <v>466</v>
       </c>
-      <c r="D59" s="363"/>
-      <c r="E59" s="363"/>
-      <c r="F59" s="363"/>
-      <c r="G59" s="363"/>
-      <c r="H59" s="363"/>
-      <c r="I59" s="363"/>
-      <c r="J59" s="363"/>
-      <c r="K59" s="363"/>
-      <c r="L59" s="364"/>
+      <c r="D59" s="343"/>
+      <c r="E59" s="343"/>
+      <c r="F59" s="343"/>
+      <c r="G59" s="343"/>
+      <c r="H59" s="343"/>
+      <c r="I59" s="343"/>
+      <c r="J59" s="343"/>
+      <c r="K59" s="343"/>
+      <c r="L59" s="344"/>
     </row>
     <row r="60" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="164"/>
       <c r="B60" s="165" t="s">
         <v>393</v>
       </c>
-      <c r="C60" s="358" t="s">
+      <c r="C60" s="342" t="s">
         <v>394</v>
       </c>
-      <c r="D60" s="358"/>
-      <c r="E60" s="358"/>
-      <c r="F60" s="358"/>
-      <c r="G60" s="358"/>
-      <c r="H60" s="358"/>
-      <c r="I60" s="358"/>
-      <c r="J60" s="358"/>
-      <c r="K60" s="358"/>
-      <c r="L60" s="359"/>
+      <c r="D60" s="342"/>
+      <c r="E60" s="342"/>
+      <c r="F60" s="342"/>
+      <c r="G60" s="342"/>
+      <c r="H60" s="342"/>
+      <c r="I60" s="342"/>
+      <c r="J60" s="342"/>
+      <c r="K60" s="342"/>
+      <c r="L60" s="363"/>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" s="164"/>
@@ -17003,25 +17003,57 @@
       </c>
     </row>
     <row r="82" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="348" t="s">
+      <c r="A82" s="388" t="s">
         <v>397</v>
       </c>
-      <c r="B82" s="348"/>
-      <c r="C82" s="348"/>
-      <c r="D82" s="348"/>
-      <c r="E82" s="348"/>
-      <c r="F82" s="348"/>
-      <c r="G82" s="348"/>
-      <c r="H82" s="348"/>
-      <c r="I82" s="348"/>
-      <c r="J82" s="348"/>
-      <c r="K82" s="348"/>
-      <c r="L82" s="348"/>
+      <c r="B82" s="388"/>
+      <c r="C82" s="388"/>
+      <c r="D82" s="388"/>
+      <c r="E82" s="388"/>
+      <c r="F82" s="388"/>
+      <c r="G82" s="388"/>
+      <c r="H82" s="388"/>
+      <c r="I82" s="388"/>
+      <c r="J82" s="388"/>
+      <c r="K82" s="388"/>
+      <c r="L82" s="388"/>
     </row>
     <row r="87" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="88" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="B15:L15"/>
+    <mergeCell ref="A82:L82"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B42:L42"/>
+    <mergeCell ref="B45:L45"/>
+    <mergeCell ref="B46:L46"/>
+    <mergeCell ref="A48:L48"/>
+    <mergeCell ref="C54:L54"/>
+    <mergeCell ref="C57:L57"/>
+    <mergeCell ref="C58:L58"/>
+    <mergeCell ref="C55:L55"/>
+    <mergeCell ref="C60:L60"/>
+    <mergeCell ref="A44:L44"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="C56:L56"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B28:L28"/>
+    <mergeCell ref="B29:L29"/>
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B31:L31"/>
+    <mergeCell ref="B32:L32"/>
+    <mergeCell ref="B33:L33"/>
+    <mergeCell ref="A34:L34"/>
+    <mergeCell ref="B35:L35"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B39:L39"/>
     <mergeCell ref="C59:L59"/>
     <mergeCell ref="A26:L26"/>
     <mergeCell ref="A1:L1"/>
@@ -17038,38 +17070,6 @@
     <mergeCell ref="B7:L7"/>
     <mergeCell ref="B8:L8"/>
     <mergeCell ref="A10:L10"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="C56:L56"/>
-    <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B27:L27"/>
-    <mergeCell ref="B28:L28"/>
-    <mergeCell ref="B29:L29"/>
-    <mergeCell ref="B30:L30"/>
-    <mergeCell ref="B31:L31"/>
-    <mergeCell ref="B32:L32"/>
-    <mergeCell ref="B33:L33"/>
-    <mergeCell ref="A34:L34"/>
-    <mergeCell ref="B35:L35"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="B38:L38"/>
-    <mergeCell ref="B37:L37"/>
-    <mergeCell ref="B39:L39"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="B14:L14"/>
-    <mergeCell ref="B15:L15"/>
-    <mergeCell ref="A82:L82"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B42:L42"/>
-    <mergeCell ref="B45:L45"/>
-    <mergeCell ref="B46:L46"/>
-    <mergeCell ref="A48:L48"/>
-    <mergeCell ref="C54:L54"/>
-    <mergeCell ref="C57:L57"/>
-    <mergeCell ref="C58:L58"/>
-    <mergeCell ref="C55:L55"/>
-    <mergeCell ref="C60:L60"/>
-    <mergeCell ref="A44:L44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A67" r:id="rId1" xr:uid="{C9866D44-2827-49D7-B9C3-89CF23FACDC1}"/>
@@ -24393,62 +24393,62 @@
       <c r="G5" s="185" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="427" t="s">
+      <c r="I5" s="422" t="s">
         <v>423</v>
       </c>
-      <c r="J5" s="428"/>
-      <c r="K5" s="428"/>
-      <c r="L5" s="428"/>
-      <c r="M5" s="428"/>
-      <c r="N5" s="428"/>
-      <c r="O5" s="428"/>
-      <c r="P5" s="428"/>
-      <c r="Q5" s="428"/>
-      <c r="R5" s="428"/>
-      <c r="S5" s="428"/>
-      <c r="T5" s="428"/>
-      <c r="U5" s="428"/>
-      <c r="V5" s="428"/>
-      <c r="W5" s="429"/>
+      <c r="J5" s="423"/>
+      <c r="K5" s="423"/>
+      <c r="L5" s="423"/>
+      <c r="M5" s="423"/>
+      <c r="N5" s="423"/>
+      <c r="O5" s="423"/>
+      <c r="P5" s="423"/>
+      <c r="Q5" s="423"/>
+      <c r="R5" s="423"/>
+      <c r="S5" s="423"/>
+      <c r="T5" s="423"/>
+      <c r="U5" s="423"/>
+      <c r="V5" s="423"/>
+      <c r="W5" s="424"/>
       <c r="Y5" s="192"/>
       <c r="Z5" s="192"/>
       <c r="AA5" s="192"/>
       <c r="AB5" s="334"/>
     </row>
     <row r="6" spans="1:53" s="184" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="416" t="s">
+      <c r="B6" s="414" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="417"/>
-      <c r="D6" s="417"/>
-      <c r="E6" s="417"/>
-      <c r="F6" s="417"/>
-      <c r="G6" s="418"/>
-      <c r="I6" s="430" t="s">
+      <c r="C6" s="415"/>
+      <c r="D6" s="415"/>
+      <c r="E6" s="415"/>
+      <c r="F6" s="415"/>
+      <c r="G6" s="416"/>
+      <c r="I6" s="425" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="414" t="s">
+      <c r="J6" s="427" t="s">
         <v>409</v>
       </c>
-      <c r="K6" s="414" t="s">
+      <c r="K6" s="427" t="s">
         <v>408</v>
       </c>
-      <c r="L6" s="432" t="s">
+      <c r="L6" s="428" t="s">
         <v>215</v>
       </c>
-      <c r="M6" s="433"/>
-      <c r="N6" s="433"/>
-      <c r="O6" s="433"/>
-      <c r="P6" s="433"/>
-      <c r="Q6" s="434"/>
-      <c r="R6" s="419" t="s">
+      <c r="M6" s="429"/>
+      <c r="N6" s="429"/>
+      <c r="O6" s="429"/>
+      <c r="P6" s="429"/>
+      <c r="Q6" s="430"/>
+      <c r="R6" s="431" t="s">
         <v>216</v>
       </c>
-      <c r="S6" s="420"/>
-      <c r="T6" s="420"/>
-      <c r="U6" s="420"/>
-      <c r="V6" s="420"/>
-      <c r="W6" s="421"/>
+      <c r="S6" s="432"/>
+      <c r="T6" s="432"/>
+      <c r="U6" s="432"/>
+      <c r="V6" s="432"/>
+      <c r="W6" s="433"/>
       <c r="Y6" s="307"/>
       <c r="Z6" s="307"/>
       <c r="AA6" s="307"/>
@@ -24474,9 +24474,9 @@
         <f>SUM(C7:F7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="431"/>
-      <c r="J7" s="431"/>
-      <c r="K7" s="431"/>
+      <c r="I7" s="426"/>
+      <c r="J7" s="426"/>
+      <c r="K7" s="426"/>
       <c r="L7" s="186" t="s">
         <v>410</v>
       </c>
@@ -24680,14 +24680,14 @@
       <c r="AZ9" s="285"/>
     </row>
     <row r="10" spans="1:53" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.3">
-      <c r="B10" s="422" t="s">
+      <c r="B10" s="417" t="s">
         <v>237</v>
       </c>
-      <c r="C10" s="422"/>
-      <c r="D10" s="422"/>
-      <c r="E10" s="422"/>
-      <c r="F10" s="422"/>
-      <c r="G10" s="422"/>
+      <c r="C10" s="417"/>
+      <c r="D10" s="417"/>
+      <c r="E10" s="417"/>
+      <c r="F10" s="417"/>
+      <c r="G10" s="417"/>
       <c r="I10" s="244" t="s">
         <v>231</v>
       </c>
@@ -25171,13 +25171,13 @@
       <c r="B16" s="193" t="s">
         <v>234</v>
       </c>
-      <c r="C16" s="423" t="s">
+      <c r="C16" s="418" t="s">
         <v>235</v>
       </c>
-      <c r="D16" s="424"/>
-      <c r="E16" s="424"/>
-      <c r="F16" s="424"/>
-      <c r="G16" s="425"/>
+      <c r="D16" s="419"/>
+      <c r="E16" s="419"/>
+      <c r="F16" s="419"/>
+      <c r="G16" s="420"/>
       <c r="I16" s="244" t="s">
         <v>404</v>
       </c>
@@ -25293,59 +25293,59 @@
     </row>
     <row r="18" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.3"/>
     <row r="19" spans="2:58" s="192" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I19" s="426" t="s">
+      <c r="I19" s="421" t="s">
         <v>424</v>
       </c>
-      <c r="J19" s="426"/>
-      <c r="K19" s="426"/>
-      <c r="L19" s="426"/>
-      <c r="M19" s="426"/>
-      <c r="N19" s="426"/>
-      <c r="O19" s="426"/>
-      <c r="P19" s="426"/>
-      <c r="Q19" s="426"/>
-      <c r="R19" s="426"/>
-      <c r="S19" s="426"/>
-      <c r="T19" s="426"/>
-      <c r="U19" s="426"/>
+      <c r="J19" s="421"/>
+      <c r="K19" s="421"/>
+      <c r="L19" s="421"/>
+      <c r="M19" s="421"/>
+      <c r="N19" s="421"/>
+      <c r="O19" s="421"/>
+      <c r="P19" s="421"/>
+      <c r="Q19" s="421"/>
+      <c r="R19" s="421"/>
+      <c r="S19" s="421"/>
+      <c r="T19" s="421"/>
+      <c r="U19" s="421"/>
       <c r="Z19" s="250"/>
       <c r="AA19" s="250"/>
       <c r="AB19" s="250"/>
       <c r="AC19" s="250"/>
     </row>
     <row r="20" spans="2:58" s="192" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="414" t="s">
+      <c r="I20" s="427" t="s">
         <v>13</v>
       </c>
-      <c r="J20" s="414" t="s">
+      <c r="J20" s="427" t="s">
         <v>213</v>
       </c>
-      <c r="K20" s="414" t="s">
+      <c r="K20" s="427" t="s">
         <v>214</v>
       </c>
-      <c r="L20" s="416" t="s">
+      <c r="L20" s="414" t="s">
         <v>215</v>
       </c>
-      <c r="M20" s="417"/>
-      <c r="N20" s="417"/>
-      <c r="O20" s="417"/>
-      <c r="P20" s="418"/>
-      <c r="Q20" s="419" t="s">
+      <c r="M20" s="415"/>
+      <c r="N20" s="415"/>
+      <c r="O20" s="415"/>
+      <c r="P20" s="416"/>
+      <c r="Q20" s="431" t="s">
         <v>216</v>
       </c>
-      <c r="R20" s="420"/>
-      <c r="S20" s="420"/>
-      <c r="T20" s="420"/>
-      <c r="U20" s="421"/>
+      <c r="R20" s="432"/>
+      <c r="S20" s="432"/>
+      <c r="T20" s="432"/>
+      <c r="U20" s="433"/>
       <c r="Z20" s="254"/>
       <c r="AA20" s="254"/>
       <c r="AB20" s="254"/>
       <c r="AC20" s="254"/>
     </row>
     <row r="21" spans="2:58" s="192" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I21" s="415"/>
-      <c r="J21" s="415"/>
-      <c r="K21" s="415"/>
+      <c r="I21" s="434"/>
+      <c r="J21" s="434"/>
+      <c r="K21" s="434"/>
       <c r="L21" s="186" t="s">
         <v>218</v>
       </c>
@@ -26367,6 +26367,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:P20"/>
+    <mergeCell ref="Q20:U20"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="C16:G16"/>
@@ -26377,11 +26382,6 @@
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:Q6"/>
     <mergeCell ref="R6:W6"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:P20"/>
-    <mergeCell ref="Q20:U20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26714,16 +26714,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="436" t="e">
+      <c r="A1" s="435" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B1" s="436"/>
-      <c r="C1" s="436"/>
-      <c r="D1" s="436"/>
-      <c r="E1" s="436"/>
-      <c r="F1" s="436"/>
-      <c r="G1" s="436"/>
+      <c r="B1" s="435"/>
+      <c r="C1" s="435"/>
+      <c r="D1" s="435"/>
+      <c r="E1" s="435"/>
+      <c r="F1" s="435"/>
+      <c r="G1" s="435"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -26832,11 +26832,11 @@
         <v>40</v>
       </c>
       <c r="B10" s="112"/>
-      <c r="C10" s="435"/>
-      <c r="D10" s="435"/>
-      <c r="E10" s="435"/>
-      <c r="F10" s="435"/>
-      <c r="G10" s="435"/>
+      <c r="C10" s="436"/>
+      <c r="D10" s="436"/>
+      <c r="E10" s="436"/>
+      <c r="F10" s="436"/>
+      <c r="G10" s="436"/>
       <c r="N10" s="139"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
@@ -28099,12 +28099,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C6:G6"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="C9:G9"/>
@@ -28112,6 +28106,12 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N4" r:id="rId1" location="step-1-assign-parties-person-playing-and-strategies" xr:uid="{726B234F-7B54-4D33-A192-8F1604C6B04C}"/>

</xml_diff>

<commit_message>
Added figure to powerpoint
</commit_message>
<xml_diff>
--- a/LakeMeadWaterBankDivideInflow.xlsx
+++ b/LakeMeadWaterBankDivideInflow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anabelle/Documents/LakeMeadDivideInflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4B68E9-7D24-0141-AE80-D899B868549C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E77140F-F2EE-6F4E-801F-6E1CF3CFDBB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-22620" windowWidth="38400" windowHeight="23500" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe-Directions" sheetId="62" r:id="rId1"/>
@@ -2235,11 +2235,6 @@
       </rPr>
       <t>enter their choices to withdraw, conserve, and trade water in response to their available water, others choices, and the real-time discussion by participants.</t>
     </r>
-  </si>
-  <si>
-    <t>We are looking at scenarios within Reclamation’s different modeling methods and scenarios. There is broad agreement that Colorado River
-flows will be more volatile, declining, and have longer-lasting periods of low flow than current adjusted February 24-month study 10th and
- 50th percentile flows</t>
   </si>
   <si>
     <t>4)</t>
@@ -2371,6 +2366,11 @@
   </si>
   <si>
     <t xml:space="preserve">    1) To improve NOAA tools to communicate and manage risks of water shortages.</t>
+  </si>
+  <si>
+    <t>We are looking at scenarios within Reclamation’s different modeling methods and scenarios. There is broad agreement that Colorado River
+flows will be more volatile, declining, and have longer-lasting periods of low flow than current adjusted February 24-month study 10th and
+ 50th percentile flows.</t>
   </si>
 </sst>
 </file>
@@ -4199,97 +4199,13 @@
     <xf numFmtId="0" fontId="1" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -4328,6 +4244,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4346,10 +4265,91 @@
     <xf numFmtId="0" fontId="1" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4412,12 +4412,6 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4426,15 +4420,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4466,6 +4451,9 @@
     <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4475,11 +4463,23 @@
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -15996,20 +15996,20 @@
       <c r="R4" s="375"/>
     </row>
     <row r="5" spans="1:18" s="52" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="350" t="s">
-        <v>483</v>
-      </c>
-      <c r="B5" s="351"/>
-      <c r="C5" s="351"/>
-      <c r="D5" s="351"/>
-      <c r="E5" s="351"/>
-      <c r="F5" s="351"/>
-      <c r="G5" s="351"/>
-      <c r="H5" s="351"/>
-      <c r="I5" s="351"/>
-      <c r="J5" s="351"/>
-      <c r="K5" s="351"/>
-      <c r="L5" s="352"/>
+      <c r="A5" s="376" t="s">
+        <v>482</v>
+      </c>
+      <c r="B5" s="377"/>
+      <c r="C5" s="377"/>
+      <c r="D5" s="377"/>
+      <c r="E5" s="377"/>
+      <c r="F5" s="377"/>
+      <c r="G5" s="377"/>
+      <c r="H5" s="377"/>
+      <c r="I5" s="377"/>
+      <c r="J5" s="377"/>
+      <c r="K5" s="377"/>
+      <c r="L5" s="378"/>
       <c r="N5" s="110"/>
       <c r="O5" s="110"/>
       <c r="P5" s="110"/>
@@ -16017,20 +16017,20 @@
       <c r="R5" s="110"/>
     </row>
     <row r="6" spans="1:18" s="52" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="350" t="s">
-        <v>481</v>
-      </c>
-      <c r="B6" s="351"/>
-      <c r="C6" s="351"/>
-      <c r="D6" s="351"/>
-      <c r="E6" s="351"/>
-      <c r="F6" s="351"/>
-      <c r="G6" s="351"/>
-      <c r="H6" s="351"/>
-      <c r="I6" s="351"/>
-      <c r="J6" s="351"/>
-      <c r="K6" s="351"/>
-      <c r="L6" s="352"/>
+      <c r="A6" s="376" t="s">
+        <v>480</v>
+      </c>
+      <c r="B6" s="377"/>
+      <c r="C6" s="377"/>
+      <c r="D6" s="377"/>
+      <c r="E6" s="377"/>
+      <c r="F6" s="377"/>
+      <c r="G6" s="377"/>
+      <c r="H6" s="377"/>
+      <c r="I6" s="377"/>
+      <c r="J6" s="377"/>
+      <c r="K6" s="377"/>
+      <c r="L6" s="378"/>
       <c r="N6" s="110"/>
       <c r="O6" s="110"/>
       <c r="P6" s="110"/>
@@ -16038,20 +16038,20 @@
       <c r="R6" s="110"/>
     </row>
     <row r="7" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="350" t="s">
-        <v>482</v>
-      </c>
-      <c r="B7" s="351"/>
-      <c r="C7" s="351"/>
-      <c r="D7" s="351"/>
-      <c r="E7" s="351"/>
-      <c r="F7" s="351"/>
-      <c r="G7" s="351"/>
-      <c r="H7" s="351"/>
-      <c r="I7" s="351"/>
-      <c r="J7" s="351"/>
-      <c r="K7" s="351"/>
-      <c r="L7" s="352"/>
+      <c r="A7" s="376" t="s">
+        <v>481</v>
+      </c>
+      <c r="B7" s="377"/>
+      <c r="C7" s="377"/>
+      <c r="D7" s="377"/>
+      <c r="E7" s="377"/>
+      <c r="F7" s="377"/>
+      <c r="G7" s="377"/>
+      <c r="H7" s="377"/>
+      <c r="I7" s="377"/>
+      <c r="J7" s="377"/>
+      <c r="K7" s="377"/>
+      <c r="L7" s="378"/>
       <c r="N7" s="110"/>
       <c r="O7" s="110"/>
       <c r="P7" s="110"/>
@@ -16060,19 +16060,19 @@
     </row>
     <row r="8" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="214"/>
-      <c r="B8" s="351" t="s">
+      <c r="B8" s="377" t="s">
         <v>296</v>
       </c>
-      <c r="C8" s="351"/>
-      <c r="D8" s="351"/>
-      <c r="E8" s="351"/>
-      <c r="F8" s="351"/>
-      <c r="G8" s="351"/>
-      <c r="H8" s="351"/>
-      <c r="I8" s="351"/>
-      <c r="J8" s="351"/>
-      <c r="K8" s="351"/>
-      <c r="L8" s="352"/>
+      <c r="C8" s="377"/>
+      <c r="D8" s="377"/>
+      <c r="E8" s="377"/>
+      <c r="F8" s="377"/>
+      <c r="G8" s="377"/>
+      <c r="H8" s="377"/>
+      <c r="I8" s="377"/>
+      <c r="J8" s="377"/>
+      <c r="K8" s="377"/>
+      <c r="L8" s="378"/>
       <c r="N8" s="110"/>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
@@ -16081,19 +16081,19 @@
     </row>
     <row r="9" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="215"/>
-      <c r="B9" s="366" t="s">
+      <c r="B9" s="379" t="s">
         <v>297</v>
       </c>
-      <c r="C9" s="366"/>
-      <c r="D9" s="366"/>
-      <c r="E9" s="366"/>
-      <c r="F9" s="366"/>
-      <c r="G9" s="366"/>
-      <c r="H9" s="366"/>
-      <c r="I9" s="366"/>
-      <c r="J9" s="366"/>
-      <c r="K9" s="366"/>
-      <c r="L9" s="367"/>
+      <c r="C9" s="379"/>
+      <c r="D9" s="379"/>
+      <c r="E9" s="379"/>
+      <c r="F9" s="379"/>
+      <c r="G9" s="379"/>
+      <c r="H9" s="379"/>
+      <c r="I9" s="379"/>
+      <c r="J9" s="379"/>
+      <c r="K9" s="379"/>
+      <c r="L9" s="380"/>
       <c r="N9" s="110"/>
       <c r="O9" s="110"/>
       <c r="P9" s="110"/>
@@ -16115,81 +16115,81 @@
       <c r="L10" s="110"/>
     </row>
     <row r="11" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="368" t="s">
+      <c r="A11" s="381" t="s">
         <v>332</v>
       </c>
-      <c r="B11" s="369"/>
-      <c r="C11" s="369"/>
-      <c r="D11" s="369"/>
-      <c r="E11" s="369"/>
-      <c r="F11" s="369"/>
-      <c r="G11" s="369"/>
-      <c r="H11" s="369"/>
-      <c r="I11" s="369"/>
-      <c r="J11" s="369"/>
-      <c r="K11" s="369"/>
-      <c r="L11" s="370"/>
+      <c r="B11" s="382"/>
+      <c r="C11" s="382"/>
+      <c r="D11" s="382"/>
+      <c r="E11" s="382"/>
+      <c r="F11" s="382"/>
+      <c r="G11" s="382"/>
+      <c r="H11" s="382"/>
+      <c r="I11" s="382"/>
+      <c r="J11" s="382"/>
+      <c r="K11" s="382"/>
+      <c r="L11" s="383"/>
     </row>
     <row r="12" spans="1:18" s="57" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="344" t="s">
         <v>333</v>
       </c>
-      <c r="B12" s="360" t="s">
-        <v>475</v>
-      </c>
-      <c r="C12" s="360"/>
-      <c r="D12" s="360"/>
-      <c r="E12" s="360"/>
-      <c r="F12" s="360"/>
-      <c r="G12" s="360"/>
-      <c r="H12" s="360"/>
-      <c r="I12" s="360"/>
-      <c r="J12" s="360"/>
-      <c r="K12" s="360"/>
-      <c r="L12" s="361"/>
+      <c r="B12" s="345" t="s">
+        <v>483</v>
+      </c>
+      <c r="C12" s="345"/>
+      <c r="D12" s="345"/>
+      <c r="E12" s="345"/>
+      <c r="F12" s="345"/>
+      <c r="G12" s="345"/>
+      <c r="H12" s="345"/>
+      <c r="I12" s="345"/>
+      <c r="J12" s="345"/>
+      <c r="K12" s="345"/>
+      <c r="L12" s="384"/>
     </row>
     <row r="13" spans="1:18" s="57" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="344"/>
-      <c r="B13" s="360" t="e" vm="1">
+      <c r="B13" s="345" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C13" s="360"/>
-      <c r="D13" s="360"/>
-      <c r="E13" s="360"/>
-      <c r="F13" s="360"/>
-      <c r="G13" s="360"/>
-      <c r="H13" s="360"/>
-      <c r="I13" s="360"/>
-      <c r="J13" s="360"/>
-      <c r="K13" s="360"/>
+      <c r="C13" s="345"/>
+      <c r="D13" s="345"/>
+      <c r="E13" s="345"/>
+      <c r="F13" s="345"/>
+      <c r="G13" s="345"/>
+      <c r="H13" s="345"/>
+      <c r="I13" s="345"/>
+      <c r="J13" s="345"/>
+      <c r="K13" s="345"/>
       <c r="L13" s="342"/>
     </row>
     <row r="14" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="235" t="s">
         <v>334</v>
       </c>
-      <c r="B14" s="360" t="s">
+      <c r="B14" s="345" t="s">
         <v>336</v>
       </c>
-      <c r="C14" s="360"/>
-      <c r="D14" s="360"/>
-      <c r="E14" s="360"/>
-      <c r="F14" s="360"/>
-      <c r="G14" s="360"/>
-      <c r="H14" s="360"/>
-      <c r="I14" s="360"/>
-      <c r="J14" s="360"/>
-      <c r="K14" s="360"/>
-      <c r="L14" s="361"/>
+      <c r="C14" s="345"/>
+      <c r="D14" s="345"/>
+      <c r="E14" s="345"/>
+      <c r="F14" s="345"/>
+      <c r="G14" s="345"/>
+      <c r="H14" s="345"/>
+      <c r="I14" s="345"/>
+      <c r="J14" s="345"/>
+      <c r="K14" s="345"/>
+      <c r="L14" s="384"/>
     </row>
     <row r="15" spans="1:18" s="57" customFormat="1" ht="176" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="227"/>
-      <c r="B15" s="362"/>
-      <c r="C15" s="362"/>
-      <c r="D15" s="362"/>
-      <c r="E15" s="362"/>
-      <c r="F15" s="362"/>
-      <c r="G15" s="362"/>
+      <c r="B15" s="346"/>
+      <c r="C15" s="346"/>
+      <c r="D15" s="346"/>
+      <c r="E15" s="346"/>
+      <c r="F15" s="346"/>
+      <c r="G15" s="346"/>
       <c r="H15" s="233"/>
       <c r="I15" s="233"/>
       <c r="J15" s="233"/>
@@ -16200,75 +16200,75 @@
       <c r="A16" s="235" t="s">
         <v>335</v>
       </c>
-      <c r="B16" s="360" t="s">
+      <c r="B16" s="345" t="s">
         <v>337</v>
       </c>
-      <c r="C16" s="360"/>
-      <c r="D16" s="360"/>
-      <c r="E16" s="360"/>
-      <c r="F16" s="360"/>
-      <c r="G16" s="360"/>
-      <c r="H16" s="360"/>
-      <c r="I16" s="360"/>
-      <c r="J16" s="360"/>
-      <c r="K16" s="360"/>
-      <c r="L16" s="361"/>
+      <c r="C16" s="345"/>
+      <c r="D16" s="345"/>
+      <c r="E16" s="345"/>
+      <c r="F16" s="345"/>
+      <c r="G16" s="345"/>
+      <c r="H16" s="345"/>
+      <c r="I16" s="345"/>
+      <c r="J16" s="345"/>
+      <c r="K16" s="345"/>
+      <c r="L16" s="384"/>
     </row>
     <row r="17" spans="1:14" s="57" customFormat="1" ht="90.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="227"/>
-      <c r="B17" s="362"/>
-      <c r="C17" s="362"/>
-      <c r="D17" s="362"/>
-      <c r="E17" s="362"/>
-      <c r="F17" s="362"/>
-      <c r="G17" s="362"/>
-      <c r="H17" s="362"/>
-      <c r="I17" s="362"/>
-      <c r="J17" s="362"/>
-      <c r="K17" s="362"/>
-      <c r="L17" s="363"/>
+      <c r="B17" s="346"/>
+      <c r="C17" s="346"/>
+      <c r="D17" s="346"/>
+      <c r="E17" s="346"/>
+      <c r="F17" s="346"/>
+      <c r="G17" s="346"/>
+      <c r="H17" s="346"/>
+      <c r="I17" s="346"/>
+      <c r="J17" s="346"/>
+      <c r="K17" s="346"/>
+      <c r="L17" s="395"/>
     </row>
     <row r="18" spans="1:14" s="56" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="235" t="s">
-        <v>476</v>
-      </c>
-      <c r="B18" s="360" t="s">
+        <v>475</v>
+      </c>
+      <c r="B18" s="345" t="s">
         <v>463</v>
       </c>
-      <c r="C18" s="360"/>
-      <c r="D18" s="360"/>
-      <c r="E18" s="360"/>
-      <c r="F18" s="360"/>
-      <c r="G18" s="360"/>
-      <c r="H18" s="360"/>
-      <c r="I18" s="360"/>
-      <c r="J18" s="360"/>
-      <c r="K18" s="360"/>
-      <c r="L18" s="361"/>
+      <c r="C18" s="345"/>
+      <c r="D18" s="345"/>
+      <c r="E18" s="345"/>
+      <c r="F18" s="345"/>
+      <c r="G18" s="345"/>
+      <c r="H18" s="345"/>
+      <c r="I18" s="345"/>
+      <c r="J18" s="345"/>
+      <c r="K18" s="345"/>
+      <c r="L18" s="384"/>
     </row>
     <row r="19" spans="1:14" s="57" customFormat="1" ht="269" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="227"/>
-      <c r="B19" s="362" t="e" vm="2">
+      <c r="B19" s="346" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="C19" s="362"/>
-      <c r="D19" s="362"/>
-      <c r="E19" s="362"/>
-      <c r="F19" s="362"/>
-      <c r="G19" s="362"/>
-      <c r="H19" s="362"/>
-      <c r="I19" s="362"/>
-      <c r="J19" s="362"/>
-      <c r="K19" s="362"/>
+      <c r="C19" s="346"/>
+      <c r="D19" s="346"/>
+      <c r="E19" s="346"/>
+      <c r="F19" s="346"/>
+      <c r="G19" s="346"/>
+      <c r="H19" s="346"/>
+      <c r="I19" s="346"/>
+      <c r="J19" s="346"/>
+      <c r="K19" s="346"/>
       <c r="L19" s="234"/>
     </row>
     <row r="20" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="394" t="s">
+      <c r="A20" s="369" t="s">
         <v>341</v>
       </c>
-      <c r="B20" s="395"/>
-      <c r="C20" s="395"/>
-      <c r="D20" s="395"/>
+      <c r="B20" s="370"/>
+      <c r="C20" s="370"/>
+      <c r="D20" s="370"/>
       <c r="E20" s="232" t="s">
         <v>342</v>
       </c>
@@ -16295,84 +16295,84 @@
       <c r="L21" s="110"/>
     </row>
     <row r="22" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="381" t="s">
+      <c r="A22" s="353" t="s">
         <v>165</v>
       </c>
-      <c r="B22" s="382"/>
-      <c r="C22" s="382"/>
-      <c r="D22" s="382"/>
-      <c r="E22" s="382"/>
-      <c r="F22" s="382"/>
-      <c r="G22" s="382"/>
-      <c r="H22" s="382"/>
-      <c r="I22" s="382"/>
-      <c r="J22" s="382"/>
-      <c r="K22" s="382"/>
-      <c r="L22" s="383"/>
+      <c r="B22" s="354"/>
+      <c r="C22" s="354"/>
+      <c r="D22" s="354"/>
+      <c r="E22" s="354"/>
+      <c r="F22" s="354"/>
+      <c r="G22" s="354"/>
+      <c r="H22" s="354"/>
+      <c r="I22" s="354"/>
+      <c r="J22" s="354"/>
+      <c r="K22" s="354"/>
+      <c r="L22" s="355"/>
     </row>
     <row r="23" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="384" t="s">
+      <c r="A23" s="356" t="s">
         <v>280</v>
       </c>
-      <c r="B23" s="385"/>
-      <c r="C23" s="385"/>
-      <c r="D23" s="385"/>
-      <c r="E23" s="385"/>
-      <c r="F23" s="385"/>
-      <c r="G23" s="385"/>
-      <c r="H23" s="385"/>
-      <c r="I23" s="385"/>
-      <c r="J23" s="385"/>
-      <c r="K23" s="385"/>
-      <c r="L23" s="386"/>
+      <c r="B23" s="357"/>
+      <c r="C23" s="357"/>
+      <c r="D23" s="357"/>
+      <c r="E23" s="357"/>
+      <c r="F23" s="357"/>
+      <c r="G23" s="357"/>
+      <c r="H23" s="357"/>
+      <c r="I23" s="357"/>
+      <c r="J23" s="357"/>
+      <c r="K23" s="357"/>
+      <c r="L23" s="358"/>
     </row>
     <row r="24" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="387" t="s">
+      <c r="A24" s="359" t="s">
         <v>281</v>
       </c>
-      <c r="B24" s="345"/>
-      <c r="C24" s="345"/>
-      <c r="D24" s="345"/>
-      <c r="E24" s="345"/>
-      <c r="F24" s="345"/>
-      <c r="G24" s="345"/>
-      <c r="H24" s="345"/>
-      <c r="I24" s="345"/>
-      <c r="J24" s="345"/>
-      <c r="K24" s="345"/>
-      <c r="L24" s="346"/>
+      <c r="B24" s="347"/>
+      <c r="C24" s="347"/>
+      <c r="D24" s="347"/>
+      <c r="E24" s="347"/>
+      <c r="F24" s="347"/>
+      <c r="G24" s="347"/>
+      <c r="H24" s="347"/>
+      <c r="I24" s="347"/>
+      <c r="J24" s="347"/>
+      <c r="K24" s="347"/>
+      <c r="L24" s="360"/>
     </row>
     <row r="25" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="387" t="s">
+      <c r="A25" s="359" t="s">
         <v>166</v>
       </c>
-      <c r="B25" s="345"/>
-      <c r="C25" s="345"/>
-      <c r="D25" s="345"/>
-      <c r="E25" s="345"/>
-      <c r="F25" s="345"/>
-      <c r="G25" s="345"/>
-      <c r="H25" s="345"/>
-      <c r="I25" s="345"/>
-      <c r="J25" s="345"/>
-      <c r="K25" s="345"/>
-      <c r="L25" s="346"/>
+      <c r="B25" s="347"/>
+      <c r="C25" s="347"/>
+      <c r="D25" s="347"/>
+      <c r="E25" s="347"/>
+      <c r="F25" s="347"/>
+      <c r="G25" s="347"/>
+      <c r="H25" s="347"/>
+      <c r="I25" s="347"/>
+      <c r="J25" s="347"/>
+      <c r="K25" s="347"/>
+      <c r="L25" s="360"/>
     </row>
     <row r="26" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="388" t="s">
+      <c r="A26" s="361" t="s">
         <v>282</v>
       </c>
-      <c r="B26" s="389"/>
-      <c r="C26" s="389"/>
-      <c r="D26" s="389"/>
-      <c r="E26" s="389"/>
-      <c r="F26" s="389"/>
-      <c r="G26" s="389"/>
-      <c r="H26" s="389"/>
-      <c r="I26" s="389"/>
-      <c r="J26" s="389"/>
-      <c r="K26" s="389"/>
-      <c r="L26" s="390"/>
+      <c r="B26" s="362"/>
+      <c r="C26" s="362"/>
+      <c r="D26" s="362"/>
+      <c r="E26" s="362"/>
+      <c r="F26" s="362"/>
+      <c r="G26" s="362"/>
+      <c r="H26" s="362"/>
+      <c r="I26" s="362"/>
+      <c r="J26" s="362"/>
+      <c r="K26" s="362"/>
+      <c r="L26" s="363"/>
     </row>
     <row r="27" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="110"/>
@@ -16389,332 +16389,332 @@
       <c r="L27" s="110"/>
     </row>
     <row r="28" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="391" t="s">
+      <c r="A28" s="364" t="s">
         <v>279</v>
       </c>
-      <c r="B28" s="392"/>
-      <c r="C28" s="392"/>
-      <c r="D28" s="392"/>
-      <c r="E28" s="392"/>
-      <c r="F28" s="392"/>
-      <c r="G28" s="392"/>
-      <c r="H28" s="392"/>
-      <c r="I28" s="392"/>
-      <c r="J28" s="392"/>
-      <c r="K28" s="392"/>
-      <c r="L28" s="393"/>
+      <c r="B28" s="365"/>
+      <c r="C28" s="365"/>
+      <c r="D28" s="365"/>
+      <c r="E28" s="365"/>
+      <c r="F28" s="365"/>
+      <c r="G28" s="365"/>
+      <c r="H28" s="365"/>
+      <c r="I28" s="365"/>
+      <c r="J28" s="365"/>
+      <c r="K28" s="365"/>
+      <c r="L28" s="366"/>
       <c r="N28" s="1"/>
     </row>
     <row r="29" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="378" t="s">
+      <c r="A29" s="350" t="s">
         <v>175</v>
       </c>
-      <c r="B29" s="379"/>
-      <c r="C29" s="379"/>
-      <c r="D29" s="379"/>
-      <c r="E29" s="379"/>
-      <c r="F29" s="379"/>
-      <c r="G29" s="379"/>
-      <c r="H29" s="379"/>
-      <c r="I29" s="379"/>
-      <c r="J29" s="379"/>
-      <c r="K29" s="379"/>
-      <c r="L29" s="380"/>
+      <c r="B29" s="351"/>
+      <c r="C29" s="351"/>
+      <c r="D29" s="351"/>
+      <c r="E29" s="351"/>
+      <c r="F29" s="351"/>
+      <c r="G29" s="351"/>
+      <c r="H29" s="351"/>
+      <c r="I29" s="351"/>
+      <c r="J29" s="351"/>
+      <c r="K29" s="351"/>
+      <c r="L29" s="352"/>
       <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="209">
         <v>1</v>
       </c>
-      <c r="B30" s="353" t="s">
+      <c r="B30" s="367" t="s">
         <v>174</v>
       </c>
-      <c r="C30" s="353"/>
-      <c r="D30" s="353"/>
-      <c r="E30" s="353"/>
-      <c r="F30" s="353"/>
-      <c r="G30" s="353"/>
-      <c r="H30" s="353"/>
-      <c r="I30" s="353"/>
-      <c r="J30" s="353"/>
-      <c r="K30" s="353"/>
-      <c r="L30" s="354"/>
+      <c r="C30" s="367"/>
+      <c r="D30" s="367"/>
+      <c r="E30" s="367"/>
+      <c r="F30" s="367"/>
+      <c r="G30" s="367"/>
+      <c r="H30" s="367"/>
+      <c r="I30" s="367"/>
+      <c r="J30" s="367"/>
+      <c r="K30" s="367"/>
+      <c r="L30" s="368"/>
     </row>
     <row r="31" spans="1:14" s="57" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="209">
         <v>2</v>
       </c>
-      <c r="B31" s="353" t="s">
+      <c r="B31" s="367" t="s">
         <v>275</v>
       </c>
-      <c r="C31" s="353"/>
-      <c r="D31" s="353"/>
-      <c r="E31" s="353"/>
-      <c r="F31" s="353"/>
-      <c r="G31" s="353"/>
-      <c r="H31" s="353"/>
-      <c r="I31" s="353"/>
-      <c r="J31" s="353"/>
-      <c r="K31" s="353"/>
-      <c r="L31" s="354"/>
+      <c r="C31" s="367"/>
+      <c r="D31" s="367"/>
+      <c r="E31" s="367"/>
+      <c r="F31" s="367"/>
+      <c r="G31" s="367"/>
+      <c r="H31" s="367"/>
+      <c r="I31" s="367"/>
+      <c r="J31" s="367"/>
+      <c r="K31" s="367"/>
+      <c r="L31" s="368"/>
       <c r="N31" s="104"/>
     </row>
     <row r="32" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="209">
         <v>3</v>
       </c>
-      <c r="B32" s="353" t="s">
+      <c r="B32" s="367" t="s">
         <v>167</v>
       </c>
-      <c r="C32" s="353"/>
-      <c r="D32" s="353"/>
-      <c r="E32" s="353"/>
-      <c r="F32" s="353"/>
-      <c r="G32" s="353"/>
-      <c r="H32" s="353"/>
-      <c r="I32" s="353"/>
-      <c r="J32" s="353"/>
-      <c r="K32" s="353"/>
-      <c r="L32" s="354"/>
+      <c r="C32" s="367"/>
+      <c r="D32" s="367"/>
+      <c r="E32" s="367"/>
+      <c r="F32" s="367"/>
+      <c r="G32" s="367"/>
+      <c r="H32" s="367"/>
+      <c r="I32" s="367"/>
+      <c r="J32" s="367"/>
+      <c r="K32" s="367"/>
+      <c r="L32" s="368"/>
       <c r="N32" s="104"/>
     </row>
     <row r="33" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="209">
         <v>4</v>
       </c>
-      <c r="B33" s="353" t="s">
+      <c r="B33" s="367" t="s">
         <v>283</v>
       </c>
-      <c r="C33" s="353"/>
-      <c r="D33" s="353"/>
-      <c r="E33" s="353"/>
-      <c r="F33" s="353"/>
-      <c r="G33" s="353"/>
-      <c r="H33" s="353"/>
-      <c r="I33" s="353"/>
-      <c r="J33" s="353"/>
-      <c r="K33" s="353"/>
-      <c r="L33" s="354"/>
+      <c r="C33" s="367"/>
+      <c r="D33" s="367"/>
+      <c r="E33" s="367"/>
+      <c r="F33" s="367"/>
+      <c r="G33" s="367"/>
+      <c r="H33" s="367"/>
+      <c r="I33" s="367"/>
+      <c r="J33" s="367"/>
+      <c r="K33" s="367"/>
+      <c r="L33" s="368"/>
       <c r="N33" s="104"/>
     </row>
     <row r="34" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="209">
         <v>5</v>
       </c>
-      <c r="B34" s="353" t="s">
+      <c r="B34" s="367" t="s">
         <v>168</v>
       </c>
-      <c r="C34" s="353"/>
-      <c r="D34" s="353"/>
-      <c r="E34" s="353"/>
-      <c r="F34" s="353"/>
-      <c r="G34" s="353"/>
-      <c r="H34" s="353"/>
-      <c r="I34" s="353"/>
-      <c r="J34" s="353"/>
-      <c r="K34" s="353"/>
-      <c r="L34" s="354"/>
+      <c r="C34" s="367"/>
+      <c r="D34" s="367"/>
+      <c r="E34" s="367"/>
+      <c r="F34" s="367"/>
+      <c r="G34" s="367"/>
+      <c r="H34" s="367"/>
+      <c r="I34" s="367"/>
+      <c r="J34" s="367"/>
+      <c r="K34" s="367"/>
+      <c r="L34" s="368"/>
       <c r="N34" s="104"/>
     </row>
     <row r="35" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="209"/>
-      <c r="B35" s="353" t="s">
+      <c r="B35" s="367" t="s">
         <v>169</v>
       </c>
-      <c r="C35" s="353"/>
-      <c r="D35" s="353"/>
-      <c r="E35" s="353"/>
-      <c r="F35" s="353"/>
-      <c r="G35" s="353"/>
-      <c r="H35" s="353"/>
-      <c r="I35" s="353"/>
-      <c r="J35" s="353"/>
-      <c r="K35" s="353"/>
-      <c r="L35" s="354"/>
+      <c r="C35" s="367"/>
+      <c r="D35" s="367"/>
+      <c r="E35" s="367"/>
+      <c r="F35" s="367"/>
+      <c r="G35" s="367"/>
+      <c r="H35" s="367"/>
+      <c r="I35" s="367"/>
+      <c r="J35" s="367"/>
+      <c r="K35" s="367"/>
+      <c r="L35" s="368"/>
       <c r="N35" s="104"/>
     </row>
     <row r="36" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="209"/>
-      <c r="B36" s="353" t="s">
+      <c r="B36" s="367" t="s">
         <v>170</v>
       </c>
-      <c r="C36" s="353"/>
-      <c r="D36" s="353"/>
-      <c r="E36" s="353"/>
-      <c r="F36" s="353"/>
-      <c r="G36" s="353"/>
-      <c r="H36" s="353"/>
-      <c r="I36" s="353"/>
-      <c r="J36" s="353"/>
-      <c r="K36" s="353"/>
-      <c r="L36" s="354"/>
+      <c r="C36" s="367"/>
+      <c r="D36" s="367"/>
+      <c r="E36" s="367"/>
+      <c r="F36" s="367"/>
+      <c r="G36" s="367"/>
+      <c r="H36" s="367"/>
+      <c r="I36" s="367"/>
+      <c r="J36" s="367"/>
+      <c r="K36" s="367"/>
+      <c r="L36" s="368"/>
       <c r="N36" s="104"/>
     </row>
     <row r="37" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="347" t="s">
+      <c r="A37" s="387" t="s">
         <v>176</v>
       </c>
-      <c r="B37" s="348"/>
-      <c r="C37" s="348"/>
-      <c r="D37" s="348"/>
-      <c r="E37" s="348"/>
-      <c r="F37" s="348"/>
-      <c r="G37" s="348"/>
-      <c r="H37" s="348"/>
-      <c r="I37" s="348"/>
-      <c r="J37" s="348"/>
-      <c r="K37" s="348"/>
-      <c r="L37" s="349"/>
+      <c r="B37" s="388"/>
+      <c r="C37" s="388"/>
+      <c r="D37" s="388"/>
+      <c r="E37" s="388"/>
+      <c r="F37" s="388"/>
+      <c r="G37" s="388"/>
+      <c r="H37" s="388"/>
+      <c r="I37" s="388"/>
+      <c r="J37" s="388"/>
+      <c r="K37" s="388"/>
+      <c r="L37" s="389"/>
       <c r="N37" s="104"/>
     </row>
     <row r="38" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="209">
         <v>1</v>
       </c>
-      <c r="B38" s="353" t="s">
+      <c r="B38" s="367" t="s">
         <v>171</v>
       </c>
-      <c r="C38" s="353"/>
-      <c r="D38" s="353"/>
-      <c r="E38" s="353"/>
-      <c r="F38" s="353"/>
-      <c r="G38" s="353"/>
-      <c r="H38" s="353"/>
-      <c r="I38" s="353"/>
-      <c r="J38" s="353"/>
-      <c r="K38" s="353"/>
-      <c r="L38" s="354"/>
+      <c r="C38" s="367"/>
+      <c r="D38" s="367"/>
+      <c r="E38" s="367"/>
+      <c r="F38" s="367"/>
+      <c r="G38" s="367"/>
+      <c r="H38" s="367"/>
+      <c r="I38" s="367"/>
+      <c r="J38" s="367"/>
+      <c r="K38" s="367"/>
+      <c r="L38" s="368"/>
       <c r="N38" s="104"/>
     </row>
     <row r="39" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="209"/>
-      <c r="B39" s="364" t="s">
+      <c r="B39" s="385" t="s">
         <v>424</v>
       </c>
-      <c r="C39" s="364"/>
-      <c r="D39" s="364"/>
-      <c r="E39" s="364"/>
-      <c r="F39" s="364"/>
-      <c r="G39" s="364"/>
-      <c r="H39" s="364"/>
-      <c r="I39" s="364"/>
-      <c r="J39" s="364"/>
-      <c r="K39" s="364"/>
-      <c r="L39" s="365"/>
+      <c r="C39" s="385"/>
+      <c r="D39" s="385"/>
+      <c r="E39" s="385"/>
+      <c r="F39" s="385"/>
+      <c r="G39" s="385"/>
+      <c r="H39" s="385"/>
+      <c r="I39" s="385"/>
+      <c r="J39" s="385"/>
+      <c r="K39" s="385"/>
+      <c r="L39" s="386"/>
       <c r="N39" s="104"/>
     </row>
     <row r="40" spans="1:14" s="57" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="209">
         <v>2</v>
       </c>
-      <c r="B40" s="353" t="s">
+      <c r="B40" s="367" t="s">
         <v>278</v>
       </c>
-      <c r="C40" s="353"/>
-      <c r="D40" s="353"/>
-      <c r="E40" s="353"/>
-      <c r="F40" s="353"/>
-      <c r="G40" s="353"/>
-      <c r="H40" s="353"/>
-      <c r="I40" s="353"/>
-      <c r="J40" s="353"/>
-      <c r="K40" s="353"/>
-      <c r="L40" s="354"/>
+      <c r="C40" s="367"/>
+      <c r="D40" s="367"/>
+      <c r="E40" s="367"/>
+      <c r="F40" s="367"/>
+      <c r="G40" s="367"/>
+      <c r="H40" s="367"/>
+      <c r="I40" s="367"/>
+      <c r="J40" s="367"/>
+      <c r="K40" s="367"/>
+      <c r="L40" s="368"/>
       <c r="N40" s="104"/>
     </row>
     <row r="41" spans="1:14" s="57" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="209">
         <v>3</v>
       </c>
-      <c r="B41" s="353" t="s">
+      <c r="B41" s="367" t="s">
         <v>473</v>
       </c>
-      <c r="C41" s="353"/>
-      <c r="D41" s="353"/>
-      <c r="E41" s="353"/>
-      <c r="F41" s="353"/>
-      <c r="G41" s="353"/>
-      <c r="H41" s="353"/>
-      <c r="I41" s="353"/>
-      <c r="J41" s="353"/>
-      <c r="K41" s="353"/>
-      <c r="L41" s="354"/>
+      <c r="C41" s="367"/>
+      <c r="D41" s="367"/>
+      <c r="E41" s="367"/>
+      <c r="F41" s="367"/>
+      <c r="G41" s="367"/>
+      <c r="H41" s="367"/>
+      <c r="I41" s="367"/>
+      <c r="J41" s="367"/>
+      <c r="K41" s="367"/>
+      <c r="L41" s="368"/>
       <c r="N41" s="104"/>
     </row>
     <row r="42" spans="1:14" s="57" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="209">
         <v>4</v>
       </c>
-      <c r="B42" s="353" t="s">
+      <c r="B42" s="367" t="s">
         <v>284</v>
       </c>
-      <c r="C42" s="353"/>
-      <c r="D42" s="353"/>
-      <c r="E42" s="353"/>
-      <c r="F42" s="353"/>
-      <c r="G42" s="353"/>
-      <c r="H42" s="353"/>
-      <c r="I42" s="353"/>
-      <c r="J42" s="353"/>
-      <c r="K42" s="353"/>
-      <c r="L42" s="354"/>
+      <c r="C42" s="367"/>
+      <c r="D42" s="367"/>
+      <c r="E42" s="367"/>
+      <c r="F42" s="367"/>
+      <c r="G42" s="367"/>
+      <c r="H42" s="367"/>
+      <c r="I42" s="367"/>
+      <c r="J42" s="367"/>
+      <c r="K42" s="367"/>
+      <c r="L42" s="368"/>
       <c r="N42" s="104"/>
     </row>
     <row r="43" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="209">
         <v>5</v>
       </c>
-      <c r="B43" s="364" t="s">
+      <c r="B43" s="385" t="s">
         <v>269</v>
       </c>
-      <c r="C43" s="364"/>
-      <c r="D43" s="364"/>
-      <c r="E43" s="364"/>
-      <c r="F43" s="364"/>
-      <c r="G43" s="364"/>
-      <c r="H43" s="364"/>
-      <c r="I43" s="364"/>
-      <c r="J43" s="364"/>
-      <c r="K43" s="364"/>
-      <c r="L43" s="365"/>
+      <c r="C43" s="385"/>
+      <c r="D43" s="385"/>
+      <c r="E43" s="385"/>
+      <c r="F43" s="385"/>
+      <c r="G43" s="385"/>
+      <c r="H43" s="385"/>
+      <c r="I43" s="385"/>
+      <c r="J43" s="385"/>
+      <c r="K43" s="385"/>
+      <c r="L43" s="386"/>
       <c r="N43" s="104"/>
     </row>
     <row r="44" spans="1:14" s="57" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="209">
         <v>6</v>
       </c>
-      <c r="B44" s="364" t="s">
+      <c r="B44" s="385" t="s">
         <v>474</v>
       </c>
-      <c r="C44" s="364"/>
-      <c r="D44" s="364"/>
-      <c r="E44" s="364"/>
-      <c r="F44" s="364"/>
-      <c r="G44" s="364"/>
-      <c r="H44" s="364"/>
-      <c r="I44" s="364"/>
-      <c r="J44" s="364"/>
-      <c r="K44" s="364"/>
-      <c r="L44" s="365"/>
+      <c r="C44" s="385"/>
+      <c r="D44" s="385"/>
+      <c r="E44" s="385"/>
+      <c r="F44" s="385"/>
+      <c r="G44" s="385"/>
+      <c r="H44" s="385"/>
+      <c r="I44" s="385"/>
+      <c r="J44" s="385"/>
+      <c r="K44" s="385"/>
+      <c r="L44" s="386"/>
       <c r="N44" s="104"/>
     </row>
     <row r="45" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="209">
         <v>7</v>
       </c>
-      <c r="B45" s="353" t="s">
+      <c r="B45" s="367" t="s">
         <v>270</v>
       </c>
-      <c r="C45" s="353"/>
-      <c r="D45" s="353"/>
-      <c r="E45" s="353"/>
-      <c r="F45" s="353"/>
-      <c r="G45" s="353"/>
-      <c r="H45" s="353"/>
-      <c r="I45" s="353"/>
-      <c r="J45" s="353"/>
-      <c r="K45" s="353"/>
-      <c r="L45" s="354"/>
+      <c r="C45" s="367"/>
+      <c r="D45" s="367"/>
+      <c r="E45" s="367"/>
+      <c r="F45" s="367"/>
+      <c r="G45" s="367"/>
+      <c r="H45" s="367"/>
+      <c r="I45" s="367"/>
+      <c r="J45" s="367"/>
+      <c r="K45" s="367"/>
+      <c r="L45" s="368"/>
     </row>
     <row r="46" spans="1:14" s="57" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="209"/>
@@ -16731,56 +16731,56 @@
       <c r="L46" s="211"/>
     </row>
     <row r="47" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="347" t="s">
+      <c r="A47" s="387" t="s">
         <v>273</v>
       </c>
-      <c r="B47" s="348"/>
-      <c r="C47" s="348"/>
-      <c r="D47" s="348"/>
-      <c r="E47" s="348"/>
-      <c r="F47" s="348"/>
-      <c r="G47" s="348"/>
-      <c r="H47" s="348"/>
-      <c r="I47" s="348"/>
-      <c r="J47" s="348"/>
-      <c r="K47" s="348"/>
-      <c r="L47" s="349"/>
+      <c r="B47" s="388"/>
+      <c r="C47" s="388"/>
+      <c r="D47" s="388"/>
+      <c r="E47" s="388"/>
+      <c r="F47" s="388"/>
+      <c r="G47" s="388"/>
+      <c r="H47" s="388"/>
+      <c r="I47" s="388"/>
+      <c r="J47" s="388"/>
+      <c r="K47" s="388"/>
+      <c r="L47" s="389"/>
     </row>
     <row r="48" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="212" t="s">
         <v>271</v>
       </c>
-      <c r="B48" s="353" t="s">
+      <c r="B48" s="367" t="s">
         <v>172</v>
       </c>
-      <c r="C48" s="353"/>
-      <c r="D48" s="353"/>
-      <c r="E48" s="353"/>
-      <c r="F48" s="353"/>
-      <c r="G48" s="353"/>
-      <c r="H48" s="353"/>
-      <c r="I48" s="353"/>
-      <c r="J48" s="353"/>
-      <c r="K48" s="353"/>
-      <c r="L48" s="354"/>
+      <c r="C48" s="367"/>
+      <c r="D48" s="367"/>
+      <c r="E48" s="367"/>
+      <c r="F48" s="367"/>
+      <c r="G48" s="367"/>
+      <c r="H48" s="367"/>
+      <c r="I48" s="367"/>
+      <c r="J48" s="367"/>
+      <c r="K48" s="367"/>
+      <c r="L48" s="368"/>
     </row>
     <row r="49" spans="1:12" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="213" t="s">
         <v>272</v>
       </c>
-      <c r="B49" s="355" t="s">
+      <c r="B49" s="390" t="s">
         <v>274</v>
       </c>
-      <c r="C49" s="355"/>
-      <c r="D49" s="355"/>
-      <c r="E49" s="355"/>
-      <c r="F49" s="355"/>
-      <c r="G49" s="355"/>
-      <c r="H49" s="355"/>
-      <c r="I49" s="355"/>
-      <c r="J49" s="355"/>
-      <c r="K49" s="355"/>
-      <c r="L49" s="356"/>
+      <c r="C49" s="390"/>
+      <c r="D49" s="390"/>
+      <c r="E49" s="390"/>
+      <c r="F49" s="390"/>
+      <c r="G49" s="390"/>
+      <c r="H49" s="390"/>
+      <c r="I49" s="390"/>
+      <c r="J49" s="390"/>
+      <c r="K49" s="390"/>
+      <c r="L49" s="391"/>
     </row>
     <row r="50" spans="1:12" s="57" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="157"/>
@@ -16797,20 +16797,20 @@
       <c r="L50" s="110"/>
     </row>
     <row r="51" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="357" t="s">
+      <c r="A51" s="392" t="s">
         <v>200</v>
       </c>
-      <c r="B51" s="358"/>
-      <c r="C51" s="358"/>
-      <c r="D51" s="358"/>
-      <c r="E51" s="358"/>
-      <c r="F51" s="358"/>
-      <c r="G51" s="358"/>
-      <c r="H51" s="358"/>
-      <c r="I51" s="358"/>
-      <c r="J51" s="358"/>
-      <c r="K51" s="358"/>
-      <c r="L51" s="359"/>
+      <c r="B51" s="393"/>
+      <c r="C51" s="393"/>
+      <c r="D51" s="393"/>
+      <c r="E51" s="393"/>
+      <c r="F51" s="393"/>
+      <c r="G51" s="393"/>
+      <c r="H51" s="393"/>
+      <c r="I51" s="393"/>
+      <c r="J51" s="393"/>
+      <c r="K51" s="393"/>
+      <c r="L51" s="394"/>
     </row>
     <row r="52" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="216" t="s">
@@ -16898,126 +16898,126 @@
       <c r="B57" s="165" t="s">
         <v>24</v>
       </c>
-      <c r="C57" s="345" t="s">
+      <c r="C57" s="347" t="s">
         <v>262</v>
       </c>
-      <c r="D57" s="345"/>
-      <c r="E57" s="345"/>
-      <c r="F57" s="345"/>
-      <c r="G57" s="345"/>
-      <c r="H57" s="345"/>
-      <c r="I57" s="345"/>
-      <c r="J57" s="345"/>
-      <c r="K57" s="345"/>
-      <c r="L57" s="346"/>
+      <c r="D57" s="347"/>
+      <c r="E57" s="347"/>
+      <c r="F57" s="347"/>
+      <c r="G57" s="347"/>
+      <c r="H57" s="347"/>
+      <c r="I57" s="347"/>
+      <c r="J57" s="347"/>
+      <c r="K57" s="347"/>
+      <c r="L57" s="360"/>
     </row>
     <row r="58" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="164"/>
       <c r="B58" s="165" t="s">
         <v>263</v>
       </c>
-      <c r="C58" s="345" t="s">
+      <c r="C58" s="347" t="s">
         <v>264</v>
       </c>
-      <c r="D58" s="345"/>
-      <c r="E58" s="345"/>
-      <c r="F58" s="345"/>
-      <c r="G58" s="345"/>
-      <c r="H58" s="345"/>
-      <c r="I58" s="345"/>
-      <c r="J58" s="345"/>
-      <c r="K58" s="345"/>
-      <c r="L58" s="346"/>
+      <c r="D58" s="347"/>
+      <c r="E58" s="347"/>
+      <c r="F58" s="347"/>
+      <c r="G58" s="347"/>
+      <c r="H58" s="347"/>
+      <c r="I58" s="347"/>
+      <c r="J58" s="347"/>
+      <c r="K58" s="347"/>
+      <c r="L58" s="360"/>
     </row>
     <row r="59" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="164"/>
       <c r="B59" s="165" t="s">
         <v>325</v>
       </c>
-      <c r="C59" s="345" t="s">
+      <c r="C59" s="347" t="s">
         <v>326</v>
       </c>
-      <c r="D59" s="345"/>
-      <c r="E59" s="345"/>
-      <c r="F59" s="345"/>
-      <c r="G59" s="345"/>
-      <c r="H59" s="345"/>
-      <c r="I59" s="345"/>
-      <c r="J59" s="345"/>
-      <c r="K59" s="345"/>
-      <c r="L59" s="346"/>
+      <c r="D59" s="347"/>
+      <c r="E59" s="347"/>
+      <c r="F59" s="347"/>
+      <c r="G59" s="347"/>
+      <c r="H59" s="347"/>
+      <c r="I59" s="347"/>
+      <c r="J59" s="347"/>
+      <c r="K59" s="347"/>
+      <c r="L59" s="360"/>
     </row>
     <row r="60" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="164"/>
       <c r="B60" s="165" t="s">
         <v>98</v>
       </c>
-      <c r="C60" s="345" t="s">
+      <c r="C60" s="347" t="s">
         <v>99</v>
       </c>
-      <c r="D60" s="345"/>
-      <c r="E60" s="345"/>
-      <c r="F60" s="345"/>
-      <c r="G60" s="345"/>
-      <c r="H60" s="345"/>
-      <c r="I60" s="345"/>
-      <c r="J60" s="345"/>
-      <c r="K60" s="345"/>
-      <c r="L60" s="346"/>
+      <c r="D60" s="347"/>
+      <c r="E60" s="347"/>
+      <c r="F60" s="347"/>
+      <c r="G60" s="347"/>
+      <c r="H60" s="347"/>
+      <c r="I60" s="347"/>
+      <c r="J60" s="347"/>
+      <c r="K60" s="347"/>
+      <c r="L60" s="360"/>
     </row>
     <row r="61" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="164"/>
       <c r="B61" s="165" t="s">
         <v>198</v>
       </c>
-      <c r="C61" s="345" t="s">
+      <c r="C61" s="347" t="s">
         <v>199</v>
       </c>
-      <c r="D61" s="345"/>
-      <c r="E61" s="345"/>
-      <c r="F61" s="345"/>
-      <c r="G61" s="345"/>
-      <c r="H61" s="345"/>
-      <c r="I61" s="345"/>
-      <c r="J61" s="345"/>
-      <c r="K61" s="345"/>
-      <c r="L61" s="346"/>
+      <c r="D61" s="347"/>
+      <c r="E61" s="347"/>
+      <c r="F61" s="347"/>
+      <c r="G61" s="347"/>
+      <c r="H61" s="347"/>
+      <c r="I61" s="347"/>
+      <c r="J61" s="347"/>
+      <c r="K61" s="347"/>
+      <c r="L61" s="360"/>
     </row>
     <row r="62" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="164"/>
       <c r="B62" s="165" t="s">
         <v>163</v>
       </c>
-      <c r="C62" s="345" t="s">
+      <c r="C62" s="347" t="s">
         <v>464</v>
       </c>
-      <c r="D62" s="376"/>
-      <c r="E62" s="376"/>
-      <c r="F62" s="376"/>
-      <c r="G62" s="376"/>
-      <c r="H62" s="376"/>
-      <c r="I62" s="376"/>
-      <c r="J62" s="376"/>
-      <c r="K62" s="376"/>
-      <c r="L62" s="377"/>
+      <c r="D62" s="348"/>
+      <c r="E62" s="348"/>
+      <c r="F62" s="348"/>
+      <c r="G62" s="348"/>
+      <c r="H62" s="348"/>
+      <c r="I62" s="348"/>
+      <c r="J62" s="348"/>
+      <c r="K62" s="348"/>
+      <c r="L62" s="349"/>
     </row>
     <row r="63" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="164"/>
       <c r="B63" s="165" t="s">
         <v>391</v>
       </c>
-      <c r="C63" s="345" t="s">
+      <c r="C63" s="347" t="s">
         <v>392</v>
       </c>
-      <c r="D63" s="345"/>
-      <c r="E63" s="345"/>
-      <c r="F63" s="345"/>
-      <c r="G63" s="345"/>
-      <c r="H63" s="345"/>
-      <c r="I63" s="345"/>
-      <c r="J63" s="345"/>
-      <c r="K63" s="345"/>
-      <c r="L63" s="346"/>
+      <c r="D63" s="347"/>
+      <c r="E63" s="347"/>
+      <c r="F63" s="347"/>
+      <c r="G63" s="347"/>
+      <c r="H63" s="347"/>
+      <c r="I63" s="347"/>
+      <c r="J63" s="347"/>
+      <c r="K63" s="347"/>
+      <c r="L63" s="360"/>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="164"/>
@@ -17103,7 +17103,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
@@ -17113,7 +17113,7 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="43" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.2">
@@ -17172,26 +17172,21 @@
     <row r="94" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="B13:K13"/>
-    <mergeCell ref="B19:K19"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="C62:L62"/>
-    <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="A25:L25"/>
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B42:L42"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="C58:L58"/>
+    <mergeCell ref="C63:L63"/>
+    <mergeCell ref="A47:L47"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="B48:L48"/>
+    <mergeCell ref="B49:L49"/>
+    <mergeCell ref="A51:L51"/>
+    <mergeCell ref="C57:L57"/>
+    <mergeCell ref="C60:L60"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B18:L18"/>
+    <mergeCell ref="B44:L44"/>
+    <mergeCell ref="B45:L45"/>
+    <mergeCell ref="B8:L8"/>
     <mergeCell ref="B9:L9"/>
     <mergeCell ref="A11:L11"/>
     <mergeCell ref="B14:L14"/>
@@ -17208,22 +17203,27 @@
     <mergeCell ref="B38:L38"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="B12:L12"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="B13:K13"/>
+    <mergeCell ref="B19:K19"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="C62:L62"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B42:L42"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="C61:L61"/>
-    <mergeCell ref="C58:L58"/>
-    <mergeCell ref="C63:L63"/>
-    <mergeCell ref="A47:L47"/>
-    <mergeCell ref="A5:L5"/>
-    <mergeCell ref="B48:L48"/>
-    <mergeCell ref="B49:L49"/>
-    <mergeCell ref="A51:L51"/>
-    <mergeCell ref="C57:L57"/>
-    <mergeCell ref="C60:L60"/>
-    <mergeCell ref="B16:L16"/>
-    <mergeCell ref="B17:L17"/>
-    <mergeCell ref="B18:L18"/>
-    <mergeCell ref="B44:L44"/>
-    <mergeCell ref="B45:L45"/>
-    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A70" r:id="rId1" xr:uid="{C9866D44-2827-49D7-B9C3-89CF23FACDC1}"/>
@@ -18766,10 +18766,10 @@
         <v>46121</v>
       </c>
       <c r="B18" s="146" t="s">
+        <v>478</v>
+      </c>
+      <c r="C18" s="54" t="s">
         <v>479</v>
-      </c>
-      <c r="C18" s="54" t="s">
-        <v>480</v>
       </c>
       <c r="D18" s="53">
         <v>0.2</v>
@@ -24562,62 +24562,62 @@
       <c r="G5" s="185" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="429" t="s">
+      <c r="I5" s="424" t="s">
         <v>421</v>
       </c>
-      <c r="J5" s="430"/>
-      <c r="K5" s="430"/>
-      <c r="L5" s="430"/>
-      <c r="M5" s="430"/>
-      <c r="N5" s="430"/>
-      <c r="O5" s="430"/>
-      <c r="P5" s="430"/>
-      <c r="Q5" s="430"/>
-      <c r="R5" s="430"/>
-      <c r="S5" s="430"/>
-      <c r="T5" s="430"/>
-      <c r="U5" s="430"/>
-      <c r="V5" s="430"/>
-      <c r="W5" s="431"/>
+      <c r="J5" s="425"/>
+      <c r="K5" s="425"/>
+      <c r="L5" s="425"/>
+      <c r="M5" s="425"/>
+      <c r="N5" s="425"/>
+      <c r="O5" s="425"/>
+      <c r="P5" s="425"/>
+      <c r="Q5" s="425"/>
+      <c r="R5" s="425"/>
+      <c r="S5" s="425"/>
+      <c r="T5" s="425"/>
+      <c r="U5" s="425"/>
+      <c r="V5" s="425"/>
+      <c r="W5" s="426"/>
       <c r="Y5" s="192"/>
       <c r="Z5" s="192"/>
       <c r="AA5" s="192"/>
       <c r="AB5" s="334"/>
     </row>
     <row r="6" spans="1:53" s="184" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B6" s="418" t="s">
+      <c r="B6" s="416" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="419"/>
-      <c r="D6" s="419"/>
-      <c r="E6" s="419"/>
-      <c r="F6" s="419"/>
-      <c r="G6" s="420"/>
-      <c r="I6" s="432" t="s">
+      <c r="C6" s="417"/>
+      <c r="D6" s="417"/>
+      <c r="E6" s="417"/>
+      <c r="F6" s="417"/>
+      <c r="G6" s="418"/>
+      <c r="I6" s="427" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="416" t="s">
+      <c r="J6" s="429" t="s">
         <v>407</v>
       </c>
-      <c r="K6" s="416" t="s">
+      <c r="K6" s="429" t="s">
         <v>406</v>
       </c>
-      <c r="L6" s="434" t="s">
+      <c r="L6" s="430" t="s">
         <v>215</v>
       </c>
-      <c r="M6" s="435"/>
-      <c r="N6" s="435"/>
-      <c r="O6" s="435"/>
-      <c r="P6" s="435"/>
-      <c r="Q6" s="436"/>
-      <c r="R6" s="421" t="s">
+      <c r="M6" s="431"/>
+      <c r="N6" s="431"/>
+      <c r="O6" s="431"/>
+      <c r="P6" s="431"/>
+      <c r="Q6" s="432"/>
+      <c r="R6" s="433" t="s">
         <v>216</v>
       </c>
-      <c r="S6" s="422"/>
-      <c r="T6" s="422"/>
-      <c r="U6" s="422"/>
-      <c r="V6" s="422"/>
-      <c r="W6" s="423"/>
+      <c r="S6" s="434"/>
+      <c r="T6" s="434"/>
+      <c r="U6" s="434"/>
+      <c r="V6" s="434"/>
+      <c r="W6" s="435"/>
       <c r="Y6" s="307"/>
       <c r="Z6" s="307"/>
       <c r="AA6" s="307"/>
@@ -24643,9 +24643,9 @@
         <f>SUM(C7:F7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="433"/>
-      <c r="J7" s="433"/>
-      <c r="K7" s="433"/>
+      <c r="I7" s="428"/>
+      <c r="J7" s="428"/>
+      <c r="K7" s="428"/>
       <c r="L7" s="186" t="s">
         <v>408</v>
       </c>
@@ -24849,14 +24849,14 @@
       <c r="AZ9" s="285"/>
     </row>
     <row r="10" spans="1:53" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="B10" s="424" t="s">
+      <c r="B10" s="419" t="s">
         <v>237</v>
       </c>
-      <c r="C10" s="424"/>
-      <c r="D10" s="424"/>
-      <c r="E10" s="424"/>
-      <c r="F10" s="424"/>
-      <c r="G10" s="424"/>
+      <c r="C10" s="419"/>
+      <c r="D10" s="419"/>
+      <c r="E10" s="419"/>
+      <c r="F10" s="419"/>
+      <c r="G10" s="419"/>
       <c r="I10" s="244" t="s">
         <v>231</v>
       </c>
@@ -25340,13 +25340,13 @@
       <c r="B16" s="193" t="s">
         <v>234</v>
       </c>
-      <c r="C16" s="425" t="s">
+      <c r="C16" s="420" t="s">
         <v>235</v>
       </c>
-      <c r="D16" s="426"/>
-      <c r="E16" s="426"/>
-      <c r="F16" s="426"/>
-      <c r="G16" s="427"/>
+      <c r="D16" s="421"/>
+      <c r="E16" s="421"/>
+      <c r="F16" s="421"/>
+      <c r="G16" s="422"/>
       <c r="I16" s="244" t="s">
         <v>402</v>
       </c>
@@ -25462,59 +25462,59 @@
     </row>
     <row r="18" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15"/>
     <row r="19" spans="2:58" s="192" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I19" s="428" t="s">
+      <c r="I19" s="423" t="s">
         <v>422</v>
       </c>
-      <c r="J19" s="428"/>
-      <c r="K19" s="428"/>
-      <c r="L19" s="428"/>
-      <c r="M19" s="428"/>
-      <c r="N19" s="428"/>
-      <c r="O19" s="428"/>
-      <c r="P19" s="428"/>
-      <c r="Q19" s="428"/>
-      <c r="R19" s="428"/>
-      <c r="S19" s="428"/>
-      <c r="T19" s="428"/>
-      <c r="U19" s="428"/>
+      <c r="J19" s="423"/>
+      <c r="K19" s="423"/>
+      <c r="L19" s="423"/>
+      <c r="M19" s="423"/>
+      <c r="N19" s="423"/>
+      <c r="O19" s="423"/>
+      <c r="P19" s="423"/>
+      <c r="Q19" s="423"/>
+      <c r="R19" s="423"/>
+      <c r="S19" s="423"/>
+      <c r="T19" s="423"/>
+      <c r="U19" s="423"/>
       <c r="Z19" s="250"/>
       <c r="AA19" s="250"/>
       <c r="AB19" s="250"/>
       <c r="AC19" s="250"/>
     </row>
     <row r="20" spans="2:58" s="192" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I20" s="416" t="s">
+      <c r="I20" s="429" t="s">
         <v>13</v>
       </c>
-      <c r="J20" s="416" t="s">
+      <c r="J20" s="429" t="s">
         <v>213</v>
       </c>
-      <c r="K20" s="416" t="s">
+      <c r="K20" s="429" t="s">
         <v>214</v>
       </c>
-      <c r="L20" s="418" t="s">
+      <c r="L20" s="416" t="s">
         <v>215</v>
       </c>
-      <c r="M20" s="419"/>
-      <c r="N20" s="419"/>
-      <c r="O20" s="419"/>
-      <c r="P20" s="420"/>
-      <c r="Q20" s="421" t="s">
+      <c r="M20" s="417"/>
+      <c r="N20" s="417"/>
+      <c r="O20" s="417"/>
+      <c r="P20" s="418"/>
+      <c r="Q20" s="433" t="s">
         <v>216</v>
       </c>
-      <c r="R20" s="422"/>
-      <c r="S20" s="422"/>
-      <c r="T20" s="422"/>
-      <c r="U20" s="423"/>
+      <c r="R20" s="434"/>
+      <c r="S20" s="434"/>
+      <c r="T20" s="434"/>
+      <c r="U20" s="435"/>
       <c r="Z20" s="254"/>
       <c r="AA20" s="254"/>
       <c r="AB20" s="254"/>
       <c r="AC20" s="254"/>
     </row>
     <row r="21" spans="2:58" s="192" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I21" s="417"/>
-      <c r="J21" s="417"/>
-      <c r="K21" s="417"/>
+      <c r="I21" s="436"/>
+      <c r="J21" s="436"/>
+      <c r="K21" s="436"/>
       <c r="L21" s="186" t="s">
         <v>218</v>
       </c>
@@ -26536,6 +26536,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:P20"/>
+    <mergeCell ref="Q20:U20"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="C16:G16"/>
@@ -26546,11 +26551,6 @@
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:Q6"/>
     <mergeCell ref="R6:W6"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:P20"/>
-    <mergeCell ref="Q20:U20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26883,16 +26883,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="438" t="e">
+      <c r="A1" s="437" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B1" s="438"/>
-      <c r="C1" s="438"/>
-      <c r="D1" s="438"/>
-      <c r="E1" s="438"/>
-      <c r="F1" s="438"/>
-      <c r="G1" s="438"/>
+      <c r="B1" s="437"/>
+      <c r="C1" s="437"/>
+      <c r="D1" s="437"/>
+      <c r="E1" s="437"/>
+      <c r="F1" s="437"/>
+      <c r="G1" s="437"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -27001,11 +27001,11 @@
         <v>40</v>
       </c>
       <c r="B10" s="112"/>
-      <c r="C10" s="437"/>
-      <c r="D10" s="437"/>
-      <c r="E10" s="437"/>
-      <c r="F10" s="437"/>
-      <c r="G10" s="437"/>
+      <c r="C10" s="438"/>
+      <c r="D10" s="438"/>
+      <c r="E10" s="438"/>
+      <c r="F10" s="438"/>
+      <c r="G10" s="438"/>
       <c r="N10" s="139"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -28268,12 +28268,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C6:G6"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="C9:G9"/>
@@ -28281,6 +28275,12 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N4" r:id="rId1" location="step-1-assign-parties-person-playing-and-strategies" xr:uid="{726B234F-7B54-4D33-A192-8F1604C6B04C}"/>

</xml_diff>

<commit_message>
Update model file to change hotlinks to new repository and Brittany's figure of hydrology scenarios.
</commit_message>
<xml_diff>
--- a/LakeMeadWaterBankDivideInflow.xlsx
+++ b/LakeMeadWaterBankDivideInflow.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2098394058039/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD78D97-C7E9-4C27-BF8C-60CA00335947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{2BD78D97-C7E9-4C27-BF8C-60CA00335947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5561AD0F-A306-4A18-9AAF-952BA0A41C05}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1200" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="479">
   <si>
     <t>Year 1</t>
   </si>
@@ -2316,6 +2316,12 @@
       </rPr>
       <t>enter their choices to withdraw, conserve, and trade water in response to their available water, others choices, and the real-time discussion by participants.</t>
     </r>
+  </si>
+  <si>
+    <t>There is borad agreement that Colorado River flows will be more volative, declining, and have longer-lasting periods of flow.</t>
+  </si>
+  <si>
+    <t>4)</t>
   </si>
 </sst>
 </file>
@@ -3226,7 +3232,7 @@
     <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="446">
+  <cellXfs count="450">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4135,7 +4141,130 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="9" xfId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="9" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="9" xfId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="13" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="11" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="12" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -4198,9 +4327,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4234,122 +4360,11 @@
     <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="9" xfId="9" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="9" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="9" xfId="9" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="13" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="11" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="12" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4359,6 +4374,15 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4390,9 +4414,6 @@
     <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4402,23 +4423,11 @@
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4447,6 +4456,13 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="20% - Accent1" xfId="12" builtinId="30"/>
@@ -15128,13 +15144,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>321469</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>11906</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>406644</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:colOff>409819</xdr:colOff>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>22141</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -15172,13 +15188,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>46832</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>121840</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:colOff>125015</xdr:colOff>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>1983971</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -15221,14 +15237,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1336343</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>261635</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>483358</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>3301237</xdr:rowOff>
+      <xdr:colOff>486533</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>3304412</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -15267,6 +15283,67 @@
             <a:schemeClr val="tx1"/>
           </a:solidFill>
         </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>232916</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>19457</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>467214</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>2808664</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="VolitileFlows">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47BD50B7-230A-6957-3E35-1BE51D728583}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="232916" y="2958367"/>
+          <a:ext cx="4624102" cy="2789207"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -15843,7 +15920,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2EA02F4-5F19-409C-8BC6-A0D8FEB3A90D}">
-  <dimension ref="A1:R88"/>
+  <dimension ref="A1:R91"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.453125" customWidth="1"/>
@@ -15861,20 +15938,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="348" t="s">
+      <c r="A1" s="389" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="348"/>
-      <c r="C1" s="348"/>
-      <c r="D1" s="348"/>
-      <c r="E1" s="348"/>
-      <c r="F1" s="348"/>
-      <c r="G1" s="348"/>
-      <c r="H1" s="348"/>
-      <c r="I1" s="348"/>
-      <c r="J1" s="348"/>
-      <c r="K1" s="348"/>
-      <c r="L1" s="348"/>
+      <c r="B1" s="389"/>
+      <c r="C1" s="389"/>
+      <c r="D1" s="389"/>
+      <c r="E1" s="389"/>
+      <c r="F1" s="389"/>
+      <c r="G1" s="389"/>
+      <c r="H1" s="389"/>
+      <c r="I1" s="389"/>
+      <c r="J1" s="389"/>
+      <c r="K1" s="389"/>
+      <c r="L1" s="389"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -15900,41 +15977,41 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:18" s="52" customFormat="1" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="349" t="s">
+      <c r="A4" s="390" t="s">
         <v>296</v>
       </c>
-      <c r="B4" s="350"/>
-      <c r="C4" s="350"/>
-      <c r="D4" s="350"/>
-      <c r="E4" s="350"/>
-      <c r="F4" s="350"/>
-      <c r="G4" s="350"/>
-      <c r="H4" s="350"/>
-      <c r="I4" s="350"/>
-      <c r="J4" s="350"/>
-      <c r="K4" s="350"/>
-      <c r="L4" s="351"/>
-      <c r="N4" s="352"/>
-      <c r="O4" s="352"/>
-      <c r="P4" s="352"/>
-      <c r="Q4" s="352"/>
-      <c r="R4" s="352"/>
+      <c r="B4" s="391"/>
+      <c r="C4" s="391"/>
+      <c r="D4" s="391"/>
+      <c r="E4" s="391"/>
+      <c r="F4" s="391"/>
+      <c r="G4" s="391"/>
+      <c r="H4" s="391"/>
+      <c r="I4" s="391"/>
+      <c r="J4" s="391"/>
+      <c r="K4" s="391"/>
+      <c r="L4" s="392"/>
+      <c r="N4" s="393"/>
+      <c r="O4" s="393"/>
+      <c r="P4" s="393"/>
+      <c r="Q4" s="393"/>
+      <c r="R4" s="393"/>
     </row>
     <row r="5" spans="1:18" s="52" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="353" t="s">
+      <c r="A5" s="394" t="s">
         <v>280</v>
       </c>
-      <c r="B5" s="354"/>
-      <c r="C5" s="354"/>
-      <c r="D5" s="354"/>
-      <c r="E5" s="354"/>
-      <c r="F5" s="354"/>
-      <c r="G5" s="354"/>
-      <c r="H5" s="354"/>
-      <c r="I5" s="354"/>
-      <c r="J5" s="354"/>
-      <c r="K5" s="354"/>
-      <c r="L5" s="355"/>
+      <c r="B5" s="395"/>
+      <c r="C5" s="395"/>
+      <c r="D5" s="395"/>
+      <c r="E5" s="395"/>
+      <c r="F5" s="395"/>
+      <c r="G5" s="395"/>
+      <c r="H5" s="395"/>
+      <c r="I5" s="395"/>
+      <c r="J5" s="395"/>
+      <c r="K5" s="395"/>
+      <c r="L5" s="396"/>
       <c r="N5" s="110"/>
       <c r="O5" s="110"/>
       <c r="P5" s="110"/>
@@ -15942,20 +16019,20 @@
       <c r="R5" s="110"/>
     </row>
     <row r="6" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="353" t="s">
+      <c r="A6" s="394" t="s">
         <v>297</v>
       </c>
-      <c r="B6" s="354"/>
-      <c r="C6" s="354"/>
-      <c r="D6" s="354"/>
-      <c r="E6" s="354"/>
-      <c r="F6" s="354"/>
-      <c r="G6" s="354"/>
-      <c r="H6" s="354"/>
-      <c r="I6" s="354"/>
-      <c r="J6" s="354"/>
-      <c r="K6" s="354"/>
-      <c r="L6" s="355"/>
+      <c r="B6" s="395"/>
+      <c r="C6" s="395"/>
+      <c r="D6" s="395"/>
+      <c r="E6" s="395"/>
+      <c r="F6" s="395"/>
+      <c r="G6" s="395"/>
+      <c r="H6" s="395"/>
+      <c r="I6" s="395"/>
+      <c r="J6" s="395"/>
+      <c r="K6" s="395"/>
+      <c r="L6" s="396"/>
       <c r="N6" s="110"/>
       <c r="O6" s="110"/>
       <c r="P6" s="110"/>
@@ -15964,19 +16041,19 @@
     </row>
     <row r="7" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="214"/>
-      <c r="B7" s="354" t="s">
+      <c r="B7" s="395" t="s">
         <v>298</v>
       </c>
-      <c r="C7" s="354"/>
-      <c r="D7" s="354"/>
-      <c r="E7" s="354"/>
-      <c r="F7" s="354"/>
-      <c r="G7" s="354"/>
-      <c r="H7" s="354"/>
-      <c r="I7" s="354"/>
-      <c r="J7" s="354"/>
-      <c r="K7" s="354"/>
-      <c r="L7" s="355"/>
+      <c r="C7" s="395"/>
+      <c r="D7" s="395"/>
+      <c r="E7" s="395"/>
+      <c r="F7" s="395"/>
+      <c r="G7" s="395"/>
+      <c r="H7" s="395"/>
+      <c r="I7" s="395"/>
+      <c r="J7" s="395"/>
+      <c r="K7" s="395"/>
+      <c r="L7" s="396"/>
       <c r="N7" s="110"/>
       <c r="O7" s="110"/>
       <c r="P7" s="110"/>
@@ -15985,19 +16062,19 @@
     </row>
     <row r="8" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="215"/>
-      <c r="B8" s="370" t="s">
+      <c r="B8" s="410" t="s">
         <v>299</v>
       </c>
-      <c r="C8" s="370"/>
-      <c r="D8" s="370"/>
-      <c r="E8" s="370"/>
-      <c r="F8" s="370"/>
-      <c r="G8" s="370"/>
-      <c r="H8" s="370"/>
-      <c r="I8" s="370"/>
-      <c r="J8" s="370"/>
-      <c r="K8" s="370"/>
-      <c r="L8" s="371"/>
+      <c r="C8" s="410"/>
+      <c r="D8" s="410"/>
+      <c r="E8" s="410"/>
+      <c r="F8" s="410"/>
+      <c r="G8" s="410"/>
+      <c r="H8" s="410"/>
+      <c r="I8" s="410"/>
+      <c r="J8" s="410"/>
+      <c r="K8" s="410"/>
+      <c r="L8" s="411"/>
       <c r="N8" s="110"/>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
@@ -16019,1067 +16096,1113 @@
       <c r="L9" s="110"/>
     </row>
     <row r="10" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="372" t="s">
+      <c r="A10" s="412" t="s">
         <v>334</v>
       </c>
-      <c r="B10" s="373"/>
-      <c r="C10" s="373"/>
-      <c r="D10" s="373"/>
-      <c r="E10" s="373"/>
-      <c r="F10" s="373"/>
-      <c r="G10" s="373"/>
-      <c r="H10" s="373"/>
-      <c r="I10" s="373"/>
-      <c r="J10" s="373"/>
-      <c r="K10" s="373"/>
-      <c r="L10" s="374"/>
-    </row>
-    <row r="11" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="235" t="s">
+      <c r="B10" s="413"/>
+      <c r="C10" s="413"/>
+      <c r="D10" s="413"/>
+      <c r="E10" s="413"/>
+      <c r="F10" s="413"/>
+      <c r="G10" s="413"/>
+      <c r="H10" s="413"/>
+      <c r="I10" s="413"/>
+      <c r="J10" s="413"/>
+      <c r="K10" s="413"/>
+      <c r="L10" s="414"/>
+    </row>
+    <row r="11" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="447"/>
+      <c r="B11" s="448"/>
+      <c r="C11" s="448"/>
+      <c r="D11" s="448"/>
+      <c r="E11" s="448"/>
+      <c r="F11" s="448"/>
+      <c r="G11" s="448"/>
+      <c r="H11" s="448"/>
+      <c r="I11" s="448"/>
+      <c r="J11" s="448"/>
+      <c r="K11" s="448"/>
+      <c r="L11" s="342"/>
+    </row>
+    <row r="12" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="447" t="s">
         <v>335</v>
       </c>
-      <c r="B11" s="375" t="s">
+      <c r="B12" s="449" t="s">
+        <v>477</v>
+      </c>
+      <c r="C12" s="448"/>
+      <c r="D12" s="448"/>
+      <c r="E12" s="448"/>
+      <c r="F12" s="448"/>
+      <c r="G12" s="448"/>
+      <c r="H12" s="448"/>
+      <c r="I12" s="448"/>
+      <c r="J12" s="448"/>
+      <c r="K12" s="448"/>
+      <c r="L12" s="342"/>
+    </row>
+    <row r="13" spans="1:18" s="57" customFormat="1" ht="224" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="447"/>
+      <c r="B13"/>
+      <c r="C13" s="448"/>
+      <c r="D13" s="448"/>
+      <c r="E13" s="448"/>
+      <c r="F13" s="448"/>
+      <c r="G13" s="448"/>
+      <c r="H13" s="448"/>
+      <c r="I13" s="448"/>
+      <c r="J13" s="448"/>
+      <c r="K13" s="448"/>
+      <c r="L13" s="342"/>
+    </row>
+    <row r="14" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="235" t="s">
+        <v>336</v>
+      </c>
+      <c r="B14" s="365" t="s">
         <v>338</v>
       </c>
-      <c r="C11" s="375"/>
-      <c r="D11" s="375"/>
-      <c r="E11" s="375"/>
-      <c r="F11" s="375"/>
-      <c r="G11" s="375"/>
-      <c r="H11" s="375"/>
-      <c r="I11" s="375"/>
-      <c r="J11" s="375"/>
-      <c r="K11" s="375"/>
-      <c r="L11" s="376"/>
-    </row>
-    <row r="12" spans="1:18" s="57" customFormat="1" ht="161.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="227"/>
-      <c r="B12" s="233"/>
-      <c r="C12" s="233"/>
-      <c r="D12" s="233"/>
-      <c r="E12" s="233"/>
-      <c r="F12" s="233"/>
-      <c r="G12" s="233"/>
-      <c r="H12" s="233"/>
-      <c r="I12" s="233"/>
-      <c r="J12" s="233"/>
-      <c r="K12" s="233"/>
-      <c r="L12" s="234"/>
-    </row>
-    <row r="13" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="235" t="s">
-        <v>336</v>
-      </c>
-      <c r="B13" s="375" t="s">
+      <c r="C14" s="365"/>
+      <c r="D14" s="365"/>
+      <c r="E14" s="365"/>
+      <c r="F14" s="365"/>
+      <c r="G14" s="365"/>
+      <c r="H14" s="365"/>
+      <c r="I14" s="365"/>
+      <c r="J14" s="365"/>
+      <c r="K14" s="365"/>
+      <c r="L14" s="366"/>
+    </row>
+    <row r="15" spans="1:18" s="57" customFormat="1" ht="161.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="227"/>
+      <c r="B15" s="233"/>
+      <c r="C15" s="233"/>
+      <c r="D15" s="233"/>
+      <c r="E15" s="233"/>
+      <c r="F15" s="233"/>
+      <c r="G15" s="233"/>
+      <c r="H15" s="233"/>
+      <c r="I15" s="233"/>
+      <c r="J15" s="233"/>
+      <c r="K15" s="233"/>
+      <c r="L15" s="234"/>
+    </row>
+    <row r="16" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="235" t="s">
+        <v>337</v>
+      </c>
+      <c r="B16" s="365" t="s">
         <v>339</v>
       </c>
-      <c r="C13" s="375"/>
-      <c r="D13" s="375"/>
-      <c r="E13" s="375"/>
-      <c r="F13" s="375"/>
-      <c r="G13" s="375"/>
-      <c r="H13" s="375"/>
-      <c r="I13" s="375"/>
-      <c r="J13" s="375"/>
-      <c r="K13" s="375"/>
-      <c r="L13" s="376"/>
-    </row>
-    <row r="14" spans="1:18" s="57" customFormat="1" ht="90.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="227"/>
-      <c r="B14" s="386"/>
-      <c r="C14" s="386"/>
-      <c r="D14" s="386"/>
-      <c r="E14" s="386"/>
-      <c r="F14" s="386"/>
-      <c r="G14" s="386"/>
-      <c r="H14" s="386"/>
-      <c r="I14" s="386"/>
-      <c r="J14" s="386"/>
-      <c r="K14" s="386"/>
-      <c r="L14" s="387"/>
-    </row>
-    <row r="15" spans="1:18" s="56" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="235" t="s">
-        <v>337</v>
-      </c>
-      <c r="B15" s="375" t="s">
+      <c r="C16" s="365"/>
+      <c r="D16" s="365"/>
+      <c r="E16" s="365"/>
+      <c r="F16" s="365"/>
+      <c r="G16" s="365"/>
+      <c r="H16" s="365"/>
+      <c r="I16" s="365"/>
+      <c r="J16" s="365"/>
+      <c r="K16" s="365"/>
+      <c r="L16" s="366"/>
+    </row>
+    <row r="17" spans="1:14" s="57" customFormat="1" ht="90.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="227"/>
+      <c r="B17" s="367"/>
+      <c r="C17" s="367"/>
+      <c r="D17" s="367"/>
+      <c r="E17" s="367"/>
+      <c r="F17" s="367"/>
+      <c r="G17" s="367"/>
+      <c r="H17" s="367"/>
+      <c r="I17" s="367"/>
+      <c r="J17" s="367"/>
+      <c r="K17" s="367"/>
+      <c r="L17" s="368"/>
+    </row>
+    <row r="18" spans="1:14" s="56" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="235" t="s">
+        <v>478</v>
+      </c>
+      <c r="B18" s="365" t="s">
         <v>465</v>
       </c>
-      <c r="C15" s="375"/>
-      <c r="D15" s="375"/>
-      <c r="E15" s="375"/>
-      <c r="F15" s="375"/>
-      <c r="G15" s="375"/>
-      <c r="H15" s="375"/>
-      <c r="I15" s="375"/>
-      <c r="J15" s="375"/>
-      <c r="K15" s="375"/>
-      <c r="L15" s="376"/>
-    </row>
-    <row r="16" spans="1:18" s="57" customFormat="1" ht="269" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="227"/>
-      <c r="B16" s="233"/>
-      <c r="C16" s="233"/>
-      <c r="D16" s="233"/>
-      <c r="E16" s="233"/>
-      <c r="F16" s="233"/>
-      <c r="G16" s="233"/>
-      <c r="H16" s="233"/>
-      <c r="I16" s="233"/>
-      <c r="J16" s="233"/>
-      <c r="K16" s="233"/>
-      <c r="L16" s="234"/>
-    </row>
-    <row r="17" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="384" t="s">
+      <c r="C18" s="365"/>
+      <c r="D18" s="365"/>
+      <c r="E18" s="365"/>
+      <c r="F18" s="365"/>
+      <c r="G18" s="365"/>
+      <c r="H18" s="365"/>
+      <c r="I18" s="365"/>
+      <c r="J18" s="365"/>
+      <c r="K18" s="365"/>
+      <c r="L18" s="366"/>
+    </row>
+    <row r="19" spans="1:14" s="57" customFormat="1" ht="269" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="227"/>
+      <c r="B19" s="233"/>
+      <c r="C19" s="233"/>
+      <c r="D19" s="233"/>
+      <c r="E19" s="233"/>
+      <c r="F19" s="233"/>
+      <c r="G19" s="233"/>
+      <c r="H19" s="233"/>
+      <c r="I19" s="233"/>
+      <c r="J19" s="233"/>
+      <c r="K19" s="233"/>
+      <c r="L19" s="234"/>
+    </row>
+    <row r="20" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="363" t="s">
         <v>343</v>
       </c>
-      <c r="B17" s="385"/>
-      <c r="C17" s="385"/>
-      <c r="D17" s="385"/>
-      <c r="E17" s="232" t="s">
+      <c r="B20" s="364"/>
+      <c r="C20" s="364"/>
+      <c r="D20" s="364"/>
+      <c r="E20" s="232" t="s">
         <v>344</v>
       </c>
-      <c r="F17" s="230"/>
-      <c r="G17" s="230"/>
-      <c r="H17" s="230"/>
-      <c r="I17" s="230"/>
-      <c r="J17" s="230"/>
-      <c r="K17" s="230"/>
-      <c r="L17" s="231"/>
-    </row>
-    <row r="18" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="110"/>
-      <c r="B18" s="110"/>
-      <c r="C18" s="110"/>
-      <c r="D18" s="110"/>
-      <c r="E18" s="110"/>
-      <c r="F18" s="110"/>
-      <c r="G18" s="110"/>
-      <c r="H18" s="110"/>
-      <c r="I18" s="110"/>
-      <c r="J18" s="110"/>
-      <c r="K18" s="110"/>
-      <c r="L18" s="110"/>
-    </row>
-    <row r="19" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="356" t="s">
+      <c r="F20" s="230"/>
+      <c r="G20" s="230"/>
+      <c r="H20" s="230"/>
+      <c r="I20" s="230"/>
+      <c r="J20" s="230"/>
+      <c r="K20" s="230"/>
+      <c r="L20" s="231"/>
+    </row>
+    <row r="21" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="110"/>
+      <c r="B21" s="110"/>
+      <c r="C21" s="110"/>
+      <c r="D21" s="110"/>
+      <c r="E21" s="110"/>
+      <c r="F21" s="110"/>
+      <c r="G21" s="110"/>
+      <c r="H21" s="110"/>
+      <c r="I21" s="110"/>
+      <c r="J21" s="110"/>
+      <c r="K21" s="110"/>
+      <c r="L21" s="110"/>
+    </row>
+    <row r="22" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="397" t="s">
         <v>165</v>
       </c>
-      <c r="B19" s="357"/>
-      <c r="C19" s="357"/>
-      <c r="D19" s="357"/>
-      <c r="E19" s="357"/>
-      <c r="F19" s="357"/>
-      <c r="G19" s="357"/>
-      <c r="H19" s="357"/>
-      <c r="I19" s="357"/>
-      <c r="J19" s="357"/>
-      <c r="K19" s="357"/>
-      <c r="L19" s="358"/>
-    </row>
-    <row r="20" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="359" t="s">
+      <c r="B22" s="398"/>
+      <c r="C22" s="398"/>
+      <c r="D22" s="398"/>
+      <c r="E22" s="398"/>
+      <c r="F22" s="398"/>
+      <c r="G22" s="398"/>
+      <c r="H22" s="398"/>
+      <c r="I22" s="398"/>
+      <c r="J22" s="398"/>
+      <c r="K22" s="398"/>
+      <c r="L22" s="399"/>
+    </row>
+    <row r="23" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="400" t="s">
         <v>281</v>
       </c>
-      <c r="B20" s="360"/>
-      <c r="C20" s="360"/>
-      <c r="D20" s="360"/>
-      <c r="E20" s="360"/>
-      <c r="F20" s="360"/>
-      <c r="G20" s="360"/>
-      <c r="H20" s="360"/>
-      <c r="I20" s="360"/>
-      <c r="J20" s="360"/>
-      <c r="K20" s="360"/>
-      <c r="L20" s="361"/>
-    </row>
-    <row r="21" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="362" t="s">
+      <c r="B23" s="401"/>
+      <c r="C23" s="401"/>
+      <c r="D23" s="401"/>
+      <c r="E23" s="401"/>
+      <c r="F23" s="401"/>
+      <c r="G23" s="401"/>
+      <c r="H23" s="401"/>
+      <c r="I23" s="401"/>
+      <c r="J23" s="401"/>
+      <c r="K23" s="401"/>
+      <c r="L23" s="402"/>
+    </row>
+    <row r="24" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="403" t="s">
         <v>282</v>
       </c>
-      <c r="B21" s="342"/>
-      <c r="C21" s="342"/>
-      <c r="D21" s="342"/>
-      <c r="E21" s="342"/>
-      <c r="F21" s="342"/>
-      <c r="G21" s="342"/>
-      <c r="H21" s="342"/>
-      <c r="I21" s="342"/>
-      <c r="J21" s="342"/>
-      <c r="K21" s="342"/>
-      <c r="L21" s="363"/>
-    </row>
-    <row r="22" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="362" t="s">
+      <c r="B24" s="379"/>
+      <c r="C24" s="379"/>
+      <c r="D24" s="379"/>
+      <c r="E24" s="379"/>
+      <c r="F24" s="379"/>
+      <c r="G24" s="379"/>
+      <c r="H24" s="379"/>
+      <c r="I24" s="379"/>
+      <c r="J24" s="379"/>
+      <c r="K24" s="379"/>
+      <c r="L24" s="380"/>
+    </row>
+    <row r="25" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="403" t="s">
         <v>166</v>
       </c>
-      <c r="B22" s="342"/>
-      <c r="C22" s="342"/>
-      <c r="D22" s="342"/>
-      <c r="E22" s="342"/>
-      <c r="F22" s="342"/>
-      <c r="G22" s="342"/>
-      <c r="H22" s="342"/>
-      <c r="I22" s="342"/>
-      <c r="J22" s="342"/>
-      <c r="K22" s="342"/>
-      <c r="L22" s="363"/>
-    </row>
-    <row r="23" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="364" t="s">
+      <c r="B25" s="379"/>
+      <c r="C25" s="379"/>
+      <c r="D25" s="379"/>
+      <c r="E25" s="379"/>
+      <c r="F25" s="379"/>
+      <c r="G25" s="379"/>
+      <c r="H25" s="379"/>
+      <c r="I25" s="379"/>
+      <c r="J25" s="379"/>
+      <c r="K25" s="379"/>
+      <c r="L25" s="380"/>
+    </row>
+    <row r="26" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="404" t="s">
         <v>283</v>
       </c>
-      <c r="B23" s="365"/>
-      <c r="C23" s="365"/>
-      <c r="D23" s="365"/>
-      <c r="E23" s="365"/>
-      <c r="F23" s="365"/>
-      <c r="G23" s="365"/>
-      <c r="H23" s="365"/>
-      <c r="I23" s="365"/>
-      <c r="J23" s="365"/>
-      <c r="K23" s="365"/>
-      <c r="L23" s="366"/>
-    </row>
-    <row r="24" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="110"/>
-      <c r="B24" s="110"/>
-      <c r="C24" s="110"/>
-      <c r="D24" s="110"/>
-      <c r="E24" s="110"/>
-      <c r="F24" s="110"/>
-      <c r="G24" s="110"/>
-      <c r="H24" s="110"/>
-      <c r="I24" s="110"/>
-      <c r="J24" s="110"/>
-      <c r="K24" s="110"/>
-      <c r="L24" s="110"/>
-    </row>
-    <row r="25" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="367" t="s">
+      <c r="B26" s="405"/>
+      <c r="C26" s="405"/>
+      <c r="D26" s="405"/>
+      <c r="E26" s="405"/>
+      <c r="F26" s="405"/>
+      <c r="G26" s="405"/>
+      <c r="H26" s="405"/>
+      <c r="I26" s="405"/>
+      <c r="J26" s="405"/>
+      <c r="K26" s="405"/>
+      <c r="L26" s="406"/>
+    </row>
+    <row r="27" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="110"/>
+      <c r="B27" s="110"/>
+      <c r="C27" s="110"/>
+      <c r="D27" s="110"/>
+      <c r="E27" s="110"/>
+      <c r="F27" s="110"/>
+      <c r="G27" s="110"/>
+      <c r="H27" s="110"/>
+      <c r="I27" s="110"/>
+      <c r="J27" s="110"/>
+      <c r="K27" s="110"/>
+      <c r="L27" s="110"/>
+    </row>
+    <row r="28" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="407" t="s">
         <v>279</v>
       </c>
-      <c r="B25" s="368"/>
-      <c r="C25" s="368"/>
-      <c r="D25" s="368"/>
-      <c r="E25" s="368"/>
-      <c r="F25" s="368"/>
-      <c r="G25" s="368"/>
-      <c r="H25" s="368"/>
-      <c r="I25" s="368"/>
-      <c r="J25" s="368"/>
-      <c r="K25" s="368"/>
-      <c r="L25" s="369"/>
-      <c r="N25" s="1"/>
-    </row>
-    <row r="26" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="345" t="s">
+      <c r="B28" s="408"/>
+      <c r="C28" s="408"/>
+      <c r="D28" s="408"/>
+      <c r="E28" s="408"/>
+      <c r="F28" s="408"/>
+      <c r="G28" s="408"/>
+      <c r="H28" s="408"/>
+      <c r="I28" s="408"/>
+      <c r="J28" s="408"/>
+      <c r="K28" s="408"/>
+      <c r="L28" s="409"/>
+      <c r="N28" s="1"/>
+    </row>
+    <row r="29" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="386" t="s">
         <v>175</v>
       </c>
-      <c r="B26" s="346"/>
-      <c r="C26" s="346"/>
-      <c r="D26" s="346"/>
-      <c r="E26" s="346"/>
-      <c r="F26" s="346"/>
-      <c r="G26" s="346"/>
-      <c r="H26" s="346"/>
-      <c r="I26" s="346"/>
-      <c r="J26" s="346"/>
-      <c r="K26" s="346"/>
-      <c r="L26" s="347"/>
-      <c r="N26" s="1"/>
-    </row>
-    <row r="27" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="209">
-        <v>1</v>
-      </c>
-      <c r="B27" s="379" t="s">
-        <v>174</v>
-      </c>
-      <c r="C27" s="379"/>
-      <c r="D27" s="379"/>
-      <c r="E27" s="379"/>
-      <c r="F27" s="379"/>
-      <c r="G27" s="379"/>
-      <c r="H27" s="379"/>
-      <c r="I27" s="379"/>
-      <c r="J27" s="379"/>
-      <c r="K27" s="379"/>
-      <c r="L27" s="380"/>
-    </row>
-    <row r="28" spans="1:14" s="57" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="209">
-        <v>2</v>
-      </c>
-      <c r="B28" s="379" t="s">
-        <v>275</v>
-      </c>
-      <c r="C28" s="379"/>
-      <c r="D28" s="379"/>
-      <c r="E28" s="379"/>
-      <c r="F28" s="379"/>
-      <c r="G28" s="379"/>
-      <c r="H28" s="379"/>
-      <c r="I28" s="379"/>
-      <c r="J28" s="379"/>
-      <c r="K28" s="379"/>
-      <c r="L28" s="380"/>
-      <c r="N28" s="104"/>
-    </row>
-    <row r="29" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="209">
-        <v>3</v>
-      </c>
-      <c r="B29" s="379" t="s">
-        <v>167</v>
-      </c>
-      <c r="C29" s="379"/>
-      <c r="D29" s="379"/>
-      <c r="E29" s="379"/>
-      <c r="F29" s="379"/>
-      <c r="G29" s="379"/>
-      <c r="H29" s="379"/>
-      <c r="I29" s="379"/>
-      <c r="J29" s="379"/>
-      <c r="K29" s="379"/>
-      <c r="L29" s="380"/>
-      <c r="N29" s="104"/>
+      <c r="B29" s="387"/>
+      <c r="C29" s="387"/>
+      <c r="D29" s="387"/>
+      <c r="E29" s="387"/>
+      <c r="F29" s="387"/>
+      <c r="G29" s="387"/>
+      <c r="H29" s="387"/>
+      <c r="I29" s="387"/>
+      <c r="J29" s="387"/>
+      <c r="K29" s="387"/>
+      <c r="L29" s="388"/>
+      <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="209">
+        <v>1</v>
+      </c>
+      <c r="B30" s="372" t="s">
+        <v>174</v>
+      </c>
+      <c r="C30" s="372"/>
+      <c r="D30" s="372"/>
+      <c r="E30" s="372"/>
+      <c r="F30" s="372"/>
+      <c r="G30" s="372"/>
+      <c r="H30" s="372"/>
+      <c r="I30" s="372"/>
+      <c r="J30" s="372"/>
+      <c r="K30" s="372"/>
+      <c r="L30" s="373"/>
+    </row>
+    <row r="31" spans="1:14" s="57" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="209">
+        <v>2</v>
+      </c>
+      <c r="B31" s="372" t="s">
+        <v>275</v>
+      </c>
+      <c r="C31" s="372"/>
+      <c r="D31" s="372"/>
+      <c r="E31" s="372"/>
+      <c r="F31" s="372"/>
+      <c r="G31" s="372"/>
+      <c r="H31" s="372"/>
+      <c r="I31" s="372"/>
+      <c r="J31" s="372"/>
+      <c r="K31" s="372"/>
+      <c r="L31" s="373"/>
+      <c r="N31" s="104"/>
+    </row>
+    <row r="32" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="209">
+        <v>3</v>
+      </c>
+      <c r="B32" s="372" t="s">
+        <v>167</v>
+      </c>
+      <c r="C32" s="372"/>
+      <c r="D32" s="372"/>
+      <c r="E32" s="372"/>
+      <c r="F32" s="372"/>
+      <c r="G32" s="372"/>
+      <c r="H32" s="372"/>
+      <c r="I32" s="372"/>
+      <c r="J32" s="372"/>
+      <c r="K32" s="372"/>
+      <c r="L32" s="373"/>
+      <c r="N32" s="104"/>
+    </row>
+    <row r="33" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="209">
         <v>4</v>
       </c>
-      <c r="B30" s="379" t="s">
+      <c r="B33" s="372" t="s">
         <v>284</v>
       </c>
-      <c r="C30" s="379"/>
-      <c r="D30" s="379"/>
-      <c r="E30" s="379"/>
-      <c r="F30" s="379"/>
-      <c r="G30" s="379"/>
-      <c r="H30" s="379"/>
-      <c r="I30" s="379"/>
-      <c r="J30" s="379"/>
-      <c r="K30" s="379"/>
-      <c r="L30" s="380"/>
-      <c r="N30" s="104"/>
-    </row>
-    <row r="31" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="209">
+      <c r="C33" s="372"/>
+      <c r="D33" s="372"/>
+      <c r="E33" s="372"/>
+      <c r="F33" s="372"/>
+      <c r="G33" s="372"/>
+      <c r="H33" s="372"/>
+      <c r="I33" s="372"/>
+      <c r="J33" s="372"/>
+      <c r="K33" s="372"/>
+      <c r="L33" s="373"/>
+      <c r="N33" s="104"/>
+    </row>
+    <row r="34" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="209">
         <v>5</v>
       </c>
-      <c r="B31" s="379" t="s">
+      <c r="B34" s="372" t="s">
         <v>168</v>
       </c>
-      <c r="C31" s="379"/>
-      <c r="D31" s="379"/>
-      <c r="E31" s="379"/>
-      <c r="F31" s="379"/>
-      <c r="G31" s="379"/>
-      <c r="H31" s="379"/>
-      <c r="I31" s="379"/>
-      <c r="J31" s="379"/>
-      <c r="K31" s="379"/>
-      <c r="L31" s="380"/>
-      <c r="N31" s="104"/>
-    </row>
-    <row r="32" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="209"/>
-      <c r="B32" s="379" t="s">
+      <c r="C34" s="372"/>
+      <c r="D34" s="372"/>
+      <c r="E34" s="372"/>
+      <c r="F34" s="372"/>
+      <c r="G34" s="372"/>
+      <c r="H34" s="372"/>
+      <c r="I34" s="372"/>
+      <c r="J34" s="372"/>
+      <c r="K34" s="372"/>
+      <c r="L34" s="373"/>
+      <c r="N34" s="104"/>
+    </row>
+    <row r="35" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="209"/>
+      <c r="B35" s="372" t="s">
         <v>169</v>
       </c>
-      <c r="C32" s="379"/>
-      <c r="D32" s="379"/>
-      <c r="E32" s="379"/>
-      <c r="F32" s="379"/>
-      <c r="G32" s="379"/>
-      <c r="H32" s="379"/>
-      <c r="I32" s="379"/>
-      <c r="J32" s="379"/>
-      <c r="K32" s="379"/>
-      <c r="L32" s="380"/>
-      <c r="N32" s="104"/>
-    </row>
-    <row r="33" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="209"/>
-      <c r="B33" s="379" t="s">
+      <c r="C35" s="372"/>
+      <c r="D35" s="372"/>
+      <c r="E35" s="372"/>
+      <c r="F35" s="372"/>
+      <c r="G35" s="372"/>
+      <c r="H35" s="372"/>
+      <c r="I35" s="372"/>
+      <c r="J35" s="372"/>
+      <c r="K35" s="372"/>
+      <c r="L35" s="373"/>
+      <c r="N35" s="104"/>
+    </row>
+    <row r="36" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="209"/>
+      <c r="B36" s="372" t="s">
         <v>170</v>
       </c>
-      <c r="C33" s="379"/>
-      <c r="D33" s="379"/>
-      <c r="E33" s="379"/>
-      <c r="F33" s="379"/>
-      <c r="G33" s="379"/>
-      <c r="H33" s="379"/>
-      <c r="I33" s="379"/>
-      <c r="J33" s="379"/>
-      <c r="K33" s="379"/>
-      <c r="L33" s="380"/>
-      <c r="N33" s="104"/>
-    </row>
-    <row r="34" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="381" t="s">
+      <c r="C36" s="372"/>
+      <c r="D36" s="372"/>
+      <c r="E36" s="372"/>
+      <c r="F36" s="372"/>
+      <c r="G36" s="372"/>
+      <c r="H36" s="372"/>
+      <c r="I36" s="372"/>
+      <c r="J36" s="372"/>
+      <c r="K36" s="372"/>
+      <c r="L36" s="373"/>
+      <c r="N36" s="104"/>
+    </row>
+    <row r="37" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="381" t="s">
         <v>176</v>
       </c>
-      <c r="B34" s="382"/>
-      <c r="C34" s="382"/>
-      <c r="D34" s="382"/>
-      <c r="E34" s="382"/>
-      <c r="F34" s="382"/>
-      <c r="G34" s="382"/>
-      <c r="H34" s="382"/>
-      <c r="I34" s="382"/>
-      <c r="J34" s="382"/>
-      <c r="K34" s="382"/>
-      <c r="L34" s="383"/>
-      <c r="N34" s="104"/>
-    </row>
-    <row r="35" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="209">
+      <c r="B37" s="382"/>
+      <c r="C37" s="382"/>
+      <c r="D37" s="382"/>
+      <c r="E37" s="382"/>
+      <c r="F37" s="382"/>
+      <c r="G37" s="382"/>
+      <c r="H37" s="382"/>
+      <c r="I37" s="382"/>
+      <c r="J37" s="382"/>
+      <c r="K37" s="382"/>
+      <c r="L37" s="383"/>
+      <c r="N37" s="104"/>
+    </row>
+    <row r="38" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="209">
         <v>1</v>
       </c>
-      <c r="B35" s="379" t="s">
+      <c r="B38" s="372" t="s">
         <v>171</v>
       </c>
-      <c r="C35" s="379"/>
-      <c r="D35" s="379"/>
-      <c r="E35" s="379"/>
-      <c r="F35" s="379"/>
-      <c r="G35" s="379"/>
-      <c r="H35" s="379"/>
-      <c r="I35" s="379"/>
-      <c r="J35" s="379"/>
-      <c r="K35" s="379"/>
-      <c r="L35" s="380"/>
-      <c r="N35" s="104"/>
-    </row>
-    <row r="36" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="209"/>
-      <c r="B36" s="377" t="s">
+      <c r="C38" s="372"/>
+      <c r="D38" s="372"/>
+      <c r="E38" s="372"/>
+      <c r="F38" s="372"/>
+      <c r="G38" s="372"/>
+      <c r="H38" s="372"/>
+      <c r="I38" s="372"/>
+      <c r="J38" s="372"/>
+      <c r="K38" s="372"/>
+      <c r="L38" s="373"/>
+      <c r="N38" s="104"/>
+    </row>
+    <row r="39" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="209"/>
+      <c r="B39" s="370" t="s">
         <v>426</v>
       </c>
-      <c r="C36" s="377"/>
-      <c r="D36" s="377"/>
-      <c r="E36" s="377"/>
-      <c r="F36" s="377"/>
-      <c r="G36" s="377"/>
-      <c r="H36" s="377"/>
-      <c r="I36" s="377"/>
-      <c r="J36" s="377"/>
-      <c r="K36" s="377"/>
-      <c r="L36" s="378"/>
-      <c r="N36" s="104"/>
-    </row>
-    <row r="37" spans="1:14" s="57" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="209">
+      <c r="C39" s="370"/>
+      <c r="D39" s="370"/>
+      <c r="E39" s="370"/>
+      <c r="F39" s="370"/>
+      <c r="G39" s="370"/>
+      <c r="H39" s="370"/>
+      <c r="I39" s="370"/>
+      <c r="J39" s="370"/>
+      <c r="K39" s="370"/>
+      <c r="L39" s="371"/>
+      <c r="N39" s="104"/>
+    </row>
+    <row r="40" spans="1:14" s="57" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="209">
         <v>2</v>
       </c>
-      <c r="B37" s="379" t="s">
+      <c r="B40" s="372" t="s">
         <v>278</v>
       </c>
-      <c r="C37" s="379"/>
-      <c r="D37" s="379"/>
-      <c r="E37" s="379"/>
-      <c r="F37" s="379"/>
-      <c r="G37" s="379"/>
-      <c r="H37" s="379"/>
-      <c r="I37" s="379"/>
-      <c r="J37" s="379"/>
-      <c r="K37" s="379"/>
-      <c r="L37" s="380"/>
-      <c r="N37" s="104"/>
-    </row>
-    <row r="38" spans="1:14" s="57" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="209">
+      <c r="C40" s="372"/>
+      <c r="D40" s="372"/>
+      <c r="E40" s="372"/>
+      <c r="F40" s="372"/>
+      <c r="G40" s="372"/>
+      <c r="H40" s="372"/>
+      <c r="I40" s="372"/>
+      <c r="J40" s="372"/>
+      <c r="K40" s="372"/>
+      <c r="L40" s="373"/>
+      <c r="N40" s="104"/>
+    </row>
+    <row r="41" spans="1:14" s="57" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="209">
         <v>3</v>
       </c>
-      <c r="B38" s="379" t="s">
+      <c r="B41" s="372" t="s">
         <v>475</v>
       </c>
-      <c r="C38" s="379"/>
-      <c r="D38" s="379"/>
-      <c r="E38" s="379"/>
-      <c r="F38" s="379"/>
-      <c r="G38" s="379"/>
-      <c r="H38" s="379"/>
-      <c r="I38" s="379"/>
-      <c r="J38" s="379"/>
-      <c r="K38" s="379"/>
-      <c r="L38" s="380"/>
-      <c r="N38" s="104"/>
-    </row>
-    <row r="39" spans="1:14" s="57" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="209">
+      <c r="C41" s="372"/>
+      <c r="D41" s="372"/>
+      <c r="E41" s="372"/>
+      <c r="F41" s="372"/>
+      <c r="G41" s="372"/>
+      <c r="H41" s="372"/>
+      <c r="I41" s="372"/>
+      <c r="J41" s="372"/>
+      <c r="K41" s="372"/>
+      <c r="L41" s="373"/>
+      <c r="N41" s="104"/>
+    </row>
+    <row r="42" spans="1:14" s="57" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="209">
         <v>4</v>
       </c>
-      <c r="B39" s="379" t="s">
+      <c r="B42" s="372" t="s">
         <v>285</v>
       </c>
-      <c r="C39" s="379"/>
-      <c r="D39" s="379"/>
-      <c r="E39" s="379"/>
-      <c r="F39" s="379"/>
-      <c r="G39" s="379"/>
-      <c r="H39" s="379"/>
-      <c r="I39" s="379"/>
-      <c r="J39" s="379"/>
-      <c r="K39" s="379"/>
-      <c r="L39" s="380"/>
-      <c r="N39" s="104"/>
-    </row>
-    <row r="40" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="209">
+      <c r="C42" s="372"/>
+      <c r="D42" s="372"/>
+      <c r="E42" s="372"/>
+      <c r="F42" s="372"/>
+      <c r="G42" s="372"/>
+      <c r="H42" s="372"/>
+      <c r="I42" s="372"/>
+      <c r="J42" s="372"/>
+      <c r="K42" s="372"/>
+      <c r="L42" s="373"/>
+      <c r="N42" s="104"/>
+    </row>
+    <row r="43" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="209">
         <v>5</v>
       </c>
-      <c r="B40" s="377" t="s">
+      <c r="B43" s="370" t="s">
         <v>269</v>
       </c>
-      <c r="C40" s="377"/>
-      <c r="D40" s="377"/>
-      <c r="E40" s="377"/>
-      <c r="F40" s="377"/>
-      <c r="G40" s="377"/>
-      <c r="H40" s="377"/>
-      <c r="I40" s="377"/>
-      <c r="J40" s="377"/>
-      <c r="K40" s="377"/>
-      <c r="L40" s="378"/>
-      <c r="N40" s="104"/>
-    </row>
-    <row r="41" spans="1:14" s="57" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="209">
+      <c r="C43" s="370"/>
+      <c r="D43" s="370"/>
+      <c r="E43" s="370"/>
+      <c r="F43" s="370"/>
+      <c r="G43" s="370"/>
+      <c r="H43" s="370"/>
+      <c r="I43" s="370"/>
+      <c r="J43" s="370"/>
+      <c r="K43" s="370"/>
+      <c r="L43" s="371"/>
+      <c r="N43" s="104"/>
+    </row>
+    <row r="44" spans="1:14" s="57" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="209">
         <v>6</v>
       </c>
-      <c r="B41" s="377" t="s">
+      <c r="B44" s="370" t="s">
         <v>476</v>
       </c>
-      <c r="C41" s="377"/>
-      <c r="D41" s="377"/>
-      <c r="E41" s="377"/>
-      <c r="F41" s="377"/>
-      <c r="G41" s="377"/>
-      <c r="H41" s="377"/>
-      <c r="I41" s="377"/>
-      <c r="J41" s="377"/>
-      <c r="K41" s="377"/>
-      <c r="L41" s="378"/>
-      <c r="N41" s="104"/>
-    </row>
-    <row r="42" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="209">
+      <c r="C44" s="370"/>
+      <c r="D44" s="370"/>
+      <c r="E44" s="370"/>
+      <c r="F44" s="370"/>
+      <c r="G44" s="370"/>
+      <c r="H44" s="370"/>
+      <c r="I44" s="370"/>
+      <c r="J44" s="370"/>
+      <c r="K44" s="370"/>
+      <c r="L44" s="371"/>
+      <c r="N44" s="104"/>
+    </row>
+    <row r="45" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="209">
         <v>7</v>
       </c>
-      <c r="B42" s="379" t="s">
+      <c r="B45" s="372" t="s">
         <v>270</v>
       </c>
-      <c r="C42" s="379"/>
-      <c r="D42" s="379"/>
-      <c r="E42" s="379"/>
-      <c r="F42" s="379"/>
-      <c r="G42" s="379"/>
-      <c r="H42" s="379"/>
-      <c r="I42" s="379"/>
-      <c r="J42" s="379"/>
-      <c r="K42" s="379"/>
-      <c r="L42" s="380"/>
-    </row>
-    <row r="43" spans="1:14" s="57" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="209"/>
-      <c r="B43" s="210"/>
-      <c r="C43" s="210"/>
-      <c r="D43" s="210"/>
-      <c r="E43" s="210"/>
-      <c r="F43" s="210"/>
-      <c r="G43" s="210"/>
-      <c r="H43" s="210"/>
-      <c r="I43" s="210"/>
-      <c r="J43" s="210"/>
-      <c r="K43" s="210"/>
-      <c r="L43" s="211"/>
-    </row>
-    <row r="44" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="381" t="s">
+      <c r="C45" s="372"/>
+      <c r="D45" s="372"/>
+      <c r="E45" s="372"/>
+      <c r="F45" s="372"/>
+      <c r="G45" s="372"/>
+      <c r="H45" s="372"/>
+      <c r="I45" s="372"/>
+      <c r="J45" s="372"/>
+      <c r="K45" s="372"/>
+      <c r="L45" s="373"/>
+    </row>
+    <row r="46" spans="1:14" s="57" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="209"/>
+      <c r="B46" s="210"/>
+      <c r="C46" s="210"/>
+      <c r="D46" s="210"/>
+      <c r="E46" s="210"/>
+      <c r="F46" s="210"/>
+      <c r="G46" s="210"/>
+      <c r="H46" s="210"/>
+      <c r="I46" s="210"/>
+      <c r="J46" s="210"/>
+      <c r="K46" s="210"/>
+      <c r="L46" s="211"/>
+    </row>
+    <row r="47" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="381" t="s">
         <v>273</v>
       </c>
-      <c r="B44" s="382"/>
-      <c r="C44" s="382"/>
-      <c r="D44" s="382"/>
-      <c r="E44" s="382"/>
-      <c r="F44" s="382"/>
-      <c r="G44" s="382"/>
-      <c r="H44" s="382"/>
-      <c r="I44" s="382"/>
-      <c r="J44" s="382"/>
-      <c r="K44" s="382"/>
-      <c r="L44" s="383"/>
-    </row>
-    <row r="45" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="212" t="s">
+      <c r="B47" s="382"/>
+      <c r="C47" s="382"/>
+      <c r="D47" s="382"/>
+      <c r="E47" s="382"/>
+      <c r="F47" s="382"/>
+      <c r="G47" s="382"/>
+      <c r="H47" s="382"/>
+      <c r="I47" s="382"/>
+      <c r="J47" s="382"/>
+      <c r="K47" s="382"/>
+      <c r="L47" s="383"/>
+    </row>
+    <row r="48" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="212" t="s">
         <v>271</v>
       </c>
-      <c r="B45" s="379" t="s">
+      <c r="B48" s="372" t="s">
         <v>172</v>
       </c>
-      <c r="C45" s="379"/>
-      <c r="D45" s="379"/>
-      <c r="E45" s="379"/>
-      <c r="F45" s="379"/>
-      <c r="G45" s="379"/>
-      <c r="H45" s="379"/>
-      <c r="I45" s="379"/>
-      <c r="J45" s="379"/>
-      <c r="K45" s="379"/>
-      <c r="L45" s="380"/>
-    </row>
-    <row r="46" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="213" t="s">
+      <c r="C48" s="372"/>
+      <c r="D48" s="372"/>
+      <c r="E48" s="372"/>
+      <c r="F48" s="372"/>
+      <c r="G48" s="372"/>
+      <c r="H48" s="372"/>
+      <c r="I48" s="372"/>
+      <c r="J48" s="372"/>
+      <c r="K48" s="372"/>
+      <c r="L48" s="373"/>
+    </row>
+    <row r="49" spans="1:12" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="213" t="s">
         <v>272</v>
       </c>
-      <c r="B46" s="389" t="s">
+      <c r="B49" s="374" t="s">
         <v>274</v>
       </c>
-      <c r="C46" s="389"/>
-      <c r="D46" s="389"/>
-      <c r="E46" s="389"/>
-      <c r="F46" s="389"/>
-      <c r="G46" s="389"/>
-      <c r="H46" s="389"/>
-      <c r="I46" s="389"/>
-      <c r="J46" s="389"/>
-      <c r="K46" s="389"/>
-      <c r="L46" s="390"/>
-    </row>
-    <row r="47" spans="1:14" s="57" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="157"/>
-      <c r="B47" s="110"/>
-      <c r="C47" s="110"/>
-      <c r="D47" s="110"/>
-      <c r="E47" s="110"/>
-      <c r="F47" s="110"/>
-      <c r="G47" s="110"/>
-      <c r="H47" s="110"/>
-      <c r="I47" s="110"/>
-      <c r="J47" s="110"/>
-      <c r="K47" s="110"/>
-      <c r="L47" s="110"/>
-    </row>
-    <row r="48" spans="1:14" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="391" t="s">
+      <c r="C49" s="374"/>
+      <c r="D49" s="374"/>
+      <c r="E49" s="374"/>
+      <c r="F49" s="374"/>
+      <c r="G49" s="374"/>
+      <c r="H49" s="374"/>
+      <c r="I49" s="374"/>
+      <c r="J49" s="374"/>
+      <c r="K49" s="374"/>
+      <c r="L49" s="375"/>
+    </row>
+    <row r="50" spans="1:12" s="57" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="157"/>
+      <c r="B50" s="110"/>
+      <c r="C50" s="110"/>
+      <c r="D50" s="110"/>
+      <c r="E50" s="110"/>
+      <c r="F50" s="110"/>
+      <c r="G50" s="110"/>
+      <c r="H50" s="110"/>
+      <c r="I50" s="110"/>
+      <c r="J50" s="110"/>
+      <c r="K50" s="110"/>
+      <c r="L50" s="110"/>
+    </row>
+    <row r="51" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="376" t="s">
         <v>200</v>
       </c>
-      <c r="B48" s="392"/>
-      <c r="C48" s="392"/>
-      <c r="D48" s="392"/>
-      <c r="E48" s="392"/>
-      <c r="F48" s="392"/>
-      <c r="G48" s="392"/>
-      <c r="H48" s="392"/>
-      <c r="I48" s="392"/>
-      <c r="J48" s="392"/>
-      <c r="K48" s="392"/>
-      <c r="L48" s="393"/>
-    </row>
-    <row r="49" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="216" t="s">
+      <c r="B51" s="377"/>
+      <c r="C51" s="377"/>
+      <c r="D51" s="377"/>
+      <c r="E51" s="377"/>
+      <c r="F51" s="377"/>
+      <c r="G51" s="377"/>
+      <c r="H51" s="377"/>
+      <c r="I51" s="377"/>
+      <c r="J51" s="377"/>
+      <c r="K51" s="377"/>
+      <c r="L51" s="378"/>
+    </row>
+    <row r="52" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="216" t="s">
         <v>173</v>
       </c>
-      <c r="B49" s="158"/>
-      <c r="C49" s="158"/>
-      <c r="D49" s="158"/>
-      <c r="E49" s="158"/>
-      <c r="F49" s="158"/>
-      <c r="G49" s="158"/>
-      <c r="H49" s="158"/>
-      <c r="I49" s="158"/>
-      <c r="J49" s="158"/>
-      <c r="K49" s="158"/>
-      <c r="L49" s="159"/>
-    </row>
-    <row r="50" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="82"/>
-      <c r="C50" s="82"/>
-      <c r="D50" s="82"/>
-      <c r="E50" s="82"/>
-      <c r="F50" s="82"/>
-      <c r="G50" s="82"/>
-      <c r="H50" s="82"/>
-      <c r="I50" s="82"/>
-      <c r="J50" s="82"/>
-      <c r="K50" s="82"/>
-      <c r="L50" s="82"/>
-    </row>
-    <row r="51" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="160" t="s">
+      <c r="B52" s="158"/>
+      <c r="C52" s="158"/>
+      <c r="D52" s="158"/>
+      <c r="E52" s="158"/>
+      <c r="F52" s="158"/>
+      <c r="G52" s="158"/>
+      <c r="H52" s="158"/>
+      <c r="I52" s="158"/>
+      <c r="J52" s="158"/>
+      <c r="K52" s="158"/>
+      <c r="L52" s="159"/>
+    </row>
+    <row r="53" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B53" s="82"/>
+      <c r="C53" s="82"/>
+      <c r="D53" s="82"/>
+      <c r="E53" s="82"/>
+      <c r="F53" s="82"/>
+      <c r="G53" s="82"/>
+      <c r="H53" s="82"/>
+      <c r="I53" s="82"/>
+      <c r="J53" s="82"/>
+      <c r="K53" s="82"/>
+      <c r="L53" s="82"/>
+    </row>
+    <row r="54" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="160" t="s">
         <v>126</v>
       </c>
-      <c r="B51" s="161"/>
-      <c r="C51" s="161"/>
-      <c r="D51" s="162"/>
-      <c r="E51" s="161"/>
-      <c r="F51" s="161"/>
-      <c r="G51" s="161"/>
-      <c r="H51" s="161"/>
-      <c r="I51" s="161"/>
-      <c r="J51" s="161"/>
-      <c r="K51" s="161"/>
-      <c r="L51" s="163"/>
-    </row>
-    <row r="52" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="164"/>
-      <c r="B52" s="165" t="s">
-        <v>24</v>
-      </c>
-      <c r="C52" s="166" t="s">
-        <v>427</v>
-      </c>
-      <c r="D52" s="166"/>
-      <c r="E52" s="166"/>
-      <c r="F52" s="166"/>
-      <c r="G52" s="166"/>
-      <c r="H52" s="166"/>
-      <c r="I52" s="166"/>
-      <c r="J52" s="166"/>
-      <c r="K52" s="166"/>
-      <c r="L52" s="167"/>
-    </row>
-    <row r="53" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="164"/>
-      <c r="B53" s="165" t="s">
-        <v>41</v>
-      </c>
-      <c r="C53" s="166" t="s">
-        <v>51</v>
-      </c>
-      <c r="D53" s="166"/>
-      <c r="E53" s="166"/>
-      <c r="F53" s="166"/>
-      <c r="G53" s="166"/>
-      <c r="H53" s="166"/>
-      <c r="I53" s="166"/>
-      <c r="J53" s="166"/>
-      <c r="K53" s="166"/>
-      <c r="L53" s="167"/>
-    </row>
-    <row r="54" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="164"/>
-      <c r="B54" s="165" t="s">
-        <v>24</v>
-      </c>
-      <c r="C54" s="342" t="s">
-        <v>262</v>
-      </c>
-      <c r="D54" s="342"/>
-      <c r="E54" s="342"/>
-      <c r="F54" s="342"/>
-      <c r="G54" s="342"/>
-      <c r="H54" s="342"/>
-      <c r="I54" s="342"/>
-      <c r="J54" s="342"/>
-      <c r="K54" s="342"/>
-      <c r="L54" s="363"/>
-    </row>
-    <row r="55" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B54" s="161"/>
+      <c r="C54" s="161"/>
+      <c r="D54" s="162"/>
+      <c r="E54" s="161"/>
+      <c r="F54" s="161"/>
+      <c r="G54" s="161"/>
+      <c r="H54" s="161"/>
+      <c r="I54" s="161"/>
+      <c r="J54" s="161"/>
+      <c r="K54" s="161"/>
+      <c r="L54" s="163"/>
+    </row>
+    <row r="55" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="164"/>
       <c r="B55" s="165" t="s">
-        <v>263</v>
-      </c>
-      <c r="C55" s="342" t="s">
-        <v>264</v>
-      </c>
-      <c r="D55" s="342"/>
-      <c r="E55" s="342"/>
-      <c r="F55" s="342"/>
-      <c r="G55" s="342"/>
-      <c r="H55" s="342"/>
-      <c r="I55" s="342"/>
-      <c r="J55" s="342"/>
-      <c r="K55" s="342"/>
-      <c r="L55" s="363"/>
-    </row>
-    <row r="56" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="C55" s="166" t="s">
+        <v>427</v>
+      </c>
+      <c r="D55" s="166"/>
+      <c r="E55" s="166"/>
+      <c r="F55" s="166"/>
+      <c r="G55" s="166"/>
+      <c r="H55" s="166"/>
+      <c r="I55" s="166"/>
+      <c r="J55" s="166"/>
+      <c r="K55" s="166"/>
+      <c r="L55" s="167"/>
+    </row>
+    <row r="56" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="164"/>
       <c r="B56" s="165" t="s">
-        <v>327</v>
-      </c>
-      <c r="C56" s="342" t="s">
-        <v>328</v>
-      </c>
-      <c r="D56" s="342"/>
-      <c r="E56" s="342"/>
-      <c r="F56" s="342"/>
-      <c r="G56" s="342"/>
-      <c r="H56" s="342"/>
-      <c r="I56" s="342"/>
-      <c r="J56" s="342"/>
-      <c r="K56" s="342"/>
-      <c r="L56" s="363"/>
-    </row>
-    <row r="57" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+      <c r="C56" s="166" t="s">
+        <v>51</v>
+      </c>
+      <c r="D56" s="166"/>
+      <c r="E56" s="166"/>
+      <c r="F56" s="166"/>
+      <c r="G56" s="166"/>
+      <c r="H56" s="166"/>
+      <c r="I56" s="166"/>
+      <c r="J56" s="166"/>
+      <c r="K56" s="166"/>
+      <c r="L56" s="167"/>
+    </row>
+    <row r="57" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="164"/>
       <c r="B57" s="165" t="s">
-        <v>98</v>
-      </c>
-      <c r="C57" s="342" t="s">
-        <v>99</v>
-      </c>
-      <c r="D57" s="342"/>
-      <c r="E57" s="342"/>
-      <c r="F57" s="342"/>
-      <c r="G57" s="342"/>
-      <c r="H57" s="342"/>
-      <c r="I57" s="342"/>
-      <c r="J57" s="342"/>
-      <c r="K57" s="342"/>
-      <c r="L57" s="363"/>
-    </row>
-    <row r="58" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="C57" s="379" t="s">
+        <v>262</v>
+      </c>
+      <c r="D57" s="379"/>
+      <c r="E57" s="379"/>
+      <c r="F57" s="379"/>
+      <c r="G57" s="379"/>
+      <c r="H57" s="379"/>
+      <c r="I57" s="379"/>
+      <c r="J57" s="379"/>
+      <c r="K57" s="379"/>
+      <c r="L57" s="380"/>
+    </row>
+    <row r="58" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="164"/>
       <c r="B58" s="165" t="s">
-        <v>198</v>
-      </c>
-      <c r="C58" s="342" t="s">
-        <v>199</v>
-      </c>
-      <c r="D58" s="342"/>
-      <c r="E58" s="342"/>
-      <c r="F58" s="342"/>
-      <c r="G58" s="342"/>
-      <c r="H58" s="342"/>
-      <c r="I58" s="342"/>
-      <c r="J58" s="342"/>
-      <c r="K58" s="342"/>
-      <c r="L58" s="363"/>
-    </row>
-    <row r="59" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+        <v>263</v>
+      </c>
+      <c r="C58" s="379" t="s">
+        <v>264</v>
+      </c>
+      <c r="D58" s="379"/>
+      <c r="E58" s="379"/>
+      <c r="F58" s="379"/>
+      <c r="G58" s="379"/>
+      <c r="H58" s="379"/>
+      <c r="I58" s="379"/>
+      <c r="J58" s="379"/>
+      <c r="K58" s="379"/>
+      <c r="L58" s="380"/>
+    </row>
+    <row r="59" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="164"/>
       <c r="B59" s="165" t="s">
-        <v>163</v>
-      </c>
-      <c r="C59" s="342" t="s">
-        <v>466</v>
-      </c>
-      <c r="D59" s="343"/>
-      <c r="E59" s="343"/>
-      <c r="F59" s="343"/>
-      <c r="G59" s="343"/>
-      <c r="H59" s="343"/>
-      <c r="I59" s="343"/>
-      <c r="J59" s="343"/>
-      <c r="K59" s="343"/>
-      <c r="L59" s="344"/>
-    </row>
-    <row r="60" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>327</v>
+      </c>
+      <c r="C59" s="379" t="s">
+        <v>328</v>
+      </c>
+      <c r="D59" s="379"/>
+      <c r="E59" s="379"/>
+      <c r="F59" s="379"/>
+      <c r="G59" s="379"/>
+      <c r="H59" s="379"/>
+      <c r="I59" s="379"/>
+      <c r="J59" s="379"/>
+      <c r="K59" s="379"/>
+      <c r="L59" s="380"/>
+    </row>
+    <row r="60" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="164"/>
       <c r="B60" s="165" t="s">
-        <v>393</v>
-      </c>
-      <c r="C60" s="342" t="s">
-        <v>394</v>
-      </c>
-      <c r="D60" s="342"/>
-      <c r="E60" s="342"/>
-      <c r="F60" s="342"/>
-      <c r="G60" s="342"/>
-      <c r="H60" s="342"/>
-      <c r="I60" s="342"/>
-      <c r="J60" s="342"/>
-      <c r="K60" s="342"/>
-      <c r="L60" s="363"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+        <v>98</v>
+      </c>
+      <c r="C60" s="379" t="s">
+        <v>99</v>
+      </c>
+      <c r="D60" s="379"/>
+      <c r="E60" s="379"/>
+      <c r="F60" s="379"/>
+      <c r="G60" s="379"/>
+      <c r="H60" s="379"/>
+      <c r="I60" s="379"/>
+      <c r="J60" s="379"/>
+      <c r="K60" s="379"/>
+      <c r="L60" s="380"/>
+    </row>
+    <row r="61" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="164"/>
       <c r="B61" s="165" t="s">
+        <v>198</v>
+      </c>
+      <c r="C61" s="379" t="s">
+        <v>199</v>
+      </c>
+      <c r="D61" s="379"/>
+      <c r="E61" s="379"/>
+      <c r="F61" s="379"/>
+      <c r="G61" s="379"/>
+      <c r="H61" s="379"/>
+      <c r="I61" s="379"/>
+      <c r="J61" s="379"/>
+      <c r="K61" s="379"/>
+      <c r="L61" s="380"/>
+    </row>
+    <row r="62" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="164"/>
+      <c r="B62" s="165" t="s">
+        <v>163</v>
+      </c>
+      <c r="C62" s="379" t="s">
+        <v>466</v>
+      </c>
+      <c r="D62" s="384"/>
+      <c r="E62" s="384"/>
+      <c r="F62" s="384"/>
+      <c r="G62" s="384"/>
+      <c r="H62" s="384"/>
+      <c r="I62" s="384"/>
+      <c r="J62" s="384"/>
+      <c r="K62" s="384"/>
+      <c r="L62" s="385"/>
+    </row>
+    <row r="63" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="164"/>
+      <c r="B63" s="165" t="s">
+        <v>393</v>
+      </c>
+      <c r="C63" s="379" t="s">
+        <v>394</v>
+      </c>
+      <c r="D63" s="379"/>
+      <c r="E63" s="379"/>
+      <c r="F63" s="379"/>
+      <c r="G63" s="379"/>
+      <c r="H63" s="379"/>
+      <c r="I63" s="379"/>
+      <c r="J63" s="379"/>
+      <c r="K63" s="379"/>
+      <c r="L63" s="380"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A64" s="164"/>
+      <c r="B64" s="165" t="s">
         <v>36</v>
       </c>
-      <c r="C61" s="166" t="s">
+      <c r="C64" s="166" t="s">
         <v>37</v>
       </c>
-      <c r="D61" s="166"/>
-      <c r="E61" s="166"/>
-      <c r="F61" s="166"/>
-      <c r="G61" s="166"/>
-      <c r="H61" s="166"/>
-      <c r="I61" s="166"/>
-      <c r="J61" s="166"/>
-      <c r="K61" s="166"/>
-      <c r="L61" s="167"/>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A62" s="168"/>
-      <c r="B62" s="169" t="s">
+      <c r="D64" s="166"/>
+      <c r="E64" s="166"/>
+      <c r="F64" s="166"/>
+      <c r="G64" s="166"/>
+      <c r="H64" s="166"/>
+      <c r="I64" s="166"/>
+      <c r="J64" s="166"/>
+      <c r="K64" s="166"/>
+      <c r="L64" s="167"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A65" s="168"/>
+      <c r="B65" s="169" t="s">
         <v>119</v>
       </c>
-      <c r="C62" s="170" t="s">
+      <c r="C65" s="170" t="s">
         <v>120</v>
       </c>
-      <c r="D62" s="170"/>
-      <c r="E62" s="170"/>
-      <c r="F62" s="170"/>
-      <c r="G62" s="170"/>
-      <c r="H62" s="170"/>
-      <c r="I62" s="170"/>
-      <c r="J62" s="170"/>
-      <c r="K62" s="170"/>
-      <c r="L62" s="171"/>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A64" s="1" t="s">
+      <c r="D65" s="170"/>
+      <c r="E65" s="170"/>
+      <c r="F65" s="170"/>
+      <c r="G65" s="170"/>
+      <c r="H65" s="170"/>
+      <c r="I65" s="170"/>
+      <c r="J65" s="170"/>
+      <c r="K65" s="170"/>
+      <c r="L65" s="171"/>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A67" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A65" s="1" t="s">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A68" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" s="43" t="s">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A70" s="43" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" s="43" t="s">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A71" s="43" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" s="43"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" s="1" t="s">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A72" s="43"/>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" s="43" t="s">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A75" s="43" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A73" s="43"/>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A74" s="229" t="s">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A76" s="43"/>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A77" s="229" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A75" s="228" t="s">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A78" s="228" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A76" s="43" t="s">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A79" s="43" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A77" s="43"/>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A78" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A79" s="43" t="s">
-        <v>265</v>
-      </c>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A80" s="43"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A82" s="43" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A84" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="388" t="s">
+    <row r="85" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A85" s="369" t="s">
         <v>397</v>
       </c>
-      <c r="B82" s="388"/>
-      <c r="C82" s="388"/>
-      <c r="D82" s="388"/>
-      <c r="E82" s="388"/>
-      <c r="F82" s="388"/>
-      <c r="G82" s="388"/>
-      <c r="H82" s="388"/>
-      <c r="I82" s="388"/>
-      <c r="J82" s="388"/>
-      <c r="K82" s="388"/>
-      <c r="L82" s="388"/>
-    </row>
-    <row r="87" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="88" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35"/>
+      <c r="B85" s="369"/>
+      <c r="C85" s="369"/>
+      <c r="D85" s="369"/>
+      <c r="E85" s="369"/>
+      <c r="F85" s="369"/>
+      <c r="G85" s="369"/>
+      <c r="H85" s="369"/>
+      <c r="I85" s="369"/>
+      <c r="J85" s="369"/>
+      <c r="K85" s="369"/>
+      <c r="L85" s="369"/>
+    </row>
+    <row r="90" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="91" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="B14:L14"/>
-    <mergeCell ref="B15:L15"/>
-    <mergeCell ref="A82:L82"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B42:L42"/>
-    <mergeCell ref="B45:L45"/>
-    <mergeCell ref="B46:L46"/>
-    <mergeCell ref="A48:L48"/>
-    <mergeCell ref="C54:L54"/>
-    <mergeCell ref="C57:L57"/>
-    <mergeCell ref="C58:L58"/>
-    <mergeCell ref="C55:L55"/>
-    <mergeCell ref="C60:L60"/>
-    <mergeCell ref="A44:L44"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="C56:L56"/>
-    <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B27:L27"/>
-    <mergeCell ref="B28:L28"/>
-    <mergeCell ref="B29:L29"/>
-    <mergeCell ref="B30:L30"/>
-    <mergeCell ref="B31:L31"/>
-    <mergeCell ref="B32:L32"/>
-    <mergeCell ref="B33:L33"/>
-    <mergeCell ref="A34:L34"/>
-    <mergeCell ref="B35:L35"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="B38:L38"/>
-    <mergeCell ref="B37:L37"/>
-    <mergeCell ref="B39:L39"/>
-    <mergeCell ref="C59:L59"/>
-    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="C62:L62"/>
+    <mergeCell ref="A29:L29"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="N4:R4"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="A20:L20"/>
-    <mergeCell ref="A21:L21"/>
     <mergeCell ref="A22:L22"/>
     <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
     <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A28:L28"/>
     <mergeCell ref="B7:L7"/>
     <mergeCell ref="B8:L8"/>
     <mergeCell ref="A10:L10"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="C59:L59"/>
+    <mergeCell ref="B43:L43"/>
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B31:L31"/>
+    <mergeCell ref="B32:L32"/>
+    <mergeCell ref="B33:L33"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="B35:L35"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B42:L42"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B18:L18"/>
+    <mergeCell ref="A85:L85"/>
+    <mergeCell ref="B44:L44"/>
+    <mergeCell ref="B45:L45"/>
+    <mergeCell ref="B48:L48"/>
+    <mergeCell ref="B49:L49"/>
+    <mergeCell ref="A51:L51"/>
+    <mergeCell ref="C57:L57"/>
+    <mergeCell ref="C60:L60"/>
+    <mergeCell ref="C61:L61"/>
+    <mergeCell ref="C58:L58"/>
+    <mergeCell ref="C63:L63"/>
+    <mergeCell ref="A47:L47"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A67" r:id="rId1" xr:uid="{C9866D44-2827-49D7-B9C3-89CF23FACDC1}"/>
-    <hyperlink ref="A68" r:id="rId2" xr:uid="{66F54200-A2AB-43DA-A0E0-F2A25A075EE5}"/>
-    <hyperlink ref="A79" r:id="rId3" xr:uid="{A0F8DE06-D9FC-495F-9A01-AA199CB82365}"/>
-    <hyperlink ref="A48:L48" r:id="rId4" display="LETS START (visual directions as pdf)" xr:uid="{0D075873-7EBB-4309-B00A-6A62EA192A0C}"/>
-    <hyperlink ref="A49" r:id="rId5" xr:uid="{25154A32-BA44-496E-9945-086DE0980DBD}"/>
-    <hyperlink ref="A76" r:id="rId6" xr:uid="{AA792CE4-4071-4CE8-87C6-993A0BA6C6A5}"/>
-    <hyperlink ref="E17" r:id="rId7" xr:uid="{218FEB9D-6782-4420-9DCE-4D6F20EDE6D5}"/>
-    <hyperlink ref="A72" r:id="rId8" xr:uid="{E4DF21D7-58D7-F94D-825D-01575427A9FE}"/>
+    <hyperlink ref="A70" r:id="rId1" xr:uid="{C9866D44-2827-49D7-B9C3-89CF23FACDC1}"/>
+    <hyperlink ref="A71" r:id="rId2" xr:uid="{66F54200-A2AB-43DA-A0E0-F2A25A075EE5}"/>
+    <hyperlink ref="A82" r:id="rId3" xr:uid="{A0F8DE06-D9FC-495F-9A01-AA199CB82365}"/>
+    <hyperlink ref="A51:L51" r:id="rId4" display="LETS START (visual directions as pdf)" xr:uid="{0D075873-7EBB-4309-B00A-6A62EA192A0C}"/>
+    <hyperlink ref="A52" r:id="rId5" xr:uid="{25154A32-BA44-496E-9945-086DE0980DBD}"/>
+    <hyperlink ref="A79" r:id="rId6" xr:uid="{AA792CE4-4071-4CE8-87C6-993A0BA6C6A5}"/>
+    <hyperlink ref="E20" r:id="rId7" xr:uid="{218FEB9D-6782-4420-9DCE-4D6F20EDE6D5}"/>
+    <hyperlink ref="A75" r:id="rId8" xr:uid="{E4DF21D7-58D7-F94D-825D-01575427A9FE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId9"/>
@@ -17102,82 +17225,82 @@
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="438" t="s">
+      <c r="A3" s="439" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="438"/>
-      <c r="C3" s="438"/>
+      <c r="B3" s="439"/>
+      <c r="C3" s="439"/>
       <c r="D3" s="125" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="439" t="s">
+      <c r="A4" s="440" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="439"/>
-      <c r="C4" s="439"/>
+      <c r="B4" s="440"/>
+      <c r="C4" s="440"/>
       <c r="D4" s="172" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="443" t="s">
+      <c r="A5" s="444" t="s">
         <v>183</v>
       </c>
-      <c r="B5" s="440"/>
-      <c r="C5" s="440"/>
+      <c r="B5" s="441"/>
+      <c r="C5" s="441"/>
       <c r="D5" s="173" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="57.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="441" t="s">
+      <c r="A6" s="442" t="s">
         <v>184</v>
       </c>
-      <c r="B6" s="441"/>
-      <c r="C6" s="441"/>
+      <c r="B6" s="442"/>
+      <c r="C6" s="442"/>
       <c r="D6" s="174" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="442" t="s">
+      <c r="A7" s="443" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="442"/>
-      <c r="C7" s="442"/>
+      <c r="B7" s="443"/>
+      <c r="C7" s="443"/>
       <c r="D7" s="175" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="439" t="s">
+      <c r="A11" s="440" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="439"/>
-      <c r="C11" s="439"/>
+      <c r="B11" s="440"/>
+      <c r="C11" s="440"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="440" t="s">
+      <c r="A12" s="441" t="s">
         <v>113</v>
       </c>
-      <c r="B12" s="440"/>
-      <c r="C12" s="440"/>
+      <c r="B12" s="441"/>
+      <c r="C12" s="441"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="441" t="s">
+      <c r="A13" s="442" t="s">
         <v>114</v>
       </c>
-      <c r="B13" s="441"/>
-      <c r="C13" s="441"/>
+      <c r="B13" s="442"/>
+      <c r="C13" s="442"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="442" t="s">
+      <c r="A14" s="443" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="442"/>
-      <c r="C14" s="442"/>
+      <c r="B14" s="443"/>
+      <c r="C14" s="443"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -17438,28 +17561,28 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="33" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="444" t="s">
+      <c r="A2" s="445" t="s">
         <v>420</v>
       </c>
-      <c r="B2" s="445"/>
-      <c r="C2" s="445"/>
-      <c r="D2" s="445"/>
-      <c r="E2" s="445"/>
-      <c r="F2" s="445"/>
-      <c r="G2" s="445"/>
-      <c r="H2" s="445"/>
-      <c r="I2" s="445"/>
-      <c r="J2" s="445"/>
-      <c r="K2" s="445"/>
-      <c r="L2" s="445"/>
-      <c r="M2" s="445"/>
-      <c r="N2" s="445"/>
-      <c r="O2" s="445"/>
-      <c r="P2" s="445"/>
-      <c r="Q2" s="445"/>
-      <c r="R2" s="445"/>
-      <c r="S2" s="445"/>
-      <c r="T2" s="445"/>
+      <c r="B2" s="446"/>
+      <c r="C2" s="446"/>
+      <c r="D2" s="446"/>
+      <c r="E2" s="446"/>
+      <c r="F2" s="446"/>
+      <c r="G2" s="446"/>
+      <c r="H2" s="446"/>
+      <c r="I2" s="446"/>
+      <c r="J2" s="446"/>
+      <c r="K2" s="446"/>
+      <c r="L2" s="446"/>
+      <c r="M2" s="446"/>
+      <c r="N2" s="446"/>
+      <c r="O2" s="446"/>
+      <c r="P2" s="446"/>
+      <c r="Q2" s="446"/>
+      <c r="R2" s="446"/>
+      <c r="S2" s="446"/>
+      <c r="T2" s="446"/>
     </row>
     <row r="3" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
@@ -18849,16 +18972,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="394" t="str">
+      <c r="A1" s="343" t="str">
         <f>'ReadMe-Directions'!A1</f>
         <v>Immersive Model for Lake Mead based on the Principle of Divide Reservoir Inflow</v>
       </c>
-      <c r="B1" s="394"/>
-      <c r="C1" s="394"/>
-      <c r="D1" s="394"/>
-      <c r="E1" s="394"/>
-      <c r="F1" s="394"/>
-      <c r="G1" s="394"/>
+      <c r="B1" s="343"/>
+      <c r="C1" s="343"/>
+      <c r="D1" s="343"/>
+      <c r="E1" s="343"/>
+      <c r="F1" s="343"/>
+      <c r="G1" s="343"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -18867,15 +18990,15 @@
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="402" t="s">
+      <c r="A3" s="351" t="s">
         <v>190</v>
       </c>
-      <c r="B3" s="402"/>
-      <c r="C3" s="402"/>
-      <c r="D3" s="402"/>
-      <c r="E3" s="402"/>
-      <c r="F3" s="402"/>
-      <c r="G3" s="402"/>
+      <c r="B3" s="351"/>
+      <c r="C3" s="351"/>
+      <c r="D3" s="351"/>
+      <c r="E3" s="351"/>
+      <c r="F3" s="351"/>
+      <c r="G3" s="351"/>
       <c r="H3" s="82"/>
       <c r="I3" s="82"/>
       <c r="J3" s="82"/>
@@ -18891,13 +19014,13 @@
       <c r="B4" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="403" t="s">
+      <c r="C4" s="352" t="s">
         <v>259</v>
       </c>
-      <c r="D4" s="404"/>
-      <c r="E4" s="404"/>
-      <c r="F4" s="404"/>
-      <c r="G4" s="405"/>
+      <c r="D4" s="353"/>
+      <c r="E4" s="353"/>
+      <c r="F4" s="353"/>
+      <c r="G4" s="354"/>
       <c r="N4" s="138" t="s">
         <v>329</v>
       </c>
@@ -18907,11 +19030,11 @@
         <v>238</v>
       </c>
       <c r="B5" s="111"/>
-      <c r="C5" s="406"/>
-      <c r="D5" s="401"/>
-      <c r="E5" s="401"/>
-      <c r="F5" s="401"/>
-      <c r="G5" s="401"/>
+      <c r="C5" s="355"/>
+      <c r="D5" s="350"/>
+      <c r="E5" s="350"/>
+      <c r="F5" s="350"/>
+      <c r="G5" s="350"/>
       <c r="N5" s="138"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -18919,11 +19042,11 @@
         <v>202</v>
       </c>
       <c r="B6" s="111"/>
-      <c r="C6" s="406"/>
-      <c r="D6" s="401"/>
-      <c r="E6" s="401"/>
-      <c r="F6" s="401"/>
-      <c r="G6" s="401"/>
+      <c r="C6" s="355"/>
+      <c r="D6" s="350"/>
+      <c r="E6" s="350"/>
+      <c r="F6" s="350"/>
+      <c r="G6" s="350"/>
       <c r="N6" s="139"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -18931,11 +19054,11 @@
         <v>203</v>
       </c>
       <c r="B7" s="111"/>
-      <c r="C7" s="406"/>
-      <c r="D7" s="401"/>
-      <c r="E7" s="401"/>
-      <c r="F7" s="401"/>
-      <c r="G7" s="401"/>
+      <c r="C7" s="355"/>
+      <c r="D7" s="350"/>
+      <c r="E7" s="350"/>
+      <c r="F7" s="350"/>
+      <c r="G7" s="350"/>
       <c r="N7" s="139"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -18943,11 +19066,11 @@
         <v>204</v>
       </c>
       <c r="B8" s="88"/>
-      <c r="C8" s="401"/>
-      <c r="D8" s="401"/>
-      <c r="E8" s="401"/>
-      <c r="F8" s="401"/>
-      <c r="G8" s="401"/>
+      <c r="C8" s="350"/>
+      <c r="D8" s="350"/>
+      <c r="E8" s="350"/>
+      <c r="F8" s="350"/>
+      <c r="G8" s="350"/>
       <c r="N8" s="139"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -18955,11 +19078,11 @@
         <v>18</v>
       </c>
       <c r="B9" s="88"/>
-      <c r="C9" s="407"/>
-      <c r="D9" s="407"/>
-      <c r="E9" s="407"/>
-      <c r="F9" s="407"/>
-      <c r="G9" s="407"/>
+      <c r="C9" s="356"/>
+      <c r="D9" s="356"/>
+      <c r="E9" s="356"/>
+      <c r="F9" s="356"/>
+      <c r="G9" s="356"/>
       <c r="N9" s="139"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -18967,11 +19090,11 @@
         <v>277</v>
       </c>
       <c r="B10" s="88"/>
-      <c r="C10" s="401"/>
-      <c r="D10" s="401"/>
-      <c r="E10" s="401"/>
-      <c r="F10" s="401"/>
-      <c r="G10" s="401"/>
+      <c r="C10" s="350"/>
+      <c r="D10" s="350"/>
+      <c r="E10" s="350"/>
+      <c r="F10" s="350"/>
+      <c r="G10" s="350"/>
       <c r="N10" s="139"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
@@ -18984,36 +19107,36 @@
       <c r="A12" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B12" s="408" t="s">
+      <c r="B12" s="357" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="409"/>
-      <c r="D12" s="410"/>
+      <c r="C12" s="358"/>
+      <c r="D12" s="359"/>
       <c r="N12" s="138" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B13" s="411" t="s">
+      <c r="B13" s="360" t="s">
         <v>189</v>
       </c>
-      <c r="C13" s="412"/>
-      <c r="D13" s="413"/>
+      <c r="C13" s="361"/>
+      <c r="D13" s="362"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B14" s="395" t="s">
+      <c r="B14" s="344" t="s">
         <v>184</v>
       </c>
-      <c r="C14" s="396"/>
-      <c r="D14" s="397"/>
+      <c r="C14" s="345"/>
+      <c r="D14" s="346"/>
       <c r="N14" s="139"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="398" t="s">
+      <c r="B15" s="347" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="399"/>
-      <c r="D15" s="400"/>
+      <c r="C15" s="348"/>
+      <c r="D15" s="349"/>
       <c r="N15" s="139"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
@@ -20722,7 +20845,7 @@
       <c r="M63" s="98" t="s">
         <v>25</v>
       </c>
-      <c r="N63" s="136" t="s">
+      <c r="N63" s="138" t="s">
         <v>146</v>
       </c>
     </row>
@@ -24393,62 +24516,62 @@
       <c r="G5" s="185" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="422" t="s">
+      <c r="I5" s="428" t="s">
         <v>423</v>
       </c>
-      <c r="J5" s="423"/>
-      <c r="K5" s="423"/>
-      <c r="L5" s="423"/>
-      <c r="M5" s="423"/>
-      <c r="N5" s="423"/>
-      <c r="O5" s="423"/>
-      <c r="P5" s="423"/>
-      <c r="Q5" s="423"/>
-      <c r="R5" s="423"/>
-      <c r="S5" s="423"/>
-      <c r="T5" s="423"/>
-      <c r="U5" s="423"/>
-      <c r="V5" s="423"/>
-      <c r="W5" s="424"/>
+      <c r="J5" s="429"/>
+      <c r="K5" s="429"/>
+      <c r="L5" s="429"/>
+      <c r="M5" s="429"/>
+      <c r="N5" s="429"/>
+      <c r="O5" s="429"/>
+      <c r="P5" s="429"/>
+      <c r="Q5" s="429"/>
+      <c r="R5" s="429"/>
+      <c r="S5" s="429"/>
+      <c r="T5" s="429"/>
+      <c r="U5" s="429"/>
+      <c r="V5" s="429"/>
+      <c r="W5" s="430"/>
       <c r="Y5" s="192"/>
       <c r="Z5" s="192"/>
       <c r="AA5" s="192"/>
       <c r="AB5" s="334"/>
     </row>
     <row r="6" spans="1:53" s="184" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="414" t="s">
+      <c r="B6" s="417" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="415"/>
-      <c r="D6" s="415"/>
-      <c r="E6" s="415"/>
-      <c r="F6" s="415"/>
-      <c r="G6" s="416"/>
-      <c r="I6" s="425" t="s">
+      <c r="C6" s="418"/>
+      <c r="D6" s="418"/>
+      <c r="E6" s="418"/>
+      <c r="F6" s="418"/>
+      <c r="G6" s="419"/>
+      <c r="I6" s="431" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="427" t="s">
+      <c r="J6" s="415" t="s">
         <v>409</v>
       </c>
-      <c r="K6" s="427" t="s">
+      <c r="K6" s="415" t="s">
         <v>408</v>
       </c>
-      <c r="L6" s="428" t="s">
+      <c r="L6" s="433" t="s">
         <v>215</v>
       </c>
-      <c r="M6" s="429"/>
-      <c r="N6" s="429"/>
-      <c r="O6" s="429"/>
-      <c r="P6" s="429"/>
-      <c r="Q6" s="430"/>
-      <c r="R6" s="431" t="s">
+      <c r="M6" s="434"/>
+      <c r="N6" s="434"/>
+      <c r="O6" s="434"/>
+      <c r="P6" s="434"/>
+      <c r="Q6" s="435"/>
+      <c r="R6" s="420" t="s">
         <v>216</v>
       </c>
-      <c r="S6" s="432"/>
-      <c r="T6" s="432"/>
-      <c r="U6" s="432"/>
-      <c r="V6" s="432"/>
-      <c r="W6" s="433"/>
+      <c r="S6" s="421"/>
+      <c r="T6" s="421"/>
+      <c r="U6" s="421"/>
+      <c r="V6" s="421"/>
+      <c r="W6" s="422"/>
       <c r="Y6" s="307"/>
       <c r="Z6" s="307"/>
       <c r="AA6" s="307"/>
@@ -24474,9 +24597,9 @@
         <f>SUM(C7:F7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="426"/>
-      <c r="J7" s="426"/>
-      <c r="K7" s="426"/>
+      <c r="I7" s="432"/>
+      <c r="J7" s="432"/>
+      <c r="K7" s="432"/>
       <c r="L7" s="186" t="s">
         <v>410</v>
       </c>
@@ -24680,14 +24803,14 @@
       <c r="AZ9" s="285"/>
     </row>
     <row r="10" spans="1:53" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.3">
-      <c r="B10" s="417" t="s">
+      <c r="B10" s="423" t="s">
         <v>237</v>
       </c>
-      <c r="C10" s="417"/>
-      <c r="D10" s="417"/>
-      <c r="E10" s="417"/>
-      <c r="F10" s="417"/>
-      <c r="G10" s="417"/>
+      <c r="C10" s="423"/>
+      <c r="D10" s="423"/>
+      <c r="E10" s="423"/>
+      <c r="F10" s="423"/>
+      <c r="G10" s="423"/>
       <c r="I10" s="244" t="s">
         <v>231</v>
       </c>
@@ -25171,13 +25294,13 @@
       <c r="B16" s="193" t="s">
         <v>234</v>
       </c>
-      <c r="C16" s="418" t="s">
+      <c r="C16" s="424" t="s">
         <v>235</v>
       </c>
-      <c r="D16" s="419"/>
-      <c r="E16" s="419"/>
-      <c r="F16" s="419"/>
-      <c r="G16" s="420"/>
+      <c r="D16" s="425"/>
+      <c r="E16" s="425"/>
+      <c r="F16" s="425"/>
+      <c r="G16" s="426"/>
       <c r="I16" s="244" t="s">
         <v>404</v>
       </c>
@@ -25293,59 +25416,59 @@
     </row>
     <row r="18" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.3"/>
     <row r="19" spans="2:58" s="192" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I19" s="421" t="s">
+      <c r="I19" s="427" t="s">
         <v>424</v>
       </c>
-      <c r="J19" s="421"/>
-      <c r="K19" s="421"/>
-      <c r="L19" s="421"/>
-      <c r="M19" s="421"/>
-      <c r="N19" s="421"/>
-      <c r="O19" s="421"/>
-      <c r="P19" s="421"/>
-      <c r="Q19" s="421"/>
-      <c r="R19" s="421"/>
-      <c r="S19" s="421"/>
-      <c r="T19" s="421"/>
-      <c r="U19" s="421"/>
+      <c r="J19" s="427"/>
+      <c r="K19" s="427"/>
+      <c r="L19" s="427"/>
+      <c r="M19" s="427"/>
+      <c r="N19" s="427"/>
+      <c r="O19" s="427"/>
+      <c r="P19" s="427"/>
+      <c r="Q19" s="427"/>
+      <c r="R19" s="427"/>
+      <c r="S19" s="427"/>
+      <c r="T19" s="427"/>
+      <c r="U19" s="427"/>
       <c r="Z19" s="250"/>
       <c r="AA19" s="250"/>
       <c r="AB19" s="250"/>
       <c r="AC19" s="250"/>
     </row>
     <row r="20" spans="2:58" s="192" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="427" t="s">
+      <c r="I20" s="415" t="s">
         <v>13</v>
       </c>
-      <c r="J20" s="427" t="s">
+      <c r="J20" s="415" t="s">
         <v>213</v>
       </c>
-      <c r="K20" s="427" t="s">
+      <c r="K20" s="415" t="s">
         <v>214</v>
       </c>
-      <c r="L20" s="414" t="s">
+      <c r="L20" s="417" t="s">
         <v>215</v>
       </c>
-      <c r="M20" s="415"/>
-      <c r="N20" s="415"/>
-      <c r="O20" s="415"/>
-      <c r="P20" s="416"/>
-      <c r="Q20" s="431" t="s">
+      <c r="M20" s="418"/>
+      <c r="N20" s="418"/>
+      <c r="O20" s="418"/>
+      <c r="P20" s="419"/>
+      <c r="Q20" s="420" t="s">
         <v>216</v>
       </c>
-      <c r="R20" s="432"/>
-      <c r="S20" s="432"/>
-      <c r="T20" s="432"/>
-      <c r="U20" s="433"/>
+      <c r="R20" s="421"/>
+      <c r="S20" s="421"/>
+      <c r="T20" s="421"/>
+      <c r="U20" s="422"/>
       <c r="Z20" s="254"/>
       <c r="AA20" s="254"/>
       <c r="AB20" s="254"/>
       <c r="AC20" s="254"/>
     </row>
     <row r="21" spans="2:58" s="192" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I21" s="434"/>
-      <c r="J21" s="434"/>
-      <c r="K21" s="434"/>
+      <c r="I21" s="416"/>
+      <c r="J21" s="416"/>
+      <c r="K21" s="416"/>
       <c r="L21" s="186" t="s">
         <v>218</v>
       </c>
@@ -26367,11 +26490,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:P20"/>
-    <mergeCell ref="Q20:U20"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="C16:G16"/>
@@ -26382,6 +26500,11 @@
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:Q6"/>
     <mergeCell ref="R6:W6"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:P20"/>
+    <mergeCell ref="Q20:U20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26714,16 +26837,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="435" t="e">
+      <c r="A1" s="437" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B1" s="435"/>
-      <c r="C1" s="435"/>
-      <c r="D1" s="435"/>
-      <c r="E1" s="435"/>
-      <c r="F1" s="435"/>
-      <c r="G1" s="435"/>
+      <c r="B1" s="437"/>
+      <c r="C1" s="437"/>
+      <c r="D1" s="437"/>
+      <c r="E1" s="437"/>
+      <c r="F1" s="437"/>
+      <c r="G1" s="437"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -26732,15 +26855,15 @@
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="402" t="s">
+      <c r="A3" s="351" t="s">
         <v>177</v>
       </c>
-      <c r="B3" s="402"/>
-      <c r="C3" s="402"/>
-      <c r="D3" s="402"/>
-      <c r="E3" s="402"/>
-      <c r="F3" s="402"/>
-      <c r="G3" s="402"/>
+      <c r="B3" s="351"/>
+      <c r="C3" s="351"/>
+      <c r="D3" s="351"/>
+      <c r="E3" s="351"/>
+      <c r="F3" s="351"/>
+      <c r="G3" s="351"/>
       <c r="H3" s="82"/>
       <c r="I3" s="82"/>
       <c r="J3" s="82"/>
@@ -26756,13 +26879,13 @@
       <c r="B4" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="403" t="s">
+      <c r="C4" s="352" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="404"/>
-      <c r="E4" s="404"/>
-      <c r="F4" s="404"/>
-      <c r="G4" s="405"/>
+      <c r="D4" s="353"/>
+      <c r="E4" s="353"/>
+      <c r="F4" s="353"/>
+      <c r="G4" s="354"/>
       <c r="N4" s="136" t="s">
         <v>128</v>
       </c>
@@ -26772,11 +26895,11 @@
         <v>16</v>
       </c>
       <c r="B5" s="111"/>
-      <c r="C5" s="406"/>
-      <c r="D5" s="401"/>
-      <c r="E5" s="401"/>
-      <c r="F5" s="401"/>
-      <c r="G5" s="401"/>
+      <c r="C5" s="355"/>
+      <c r="D5" s="350"/>
+      <c r="E5" s="350"/>
+      <c r="F5" s="350"/>
+      <c r="G5" s="350"/>
       <c r="N5" s="139"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -26784,11 +26907,11 @@
         <v>17</v>
       </c>
       <c r="B6" s="111"/>
-      <c r="C6" s="406"/>
-      <c r="D6" s="401"/>
-      <c r="E6" s="401"/>
-      <c r="F6" s="401"/>
-      <c r="G6" s="401"/>
+      <c r="C6" s="355"/>
+      <c r="D6" s="350"/>
+      <c r="E6" s="350"/>
+      <c r="F6" s="350"/>
+      <c r="G6" s="350"/>
       <c r="N6" s="139"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -26796,11 +26919,11 @@
         <v>18</v>
       </c>
       <c r="B7" s="111"/>
-      <c r="C7" s="406"/>
-      <c r="D7" s="401"/>
-      <c r="E7" s="401"/>
-      <c r="F7" s="401"/>
-      <c r="G7" s="401"/>
+      <c r="C7" s="355"/>
+      <c r="D7" s="350"/>
+      <c r="E7" s="350"/>
+      <c r="F7" s="350"/>
+      <c r="G7" s="350"/>
       <c r="N7" s="139"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -26808,11 +26931,11 @@
         <v>39</v>
       </c>
       <c r="B8" s="88"/>
-      <c r="C8" s="401"/>
-      <c r="D8" s="401"/>
-      <c r="E8" s="401"/>
-      <c r="F8" s="401"/>
-      <c r="G8" s="401"/>
+      <c r="C8" s="350"/>
+      <c r="D8" s="350"/>
+      <c r="E8" s="350"/>
+      <c r="F8" s="350"/>
+      <c r="G8" s="350"/>
       <c r="N8" s="139"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -26820,11 +26943,11 @@
         <v>162</v>
       </c>
       <c r="B9" s="88"/>
-      <c r="C9" s="407"/>
-      <c r="D9" s="407"/>
-      <c r="E9" s="407"/>
-      <c r="F9" s="407"/>
-      <c r="G9" s="407"/>
+      <c r="C9" s="356"/>
+      <c r="D9" s="356"/>
+      <c r="E9" s="356"/>
+      <c r="F9" s="356"/>
+      <c r="G9" s="356"/>
       <c r="N9" s="139"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -26849,37 +26972,37 @@
       <c r="A12" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B12" s="408" t="s">
+      <c r="B12" s="357" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="409"/>
-      <c r="D12" s="410"/>
+      <c r="C12" s="358"/>
+      <c r="D12" s="359"/>
       <c r="N12" s="138" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B13" s="411" t="s">
+      <c r="B13" s="360" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="412"/>
-      <c r="D13" s="413"/>
+      <c r="C13" s="361"/>
+      <c r="D13" s="362"/>
       <c r="N13" s="139"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B14" s="395" t="s">
+      <c r="B14" s="344" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="396"/>
-      <c r="D14" s="397"/>
+      <c r="C14" s="345"/>
+      <c r="D14" s="346"/>
       <c r="N14" s="139"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="398" t="s">
+      <c r="B15" s="347" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="399"/>
-      <c r="D15" s="400"/>
+      <c r="C15" s="348"/>
+      <c r="D15" s="349"/>
       <c r="N15" s="139"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
@@ -28099,6 +28222,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:G6"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="C9:G9"/>
@@ -28106,12 +28235,6 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N4" r:id="rId1" location="step-1-assign-parties-person-playing-and-strategies" xr:uid="{726B234F-7B54-4D33-A192-8F1604C6B04C}"/>
@@ -28166,26 +28289,26 @@
       </c>
     </row>
     <row r="3" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D3" s="437" t="s">
+      <c r="D3" s="438" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="437"/>
-      <c r="F3" s="437" t="s">
+      <c r="E3" s="438"/>
+      <c r="F3" s="438" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="437"/>
-      <c r="H3" s="437"/>
-      <c r="I3" s="437" t="s">
+      <c r="G3" s="438"/>
+      <c r="H3" s="438"/>
+      <c r="I3" s="438" t="s">
         <v>61</v>
       </c>
-      <c r="J3" s="437"/>
-      <c r="K3" s="437"/>
+      <c r="J3" s="438"/>
+      <c r="K3" s="438"/>
       <c r="L3" s="131"/>
-      <c r="M3" s="437" t="s">
+      <c r="M3" s="438" t="s">
         <v>18</v>
       </c>
-      <c r="N3" s="437"/>
-      <c r="O3" s="437"/>
+      <c r="N3" s="438"/>
+      <c r="O3" s="438"/>
     </row>
     <row r="4" spans="1:16" s="45" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="44" t="s">

</xml_diff>

<commit_message>
changed 2 to 3 purposes
</commit_message>
<xml_diff>
--- a/LakeMeadWaterBankDivideInflow.xlsx
+++ b/LakeMeadWaterBankDivideInflow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anabelle/Documents/LakeMeadDivideInflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E77140F-F2EE-6F4E-801F-6E1CF3CFDBB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0B80CA-4D82-2A47-895F-9A24BEB18854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe-Directions" sheetId="62" r:id="rId1"/>
@@ -1434,74 +1434,6 @@
   </si>
   <si>
     <t>Immersive Model for Lake Mead based on the Principle of Divide Reservoir Inflow</t>
-  </si>
-  <si>
-    <r>
-      <t>The purpose of this tool is to give collaborators the opportunity to immerse in and personify water user roles for a Lake Mead model based on the principle of divide reservoir inflow. The process is:</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A) Divide reservoir inflow</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>B) Subtract evaporation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, and</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> C) Users withdraw and conserve within their available water</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, others choices, and real-time discussion of choices. We see uses of the tool for two purposes:</t>
-    </r>
   </si>
   <si>
     <r>
@@ -2371,6 +2303,74 @@
     <t>We are looking at scenarios within Reclamation’s different modeling methods and scenarios. There is broad agreement that Colorado River
 flows will be more volatile, declining, and have longer-lasting periods of low flow than current adjusted February 24-month study 10th and
  50th percentile flows.</t>
+  </si>
+  <si>
+    <r>
+      <t>The purpose of this tool is to give collaborators the opportunity to immerse in and personify water user roles for a Lake Mead model based on the principle of divide reservoir inflow. The process is:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A) Divide reservoir inflow</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>B) Subtract evaporation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, and</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> C) Users withdraw and conserve within their available water</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, others choices, and real-time discussion of choices. We see uses of the tool for three purposes:</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -4199,13 +4199,97 @@
     <xf numFmtId="0" fontId="1" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -4244,9 +4328,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4265,91 +4346,10 @@
     <xf numFmtId="0" fontId="1" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4412,6 +4412,12 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4420,6 +4426,15 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4451,9 +4466,6 @@
     <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4463,23 +4475,11 @@
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -15976,7 +15976,7 @@
     </row>
     <row r="4" spans="1:18" s="52" customFormat="1" ht="53.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="372" t="s">
-        <v>295</v>
+        <v>483</v>
       </c>
       <c r="B4" s="373"/>
       <c r="C4" s="373"/>
@@ -15996,20 +15996,20 @@
       <c r="R4" s="375"/>
     </row>
     <row r="5" spans="1:18" s="52" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="376" t="s">
-        <v>482</v>
-      </c>
-      <c r="B5" s="377"/>
-      <c r="C5" s="377"/>
-      <c r="D5" s="377"/>
-      <c r="E5" s="377"/>
-      <c r="F5" s="377"/>
-      <c r="G5" s="377"/>
-      <c r="H5" s="377"/>
-      <c r="I5" s="377"/>
-      <c r="J5" s="377"/>
-      <c r="K5" s="377"/>
-      <c r="L5" s="378"/>
+      <c r="A5" s="350" t="s">
+        <v>481</v>
+      </c>
+      <c r="B5" s="351"/>
+      <c r="C5" s="351"/>
+      <c r="D5" s="351"/>
+      <c r="E5" s="351"/>
+      <c r="F5" s="351"/>
+      <c r="G5" s="351"/>
+      <c r="H5" s="351"/>
+      <c r="I5" s="351"/>
+      <c r="J5" s="351"/>
+      <c r="K5" s="351"/>
+      <c r="L5" s="352"/>
       <c r="N5" s="110"/>
       <c r="O5" s="110"/>
       <c r="P5" s="110"/>
@@ -16017,20 +16017,20 @@
       <c r="R5" s="110"/>
     </row>
     <row r="6" spans="1:18" s="52" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="376" t="s">
-        <v>480</v>
-      </c>
-      <c r="B6" s="377"/>
-      <c r="C6" s="377"/>
-      <c r="D6" s="377"/>
-      <c r="E6" s="377"/>
-      <c r="F6" s="377"/>
-      <c r="G6" s="377"/>
-      <c r="H6" s="377"/>
-      <c r="I6" s="377"/>
-      <c r="J6" s="377"/>
-      <c r="K6" s="377"/>
-      <c r="L6" s="378"/>
+      <c r="A6" s="350" t="s">
+        <v>479</v>
+      </c>
+      <c r="B6" s="351"/>
+      <c r="C6" s="351"/>
+      <c r="D6" s="351"/>
+      <c r="E6" s="351"/>
+      <c r="F6" s="351"/>
+      <c r="G6" s="351"/>
+      <c r="H6" s="351"/>
+      <c r="I6" s="351"/>
+      <c r="J6" s="351"/>
+      <c r="K6" s="351"/>
+      <c r="L6" s="352"/>
       <c r="N6" s="110"/>
       <c r="O6" s="110"/>
       <c r="P6" s="110"/>
@@ -16038,20 +16038,20 @@
       <c r="R6" s="110"/>
     </row>
     <row r="7" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="376" t="s">
-        <v>481</v>
-      </c>
-      <c r="B7" s="377"/>
-      <c r="C7" s="377"/>
-      <c r="D7" s="377"/>
-      <c r="E7" s="377"/>
-      <c r="F7" s="377"/>
-      <c r="G7" s="377"/>
-      <c r="H7" s="377"/>
-      <c r="I7" s="377"/>
-      <c r="J7" s="377"/>
-      <c r="K7" s="377"/>
-      <c r="L7" s="378"/>
+      <c r="A7" s="350" t="s">
+        <v>480</v>
+      </c>
+      <c r="B7" s="351"/>
+      <c r="C7" s="351"/>
+      <c r="D7" s="351"/>
+      <c r="E7" s="351"/>
+      <c r="F7" s="351"/>
+      <c r="G7" s="351"/>
+      <c r="H7" s="351"/>
+      <c r="I7" s="351"/>
+      <c r="J7" s="351"/>
+      <c r="K7" s="351"/>
+      <c r="L7" s="352"/>
       <c r="N7" s="110"/>
       <c r="O7" s="110"/>
       <c r="P7" s="110"/>
@@ -16060,19 +16060,19 @@
     </row>
     <row r="8" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="214"/>
-      <c r="B8" s="377" t="s">
-        <v>296</v>
-      </c>
-      <c r="C8" s="377"/>
-      <c r="D8" s="377"/>
-      <c r="E8" s="377"/>
-      <c r="F8" s="377"/>
-      <c r="G8" s="377"/>
-      <c r="H8" s="377"/>
-      <c r="I8" s="377"/>
-      <c r="J8" s="377"/>
-      <c r="K8" s="377"/>
-      <c r="L8" s="378"/>
+      <c r="B8" s="351" t="s">
+        <v>295</v>
+      </c>
+      <c r="C8" s="351"/>
+      <c r="D8" s="351"/>
+      <c r="E8" s="351"/>
+      <c r="F8" s="351"/>
+      <c r="G8" s="351"/>
+      <c r="H8" s="351"/>
+      <c r="I8" s="351"/>
+      <c r="J8" s="351"/>
+      <c r="K8" s="351"/>
+      <c r="L8" s="352"/>
       <c r="N8" s="110"/>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
@@ -16081,19 +16081,19 @@
     </row>
     <row r="9" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="215"/>
-      <c r="B9" s="379" t="s">
-        <v>297</v>
-      </c>
-      <c r="C9" s="379"/>
-      <c r="D9" s="379"/>
-      <c r="E9" s="379"/>
-      <c r="F9" s="379"/>
-      <c r="G9" s="379"/>
-      <c r="H9" s="379"/>
-      <c r="I9" s="379"/>
-      <c r="J9" s="379"/>
-      <c r="K9" s="379"/>
-      <c r="L9" s="380"/>
+      <c r="B9" s="366" t="s">
+        <v>296</v>
+      </c>
+      <c r="C9" s="366"/>
+      <c r="D9" s="366"/>
+      <c r="E9" s="366"/>
+      <c r="F9" s="366"/>
+      <c r="G9" s="366"/>
+      <c r="H9" s="366"/>
+      <c r="I9" s="366"/>
+      <c r="J9" s="366"/>
+      <c r="K9" s="366"/>
+      <c r="L9" s="367"/>
       <c r="N9" s="110"/>
       <c r="O9" s="110"/>
       <c r="P9" s="110"/>
@@ -16115,81 +16115,81 @@
       <c r="L10" s="110"/>
     </row>
     <row r="11" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="381" t="s">
-        <v>332</v>
-      </c>
-      <c r="B11" s="382"/>
-      <c r="C11" s="382"/>
-      <c r="D11" s="382"/>
-      <c r="E11" s="382"/>
-      <c r="F11" s="382"/>
-      <c r="G11" s="382"/>
-      <c r="H11" s="382"/>
-      <c r="I11" s="382"/>
-      <c r="J11" s="382"/>
-      <c r="K11" s="382"/>
-      <c r="L11" s="383"/>
+      <c r="A11" s="368" t="s">
+        <v>331</v>
+      </c>
+      <c r="B11" s="369"/>
+      <c r="C11" s="369"/>
+      <c r="D11" s="369"/>
+      <c r="E11" s="369"/>
+      <c r="F11" s="369"/>
+      <c r="G11" s="369"/>
+      <c r="H11" s="369"/>
+      <c r="I11" s="369"/>
+      <c r="J11" s="369"/>
+      <c r="K11" s="369"/>
+      <c r="L11" s="370"/>
     </row>
     <row r="12" spans="1:18" s="57" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="344" t="s">
-        <v>333</v>
-      </c>
-      <c r="B12" s="345" t="s">
-        <v>483</v>
-      </c>
-      <c r="C12" s="345"/>
-      <c r="D12" s="345"/>
-      <c r="E12" s="345"/>
-      <c r="F12" s="345"/>
-      <c r="G12" s="345"/>
-      <c r="H12" s="345"/>
-      <c r="I12" s="345"/>
-      <c r="J12" s="345"/>
-      <c r="K12" s="345"/>
-      <c r="L12" s="384"/>
+        <v>332</v>
+      </c>
+      <c r="B12" s="360" t="s">
+        <v>482</v>
+      </c>
+      <c r="C12" s="360"/>
+      <c r="D12" s="360"/>
+      <c r="E12" s="360"/>
+      <c r="F12" s="360"/>
+      <c r="G12" s="360"/>
+      <c r="H12" s="360"/>
+      <c r="I12" s="360"/>
+      <c r="J12" s="360"/>
+      <c r="K12" s="360"/>
+      <c r="L12" s="361"/>
     </row>
     <row r="13" spans="1:18" s="57" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="344"/>
-      <c r="B13" s="345" t="e" vm="1">
+      <c r="B13" s="360" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C13" s="345"/>
-      <c r="D13" s="345"/>
-      <c r="E13" s="345"/>
-      <c r="F13" s="345"/>
-      <c r="G13" s="345"/>
-      <c r="H13" s="345"/>
-      <c r="I13" s="345"/>
-      <c r="J13" s="345"/>
-      <c r="K13" s="345"/>
+      <c r="C13" s="360"/>
+      <c r="D13" s="360"/>
+      <c r="E13" s="360"/>
+      <c r="F13" s="360"/>
+      <c r="G13" s="360"/>
+      <c r="H13" s="360"/>
+      <c r="I13" s="360"/>
+      <c r="J13" s="360"/>
+      <c r="K13" s="360"/>
       <c r="L13" s="342"/>
     </row>
     <row r="14" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="235" t="s">
-        <v>334</v>
-      </c>
-      <c r="B14" s="345" t="s">
-        <v>336</v>
-      </c>
-      <c r="C14" s="345"/>
-      <c r="D14" s="345"/>
-      <c r="E14" s="345"/>
-      <c r="F14" s="345"/>
-      <c r="G14" s="345"/>
-      <c r="H14" s="345"/>
-      <c r="I14" s="345"/>
-      <c r="J14" s="345"/>
-      <c r="K14" s="345"/>
-      <c r="L14" s="384"/>
+        <v>333</v>
+      </c>
+      <c r="B14" s="360" t="s">
+        <v>335</v>
+      </c>
+      <c r="C14" s="360"/>
+      <c r="D14" s="360"/>
+      <c r="E14" s="360"/>
+      <c r="F14" s="360"/>
+      <c r="G14" s="360"/>
+      <c r="H14" s="360"/>
+      <c r="I14" s="360"/>
+      <c r="J14" s="360"/>
+      <c r="K14" s="360"/>
+      <c r="L14" s="361"/>
     </row>
     <row r="15" spans="1:18" s="57" customFormat="1" ht="176" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="227"/>
-      <c r="B15" s="346"/>
-      <c r="C15" s="346"/>
-      <c r="D15" s="346"/>
-      <c r="E15" s="346"/>
-      <c r="F15" s="346"/>
-      <c r="G15" s="346"/>
+      <c r="B15" s="362"/>
+      <c r="C15" s="362"/>
+      <c r="D15" s="362"/>
+      <c r="E15" s="362"/>
+      <c r="F15" s="362"/>
+      <c r="G15" s="362"/>
       <c r="H15" s="233"/>
       <c r="I15" s="233"/>
       <c r="J15" s="233"/>
@@ -16198,79 +16198,79 @@
     </row>
     <row r="16" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="235" t="s">
-        <v>335</v>
-      </c>
-      <c r="B16" s="345" t="s">
-        <v>337</v>
-      </c>
-      <c r="C16" s="345"/>
-      <c r="D16" s="345"/>
-      <c r="E16" s="345"/>
-      <c r="F16" s="345"/>
-      <c r="G16" s="345"/>
-      <c r="H16" s="345"/>
-      <c r="I16" s="345"/>
-      <c r="J16" s="345"/>
-      <c r="K16" s="345"/>
-      <c r="L16" s="384"/>
+        <v>334</v>
+      </c>
+      <c r="B16" s="360" t="s">
+        <v>336</v>
+      </c>
+      <c r="C16" s="360"/>
+      <c r="D16" s="360"/>
+      <c r="E16" s="360"/>
+      <c r="F16" s="360"/>
+      <c r="G16" s="360"/>
+      <c r="H16" s="360"/>
+      <c r="I16" s="360"/>
+      <c r="J16" s="360"/>
+      <c r="K16" s="360"/>
+      <c r="L16" s="361"/>
     </row>
     <row r="17" spans="1:14" s="57" customFormat="1" ht="90.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="227"/>
-      <c r="B17" s="346"/>
-      <c r="C17" s="346"/>
-      <c r="D17" s="346"/>
-      <c r="E17" s="346"/>
-      <c r="F17" s="346"/>
-      <c r="G17" s="346"/>
-      <c r="H17" s="346"/>
-      <c r="I17" s="346"/>
-      <c r="J17" s="346"/>
-      <c r="K17" s="346"/>
-      <c r="L17" s="395"/>
+      <c r="B17" s="362"/>
+      <c r="C17" s="362"/>
+      <c r="D17" s="362"/>
+      <c r="E17" s="362"/>
+      <c r="F17" s="362"/>
+      <c r="G17" s="362"/>
+      <c r="H17" s="362"/>
+      <c r="I17" s="362"/>
+      <c r="J17" s="362"/>
+      <c r="K17" s="362"/>
+      <c r="L17" s="363"/>
     </row>
     <row r="18" spans="1:14" s="56" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="235" t="s">
-        <v>475</v>
-      </c>
-      <c r="B18" s="345" t="s">
-        <v>463</v>
-      </c>
-      <c r="C18" s="345"/>
-      <c r="D18" s="345"/>
-      <c r="E18" s="345"/>
-      <c r="F18" s="345"/>
-      <c r="G18" s="345"/>
-      <c r="H18" s="345"/>
-      <c r="I18" s="345"/>
-      <c r="J18" s="345"/>
-      <c r="K18" s="345"/>
-      <c r="L18" s="384"/>
+        <v>474</v>
+      </c>
+      <c r="B18" s="360" t="s">
+        <v>462</v>
+      </c>
+      <c r="C18" s="360"/>
+      <c r="D18" s="360"/>
+      <c r="E18" s="360"/>
+      <c r="F18" s="360"/>
+      <c r="G18" s="360"/>
+      <c r="H18" s="360"/>
+      <c r="I18" s="360"/>
+      <c r="J18" s="360"/>
+      <c r="K18" s="360"/>
+      <c r="L18" s="361"/>
     </row>
     <row r="19" spans="1:14" s="57" customFormat="1" ht="269" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="227"/>
-      <c r="B19" s="346" t="e" vm="2">
+      <c r="B19" s="362" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="C19" s="346"/>
-      <c r="D19" s="346"/>
-      <c r="E19" s="346"/>
-      <c r="F19" s="346"/>
-      <c r="G19" s="346"/>
-      <c r="H19" s="346"/>
-      <c r="I19" s="346"/>
-      <c r="J19" s="346"/>
-      <c r="K19" s="346"/>
+      <c r="C19" s="362"/>
+      <c r="D19" s="362"/>
+      <c r="E19" s="362"/>
+      <c r="F19" s="362"/>
+      <c r="G19" s="362"/>
+      <c r="H19" s="362"/>
+      <c r="I19" s="362"/>
+      <c r="J19" s="362"/>
+      <c r="K19" s="362"/>
       <c r="L19" s="234"/>
     </row>
     <row r="20" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="369" t="s">
+      <c r="A20" s="394" t="s">
+        <v>340</v>
+      </c>
+      <c r="B20" s="395"/>
+      <c r="C20" s="395"/>
+      <c r="D20" s="395"/>
+      <c r="E20" s="232" t="s">
         <v>341</v>
-      </c>
-      <c r="B20" s="370"/>
-      <c r="C20" s="370"/>
-      <c r="D20" s="370"/>
-      <c r="E20" s="232" t="s">
-        <v>342</v>
       </c>
       <c r="F20" s="230"/>
       <c r="G20" s="230"/>
@@ -16295,84 +16295,84 @@
       <c r="L21" s="110"/>
     </row>
     <row r="22" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="353" t="s">
+      <c r="A22" s="381" t="s">
         <v>165</v>
       </c>
-      <c r="B22" s="354"/>
-      <c r="C22" s="354"/>
-      <c r="D22" s="354"/>
-      <c r="E22" s="354"/>
-      <c r="F22" s="354"/>
-      <c r="G22" s="354"/>
-      <c r="H22" s="354"/>
-      <c r="I22" s="354"/>
-      <c r="J22" s="354"/>
-      <c r="K22" s="354"/>
-      <c r="L22" s="355"/>
+      <c r="B22" s="382"/>
+      <c r="C22" s="382"/>
+      <c r="D22" s="382"/>
+      <c r="E22" s="382"/>
+      <c r="F22" s="382"/>
+      <c r="G22" s="382"/>
+      <c r="H22" s="382"/>
+      <c r="I22" s="382"/>
+      <c r="J22" s="382"/>
+      <c r="K22" s="382"/>
+      <c r="L22" s="383"/>
     </row>
     <row r="23" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="356" t="s">
+      <c r="A23" s="384" t="s">
         <v>280</v>
       </c>
-      <c r="B23" s="357"/>
-      <c r="C23" s="357"/>
-      <c r="D23" s="357"/>
-      <c r="E23" s="357"/>
-      <c r="F23" s="357"/>
-      <c r="G23" s="357"/>
-      <c r="H23" s="357"/>
-      <c r="I23" s="357"/>
-      <c r="J23" s="357"/>
-      <c r="K23" s="357"/>
-      <c r="L23" s="358"/>
+      <c r="B23" s="385"/>
+      <c r="C23" s="385"/>
+      <c r="D23" s="385"/>
+      <c r="E23" s="385"/>
+      <c r="F23" s="385"/>
+      <c r="G23" s="385"/>
+      <c r="H23" s="385"/>
+      <c r="I23" s="385"/>
+      <c r="J23" s="385"/>
+      <c r="K23" s="385"/>
+      <c r="L23" s="386"/>
     </row>
     <row r="24" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="359" t="s">
+      <c r="A24" s="387" t="s">
         <v>281</v>
       </c>
-      <c r="B24" s="347"/>
-      <c r="C24" s="347"/>
-      <c r="D24" s="347"/>
-      <c r="E24" s="347"/>
-      <c r="F24" s="347"/>
-      <c r="G24" s="347"/>
-      <c r="H24" s="347"/>
-      <c r="I24" s="347"/>
-      <c r="J24" s="347"/>
-      <c r="K24" s="347"/>
-      <c r="L24" s="360"/>
+      <c r="B24" s="345"/>
+      <c r="C24" s="345"/>
+      <c r="D24" s="345"/>
+      <c r="E24" s="345"/>
+      <c r="F24" s="345"/>
+      <c r="G24" s="345"/>
+      <c r="H24" s="345"/>
+      <c r="I24" s="345"/>
+      <c r="J24" s="345"/>
+      <c r="K24" s="345"/>
+      <c r="L24" s="346"/>
     </row>
     <row r="25" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="359" t="s">
+      <c r="A25" s="387" t="s">
         <v>166</v>
       </c>
-      <c r="B25" s="347"/>
-      <c r="C25" s="347"/>
-      <c r="D25" s="347"/>
-      <c r="E25" s="347"/>
-      <c r="F25" s="347"/>
-      <c r="G25" s="347"/>
-      <c r="H25" s="347"/>
-      <c r="I25" s="347"/>
-      <c r="J25" s="347"/>
-      <c r="K25" s="347"/>
-      <c r="L25" s="360"/>
+      <c r="B25" s="345"/>
+      <c r="C25" s="345"/>
+      <c r="D25" s="345"/>
+      <c r="E25" s="345"/>
+      <c r="F25" s="345"/>
+      <c r="G25" s="345"/>
+      <c r="H25" s="345"/>
+      <c r="I25" s="345"/>
+      <c r="J25" s="345"/>
+      <c r="K25" s="345"/>
+      <c r="L25" s="346"/>
     </row>
     <row r="26" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="361" t="s">
+      <c r="A26" s="388" t="s">
         <v>282</v>
       </c>
-      <c r="B26" s="362"/>
-      <c r="C26" s="362"/>
-      <c r="D26" s="362"/>
-      <c r="E26" s="362"/>
-      <c r="F26" s="362"/>
-      <c r="G26" s="362"/>
-      <c r="H26" s="362"/>
-      <c r="I26" s="362"/>
-      <c r="J26" s="362"/>
-      <c r="K26" s="362"/>
-      <c r="L26" s="363"/>
+      <c r="B26" s="389"/>
+      <c r="C26" s="389"/>
+      <c r="D26" s="389"/>
+      <c r="E26" s="389"/>
+      <c r="F26" s="389"/>
+      <c r="G26" s="389"/>
+      <c r="H26" s="389"/>
+      <c r="I26" s="389"/>
+      <c r="J26" s="389"/>
+      <c r="K26" s="389"/>
+      <c r="L26" s="390"/>
     </row>
     <row r="27" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="110"/>
@@ -16389,332 +16389,332 @@
       <c r="L27" s="110"/>
     </row>
     <row r="28" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="364" t="s">
+      <c r="A28" s="391" t="s">
         <v>279</v>
       </c>
-      <c r="B28" s="365"/>
-      <c r="C28" s="365"/>
-      <c r="D28" s="365"/>
-      <c r="E28" s="365"/>
-      <c r="F28" s="365"/>
-      <c r="G28" s="365"/>
-      <c r="H28" s="365"/>
-      <c r="I28" s="365"/>
-      <c r="J28" s="365"/>
-      <c r="K28" s="365"/>
-      <c r="L28" s="366"/>
+      <c r="B28" s="392"/>
+      <c r="C28" s="392"/>
+      <c r="D28" s="392"/>
+      <c r="E28" s="392"/>
+      <c r="F28" s="392"/>
+      <c r="G28" s="392"/>
+      <c r="H28" s="392"/>
+      <c r="I28" s="392"/>
+      <c r="J28" s="392"/>
+      <c r="K28" s="392"/>
+      <c r="L28" s="393"/>
       <c r="N28" s="1"/>
     </row>
     <row r="29" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="350" t="s">
+      <c r="A29" s="378" t="s">
         <v>175</v>
       </c>
-      <c r="B29" s="351"/>
-      <c r="C29" s="351"/>
-      <c r="D29" s="351"/>
-      <c r="E29" s="351"/>
-      <c r="F29" s="351"/>
-      <c r="G29" s="351"/>
-      <c r="H29" s="351"/>
-      <c r="I29" s="351"/>
-      <c r="J29" s="351"/>
-      <c r="K29" s="351"/>
-      <c r="L29" s="352"/>
+      <c r="B29" s="379"/>
+      <c r="C29" s="379"/>
+      <c r="D29" s="379"/>
+      <c r="E29" s="379"/>
+      <c r="F29" s="379"/>
+      <c r="G29" s="379"/>
+      <c r="H29" s="379"/>
+      <c r="I29" s="379"/>
+      <c r="J29" s="379"/>
+      <c r="K29" s="379"/>
+      <c r="L29" s="380"/>
       <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="209">
         <v>1</v>
       </c>
-      <c r="B30" s="367" t="s">
+      <c r="B30" s="353" t="s">
         <v>174</v>
       </c>
-      <c r="C30" s="367"/>
-      <c r="D30" s="367"/>
-      <c r="E30" s="367"/>
-      <c r="F30" s="367"/>
-      <c r="G30" s="367"/>
-      <c r="H30" s="367"/>
-      <c r="I30" s="367"/>
-      <c r="J30" s="367"/>
-      <c r="K30" s="367"/>
-      <c r="L30" s="368"/>
+      <c r="C30" s="353"/>
+      <c r="D30" s="353"/>
+      <c r="E30" s="353"/>
+      <c r="F30" s="353"/>
+      <c r="G30" s="353"/>
+      <c r="H30" s="353"/>
+      <c r="I30" s="353"/>
+      <c r="J30" s="353"/>
+      <c r="K30" s="353"/>
+      <c r="L30" s="354"/>
     </row>
     <row r="31" spans="1:14" s="57" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="209">
         <v>2</v>
       </c>
-      <c r="B31" s="367" t="s">
+      <c r="B31" s="353" t="s">
         <v>275</v>
       </c>
-      <c r="C31" s="367"/>
-      <c r="D31" s="367"/>
-      <c r="E31" s="367"/>
-      <c r="F31" s="367"/>
-      <c r="G31" s="367"/>
-      <c r="H31" s="367"/>
-      <c r="I31" s="367"/>
-      <c r="J31" s="367"/>
-      <c r="K31" s="367"/>
-      <c r="L31" s="368"/>
+      <c r="C31" s="353"/>
+      <c r="D31" s="353"/>
+      <c r="E31" s="353"/>
+      <c r="F31" s="353"/>
+      <c r="G31" s="353"/>
+      <c r="H31" s="353"/>
+      <c r="I31" s="353"/>
+      <c r="J31" s="353"/>
+      <c r="K31" s="353"/>
+      <c r="L31" s="354"/>
       <c r="N31" s="104"/>
     </row>
     <row r="32" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="209">
         <v>3</v>
       </c>
-      <c r="B32" s="367" t="s">
+      <c r="B32" s="353" t="s">
         <v>167</v>
       </c>
-      <c r="C32" s="367"/>
-      <c r="D32" s="367"/>
-      <c r="E32" s="367"/>
-      <c r="F32" s="367"/>
-      <c r="G32" s="367"/>
-      <c r="H32" s="367"/>
-      <c r="I32" s="367"/>
-      <c r="J32" s="367"/>
-      <c r="K32" s="367"/>
-      <c r="L32" s="368"/>
+      <c r="C32" s="353"/>
+      <c r="D32" s="353"/>
+      <c r="E32" s="353"/>
+      <c r="F32" s="353"/>
+      <c r="G32" s="353"/>
+      <c r="H32" s="353"/>
+      <c r="I32" s="353"/>
+      <c r="J32" s="353"/>
+      <c r="K32" s="353"/>
+      <c r="L32" s="354"/>
       <c r="N32" s="104"/>
     </row>
     <row r="33" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="209">
         <v>4</v>
       </c>
-      <c r="B33" s="367" t="s">
+      <c r="B33" s="353" t="s">
         <v>283</v>
       </c>
-      <c r="C33" s="367"/>
-      <c r="D33" s="367"/>
-      <c r="E33" s="367"/>
-      <c r="F33" s="367"/>
-      <c r="G33" s="367"/>
-      <c r="H33" s="367"/>
-      <c r="I33" s="367"/>
-      <c r="J33" s="367"/>
-      <c r="K33" s="367"/>
-      <c r="L33" s="368"/>
+      <c r="C33" s="353"/>
+      <c r="D33" s="353"/>
+      <c r="E33" s="353"/>
+      <c r="F33" s="353"/>
+      <c r="G33" s="353"/>
+      <c r="H33" s="353"/>
+      <c r="I33" s="353"/>
+      <c r="J33" s="353"/>
+      <c r="K33" s="353"/>
+      <c r="L33" s="354"/>
       <c r="N33" s="104"/>
     </row>
     <row r="34" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="209">
         <v>5</v>
       </c>
-      <c r="B34" s="367" t="s">
+      <c r="B34" s="353" t="s">
         <v>168</v>
       </c>
-      <c r="C34" s="367"/>
-      <c r="D34" s="367"/>
-      <c r="E34" s="367"/>
-      <c r="F34" s="367"/>
-      <c r="G34" s="367"/>
-      <c r="H34" s="367"/>
-      <c r="I34" s="367"/>
-      <c r="J34" s="367"/>
-      <c r="K34" s="367"/>
-      <c r="L34" s="368"/>
+      <c r="C34" s="353"/>
+      <c r="D34" s="353"/>
+      <c r="E34" s="353"/>
+      <c r="F34" s="353"/>
+      <c r="G34" s="353"/>
+      <c r="H34" s="353"/>
+      <c r="I34" s="353"/>
+      <c r="J34" s="353"/>
+      <c r="K34" s="353"/>
+      <c r="L34" s="354"/>
       <c r="N34" s="104"/>
     </row>
     <row r="35" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="209"/>
-      <c r="B35" s="367" t="s">
+      <c r="B35" s="353" t="s">
         <v>169</v>
       </c>
-      <c r="C35" s="367"/>
-      <c r="D35" s="367"/>
-      <c r="E35" s="367"/>
-      <c r="F35" s="367"/>
-      <c r="G35" s="367"/>
-      <c r="H35" s="367"/>
-      <c r="I35" s="367"/>
-      <c r="J35" s="367"/>
-      <c r="K35" s="367"/>
-      <c r="L35" s="368"/>
+      <c r="C35" s="353"/>
+      <c r="D35" s="353"/>
+      <c r="E35" s="353"/>
+      <c r="F35" s="353"/>
+      <c r="G35" s="353"/>
+      <c r="H35" s="353"/>
+      <c r="I35" s="353"/>
+      <c r="J35" s="353"/>
+      <c r="K35" s="353"/>
+      <c r="L35" s="354"/>
       <c r="N35" s="104"/>
     </row>
     <row r="36" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="209"/>
-      <c r="B36" s="367" t="s">
+      <c r="B36" s="353" t="s">
         <v>170</v>
       </c>
-      <c r="C36" s="367"/>
-      <c r="D36" s="367"/>
-      <c r="E36" s="367"/>
-      <c r="F36" s="367"/>
-      <c r="G36" s="367"/>
-      <c r="H36" s="367"/>
-      <c r="I36" s="367"/>
-      <c r="J36" s="367"/>
-      <c r="K36" s="367"/>
-      <c r="L36" s="368"/>
+      <c r="C36" s="353"/>
+      <c r="D36" s="353"/>
+      <c r="E36" s="353"/>
+      <c r="F36" s="353"/>
+      <c r="G36" s="353"/>
+      <c r="H36" s="353"/>
+      <c r="I36" s="353"/>
+      <c r="J36" s="353"/>
+      <c r="K36" s="353"/>
+      <c r="L36" s="354"/>
       <c r="N36" s="104"/>
     </row>
     <row r="37" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="387" t="s">
+      <c r="A37" s="347" t="s">
         <v>176</v>
       </c>
-      <c r="B37" s="388"/>
-      <c r="C37" s="388"/>
-      <c r="D37" s="388"/>
-      <c r="E37" s="388"/>
-      <c r="F37" s="388"/>
-      <c r="G37" s="388"/>
-      <c r="H37" s="388"/>
-      <c r="I37" s="388"/>
-      <c r="J37" s="388"/>
-      <c r="K37" s="388"/>
-      <c r="L37" s="389"/>
+      <c r="B37" s="348"/>
+      <c r="C37" s="348"/>
+      <c r="D37" s="348"/>
+      <c r="E37" s="348"/>
+      <c r="F37" s="348"/>
+      <c r="G37" s="348"/>
+      <c r="H37" s="348"/>
+      <c r="I37" s="348"/>
+      <c r="J37" s="348"/>
+      <c r="K37" s="348"/>
+      <c r="L37" s="349"/>
       <c r="N37" s="104"/>
     </row>
     <row r="38" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="209">
         <v>1</v>
       </c>
-      <c r="B38" s="367" t="s">
+      <c r="B38" s="353" t="s">
         <v>171</v>
       </c>
-      <c r="C38" s="367"/>
-      <c r="D38" s="367"/>
-      <c r="E38" s="367"/>
-      <c r="F38" s="367"/>
-      <c r="G38" s="367"/>
-      <c r="H38" s="367"/>
-      <c r="I38" s="367"/>
-      <c r="J38" s="367"/>
-      <c r="K38" s="367"/>
-      <c r="L38" s="368"/>
+      <c r="C38" s="353"/>
+      <c r="D38" s="353"/>
+      <c r="E38" s="353"/>
+      <c r="F38" s="353"/>
+      <c r="G38" s="353"/>
+      <c r="H38" s="353"/>
+      <c r="I38" s="353"/>
+      <c r="J38" s="353"/>
+      <c r="K38" s="353"/>
+      <c r="L38" s="354"/>
       <c r="N38" s="104"/>
     </row>
     <row r="39" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="209"/>
-      <c r="B39" s="385" t="s">
-        <v>424</v>
-      </c>
-      <c r="C39" s="385"/>
-      <c r="D39" s="385"/>
-      <c r="E39" s="385"/>
-      <c r="F39" s="385"/>
-      <c r="G39" s="385"/>
-      <c r="H39" s="385"/>
-      <c r="I39" s="385"/>
-      <c r="J39" s="385"/>
-      <c r="K39" s="385"/>
-      <c r="L39" s="386"/>
+      <c r="B39" s="364" t="s">
+        <v>423</v>
+      </c>
+      <c r="C39" s="364"/>
+      <c r="D39" s="364"/>
+      <c r="E39" s="364"/>
+      <c r="F39" s="364"/>
+      <c r="G39" s="364"/>
+      <c r="H39" s="364"/>
+      <c r="I39" s="364"/>
+      <c r="J39" s="364"/>
+      <c r="K39" s="364"/>
+      <c r="L39" s="365"/>
       <c r="N39" s="104"/>
     </row>
     <row r="40" spans="1:14" s="57" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="209">
         <v>2</v>
       </c>
-      <c r="B40" s="367" t="s">
+      <c r="B40" s="353" t="s">
         <v>278</v>
       </c>
-      <c r="C40" s="367"/>
-      <c r="D40" s="367"/>
-      <c r="E40" s="367"/>
-      <c r="F40" s="367"/>
-      <c r="G40" s="367"/>
-      <c r="H40" s="367"/>
-      <c r="I40" s="367"/>
-      <c r="J40" s="367"/>
-      <c r="K40" s="367"/>
-      <c r="L40" s="368"/>
+      <c r="C40" s="353"/>
+      <c r="D40" s="353"/>
+      <c r="E40" s="353"/>
+      <c r="F40" s="353"/>
+      <c r="G40" s="353"/>
+      <c r="H40" s="353"/>
+      <c r="I40" s="353"/>
+      <c r="J40" s="353"/>
+      <c r="K40" s="353"/>
+      <c r="L40" s="354"/>
       <c r="N40" s="104"/>
     </row>
     <row r="41" spans="1:14" s="57" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="209">
         <v>3</v>
       </c>
-      <c r="B41" s="367" t="s">
-        <v>473</v>
-      </c>
-      <c r="C41" s="367"/>
-      <c r="D41" s="367"/>
-      <c r="E41" s="367"/>
-      <c r="F41" s="367"/>
-      <c r="G41" s="367"/>
-      <c r="H41" s="367"/>
-      <c r="I41" s="367"/>
-      <c r="J41" s="367"/>
-      <c r="K41" s="367"/>
-      <c r="L41" s="368"/>
+      <c r="B41" s="353" t="s">
+        <v>472</v>
+      </c>
+      <c r="C41" s="353"/>
+      <c r="D41" s="353"/>
+      <c r="E41" s="353"/>
+      <c r="F41" s="353"/>
+      <c r="G41" s="353"/>
+      <c r="H41" s="353"/>
+      <c r="I41" s="353"/>
+      <c r="J41" s="353"/>
+      <c r="K41" s="353"/>
+      <c r="L41" s="354"/>
       <c r="N41" s="104"/>
     </row>
     <row r="42" spans="1:14" s="57" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="209">
         <v>4</v>
       </c>
-      <c r="B42" s="367" t="s">
+      <c r="B42" s="353" t="s">
         <v>284</v>
       </c>
-      <c r="C42" s="367"/>
-      <c r="D42" s="367"/>
-      <c r="E42" s="367"/>
-      <c r="F42" s="367"/>
-      <c r="G42" s="367"/>
-      <c r="H42" s="367"/>
-      <c r="I42" s="367"/>
-      <c r="J42" s="367"/>
-      <c r="K42" s="367"/>
-      <c r="L42" s="368"/>
+      <c r="C42" s="353"/>
+      <c r="D42" s="353"/>
+      <c r="E42" s="353"/>
+      <c r="F42" s="353"/>
+      <c r="G42" s="353"/>
+      <c r="H42" s="353"/>
+      <c r="I42" s="353"/>
+      <c r="J42" s="353"/>
+      <c r="K42" s="353"/>
+      <c r="L42" s="354"/>
       <c r="N42" s="104"/>
     </row>
     <row r="43" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="209">
         <v>5</v>
       </c>
-      <c r="B43" s="385" t="s">
+      <c r="B43" s="364" t="s">
         <v>269</v>
       </c>
-      <c r="C43" s="385"/>
-      <c r="D43" s="385"/>
-      <c r="E43" s="385"/>
-      <c r="F43" s="385"/>
-      <c r="G43" s="385"/>
-      <c r="H43" s="385"/>
-      <c r="I43" s="385"/>
-      <c r="J43" s="385"/>
-      <c r="K43" s="385"/>
-      <c r="L43" s="386"/>
+      <c r="C43" s="364"/>
+      <c r="D43" s="364"/>
+      <c r="E43" s="364"/>
+      <c r="F43" s="364"/>
+      <c r="G43" s="364"/>
+      <c r="H43" s="364"/>
+      <c r="I43" s="364"/>
+      <c r="J43" s="364"/>
+      <c r="K43" s="364"/>
+      <c r="L43" s="365"/>
       <c r="N43" s="104"/>
     </row>
     <row r="44" spans="1:14" s="57" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="209">
         <v>6</v>
       </c>
-      <c r="B44" s="385" t="s">
-        <v>474</v>
-      </c>
-      <c r="C44" s="385"/>
-      <c r="D44" s="385"/>
-      <c r="E44" s="385"/>
-      <c r="F44" s="385"/>
-      <c r="G44" s="385"/>
-      <c r="H44" s="385"/>
-      <c r="I44" s="385"/>
-      <c r="J44" s="385"/>
-      <c r="K44" s="385"/>
-      <c r="L44" s="386"/>
+      <c r="B44" s="364" t="s">
+        <v>473</v>
+      </c>
+      <c r="C44" s="364"/>
+      <c r="D44" s="364"/>
+      <c r="E44" s="364"/>
+      <c r="F44" s="364"/>
+      <c r="G44" s="364"/>
+      <c r="H44" s="364"/>
+      <c r="I44" s="364"/>
+      <c r="J44" s="364"/>
+      <c r="K44" s="364"/>
+      <c r="L44" s="365"/>
       <c r="N44" s="104"/>
     </row>
     <row r="45" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="209">
         <v>7</v>
       </c>
-      <c r="B45" s="367" t="s">
+      <c r="B45" s="353" t="s">
         <v>270</v>
       </c>
-      <c r="C45" s="367"/>
-      <c r="D45" s="367"/>
-      <c r="E45" s="367"/>
-      <c r="F45" s="367"/>
-      <c r="G45" s="367"/>
-      <c r="H45" s="367"/>
-      <c r="I45" s="367"/>
-      <c r="J45" s="367"/>
-      <c r="K45" s="367"/>
-      <c r="L45" s="368"/>
+      <c r="C45" s="353"/>
+      <c r="D45" s="353"/>
+      <c r="E45" s="353"/>
+      <c r="F45" s="353"/>
+      <c r="G45" s="353"/>
+      <c r="H45" s="353"/>
+      <c r="I45" s="353"/>
+      <c r="J45" s="353"/>
+      <c r="K45" s="353"/>
+      <c r="L45" s="354"/>
     </row>
     <row r="46" spans="1:14" s="57" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="209"/>
@@ -16731,56 +16731,56 @@
       <c r="L46" s="211"/>
     </row>
     <row r="47" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="387" t="s">
+      <c r="A47" s="347" t="s">
         <v>273</v>
       </c>
-      <c r="B47" s="388"/>
-      <c r="C47" s="388"/>
-      <c r="D47" s="388"/>
-      <c r="E47" s="388"/>
-      <c r="F47" s="388"/>
-      <c r="G47" s="388"/>
-      <c r="H47" s="388"/>
-      <c r="I47" s="388"/>
-      <c r="J47" s="388"/>
-      <c r="K47" s="388"/>
-      <c r="L47" s="389"/>
+      <c r="B47" s="348"/>
+      <c r="C47" s="348"/>
+      <c r="D47" s="348"/>
+      <c r="E47" s="348"/>
+      <c r="F47" s="348"/>
+      <c r="G47" s="348"/>
+      <c r="H47" s="348"/>
+      <c r="I47" s="348"/>
+      <c r="J47" s="348"/>
+      <c r="K47" s="348"/>
+      <c r="L47" s="349"/>
     </row>
     <row r="48" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="212" t="s">
         <v>271</v>
       </c>
-      <c r="B48" s="367" t="s">
+      <c r="B48" s="353" t="s">
         <v>172</v>
       </c>
-      <c r="C48" s="367"/>
-      <c r="D48" s="367"/>
-      <c r="E48" s="367"/>
-      <c r="F48" s="367"/>
-      <c r="G48" s="367"/>
-      <c r="H48" s="367"/>
-      <c r="I48" s="367"/>
-      <c r="J48" s="367"/>
-      <c r="K48" s="367"/>
-      <c r="L48" s="368"/>
+      <c r="C48" s="353"/>
+      <c r="D48" s="353"/>
+      <c r="E48" s="353"/>
+      <c r="F48" s="353"/>
+      <c r="G48" s="353"/>
+      <c r="H48" s="353"/>
+      <c r="I48" s="353"/>
+      <c r="J48" s="353"/>
+      <c r="K48" s="353"/>
+      <c r="L48" s="354"/>
     </row>
     <row r="49" spans="1:12" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="213" t="s">
         <v>272</v>
       </c>
-      <c r="B49" s="390" t="s">
+      <c r="B49" s="355" t="s">
         <v>274</v>
       </c>
-      <c r="C49" s="390"/>
-      <c r="D49" s="390"/>
-      <c r="E49" s="390"/>
-      <c r="F49" s="390"/>
-      <c r="G49" s="390"/>
-      <c r="H49" s="390"/>
-      <c r="I49" s="390"/>
-      <c r="J49" s="390"/>
-      <c r="K49" s="390"/>
-      <c r="L49" s="391"/>
+      <c r="C49" s="355"/>
+      <c r="D49" s="355"/>
+      <c r="E49" s="355"/>
+      <c r="F49" s="355"/>
+      <c r="G49" s="355"/>
+      <c r="H49" s="355"/>
+      <c r="I49" s="355"/>
+      <c r="J49" s="355"/>
+      <c r="K49" s="355"/>
+      <c r="L49" s="356"/>
     </row>
     <row r="50" spans="1:12" s="57" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="157"/>
@@ -16797,20 +16797,20 @@
       <c r="L50" s="110"/>
     </row>
     <row r="51" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="392" t="s">
+      <c r="A51" s="357" t="s">
         <v>200</v>
       </c>
-      <c r="B51" s="393"/>
-      <c r="C51" s="393"/>
-      <c r="D51" s="393"/>
-      <c r="E51" s="393"/>
-      <c r="F51" s="393"/>
-      <c r="G51" s="393"/>
-      <c r="H51" s="393"/>
-      <c r="I51" s="393"/>
-      <c r="J51" s="393"/>
-      <c r="K51" s="393"/>
-      <c r="L51" s="394"/>
+      <c r="B51" s="358"/>
+      <c r="C51" s="358"/>
+      <c r="D51" s="358"/>
+      <c r="E51" s="358"/>
+      <c r="F51" s="358"/>
+      <c r="G51" s="358"/>
+      <c r="H51" s="358"/>
+      <c r="I51" s="358"/>
+      <c r="J51" s="358"/>
+      <c r="K51" s="358"/>
+      <c r="L51" s="359"/>
     </row>
     <row r="52" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="216" t="s">
@@ -16863,7 +16863,7 @@
         <v>24</v>
       </c>
       <c r="C55" s="166" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D55" s="166"/>
       <c r="E55" s="166"/>
@@ -16898,126 +16898,126 @@
       <c r="B57" s="165" t="s">
         <v>24</v>
       </c>
-      <c r="C57" s="347" t="s">
+      <c r="C57" s="345" t="s">
         <v>262</v>
       </c>
-      <c r="D57" s="347"/>
-      <c r="E57" s="347"/>
-      <c r="F57" s="347"/>
-      <c r="G57" s="347"/>
-      <c r="H57" s="347"/>
-      <c r="I57" s="347"/>
-      <c r="J57" s="347"/>
-      <c r="K57" s="347"/>
-      <c r="L57" s="360"/>
+      <c r="D57" s="345"/>
+      <c r="E57" s="345"/>
+      <c r="F57" s="345"/>
+      <c r="G57" s="345"/>
+      <c r="H57" s="345"/>
+      <c r="I57" s="345"/>
+      <c r="J57" s="345"/>
+      <c r="K57" s="345"/>
+      <c r="L57" s="346"/>
     </row>
     <row r="58" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="164"/>
       <c r="B58" s="165" t="s">
         <v>263</v>
       </c>
-      <c r="C58" s="347" t="s">
+      <c r="C58" s="345" t="s">
         <v>264</v>
       </c>
-      <c r="D58" s="347"/>
-      <c r="E58" s="347"/>
-      <c r="F58" s="347"/>
-      <c r="G58" s="347"/>
-      <c r="H58" s="347"/>
-      <c r="I58" s="347"/>
-      <c r="J58" s="347"/>
-      <c r="K58" s="347"/>
-      <c r="L58" s="360"/>
+      <c r="D58" s="345"/>
+      <c r="E58" s="345"/>
+      <c r="F58" s="345"/>
+      <c r="G58" s="345"/>
+      <c r="H58" s="345"/>
+      <c r="I58" s="345"/>
+      <c r="J58" s="345"/>
+      <c r="K58" s="345"/>
+      <c r="L58" s="346"/>
     </row>
     <row r="59" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="164"/>
       <c r="B59" s="165" t="s">
+        <v>324</v>
+      </c>
+      <c r="C59" s="345" t="s">
         <v>325</v>
       </c>
-      <c r="C59" s="347" t="s">
-        <v>326</v>
-      </c>
-      <c r="D59" s="347"/>
-      <c r="E59" s="347"/>
-      <c r="F59" s="347"/>
-      <c r="G59" s="347"/>
-      <c r="H59" s="347"/>
-      <c r="I59" s="347"/>
-      <c r="J59" s="347"/>
-      <c r="K59" s="347"/>
-      <c r="L59" s="360"/>
+      <c r="D59" s="345"/>
+      <c r="E59" s="345"/>
+      <c r="F59" s="345"/>
+      <c r="G59" s="345"/>
+      <c r="H59" s="345"/>
+      <c r="I59" s="345"/>
+      <c r="J59" s="345"/>
+      <c r="K59" s="345"/>
+      <c r="L59" s="346"/>
     </row>
     <row r="60" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="164"/>
       <c r="B60" s="165" t="s">
         <v>98</v>
       </c>
-      <c r="C60" s="347" t="s">
+      <c r="C60" s="345" t="s">
         <v>99</v>
       </c>
-      <c r="D60" s="347"/>
-      <c r="E60" s="347"/>
-      <c r="F60" s="347"/>
-      <c r="G60" s="347"/>
-      <c r="H60" s="347"/>
-      <c r="I60" s="347"/>
-      <c r="J60" s="347"/>
-      <c r="K60" s="347"/>
-      <c r="L60" s="360"/>
+      <c r="D60" s="345"/>
+      <c r="E60" s="345"/>
+      <c r="F60" s="345"/>
+      <c r="G60" s="345"/>
+      <c r="H60" s="345"/>
+      <c r="I60" s="345"/>
+      <c r="J60" s="345"/>
+      <c r="K60" s="345"/>
+      <c r="L60" s="346"/>
     </row>
     <row r="61" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="164"/>
       <c r="B61" s="165" t="s">
         <v>198</v>
       </c>
-      <c r="C61" s="347" t="s">
+      <c r="C61" s="345" t="s">
         <v>199</v>
       </c>
-      <c r="D61" s="347"/>
-      <c r="E61" s="347"/>
-      <c r="F61" s="347"/>
-      <c r="G61" s="347"/>
-      <c r="H61" s="347"/>
-      <c r="I61" s="347"/>
-      <c r="J61" s="347"/>
-      <c r="K61" s="347"/>
-      <c r="L61" s="360"/>
+      <c r="D61" s="345"/>
+      <c r="E61" s="345"/>
+      <c r="F61" s="345"/>
+      <c r="G61" s="345"/>
+      <c r="H61" s="345"/>
+      <c r="I61" s="345"/>
+      <c r="J61" s="345"/>
+      <c r="K61" s="345"/>
+      <c r="L61" s="346"/>
     </row>
     <row r="62" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="164"/>
       <c r="B62" s="165" t="s">
         <v>163</v>
       </c>
-      <c r="C62" s="347" t="s">
-        <v>464</v>
-      </c>
-      <c r="D62" s="348"/>
-      <c r="E62" s="348"/>
-      <c r="F62" s="348"/>
-      <c r="G62" s="348"/>
-      <c r="H62" s="348"/>
-      <c r="I62" s="348"/>
-      <c r="J62" s="348"/>
-      <c r="K62" s="348"/>
-      <c r="L62" s="349"/>
+      <c r="C62" s="345" t="s">
+        <v>463</v>
+      </c>
+      <c r="D62" s="376"/>
+      <c r="E62" s="376"/>
+      <c r="F62" s="376"/>
+      <c r="G62" s="376"/>
+      <c r="H62" s="376"/>
+      <c r="I62" s="376"/>
+      <c r="J62" s="376"/>
+      <c r="K62" s="376"/>
+      <c r="L62" s="377"/>
     </row>
     <row r="63" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="164"/>
       <c r="B63" s="165" t="s">
+        <v>390</v>
+      </c>
+      <c r="C63" s="345" t="s">
         <v>391</v>
       </c>
-      <c r="C63" s="347" t="s">
-        <v>392</v>
-      </c>
-      <c r="D63" s="347"/>
-      <c r="E63" s="347"/>
-      <c r="F63" s="347"/>
-      <c r="G63" s="347"/>
-      <c r="H63" s="347"/>
-      <c r="I63" s="347"/>
-      <c r="J63" s="347"/>
-      <c r="K63" s="347"/>
-      <c r="L63" s="360"/>
+      <c r="D63" s="345"/>
+      <c r="E63" s="345"/>
+      <c r="F63" s="345"/>
+      <c r="G63" s="345"/>
+      <c r="H63" s="345"/>
+      <c r="I63" s="345"/>
+      <c r="J63" s="345"/>
+      <c r="K63" s="345"/>
+      <c r="L63" s="346"/>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="164"/>
@@ -17085,7 +17085,7 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.2">
@@ -17095,7 +17095,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="43" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.2">
@@ -17103,7 +17103,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
@@ -17113,7 +17113,7 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="43" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.2">
@@ -17121,17 +17121,17 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="229" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="228" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="43" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.2">
@@ -17165,13 +17165,49 @@
     </row>
     <row r="89" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A89" s="343" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="93" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="94" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="B19:K19"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="C62:L62"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B42:L42"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="C61:L61"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="C59:L59"/>
+    <mergeCell ref="B43:L43"/>
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B31:L31"/>
+    <mergeCell ref="B32:L32"/>
+    <mergeCell ref="B33:L33"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="B35:L35"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="B12:L12"/>
+    <mergeCell ref="B13:K13"/>
     <mergeCell ref="C58:L58"/>
     <mergeCell ref="C63:L63"/>
     <mergeCell ref="A47:L47"/>
@@ -17188,42 +17224,6 @@
     <mergeCell ref="B45:L45"/>
     <mergeCell ref="B8:L8"/>
     <mergeCell ref="B9:L9"/>
-    <mergeCell ref="A11:L11"/>
-    <mergeCell ref="B14:L14"/>
-    <mergeCell ref="C59:L59"/>
-    <mergeCell ref="B43:L43"/>
-    <mergeCell ref="B30:L30"/>
-    <mergeCell ref="B31:L31"/>
-    <mergeCell ref="B32:L32"/>
-    <mergeCell ref="B33:L33"/>
-    <mergeCell ref="B34:L34"/>
-    <mergeCell ref="B35:L35"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="A37:L37"/>
-    <mergeCell ref="B38:L38"/>
-    <mergeCell ref="B39:L39"/>
-    <mergeCell ref="B12:L12"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A7:L7"/>
-    <mergeCell ref="B13:K13"/>
-    <mergeCell ref="B19:K19"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="C62:L62"/>
-    <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="A25:L25"/>
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B42:L42"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="C61:L61"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A70" r:id="rId1" xr:uid="{C9866D44-2827-49D7-B9C3-89CF23FACDC1}"/>
@@ -17365,35 +17365,35 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="36" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D3" s="35" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="E3" s="35" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="F3" s="321"/>
     </row>
     <row r="4" spans="1:6" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="323" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B4" s="322"/>
       <c r="C4" s="322"/>
@@ -17403,7 +17403,7 @@
     </row>
     <row r="5" spans="1:6" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="319" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B5" s="320"/>
       <c r="C5" s="320"/>
@@ -17413,16 +17413,16 @@
     </row>
     <row r="6" spans="1:6" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="37" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C6" s="311">
         <v>0.17499999999999999</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="E6" s="309">
         <v>29.8</v>
@@ -17431,7 +17431,7 @@
     </row>
     <row r="7" spans="1:6" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="37" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B7" s="38">
         <v>2023</v>
@@ -17441,7 +17441,7 @@
         <v>3.7811999999999998E-2</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E7" s="309">
         <f>0.992+1.205+5.344+8.335</f>
@@ -17451,16 +17451,16 @@
     </row>
     <row r="8" spans="1:6" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="37" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C8" s="311">
         <v>2.2116E-2</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E8" s="309">
         <v>4.5599999999999996</v>
@@ -17469,7 +17469,7 @@
     </row>
     <row r="9" spans="1:6" s="57" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="319" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B9" s="320"/>
       <c r="C9" s="320"/>
@@ -17478,43 +17478,43 @@
     </row>
     <row r="10" spans="1:6" s="57" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="37" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C10" s="311">
         <v>4.0999999999999996</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E10" s="309" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="F10" s="318"/>
     </row>
     <row r="11" spans="1:6" s="57" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="37" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C11" s="311">
         <v>0.63121000000000005</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E11" s="309" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="F11" s="318"/>
     </row>
     <row r="12" spans="1:6" s="56" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="317" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B12" s="315"/>
       <c r="C12" s="316"/>
@@ -17524,44 +17524,44 @@
     </row>
     <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="37" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B13" s="21">
         <v>2021</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="37" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B14" s="21">
         <v>2021</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D14" s="312">
         <v>2000</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="37" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C15" s="311">
         <v>1</v>
@@ -17589,12 +17589,12 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="446" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B2" s="447"/>
       <c r="C2" s="447"/>
@@ -17619,36 +17619,36 @@
     <row r="3" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:20" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="262" t="s">
+        <v>348</v>
+      </c>
+      <c r="B4" s="263" t="s">
         <v>349</v>
       </c>
-      <c r="B4" s="263" t="s">
+      <c r="C4" s="264" t="s">
+        <v>416</v>
+      </c>
+      <c r="D4" s="265" t="s">
         <v>350</v>
       </c>
-      <c r="C4" s="264" t="s">
-        <v>417</v>
-      </c>
-      <c r="D4" s="265" t="s">
+      <c r="E4" s="265" t="s">
         <v>351</v>
       </c>
-      <c r="E4" s="265" t="s">
+      <c r="F4" s="265" t="s">
         <v>352</v>
       </c>
-      <c r="F4" s="265" t="s">
+      <c r="G4" s="265" t="s">
         <v>353</v>
       </c>
-      <c r="G4" s="265" t="s">
+      <c r="H4" s="265" t="s">
         <v>354</v>
       </c>
-      <c r="H4" s="265" t="s">
+      <c r="I4" s="266" t="s">
         <v>355</v>
-      </c>
-      <c r="I4" s="266" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="267" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B5" s="237">
         <v>64</v>
@@ -17678,7 +17678,7 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="268" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B6" s="237">
         <v>112</v>
@@ -17687,7 +17687,7 @@
         <v>11.6</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E6">
         <v>81</v>
@@ -17708,7 +17708,7 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="268" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B7" s="237">
         <v>100</v>
@@ -17717,7 +17717,7 @@
         <v>14.1</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E7">
         <v>13</v>
@@ -17738,7 +17738,7 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" s="268" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B8" s="237">
         <v>97</v>
@@ -17747,7 +17747,7 @@
         <v>14.1</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E8">
         <v>147</v>
@@ -17766,12 +17766,12 @@
         <v>4.7</v>
       </c>
       <c r="J8" s="270" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="268" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B9" s="237">
         <v>112</v>
@@ -17780,7 +17780,7 @@
         <v>16.5</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E9">
         <v>103</v>
@@ -17799,12 +17799,12 @@
         <v>5.5</v>
       </c>
       <c r="J9" s="270" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" s="268" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B10" s="237">
         <v>100</v>
@@ -17813,7 +17813,7 @@
         <v>16.600000000000001</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E10">
         <v>26</v>
@@ -17834,7 +17834,7 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="268" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B11" s="237">
         <v>112</v>
@@ -17843,7 +17843,7 @@
         <v>16.600000000000001</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E11">
         <v>81</v>
@@ -17862,12 +17862,12 @@
         <v>5.5</v>
       </c>
       <c r="J11" s="270" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" s="268" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B12" s="237">
         <v>100</v>
@@ -17876,7 +17876,7 @@
         <v>17.8</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E12">
         <v>31</v>
@@ -17897,7 +17897,7 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="268" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B13" s="237">
         <v>100</v>
@@ -17906,7 +17906,7 @@
         <v>18</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E13">
         <v>18</v>
@@ -17927,7 +17927,7 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="268" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B14" s="237">
         <v>112</v>
@@ -17936,7 +17936,7 @@
         <v>19.3</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E14">
         <v>81</v>
@@ -17957,7 +17957,7 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="268" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B15" s="237">
         <v>100</v>
@@ -17966,7 +17966,7 @@
         <v>20.399999999999999</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E15">
         <v>48</v>
@@ -17987,7 +17987,7 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" s="268" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B16" s="237">
         <v>100</v>
@@ -17996,7 +17996,7 @@
         <v>20.399999999999999</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E16">
         <v>45</v>
@@ -18017,7 +18017,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="268" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B17" s="237">
         <v>100</v>
@@ -18026,7 +18026,7 @@
         <v>20.5</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E17">
         <v>2</v>
@@ -18047,7 +18047,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="268" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B18" s="237">
         <v>1</v>
@@ -18056,7 +18056,7 @@
         <v>20.9</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E18">
         <v>430</v>
@@ -18077,7 +18077,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="268" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B19" s="237">
         <v>1</v>
@@ -18086,7 +18086,7 @@
         <v>20.9</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E19">
         <v>430</v>
@@ -18107,7 +18107,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="268" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B20" s="237">
         <v>112</v>
@@ -18116,7 +18116,7 @@
         <v>21.7</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E20">
         <v>81</v>
@@ -18137,7 +18137,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="268" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B21" s="237">
         <v>112</v>
@@ -18146,7 +18146,7 @@
         <v>21.8</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E21">
         <v>81</v>
@@ -18167,7 +18167,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="268" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B22" s="237">
         <v>112</v>
@@ -18176,7 +18176,7 @@
         <v>24.2</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E22">
         <v>80</v>
@@ -18197,7 +18197,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="268" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B23" s="237">
         <v>100</v>
@@ -18206,7 +18206,7 @@
         <v>24.8</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E23">
         <v>5</v>
@@ -18227,7 +18227,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="268" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B24" s="237">
         <v>1</v>
@@ -18236,7 +18236,7 @@
         <v>26.1</v>
       </c>
       <c r="D24" s="239" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E24" s="237">
         <v>97</v>
@@ -18257,7 +18257,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="268" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B25" s="237">
         <v>1</v>
@@ -18266,7 +18266,7 @@
         <v>26.1</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E25">
         <v>72</v>
@@ -18287,7 +18287,7 @@
     </row>
     <row r="26" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="269" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B26" s="240">
         <v>1</v>
@@ -18296,7 +18296,7 @@
         <v>26.1</v>
       </c>
       <c r="D26" s="242" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E26" s="241">
         <v>15</v>
@@ -18473,10 +18473,10 @@
         <v>45666</v>
       </c>
       <c r="B6" s="146" t="s">
+        <v>297</v>
+      </c>
+      <c r="C6" s="54" t="s">
         <v>298</v>
-      </c>
-      <c r="C6" s="54" t="s">
-        <v>299</v>
       </c>
       <c r="D6" s="53">
         <v>3</v>
@@ -18497,10 +18497,10 @@
         <v>45670</v>
       </c>
       <c r="B7" s="146" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D7" s="53">
         <v>0.5</v>
@@ -18521,10 +18521,10 @@
         <v>45671</v>
       </c>
       <c r="B8" s="146" t="s">
+        <v>329</v>
+      </c>
+      <c r="C8" s="54" t="s">
         <v>330</v>
-      </c>
-      <c r="C8" s="54" t="s">
-        <v>331</v>
       </c>
       <c r="D8" s="53">
         <v>0.5</v>
@@ -18545,10 +18545,10 @@
         <v>45681</v>
       </c>
       <c r="B9" s="146" t="s">
+        <v>342</v>
+      </c>
+      <c r="C9" s="54" t="s">
         <v>343</v>
-      </c>
-      <c r="C9" s="54" t="s">
-        <v>344</v>
       </c>
       <c r="D9" s="53">
         <v>0.25</v>
@@ -18569,10 +18569,10 @@
         <v>45681</v>
       </c>
       <c r="B10" s="146" t="s">
+        <v>346</v>
+      </c>
+      <c r="C10" s="54" t="s">
         <v>347</v>
-      </c>
-      <c r="C10" s="54" t="s">
-        <v>348</v>
       </c>
       <c r="D10" s="53">
         <v>1</v>
@@ -18581,7 +18581,7 @@
         <v>240</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G10" s="55">
         <v>45678</v>
@@ -18598,16 +18598,16 @@
         <v>1.5</v>
       </c>
       <c r="C11" s="54" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D11" s="53">
         <v>12</v>
       </c>
       <c r="E11" s="53" t="s">
+        <v>396</v>
+      </c>
+      <c r="F11" s="53" t="s">
         <v>397</v>
-      </c>
-      <c r="F11" s="53" t="s">
-        <v>398</v>
       </c>
       <c r="G11" s="55">
         <v>45702</v>
@@ -18624,16 +18624,16 @@
         <v>1.6</v>
       </c>
       <c r="C12" s="54" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D12" s="53">
         <v>6</v>
       </c>
       <c r="E12" s="53" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F12" s="53" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G12" s="55">
         <v>45702</v>
@@ -18647,19 +18647,19 @@
         <v>45827</v>
       </c>
       <c r="B13" s="146" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C13" s="54" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D13" s="53">
         <v>5</v>
       </c>
       <c r="E13" s="53" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F13" s="53" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G13" s="55">
         <v>45702</v>
@@ -18676,13 +18676,13 @@
         <v>1.7</v>
       </c>
       <c r="C14" s="54" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D14" s="53">
         <v>1.5</v>
       </c>
       <c r="E14" s="53" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F14" s="53" t="s">
         <v>240</v>
@@ -18699,10 +18699,10 @@
         <v>45895</v>
       </c>
       <c r="B15" s="146" t="s">
+        <v>465</v>
+      </c>
+      <c r="C15" s="54" t="s">
         <v>466</v>
-      </c>
-      <c r="C15" s="54" t="s">
-        <v>467</v>
       </c>
       <c r="D15" s="53">
         <v>0.5</v>
@@ -18721,10 +18721,10 @@
         <v>45895</v>
       </c>
       <c r="B16" s="146" t="s">
+        <v>467</v>
+      </c>
+      <c r="C16" s="54" t="s">
         <v>468</v>
-      </c>
-      <c r="C16" s="54" t="s">
-        <v>469</v>
       </c>
       <c r="D16" s="53">
         <v>1</v>
@@ -18743,16 +18743,16 @@
         <v>45993</v>
       </c>
       <c r="B17" s="146" t="s">
+        <v>469</v>
+      </c>
+      <c r="C17" s="54" t="s">
         <v>470</v>
-      </c>
-      <c r="C17" s="54" t="s">
-        <v>471</v>
       </c>
       <c r="D17" s="53">
         <v>0.5</v>
       </c>
       <c r="E17" s="53" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F17" s="53" t="s">
         <v>240</v>
@@ -18766,16 +18766,16 @@
         <v>46121</v>
       </c>
       <c r="B18" s="146" t="s">
+        <v>477</v>
+      </c>
+      <c r="C18" s="54" t="s">
         <v>478</v>
-      </c>
-      <c r="C18" s="54" t="s">
-        <v>479</v>
       </c>
       <c r="D18" s="53">
         <v>0.2</v>
       </c>
       <c r="E18" s="53" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F18" s="53" t="s">
         <v>240</v>
@@ -19068,7 +19068,7 @@
       <c r="F4" s="406"/>
       <c r="G4" s="407"/>
       <c r="N4" s="138" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -19226,7 +19226,7 @@
         <v>5.981122</v>
       </c>
       <c r="D19" s="126" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F19" s="236" t="s">
         <v>208</v>
@@ -19297,7 +19297,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B24" s="92">
         <f>TribalWater!H7</f>
@@ -19307,12 +19307,12 @@
       <c r="D24" s="109"/>
       <c r="E24" s="27"/>
       <c r="N24" s="138" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B25" s="217">
         <f>1-B24</f>
@@ -19322,7 +19322,7 @@
       <c r="D25" s="109"/>
       <c r="E25" s="27"/>
       <c r="N25" s="138" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
@@ -20897,7 +20897,7 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C64" s="12" t="str">
         <f>IF(OR(C$28="",$A69=""),"",C36+C53-C46)</f>
@@ -20981,12 +20981,12 @@
       <c r="L66" s="325"/>
       <c r="M66" s="326"/>
       <c r="N66" s="338" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C67" s="324" t="str">
         <f>IF(OR(C65="",C66=""),"",IF(C66&gt;0,ABS(C65*C66),C65*C66)
@@ -21223,7 +21223,7 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C74" s="12" t="str">
         <f>IF(OR(C$28="",$A79=""),"",C37+C55-C47)</f>
@@ -21307,12 +21307,12 @@
       <c r="L76" s="325"/>
       <c r="M76" s="326"/>
       <c r="N76" s="338" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C77" s="324" t="str">
         <f>IF(OR(C75="",C76=""),"",IF(C76&gt;0,ABS(C75*C76),C75*C76)
@@ -21548,7 +21548,7 @@
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C84" s="12" t="str">
         <f>IF(OR(C$28="",$A89=""),"",C38+C56-C48)</f>
@@ -21632,12 +21632,12 @@
       <c r="L86" s="325"/>
       <c r="M86" s="326"/>
       <c r="N86" s="338" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C87" s="324" t="str">
         <f>IF(OR(C85="",C86=""),"",IF(C86&gt;0,ABS(C85*C86),C85*C86)
@@ -21873,7 +21873,7 @@
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C94" s="12" t="str">
         <f>IF(OR(C$28="",$A99=""),"",C39+C57-C49)</f>
@@ -21957,12 +21957,12 @@
       <c r="L96" s="325"/>
       <c r="M96" s="326"/>
       <c r="N96" s="338" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C97" s="324" t="str">
         <f>IF(OR(C95="",C96=""),"",IF(C96&gt;0,ABS(C95*C96),C95*C96)
@@ -22198,7 +22198,7 @@
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C104" s="12" t="str">
         <f>IF(OR(C$28="",$A109=""),"",C40+C58-C50)</f>
@@ -22244,7 +22244,7 @@
     </row>
     <row r="105" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A105" s="123" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B105" s="237"/>
       <c r="C105" s="89"/>
@@ -22269,7 +22269,7 @@
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A106" s="123" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B106" s="237"/>
       <c r="C106" s="90"/>
@@ -22284,12 +22284,12 @@
       <c r="L106" s="90"/>
       <c r="M106" s="326"/>
       <c r="N106" s="338" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="107" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B107" s="237"/>
       <c r="C107" s="324" t="str">
@@ -22528,7 +22528,7 @@
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C114" s="12" t="str">
         <f>IF(OR(C$28="",$A119=""),"",C41+C59-C51)</f>
@@ -22574,7 +22574,7 @@
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A115" s="123" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B115" s="237"/>
       <c r="C115" s="89"/>
@@ -22599,7 +22599,7 @@
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A116" s="123" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B116" s="237"/>
       <c r="C116" s="90"/>
@@ -22614,12 +22614,12 @@
       <c r="L116" s="90"/>
       <c r="M116" s="326"/>
       <c r="N116" s="338" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B117" s="237"/>
       <c r="C117" s="324" t="str">
@@ -24562,62 +24562,62 @@
       <c r="G5" s="185" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="424" t="s">
-        <v>421</v>
-      </c>
-      <c r="J5" s="425"/>
-      <c r="K5" s="425"/>
-      <c r="L5" s="425"/>
-      <c r="M5" s="425"/>
-      <c r="N5" s="425"/>
-      <c r="O5" s="425"/>
-      <c r="P5" s="425"/>
-      <c r="Q5" s="425"/>
-      <c r="R5" s="425"/>
-      <c r="S5" s="425"/>
-      <c r="T5" s="425"/>
-      <c r="U5" s="425"/>
-      <c r="V5" s="425"/>
-      <c r="W5" s="426"/>
+      <c r="I5" s="429" t="s">
+        <v>420</v>
+      </c>
+      <c r="J5" s="430"/>
+      <c r="K5" s="430"/>
+      <c r="L5" s="430"/>
+      <c r="M5" s="430"/>
+      <c r="N5" s="430"/>
+      <c r="O5" s="430"/>
+      <c r="P5" s="430"/>
+      <c r="Q5" s="430"/>
+      <c r="R5" s="430"/>
+      <c r="S5" s="430"/>
+      <c r="T5" s="430"/>
+      <c r="U5" s="430"/>
+      <c r="V5" s="430"/>
+      <c r="W5" s="431"/>
       <c r="Y5" s="192"/>
       <c r="Z5" s="192"/>
       <c r="AA5" s="192"/>
       <c r="AB5" s="334"/>
     </row>
     <row r="6" spans="1:53" s="184" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B6" s="416" t="s">
+      <c r="B6" s="418" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="417"/>
-      <c r="D6" s="417"/>
-      <c r="E6" s="417"/>
-      <c r="F6" s="417"/>
-      <c r="G6" s="418"/>
-      <c r="I6" s="427" t="s">
+      <c r="C6" s="419"/>
+      <c r="D6" s="419"/>
+      <c r="E6" s="419"/>
+      <c r="F6" s="419"/>
+      <c r="G6" s="420"/>
+      <c r="I6" s="432" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="429" t="s">
-        <v>407</v>
-      </c>
-      <c r="K6" s="429" t="s">
+      <c r="J6" s="416" t="s">
         <v>406</v>
       </c>
-      <c r="L6" s="430" t="s">
+      <c r="K6" s="416" t="s">
+        <v>405</v>
+      </c>
+      <c r="L6" s="434" t="s">
         <v>215</v>
       </c>
-      <c r="M6" s="431"/>
-      <c r="N6" s="431"/>
-      <c r="O6" s="431"/>
-      <c r="P6" s="431"/>
-      <c r="Q6" s="432"/>
-      <c r="R6" s="433" t="s">
+      <c r="M6" s="435"/>
+      <c r="N6" s="435"/>
+      <c r="O6" s="435"/>
+      <c r="P6" s="435"/>
+      <c r="Q6" s="436"/>
+      <c r="R6" s="421" t="s">
         <v>216</v>
       </c>
-      <c r="S6" s="434"/>
-      <c r="T6" s="434"/>
-      <c r="U6" s="434"/>
-      <c r="V6" s="434"/>
-      <c r="W6" s="435"/>
+      <c r="S6" s="422"/>
+      <c r="T6" s="422"/>
+      <c r="U6" s="422"/>
+      <c r="V6" s="422"/>
+      <c r="W6" s="423"/>
       <c r="Y6" s="307"/>
       <c r="Z6" s="307"/>
       <c r="AA6" s="307"/>
@@ -24643,41 +24643,41 @@
         <f>SUM(C7:F7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="428"/>
-      <c r="J7" s="428"/>
-      <c r="K7" s="428"/>
+      <c r="I7" s="433"/>
+      <c r="J7" s="433"/>
+      <c r="K7" s="433"/>
       <c r="L7" s="186" t="s">
+        <v>407</v>
+      </c>
+      <c r="M7" s="186" t="s">
         <v>408</v>
       </c>
-      <c r="M7" s="186" t="s">
+      <c r="N7" s="186" t="s">
         <v>409</v>
       </c>
-      <c r="N7" s="186" t="s">
-        <v>410</v>
-      </c>
       <c r="O7" s="186" t="s">
+        <v>403</v>
+      </c>
+      <c r="P7" s="186" t="s">
         <v>404</v>
-      </c>
-      <c r="P7" s="186" t="s">
-        <v>405</v>
       </c>
       <c r="Q7" s="261" t="s">
         <v>222</v>
       </c>
       <c r="R7" s="187" t="s">
+        <v>410</v>
+      </c>
+      <c r="S7" s="187" t="s">
         <v>411</v>
       </c>
-      <c r="S7" s="187" t="s">
+      <c r="T7" s="187" t="s">
         <v>412</v>
       </c>
-      <c r="T7" s="187" t="s">
+      <c r="U7" s="187" t="s">
         <v>413</v>
       </c>
-      <c r="U7" s="187" t="s">
-        <v>414</v>
-      </c>
       <c r="V7" s="187" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="W7" s="247" t="s">
         <v>227</v>
@@ -24708,7 +24708,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="297" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J8" s="292">
         <v>0</v>
@@ -24765,7 +24765,7 @@
         <v>1</v>
       </c>
       <c r="X8" s="192" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="Y8" s="308"/>
     </row>
@@ -24849,14 +24849,14 @@
       <c r="AZ9" s="285"/>
     </row>
     <row r="10" spans="1:53" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="B10" s="419" t="s">
+      <c r="B10" s="424" t="s">
         <v>237</v>
       </c>
-      <c r="C10" s="419"/>
-      <c r="D10" s="419"/>
-      <c r="E10" s="419"/>
-      <c r="F10" s="419"/>
-      <c r="G10" s="419"/>
+      <c r="C10" s="424"/>
+      <c r="D10" s="424"/>
+      <c r="E10" s="424"/>
+      <c r="F10" s="424"/>
+      <c r="G10" s="424"/>
       <c r="I10" s="244" t="s">
         <v>231</v>
       </c>
@@ -25074,7 +25074,7 @@
         <v>1.0000066666666667</v>
       </c>
       <c r="X12" s="192" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="AP12" s="277"/>
       <c r="AQ12" s="277"/>
@@ -25111,7 +25111,7 @@
         <v>0.40000000000000008</v>
       </c>
       <c r="I13" s="244" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J13" s="246">
         <v>2.7</v>
@@ -25201,7 +25201,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="244" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J14" s="246">
         <v>4</v>
@@ -25281,7 +25281,7 @@
         <v>1.5</v>
       </c>
       <c r="I15" s="244" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J15" s="246">
         <v>4.4000000000000004</v>
@@ -25340,15 +25340,15 @@
       <c r="B16" s="193" t="s">
         <v>234</v>
       </c>
-      <c r="C16" s="420" t="s">
+      <c r="C16" s="425" t="s">
         <v>235</v>
       </c>
-      <c r="D16" s="421"/>
-      <c r="E16" s="421"/>
-      <c r="F16" s="421"/>
-      <c r="G16" s="422"/>
+      <c r="D16" s="426"/>
+      <c r="E16" s="426"/>
+      <c r="F16" s="426"/>
+      <c r="G16" s="427"/>
       <c r="I16" s="244" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J16" s="246">
         <v>5.2</v>
@@ -25405,7 +25405,7 @@
     </row>
     <row r="17" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="I17" s="244" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J17" s="246">
         <v>8</v>
@@ -25462,59 +25462,59 @@
     </row>
     <row r="18" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15"/>
     <row r="19" spans="2:58" s="192" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I19" s="423" t="s">
-        <v>422</v>
-      </c>
-      <c r="J19" s="423"/>
-      <c r="K19" s="423"/>
-      <c r="L19" s="423"/>
-      <c r="M19" s="423"/>
-      <c r="N19" s="423"/>
-      <c r="O19" s="423"/>
-      <c r="P19" s="423"/>
-      <c r="Q19" s="423"/>
-      <c r="R19" s="423"/>
-      <c r="S19" s="423"/>
-      <c r="T19" s="423"/>
-      <c r="U19" s="423"/>
+      <c r="I19" s="428" t="s">
+        <v>421</v>
+      </c>
+      <c r="J19" s="428"/>
+      <c r="K19" s="428"/>
+      <c r="L19" s="428"/>
+      <c r="M19" s="428"/>
+      <c r="N19" s="428"/>
+      <c r="O19" s="428"/>
+      <c r="P19" s="428"/>
+      <c r="Q19" s="428"/>
+      <c r="R19" s="428"/>
+      <c r="S19" s="428"/>
+      <c r="T19" s="428"/>
+      <c r="U19" s="428"/>
       <c r="Z19" s="250"/>
       <c r="AA19" s="250"/>
       <c r="AB19" s="250"/>
       <c r="AC19" s="250"/>
     </row>
     <row r="20" spans="2:58" s="192" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I20" s="429" t="s">
+      <c r="I20" s="416" t="s">
         <v>13</v>
       </c>
-      <c r="J20" s="429" t="s">
+      <c r="J20" s="416" t="s">
         <v>213</v>
       </c>
-      <c r="K20" s="429" t="s">
+      <c r="K20" s="416" t="s">
         <v>214</v>
       </c>
-      <c r="L20" s="416" t="s">
+      <c r="L20" s="418" t="s">
         <v>215</v>
       </c>
-      <c r="M20" s="417"/>
-      <c r="N20" s="417"/>
-      <c r="O20" s="417"/>
-      <c r="P20" s="418"/>
-      <c r="Q20" s="433" t="s">
+      <c r="M20" s="419"/>
+      <c r="N20" s="419"/>
+      <c r="O20" s="419"/>
+      <c r="P20" s="420"/>
+      <c r="Q20" s="421" t="s">
         <v>216</v>
       </c>
-      <c r="R20" s="434"/>
-      <c r="S20" s="434"/>
-      <c r="T20" s="434"/>
-      <c r="U20" s="435"/>
+      <c r="R20" s="422"/>
+      <c r="S20" s="422"/>
+      <c r="T20" s="422"/>
+      <c r="U20" s="423"/>
       <c r="Z20" s="254"/>
       <c r="AA20" s="254"/>
       <c r="AB20" s="254"/>
       <c r="AC20" s="254"/>
     </row>
     <row r="21" spans="2:58" s="192" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I21" s="436"/>
-      <c r="J21" s="436"/>
-      <c r="K21" s="436"/>
+      <c r="I21" s="417"/>
+      <c r="J21" s="417"/>
+      <c r="K21" s="417"/>
       <c r="L21" s="186" t="s">
         <v>218</v>
       </c>
@@ -25551,7 +25551,7 @@
     </row>
     <row r="22" spans="2:58" s="192" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.15">
       <c r="I22" s="297" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J22" s="288">
         <f>B11</f>
@@ -25597,7 +25597,7 @@
         <v>1</v>
       </c>
       <c r="V22" s="192" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="W22" s="258"/>
       <c r="AF22" s="336"/>
@@ -25848,7 +25848,7 @@
       <c r="F27" s="287"/>
       <c r="G27" s="287"/>
       <c r="I27" s="244" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J27" s="188">
         <v>2.7</v>
@@ -25902,7 +25902,7 @@
     </row>
     <row r="28" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="I28" s="244" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J28" s="244">
         <f>9-K28</f>
@@ -25952,7 +25952,7 @@
         <v>1</v>
       </c>
       <c r="V28" s="306" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="W28" s="256"/>
     </row>
@@ -25963,7 +25963,7 @@
       <c r="F29" s="287"/>
       <c r="G29" s="287"/>
       <c r="I29" s="244" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J29" s="244">
         <f>9-K29</f>
@@ -26022,7 +26022,7 @@
       <c r="F30" s="287"/>
       <c r="G30" s="287"/>
       <c r="I30" s="244" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J30" s="244">
         <f>9-K30</f>
@@ -26081,7 +26081,7 @@
       <c r="F31" s="287"/>
       <c r="G31" s="287"/>
       <c r="I31" s="244" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J31" s="188">
         <v>8</v>
@@ -26131,7 +26131,7 @@
         <v>1</v>
       </c>
       <c r="V31" s="304" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="W31" s="256"/>
     </row>
@@ -26536,11 +26536,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:P20"/>
-    <mergeCell ref="Q20:U20"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="C16:G16"/>
@@ -26551,6 +26546,11 @@
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:Q6"/>
     <mergeCell ref="R6:W6"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:P20"/>
+    <mergeCell ref="Q20:U20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26570,40 +26570,40 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="218" t="s">
+        <v>304</v>
+      </c>
+      <c r="B4" s="218" t="s">
         <v>305</v>
       </c>
-      <c r="B4" s="218" t="s">
+      <c r="C4" s="219" t="s">
         <v>306</v>
       </c>
-      <c r="C4" s="219" t="s">
+      <c r="D4" s="219" t="s">
         <v>307</v>
       </c>
-      <c r="D4" s="219" t="s">
-        <v>308</v>
-      </c>
       <c r="F4" s="219" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G4" s="219" t="s">
+        <v>314</v>
+      </c>
+      <c r="H4" s="219" t="s">
         <v>315</v>
-      </c>
-      <c r="H4" s="219" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="22" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B5" s="22" t="s">
         <v>204</v>
@@ -26626,7 +26626,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B6" s="22" t="s">
         <v>203</v>
@@ -26649,7 +26649,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B7" s="22" t="s">
         <v>202</v>
@@ -26672,7 +26672,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B8" s="22" t="s">
         <v>202</v>
@@ -26695,7 +26695,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B9" s="22" t="s">
         <v>203</v>
@@ -26707,7 +26707,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B10" s="22" t="s">
         <v>202</v>
@@ -26720,7 +26720,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B11" s="22" t="s">
         <v>203</v>
@@ -26732,7 +26732,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B12" s="22" t="s">
         <v>202</v>
@@ -26750,7 +26750,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B13" s="22" t="s">
         <v>203</v>
@@ -26778,23 +26778,23 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="218" t="s">
+        <v>317</v>
+      </c>
+      <c r="B18" s="226" t="s">
         <v>318</v>
       </c>
-      <c r="B18" s="226" t="s">
+      <c r="C18" s="226" t="s">
         <v>319</v>
-      </c>
-      <c r="C18" s="226" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="22" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B19" s="23">
         <v>769208</v>
@@ -26805,7 +26805,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="22" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B20" s="23">
         <v>15340</v>
@@ -26816,7 +26816,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="22" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B21" s="23">
         <v>2844</v>
@@ -26827,7 +26827,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="22" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B22" s="23">
         <v>13000</v>
@@ -26883,16 +26883,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="437" t="e">
+      <c r="A1" s="438" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B1" s="437"/>
-      <c r="C1" s="437"/>
-      <c r="D1" s="437"/>
-      <c r="E1" s="437"/>
-      <c r="F1" s="437"/>
-      <c r="G1" s="437"/>
+      <c r="B1" s="438"/>
+      <c r="C1" s="438"/>
+      <c r="D1" s="438"/>
+      <c r="E1" s="438"/>
+      <c r="F1" s="438"/>
+      <c r="G1" s="438"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -27001,11 +27001,11 @@
         <v>40</v>
       </c>
       <c r="B10" s="112"/>
-      <c r="C10" s="438"/>
-      <c r="D10" s="438"/>
-      <c r="E10" s="438"/>
-      <c r="F10" s="438"/>
-      <c r="G10" s="438"/>
+      <c r="C10" s="437"/>
+      <c r="D10" s="437"/>
+      <c r="E10" s="437"/>
+      <c r="F10" s="437"/>
+      <c r="G10" s="437"/>
       <c r="N10" s="139"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -28268,6 +28268,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:G6"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="C9:G9"/>
@@ -28275,12 +28281,6 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N4" r:id="rId1" location="step-1-assign-parties-person-playing-and-strategies" xr:uid="{726B234F-7B54-4D33-A192-8F1604C6B04C}"/>

</xml_diff>

<commit_message>
Updated media and model file with June inflows scenarios
</commit_message>
<xml_diff>
--- a/LakeMeadWaterBankDivideInflow.xlsx
+++ b/LakeMeadWaterBankDivideInflow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anabelle/Documents/LakeMeadDivideInflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FB57E1-6E5B-6345-AF43-F096115C30E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E27EC66-DD37-A44B-A760-FBC9FBA0AAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="2" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe-Directions" sheetId="62" r:id="rId1"/>
@@ -52,7 +52,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="2">
+  <futureMetadata name="XLRICHVALUE" count="1">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -60,20 +60,10 @@
         </ext>
       </extLst>
     </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
   </futureMetadata>
-  <valueMetadata count="2">
+  <valueMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -4199,10 +4189,97 @@
     <xf numFmtId="0" fontId="1" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -4241,9 +4318,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4262,94 +4336,10 @@
     <xf numFmtId="0" fontId="1" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="1" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="4" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4412,6 +4402,12 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4420,6 +4416,15 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4451,9 +4456,6 @@
     <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4463,23 +4465,11 @@
     <xf numFmtId="0" fontId="18" fillId="19" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -15277,6 +15267,55 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9769</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>605693</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>70221</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>2427654</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{434A8A38-C447-049F-82C0-23B5FF43D938}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="273538" y="3350847"/>
+          <a:ext cx="4056068" cy="2456961"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -15593,13 +15632,9 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
   <rv s="0">
     <v>0</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>1</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -15617,7 +15652,6 @@
 <file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
 <richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <rel r:id="rId1"/>
-  <rel r:id="rId2"/>
 </richValueRels>
 </file>
 
@@ -15936,20 +15970,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="370" t="s">
+      <c r="A1" s="371" t="s">
         <v>294</v>
       </c>
-      <c r="B1" s="370"/>
-      <c r="C1" s="370"/>
-      <c r="D1" s="370"/>
-      <c r="E1" s="370"/>
-      <c r="F1" s="370"/>
-      <c r="G1" s="370"/>
-      <c r="H1" s="370"/>
-      <c r="I1" s="370"/>
-      <c r="J1" s="370"/>
-      <c r="K1" s="370"/>
-      <c r="L1" s="370"/>
+      <c r="B1" s="371"/>
+      <c r="C1" s="371"/>
+      <c r="D1" s="371"/>
+      <c r="E1" s="371"/>
+      <c r="F1" s="371"/>
+      <c r="G1" s="371"/>
+      <c r="H1" s="371"/>
+      <c r="I1" s="371"/>
+      <c r="J1" s="371"/>
+      <c r="K1" s="371"/>
+      <c r="L1" s="371"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
@@ -15975,41 +16009,41 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:18" s="52" customFormat="1" ht="53.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="371" t="s">
+      <c r="A4" s="372" t="s">
         <v>482</v>
       </c>
-      <c r="B4" s="372"/>
-      <c r="C4" s="372"/>
-      <c r="D4" s="372"/>
-      <c r="E4" s="372"/>
-      <c r="F4" s="372"/>
-      <c r="G4" s="372"/>
-      <c r="H4" s="372"/>
-      <c r="I4" s="372"/>
-      <c r="J4" s="372"/>
-      <c r="K4" s="372"/>
-      <c r="L4" s="373"/>
-      <c r="N4" s="374"/>
-      <c r="O4" s="374"/>
-      <c r="P4" s="374"/>
-      <c r="Q4" s="374"/>
-      <c r="R4" s="374"/>
+      <c r="B4" s="373"/>
+      <c r="C4" s="373"/>
+      <c r="D4" s="373"/>
+      <c r="E4" s="373"/>
+      <c r="F4" s="373"/>
+      <c r="G4" s="373"/>
+      <c r="H4" s="373"/>
+      <c r="I4" s="373"/>
+      <c r="J4" s="373"/>
+      <c r="K4" s="373"/>
+      <c r="L4" s="374"/>
+      <c r="N4" s="375"/>
+      <c r="O4" s="375"/>
+      <c r="P4" s="375"/>
+      <c r="Q4" s="375"/>
+      <c r="R4" s="375"/>
     </row>
     <row r="5" spans="1:18" s="52" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="375" t="s">
+      <c r="A5" s="350" t="s">
         <v>480</v>
       </c>
-      <c r="B5" s="376"/>
-      <c r="C5" s="376"/>
-      <c r="D5" s="376"/>
-      <c r="E5" s="376"/>
-      <c r="F5" s="376"/>
-      <c r="G5" s="376"/>
-      <c r="H5" s="376"/>
-      <c r="I5" s="376"/>
-      <c r="J5" s="376"/>
-      <c r="K5" s="376"/>
-      <c r="L5" s="377"/>
+      <c r="B5" s="351"/>
+      <c r="C5" s="351"/>
+      <c r="D5" s="351"/>
+      <c r="E5" s="351"/>
+      <c r="F5" s="351"/>
+      <c r="G5" s="351"/>
+      <c r="H5" s="351"/>
+      <c r="I5" s="351"/>
+      <c r="J5" s="351"/>
+      <c r="K5" s="351"/>
+      <c r="L5" s="352"/>
       <c r="N5" s="110"/>
       <c r="O5" s="110"/>
       <c r="P5" s="110"/>
@@ -16017,20 +16051,20 @@
       <c r="R5" s="110"/>
     </row>
     <row r="6" spans="1:18" s="52" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="375" t="s">
+      <c r="A6" s="350" t="s">
         <v>478</v>
       </c>
-      <c r="B6" s="376"/>
-      <c r="C6" s="376"/>
-      <c r="D6" s="376"/>
-      <c r="E6" s="376"/>
-      <c r="F6" s="376"/>
-      <c r="G6" s="376"/>
-      <c r="H6" s="376"/>
-      <c r="I6" s="376"/>
-      <c r="J6" s="376"/>
-      <c r="K6" s="376"/>
-      <c r="L6" s="377"/>
+      <c r="B6" s="351"/>
+      <c r="C6" s="351"/>
+      <c r="D6" s="351"/>
+      <c r="E6" s="351"/>
+      <c r="F6" s="351"/>
+      <c r="G6" s="351"/>
+      <c r="H6" s="351"/>
+      <c r="I6" s="351"/>
+      <c r="J6" s="351"/>
+      <c r="K6" s="351"/>
+      <c r="L6" s="352"/>
       <c r="N6" s="110"/>
       <c r="O6" s="110"/>
       <c r="P6" s="110"/>
@@ -16038,20 +16072,20 @@
       <c r="R6" s="110"/>
     </row>
     <row r="7" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="375" t="s">
+      <c r="A7" s="350" t="s">
         <v>479</v>
       </c>
-      <c r="B7" s="376"/>
-      <c r="C7" s="376"/>
-      <c r="D7" s="376"/>
-      <c r="E7" s="376"/>
-      <c r="F7" s="376"/>
-      <c r="G7" s="376"/>
-      <c r="H7" s="376"/>
-      <c r="I7" s="376"/>
-      <c r="J7" s="376"/>
-      <c r="K7" s="376"/>
-      <c r="L7" s="377"/>
+      <c r="B7" s="351"/>
+      <c r="C7" s="351"/>
+      <c r="D7" s="351"/>
+      <c r="E7" s="351"/>
+      <c r="F7" s="351"/>
+      <c r="G7" s="351"/>
+      <c r="H7" s="351"/>
+      <c r="I7" s="351"/>
+      <c r="J7" s="351"/>
+      <c r="K7" s="351"/>
+      <c r="L7" s="352"/>
       <c r="N7" s="110"/>
       <c r="O7" s="110"/>
       <c r="P7" s="110"/>
@@ -16060,19 +16094,19 @@
     </row>
     <row r="8" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="214"/>
-      <c r="B8" s="376" t="s">
+      <c r="B8" s="351" t="s">
         <v>295</v>
       </c>
-      <c r="C8" s="376"/>
-      <c r="D8" s="376"/>
-      <c r="E8" s="376"/>
-      <c r="F8" s="376"/>
-      <c r="G8" s="376"/>
-      <c r="H8" s="376"/>
-      <c r="I8" s="376"/>
-      <c r="J8" s="376"/>
-      <c r="K8" s="376"/>
-      <c r="L8" s="377"/>
+      <c r="C8" s="351"/>
+      <c r="D8" s="351"/>
+      <c r="E8" s="351"/>
+      <c r="F8" s="351"/>
+      <c r="G8" s="351"/>
+      <c r="H8" s="351"/>
+      <c r="I8" s="351"/>
+      <c r="J8" s="351"/>
+      <c r="K8" s="351"/>
+      <c r="L8" s="352"/>
       <c r="N8" s="110"/>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
@@ -16081,19 +16115,19 @@
     </row>
     <row r="9" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="215"/>
-      <c r="B9" s="394" t="s">
+      <c r="B9" s="366" t="s">
         <v>296</v>
       </c>
-      <c r="C9" s="394"/>
-      <c r="D9" s="394"/>
-      <c r="E9" s="394"/>
-      <c r="F9" s="394"/>
-      <c r="G9" s="394"/>
-      <c r="H9" s="394"/>
-      <c r="I9" s="394"/>
-      <c r="J9" s="394"/>
-      <c r="K9" s="394"/>
-      <c r="L9" s="395"/>
+      <c r="C9" s="366"/>
+      <c r="D9" s="366"/>
+      <c r="E9" s="366"/>
+      <c r="F9" s="366"/>
+      <c r="G9" s="366"/>
+      <c r="H9" s="366"/>
+      <c r="I9" s="366"/>
+      <c r="J9" s="366"/>
+      <c r="K9" s="366"/>
+      <c r="L9" s="367"/>
       <c r="N9" s="110"/>
       <c r="O9" s="110"/>
       <c r="P9" s="110"/>
@@ -16115,81 +16149,79 @@
       <c r="L10" s="110"/>
     </row>
     <row r="11" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="378" t="s">
+      <c r="A11" s="368" t="s">
         <v>331</v>
       </c>
-      <c r="B11" s="379"/>
-      <c r="C11" s="379"/>
-      <c r="D11" s="379"/>
-      <c r="E11" s="379"/>
-      <c r="F11" s="379"/>
-      <c r="G11" s="379"/>
-      <c r="H11" s="379"/>
-      <c r="I11" s="379"/>
-      <c r="J11" s="379"/>
-      <c r="K11" s="379"/>
-      <c r="L11" s="380"/>
+      <c r="B11" s="369"/>
+      <c r="C11" s="369"/>
+      <c r="D11" s="369"/>
+      <c r="E11" s="369"/>
+      <c r="F11" s="369"/>
+      <c r="G11" s="369"/>
+      <c r="H11" s="369"/>
+      <c r="I11" s="369"/>
+      <c r="J11" s="369"/>
+      <c r="K11" s="369"/>
+      <c r="L11" s="370"/>
     </row>
     <row r="12" spans="1:18" s="57" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="344" t="s">
         <v>332</v>
       </c>
-      <c r="B12" s="381" t="s">
+      <c r="B12" s="360" t="s">
         <v>481</v>
       </c>
-      <c r="C12" s="381"/>
-      <c r="D12" s="381"/>
-      <c r="E12" s="381"/>
-      <c r="F12" s="381"/>
-      <c r="G12" s="381"/>
-      <c r="H12" s="381"/>
-      <c r="I12" s="381"/>
-      <c r="J12" s="381"/>
-      <c r="K12" s="381"/>
-      <c r="L12" s="382"/>
+      <c r="C12" s="360"/>
+      <c r="D12" s="360"/>
+      <c r="E12" s="360"/>
+      <c r="F12" s="360"/>
+      <c r="G12" s="360"/>
+      <c r="H12" s="360"/>
+      <c r="I12" s="360"/>
+      <c r="J12" s="360"/>
+      <c r="K12" s="360"/>
+      <c r="L12" s="361"/>
     </row>
     <row r="13" spans="1:18" s="57" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="344"/>
-      <c r="B13" s="381" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C13" s="381"/>
-      <c r="D13" s="381"/>
-      <c r="E13" s="381"/>
-      <c r="F13" s="381"/>
-      <c r="G13" s="381"/>
-      <c r="H13" s="381"/>
-      <c r="I13" s="381"/>
-      <c r="J13" s="381"/>
-      <c r="K13" s="381"/>
+      <c r="B13" s="360"/>
+      <c r="C13" s="360"/>
+      <c r="D13" s="360"/>
+      <c r="E13" s="360"/>
+      <c r="F13" s="360"/>
+      <c r="G13" s="360"/>
+      <c r="H13" s="360"/>
+      <c r="I13" s="360"/>
+      <c r="J13" s="360"/>
+      <c r="K13" s="360"/>
       <c r="L13" s="342"/>
     </row>
-    <row r="14" spans="1:18" s="56" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" s="56" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="235" t="s">
         <v>333</v>
       </c>
-      <c r="B14" s="381" t="s">
+      <c r="B14" s="360" t="s">
         <v>335</v>
       </c>
-      <c r="C14" s="381"/>
-      <c r="D14" s="381"/>
-      <c r="E14" s="381"/>
-      <c r="F14" s="381"/>
-      <c r="G14" s="381"/>
-      <c r="H14" s="381"/>
-      <c r="I14" s="381"/>
-      <c r="J14" s="381"/>
-      <c r="K14" s="381"/>
-      <c r="L14" s="382"/>
+      <c r="C14" s="360"/>
+      <c r="D14" s="360"/>
+      <c r="E14" s="360"/>
+      <c r="F14" s="360"/>
+      <c r="G14" s="360"/>
+      <c r="H14" s="360"/>
+      <c r="I14" s="360"/>
+      <c r="J14" s="360"/>
+      <c r="K14" s="360"/>
+      <c r="L14" s="361"/>
     </row>
     <row r="15" spans="1:18" s="57" customFormat="1" ht="176" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="227"/>
-      <c r="B15" s="345"/>
-      <c r="C15" s="345"/>
-      <c r="D15" s="345"/>
-      <c r="E15" s="345"/>
-      <c r="F15" s="345"/>
-      <c r="G15" s="345"/>
+      <c r="B15" s="362"/>
+      <c r="C15" s="362"/>
+      <c r="D15" s="362"/>
+      <c r="E15" s="362"/>
+      <c r="F15" s="362"/>
+      <c r="G15" s="362"/>
       <c r="H15" s="233"/>
       <c r="I15" s="233"/>
       <c r="J15" s="233"/>
@@ -16200,75 +16232,75 @@
       <c r="A16" s="235" t="s">
         <v>334</v>
       </c>
-      <c r="B16" s="381" t="s">
+      <c r="B16" s="360" t="s">
         <v>336</v>
       </c>
-      <c r="C16" s="381"/>
-      <c r="D16" s="381"/>
-      <c r="E16" s="381"/>
-      <c r="F16" s="381"/>
-      <c r="G16" s="381"/>
-      <c r="H16" s="381"/>
-      <c r="I16" s="381"/>
-      <c r="J16" s="381"/>
-      <c r="K16" s="381"/>
-      <c r="L16" s="382"/>
+      <c r="C16" s="360"/>
+      <c r="D16" s="360"/>
+      <c r="E16" s="360"/>
+      <c r="F16" s="360"/>
+      <c r="G16" s="360"/>
+      <c r="H16" s="360"/>
+      <c r="I16" s="360"/>
+      <c r="J16" s="360"/>
+      <c r="K16" s="360"/>
+      <c r="L16" s="361"/>
     </row>
     <row r="17" spans="1:14" s="57" customFormat="1" ht="90.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="227"/>
-      <c r="B17" s="345"/>
-      <c r="C17" s="345"/>
-      <c r="D17" s="345"/>
-      <c r="E17" s="345"/>
-      <c r="F17" s="345"/>
-      <c r="G17" s="345"/>
-      <c r="H17" s="345"/>
-      <c r="I17" s="345"/>
-      <c r="J17" s="345"/>
-      <c r="K17" s="345"/>
-      <c r="L17" s="393"/>
+      <c r="B17" s="362"/>
+      <c r="C17" s="362"/>
+      <c r="D17" s="362"/>
+      <c r="E17" s="362"/>
+      <c r="F17" s="362"/>
+      <c r="G17" s="362"/>
+      <c r="H17" s="362"/>
+      <c r="I17" s="362"/>
+      <c r="J17" s="362"/>
+      <c r="K17" s="362"/>
+      <c r="L17" s="363"/>
     </row>
     <row r="18" spans="1:14" s="56" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="235" t="s">
         <v>474</v>
       </c>
-      <c r="B18" s="381" t="s">
+      <c r="B18" s="360" t="s">
         <v>462</v>
       </c>
-      <c r="C18" s="381"/>
-      <c r="D18" s="381"/>
-      <c r="E18" s="381"/>
-      <c r="F18" s="381"/>
-      <c r="G18" s="381"/>
-      <c r="H18" s="381"/>
-      <c r="I18" s="381"/>
-      <c r="J18" s="381"/>
-      <c r="K18" s="381"/>
-      <c r="L18" s="382"/>
+      <c r="C18" s="360"/>
+      <c r="D18" s="360"/>
+      <c r="E18" s="360"/>
+      <c r="F18" s="360"/>
+      <c r="G18" s="360"/>
+      <c r="H18" s="360"/>
+      <c r="I18" s="360"/>
+      <c r="J18" s="360"/>
+      <c r="K18" s="360"/>
+      <c r="L18" s="361"/>
     </row>
     <row r="19" spans="1:14" s="57" customFormat="1" ht="269" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="227"/>
-      <c r="B19" s="345" t="e" vm="2">
+      <c r="B19" s="362" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C19" s="345"/>
-      <c r="D19" s="345"/>
-      <c r="E19" s="345"/>
-      <c r="F19" s="345"/>
-      <c r="G19" s="345"/>
-      <c r="H19" s="345"/>
-      <c r="I19" s="345"/>
-      <c r="J19" s="345"/>
-      <c r="K19" s="345"/>
+      <c r="C19" s="362"/>
+      <c r="D19" s="362"/>
+      <c r="E19" s="362"/>
+      <c r="F19" s="362"/>
+      <c r="G19" s="362"/>
+      <c r="H19" s="362"/>
+      <c r="I19" s="362"/>
+      <c r="J19" s="362"/>
+      <c r="K19" s="362"/>
       <c r="L19" s="234"/>
     </row>
     <row r="20" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="368" t="s">
+      <c r="A20" s="394" t="s">
         <v>340</v>
       </c>
-      <c r="B20" s="369"/>
-      <c r="C20" s="369"/>
-      <c r="D20" s="369"/>
+      <c r="B20" s="395"/>
+      <c r="C20" s="395"/>
+      <c r="D20" s="395"/>
       <c r="E20" s="232" t="s">
         <v>341</v>
       </c>
@@ -16295,84 +16327,84 @@
       <c r="L21" s="110"/>
     </row>
     <row r="22" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="352" t="s">
+      <c r="A22" s="381" t="s">
         <v>165</v>
       </c>
-      <c r="B22" s="353"/>
-      <c r="C22" s="353"/>
-      <c r="D22" s="353"/>
-      <c r="E22" s="353"/>
-      <c r="F22" s="353"/>
-      <c r="G22" s="353"/>
-      <c r="H22" s="353"/>
-      <c r="I22" s="353"/>
-      <c r="J22" s="353"/>
-      <c r="K22" s="353"/>
-      <c r="L22" s="354"/>
+      <c r="B22" s="382"/>
+      <c r="C22" s="382"/>
+      <c r="D22" s="382"/>
+      <c r="E22" s="382"/>
+      <c r="F22" s="382"/>
+      <c r="G22" s="382"/>
+      <c r="H22" s="382"/>
+      <c r="I22" s="382"/>
+      <c r="J22" s="382"/>
+      <c r="K22" s="382"/>
+      <c r="L22" s="383"/>
     </row>
     <row r="23" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="355" t="s">
+      <c r="A23" s="384" t="s">
         <v>280</v>
       </c>
-      <c r="B23" s="356"/>
-      <c r="C23" s="356"/>
-      <c r="D23" s="356"/>
-      <c r="E23" s="356"/>
-      <c r="F23" s="356"/>
-      <c r="G23" s="356"/>
-      <c r="H23" s="356"/>
-      <c r="I23" s="356"/>
-      <c r="J23" s="356"/>
-      <c r="K23" s="356"/>
-      <c r="L23" s="357"/>
+      <c r="B23" s="385"/>
+      <c r="C23" s="385"/>
+      <c r="D23" s="385"/>
+      <c r="E23" s="385"/>
+      <c r="F23" s="385"/>
+      <c r="G23" s="385"/>
+      <c r="H23" s="385"/>
+      <c r="I23" s="385"/>
+      <c r="J23" s="385"/>
+      <c r="K23" s="385"/>
+      <c r="L23" s="386"/>
     </row>
     <row r="24" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="358" t="s">
+      <c r="A24" s="387" t="s">
         <v>281</v>
       </c>
-      <c r="B24" s="346"/>
-      <c r="C24" s="346"/>
-      <c r="D24" s="346"/>
-      <c r="E24" s="346"/>
-      <c r="F24" s="346"/>
-      <c r="G24" s="346"/>
-      <c r="H24" s="346"/>
-      <c r="I24" s="346"/>
-      <c r="J24" s="346"/>
-      <c r="K24" s="346"/>
-      <c r="L24" s="359"/>
+      <c r="B24" s="345"/>
+      <c r="C24" s="345"/>
+      <c r="D24" s="345"/>
+      <c r="E24" s="345"/>
+      <c r="F24" s="345"/>
+      <c r="G24" s="345"/>
+      <c r="H24" s="345"/>
+      <c r="I24" s="345"/>
+      <c r="J24" s="345"/>
+      <c r="K24" s="345"/>
+      <c r="L24" s="346"/>
     </row>
     <row r="25" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="358" t="s">
+      <c r="A25" s="387" t="s">
         <v>166</v>
       </c>
-      <c r="B25" s="346"/>
-      <c r="C25" s="346"/>
-      <c r="D25" s="346"/>
-      <c r="E25" s="346"/>
-      <c r="F25" s="346"/>
-      <c r="G25" s="346"/>
-      <c r="H25" s="346"/>
-      <c r="I25" s="346"/>
-      <c r="J25" s="346"/>
-      <c r="K25" s="346"/>
-      <c r="L25" s="359"/>
+      <c r="B25" s="345"/>
+      <c r="C25" s="345"/>
+      <c r="D25" s="345"/>
+      <c r="E25" s="345"/>
+      <c r="F25" s="345"/>
+      <c r="G25" s="345"/>
+      <c r="H25" s="345"/>
+      <c r="I25" s="345"/>
+      <c r="J25" s="345"/>
+      <c r="K25" s="345"/>
+      <c r="L25" s="346"/>
     </row>
     <row r="26" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="360" t="s">
+      <c r="A26" s="388" t="s">
         <v>282</v>
       </c>
-      <c r="B26" s="361"/>
-      <c r="C26" s="361"/>
-      <c r="D26" s="361"/>
-      <c r="E26" s="361"/>
-      <c r="F26" s="361"/>
-      <c r="G26" s="361"/>
-      <c r="H26" s="361"/>
-      <c r="I26" s="361"/>
-      <c r="J26" s="361"/>
-      <c r="K26" s="361"/>
-      <c r="L26" s="362"/>
+      <c r="B26" s="389"/>
+      <c r="C26" s="389"/>
+      <c r="D26" s="389"/>
+      <c r="E26" s="389"/>
+      <c r="F26" s="389"/>
+      <c r="G26" s="389"/>
+      <c r="H26" s="389"/>
+      <c r="I26" s="389"/>
+      <c r="J26" s="389"/>
+      <c r="K26" s="389"/>
+      <c r="L26" s="390"/>
     </row>
     <row r="27" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="110"/>
@@ -16389,332 +16421,332 @@
       <c r="L27" s="110"/>
     </row>
     <row r="28" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="363" t="s">
+      <c r="A28" s="391" t="s">
         <v>279</v>
       </c>
-      <c r="B28" s="364"/>
-      <c r="C28" s="364"/>
-      <c r="D28" s="364"/>
-      <c r="E28" s="364"/>
-      <c r="F28" s="364"/>
-      <c r="G28" s="364"/>
-      <c r="H28" s="364"/>
-      <c r="I28" s="364"/>
-      <c r="J28" s="364"/>
-      <c r="K28" s="364"/>
-      <c r="L28" s="365"/>
+      <c r="B28" s="392"/>
+      <c r="C28" s="392"/>
+      <c r="D28" s="392"/>
+      <c r="E28" s="392"/>
+      <c r="F28" s="392"/>
+      <c r="G28" s="392"/>
+      <c r="H28" s="392"/>
+      <c r="I28" s="392"/>
+      <c r="J28" s="392"/>
+      <c r="K28" s="392"/>
+      <c r="L28" s="393"/>
       <c r="N28" s="1"/>
     </row>
     <row r="29" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="349" t="s">
+      <c r="A29" s="378" t="s">
         <v>175</v>
       </c>
-      <c r="B29" s="350"/>
-      <c r="C29" s="350"/>
-      <c r="D29" s="350"/>
-      <c r="E29" s="350"/>
-      <c r="F29" s="350"/>
-      <c r="G29" s="350"/>
-      <c r="H29" s="350"/>
-      <c r="I29" s="350"/>
-      <c r="J29" s="350"/>
-      <c r="K29" s="350"/>
-      <c r="L29" s="351"/>
+      <c r="B29" s="379"/>
+      <c r="C29" s="379"/>
+      <c r="D29" s="379"/>
+      <c r="E29" s="379"/>
+      <c r="F29" s="379"/>
+      <c r="G29" s="379"/>
+      <c r="H29" s="379"/>
+      <c r="I29" s="379"/>
+      <c r="J29" s="379"/>
+      <c r="K29" s="379"/>
+      <c r="L29" s="380"/>
       <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="209">
         <v>1</v>
       </c>
-      <c r="B30" s="366" t="s">
+      <c r="B30" s="353" t="s">
         <v>174</v>
       </c>
-      <c r="C30" s="366"/>
-      <c r="D30" s="366"/>
-      <c r="E30" s="366"/>
-      <c r="F30" s="366"/>
-      <c r="G30" s="366"/>
-      <c r="H30" s="366"/>
-      <c r="I30" s="366"/>
-      <c r="J30" s="366"/>
-      <c r="K30" s="366"/>
-      <c r="L30" s="367"/>
+      <c r="C30" s="353"/>
+      <c r="D30" s="353"/>
+      <c r="E30" s="353"/>
+      <c r="F30" s="353"/>
+      <c r="G30" s="353"/>
+      <c r="H30" s="353"/>
+      <c r="I30" s="353"/>
+      <c r="J30" s="353"/>
+      <c r="K30" s="353"/>
+      <c r="L30" s="354"/>
     </row>
     <row r="31" spans="1:14" s="57" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="209">
         <v>2</v>
       </c>
-      <c r="B31" s="366" t="s">
+      <c r="B31" s="353" t="s">
         <v>275</v>
       </c>
-      <c r="C31" s="366"/>
-      <c r="D31" s="366"/>
-      <c r="E31" s="366"/>
-      <c r="F31" s="366"/>
-      <c r="G31" s="366"/>
-      <c r="H31" s="366"/>
-      <c r="I31" s="366"/>
-      <c r="J31" s="366"/>
-      <c r="K31" s="366"/>
-      <c r="L31" s="367"/>
+      <c r="C31" s="353"/>
+      <c r="D31" s="353"/>
+      <c r="E31" s="353"/>
+      <c r="F31" s="353"/>
+      <c r="G31" s="353"/>
+      <c r="H31" s="353"/>
+      <c r="I31" s="353"/>
+      <c r="J31" s="353"/>
+      <c r="K31" s="353"/>
+      <c r="L31" s="354"/>
       <c r="N31" s="104"/>
     </row>
     <row r="32" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="209">
         <v>3</v>
       </c>
-      <c r="B32" s="366" t="s">
+      <c r="B32" s="353" t="s">
         <v>167</v>
       </c>
-      <c r="C32" s="366"/>
-      <c r="D32" s="366"/>
-      <c r="E32" s="366"/>
-      <c r="F32" s="366"/>
-      <c r="G32" s="366"/>
-      <c r="H32" s="366"/>
-      <c r="I32" s="366"/>
-      <c r="J32" s="366"/>
-      <c r="K32" s="366"/>
-      <c r="L32" s="367"/>
+      <c r="C32" s="353"/>
+      <c r="D32" s="353"/>
+      <c r="E32" s="353"/>
+      <c r="F32" s="353"/>
+      <c r="G32" s="353"/>
+      <c r="H32" s="353"/>
+      <c r="I32" s="353"/>
+      <c r="J32" s="353"/>
+      <c r="K32" s="353"/>
+      <c r="L32" s="354"/>
       <c r="N32" s="104"/>
     </row>
     <row r="33" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="209">
         <v>4</v>
       </c>
-      <c r="B33" s="366" t="s">
+      <c r="B33" s="353" t="s">
         <v>283</v>
       </c>
-      <c r="C33" s="366"/>
-      <c r="D33" s="366"/>
-      <c r="E33" s="366"/>
-      <c r="F33" s="366"/>
-      <c r="G33" s="366"/>
-      <c r="H33" s="366"/>
-      <c r="I33" s="366"/>
-      <c r="J33" s="366"/>
-      <c r="K33" s="366"/>
-      <c r="L33" s="367"/>
+      <c r="C33" s="353"/>
+      <c r="D33" s="353"/>
+      <c r="E33" s="353"/>
+      <c r="F33" s="353"/>
+      <c r="G33" s="353"/>
+      <c r="H33" s="353"/>
+      <c r="I33" s="353"/>
+      <c r="J33" s="353"/>
+      <c r="K33" s="353"/>
+      <c r="L33" s="354"/>
       <c r="N33" s="104"/>
     </row>
     <row r="34" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="209">
         <v>5</v>
       </c>
-      <c r="B34" s="366" t="s">
+      <c r="B34" s="353" t="s">
         <v>168</v>
       </c>
-      <c r="C34" s="366"/>
-      <c r="D34" s="366"/>
-      <c r="E34" s="366"/>
-      <c r="F34" s="366"/>
-      <c r="G34" s="366"/>
-      <c r="H34" s="366"/>
-      <c r="I34" s="366"/>
-      <c r="J34" s="366"/>
-      <c r="K34" s="366"/>
-      <c r="L34" s="367"/>
+      <c r="C34" s="353"/>
+      <c r="D34" s="353"/>
+      <c r="E34" s="353"/>
+      <c r="F34" s="353"/>
+      <c r="G34" s="353"/>
+      <c r="H34" s="353"/>
+      <c r="I34" s="353"/>
+      <c r="J34" s="353"/>
+      <c r="K34" s="353"/>
+      <c r="L34" s="354"/>
       <c r="N34" s="104"/>
     </row>
     <row r="35" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="209"/>
-      <c r="B35" s="366" t="s">
+      <c r="B35" s="353" t="s">
         <v>169</v>
       </c>
-      <c r="C35" s="366"/>
-      <c r="D35" s="366"/>
-      <c r="E35" s="366"/>
-      <c r="F35" s="366"/>
-      <c r="G35" s="366"/>
-      <c r="H35" s="366"/>
-      <c r="I35" s="366"/>
-      <c r="J35" s="366"/>
-      <c r="K35" s="366"/>
-      <c r="L35" s="367"/>
+      <c r="C35" s="353"/>
+      <c r="D35" s="353"/>
+      <c r="E35" s="353"/>
+      <c r="F35" s="353"/>
+      <c r="G35" s="353"/>
+      <c r="H35" s="353"/>
+      <c r="I35" s="353"/>
+      <c r="J35" s="353"/>
+      <c r="K35" s="353"/>
+      <c r="L35" s="354"/>
       <c r="N35" s="104"/>
     </row>
     <row r="36" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="209"/>
-      <c r="B36" s="366" t="s">
+      <c r="B36" s="353" t="s">
         <v>170</v>
       </c>
-      <c r="C36" s="366"/>
-      <c r="D36" s="366"/>
-      <c r="E36" s="366"/>
-      <c r="F36" s="366"/>
-      <c r="G36" s="366"/>
-      <c r="H36" s="366"/>
-      <c r="I36" s="366"/>
-      <c r="J36" s="366"/>
-      <c r="K36" s="366"/>
-      <c r="L36" s="367"/>
+      <c r="C36" s="353"/>
+      <c r="D36" s="353"/>
+      <c r="E36" s="353"/>
+      <c r="F36" s="353"/>
+      <c r="G36" s="353"/>
+      <c r="H36" s="353"/>
+      <c r="I36" s="353"/>
+      <c r="J36" s="353"/>
+      <c r="K36" s="353"/>
+      <c r="L36" s="354"/>
       <c r="N36" s="104"/>
     </row>
     <row r="37" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="385" t="s">
+      <c r="A37" s="347" t="s">
         <v>176</v>
       </c>
-      <c r="B37" s="386"/>
-      <c r="C37" s="386"/>
-      <c r="D37" s="386"/>
-      <c r="E37" s="386"/>
-      <c r="F37" s="386"/>
-      <c r="G37" s="386"/>
-      <c r="H37" s="386"/>
-      <c r="I37" s="386"/>
-      <c r="J37" s="386"/>
-      <c r="K37" s="386"/>
-      <c r="L37" s="387"/>
+      <c r="B37" s="348"/>
+      <c r="C37" s="348"/>
+      <c r="D37" s="348"/>
+      <c r="E37" s="348"/>
+      <c r="F37" s="348"/>
+      <c r="G37" s="348"/>
+      <c r="H37" s="348"/>
+      <c r="I37" s="348"/>
+      <c r="J37" s="348"/>
+      <c r="K37" s="348"/>
+      <c r="L37" s="349"/>
       <c r="N37" s="104"/>
     </row>
     <row r="38" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="209">
         <v>1</v>
       </c>
-      <c r="B38" s="366" t="s">
+      <c r="B38" s="353" t="s">
         <v>171</v>
       </c>
-      <c r="C38" s="366"/>
-      <c r="D38" s="366"/>
-      <c r="E38" s="366"/>
-      <c r="F38" s="366"/>
-      <c r="G38" s="366"/>
-      <c r="H38" s="366"/>
-      <c r="I38" s="366"/>
-      <c r="J38" s="366"/>
-      <c r="K38" s="366"/>
-      <c r="L38" s="367"/>
+      <c r="C38" s="353"/>
+      <c r="D38" s="353"/>
+      <c r="E38" s="353"/>
+      <c r="F38" s="353"/>
+      <c r="G38" s="353"/>
+      <c r="H38" s="353"/>
+      <c r="I38" s="353"/>
+      <c r="J38" s="353"/>
+      <c r="K38" s="353"/>
+      <c r="L38" s="354"/>
       <c r="N38" s="104"/>
     </row>
     <row r="39" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="209"/>
-      <c r="B39" s="383" t="s">
+      <c r="B39" s="364" t="s">
         <v>423</v>
       </c>
-      <c r="C39" s="383"/>
-      <c r="D39" s="383"/>
-      <c r="E39" s="383"/>
-      <c r="F39" s="383"/>
-      <c r="G39" s="383"/>
-      <c r="H39" s="383"/>
-      <c r="I39" s="383"/>
-      <c r="J39" s="383"/>
-      <c r="K39" s="383"/>
-      <c r="L39" s="384"/>
+      <c r="C39" s="364"/>
+      <c r="D39" s="364"/>
+      <c r="E39" s="364"/>
+      <c r="F39" s="364"/>
+      <c r="G39" s="364"/>
+      <c r="H39" s="364"/>
+      <c r="I39" s="364"/>
+      <c r="J39" s="364"/>
+      <c r="K39" s="364"/>
+      <c r="L39" s="365"/>
       <c r="N39" s="104"/>
     </row>
     <row r="40" spans="1:14" s="57" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="209">
         <v>2</v>
       </c>
-      <c r="B40" s="366" t="s">
+      <c r="B40" s="353" t="s">
         <v>278</v>
       </c>
-      <c r="C40" s="366"/>
-      <c r="D40" s="366"/>
-      <c r="E40" s="366"/>
-      <c r="F40" s="366"/>
-      <c r="G40" s="366"/>
-      <c r="H40" s="366"/>
-      <c r="I40" s="366"/>
-      <c r="J40" s="366"/>
-      <c r="K40" s="366"/>
-      <c r="L40" s="367"/>
+      <c r="C40" s="353"/>
+      <c r="D40" s="353"/>
+      <c r="E40" s="353"/>
+      <c r="F40" s="353"/>
+      <c r="G40" s="353"/>
+      <c r="H40" s="353"/>
+      <c r="I40" s="353"/>
+      <c r="J40" s="353"/>
+      <c r="K40" s="353"/>
+      <c r="L40" s="354"/>
       <c r="N40" s="104"/>
     </row>
     <row r="41" spans="1:14" s="57" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="209">
         <v>3</v>
       </c>
-      <c r="B41" s="366" t="s">
+      <c r="B41" s="353" t="s">
         <v>472</v>
       </c>
-      <c r="C41" s="366"/>
-      <c r="D41" s="366"/>
-      <c r="E41" s="366"/>
-      <c r="F41" s="366"/>
-      <c r="G41" s="366"/>
-      <c r="H41" s="366"/>
-      <c r="I41" s="366"/>
-      <c r="J41" s="366"/>
-      <c r="K41" s="366"/>
-      <c r="L41" s="367"/>
+      <c r="C41" s="353"/>
+      <c r="D41" s="353"/>
+      <c r="E41" s="353"/>
+      <c r="F41" s="353"/>
+      <c r="G41" s="353"/>
+      <c r="H41" s="353"/>
+      <c r="I41" s="353"/>
+      <c r="J41" s="353"/>
+      <c r="K41" s="353"/>
+      <c r="L41" s="354"/>
       <c r="N41" s="104"/>
     </row>
     <row r="42" spans="1:14" s="57" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="209">
         <v>4</v>
       </c>
-      <c r="B42" s="366" t="s">
+      <c r="B42" s="353" t="s">
         <v>284</v>
       </c>
-      <c r="C42" s="366"/>
-      <c r="D42" s="366"/>
-      <c r="E42" s="366"/>
-      <c r="F42" s="366"/>
-      <c r="G42" s="366"/>
-      <c r="H42" s="366"/>
-      <c r="I42" s="366"/>
-      <c r="J42" s="366"/>
-      <c r="K42" s="366"/>
-      <c r="L42" s="367"/>
+      <c r="C42" s="353"/>
+      <c r="D42" s="353"/>
+      <c r="E42" s="353"/>
+      <c r="F42" s="353"/>
+      <c r="G42" s="353"/>
+      <c r="H42" s="353"/>
+      <c r="I42" s="353"/>
+      <c r="J42" s="353"/>
+      <c r="K42" s="353"/>
+      <c r="L42" s="354"/>
       <c r="N42" s="104"/>
     </row>
     <row r="43" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="209">
         <v>5</v>
       </c>
-      <c r="B43" s="383" t="s">
+      <c r="B43" s="364" t="s">
         <v>269</v>
       </c>
-      <c r="C43" s="383"/>
-      <c r="D43" s="383"/>
-      <c r="E43" s="383"/>
-      <c r="F43" s="383"/>
-      <c r="G43" s="383"/>
-      <c r="H43" s="383"/>
-      <c r="I43" s="383"/>
-      <c r="J43" s="383"/>
-      <c r="K43" s="383"/>
-      <c r="L43" s="384"/>
+      <c r="C43" s="364"/>
+      <c r="D43" s="364"/>
+      <c r="E43" s="364"/>
+      <c r="F43" s="364"/>
+      <c r="G43" s="364"/>
+      <c r="H43" s="364"/>
+      <c r="I43" s="364"/>
+      <c r="J43" s="364"/>
+      <c r="K43" s="364"/>
+      <c r="L43" s="365"/>
       <c r="N43" s="104"/>
     </row>
     <row r="44" spans="1:14" s="57" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="209">
         <v>6</v>
       </c>
-      <c r="B44" s="383" t="s">
+      <c r="B44" s="364" t="s">
         <v>473</v>
       </c>
-      <c r="C44" s="383"/>
-      <c r="D44" s="383"/>
-      <c r="E44" s="383"/>
-      <c r="F44" s="383"/>
-      <c r="G44" s="383"/>
-      <c r="H44" s="383"/>
-      <c r="I44" s="383"/>
-      <c r="J44" s="383"/>
-      <c r="K44" s="383"/>
-      <c r="L44" s="384"/>
+      <c r="C44" s="364"/>
+      <c r="D44" s="364"/>
+      <c r="E44" s="364"/>
+      <c r="F44" s="364"/>
+      <c r="G44" s="364"/>
+      <c r="H44" s="364"/>
+      <c r="I44" s="364"/>
+      <c r="J44" s="364"/>
+      <c r="K44" s="364"/>
+      <c r="L44" s="365"/>
       <c r="N44" s="104"/>
     </row>
     <row r="45" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="209">
         <v>7</v>
       </c>
-      <c r="B45" s="366" t="s">
+      <c r="B45" s="353" t="s">
         <v>270</v>
       </c>
-      <c r="C45" s="366"/>
-      <c r="D45" s="366"/>
-      <c r="E45" s="366"/>
-      <c r="F45" s="366"/>
-      <c r="G45" s="366"/>
-      <c r="H45" s="366"/>
-      <c r="I45" s="366"/>
-      <c r="J45" s="366"/>
-      <c r="K45" s="366"/>
-      <c r="L45" s="367"/>
+      <c r="C45" s="353"/>
+      <c r="D45" s="353"/>
+      <c r="E45" s="353"/>
+      <c r="F45" s="353"/>
+      <c r="G45" s="353"/>
+      <c r="H45" s="353"/>
+      <c r="I45" s="353"/>
+      <c r="J45" s="353"/>
+      <c r="K45" s="353"/>
+      <c r="L45" s="354"/>
     </row>
     <row r="46" spans="1:14" s="57" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="209"/>
@@ -16731,56 +16763,56 @@
       <c r="L46" s="211"/>
     </row>
     <row r="47" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="385" t="s">
+      <c r="A47" s="347" t="s">
         <v>273</v>
       </c>
-      <c r="B47" s="386"/>
-      <c r="C47" s="386"/>
-      <c r="D47" s="386"/>
-      <c r="E47" s="386"/>
-      <c r="F47" s="386"/>
-      <c r="G47" s="386"/>
-      <c r="H47" s="386"/>
-      <c r="I47" s="386"/>
-      <c r="J47" s="386"/>
-      <c r="K47" s="386"/>
-      <c r="L47" s="387"/>
+      <c r="B47" s="348"/>
+      <c r="C47" s="348"/>
+      <c r="D47" s="348"/>
+      <c r="E47" s="348"/>
+      <c r="F47" s="348"/>
+      <c r="G47" s="348"/>
+      <c r="H47" s="348"/>
+      <c r="I47" s="348"/>
+      <c r="J47" s="348"/>
+      <c r="K47" s="348"/>
+      <c r="L47" s="349"/>
     </row>
     <row r="48" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="212" t="s">
         <v>271</v>
       </c>
-      <c r="B48" s="366" t="s">
+      <c r="B48" s="353" t="s">
         <v>172</v>
       </c>
-      <c r="C48" s="366"/>
-      <c r="D48" s="366"/>
-      <c r="E48" s="366"/>
-      <c r="F48" s="366"/>
-      <c r="G48" s="366"/>
-      <c r="H48" s="366"/>
-      <c r="I48" s="366"/>
-      <c r="J48" s="366"/>
-      <c r="K48" s="366"/>
-      <c r="L48" s="367"/>
+      <c r="C48" s="353"/>
+      <c r="D48" s="353"/>
+      <c r="E48" s="353"/>
+      <c r="F48" s="353"/>
+      <c r="G48" s="353"/>
+      <c r="H48" s="353"/>
+      <c r="I48" s="353"/>
+      <c r="J48" s="353"/>
+      <c r="K48" s="353"/>
+      <c r="L48" s="354"/>
     </row>
     <row r="49" spans="1:12" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="213" t="s">
         <v>272</v>
       </c>
-      <c r="B49" s="388" t="s">
+      <c r="B49" s="355" t="s">
         <v>274</v>
       </c>
-      <c r="C49" s="388"/>
-      <c r="D49" s="388"/>
-      <c r="E49" s="388"/>
-      <c r="F49" s="388"/>
-      <c r="G49" s="388"/>
-      <c r="H49" s="388"/>
-      <c r="I49" s="388"/>
-      <c r="J49" s="388"/>
-      <c r="K49" s="388"/>
-      <c r="L49" s="389"/>
+      <c r="C49" s="355"/>
+      <c r="D49" s="355"/>
+      <c r="E49" s="355"/>
+      <c r="F49" s="355"/>
+      <c r="G49" s="355"/>
+      <c r="H49" s="355"/>
+      <c r="I49" s="355"/>
+      <c r="J49" s="355"/>
+      <c r="K49" s="355"/>
+      <c r="L49" s="356"/>
     </row>
     <row r="50" spans="1:12" s="57" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="157"/>
@@ -16797,20 +16829,20 @@
       <c r="L50" s="110"/>
     </row>
     <row r="51" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="390" t="s">
+      <c r="A51" s="357" t="s">
         <v>200</v>
       </c>
-      <c r="B51" s="391"/>
-      <c r="C51" s="391"/>
-      <c r="D51" s="391"/>
-      <c r="E51" s="391"/>
-      <c r="F51" s="391"/>
-      <c r="G51" s="391"/>
-      <c r="H51" s="391"/>
-      <c r="I51" s="391"/>
-      <c r="J51" s="391"/>
-      <c r="K51" s="391"/>
-      <c r="L51" s="392"/>
+      <c r="B51" s="358"/>
+      <c r="C51" s="358"/>
+      <c r="D51" s="358"/>
+      <c r="E51" s="358"/>
+      <c r="F51" s="358"/>
+      <c r="G51" s="358"/>
+      <c r="H51" s="358"/>
+      <c r="I51" s="358"/>
+      <c r="J51" s="358"/>
+      <c r="K51" s="358"/>
+      <c r="L51" s="359"/>
     </row>
     <row r="52" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="216" t="s">
@@ -16898,126 +16930,126 @@
       <c r="B57" s="165" t="s">
         <v>24</v>
       </c>
-      <c r="C57" s="346" t="s">
+      <c r="C57" s="345" t="s">
         <v>262</v>
       </c>
-      <c r="D57" s="346"/>
-      <c r="E57" s="346"/>
-      <c r="F57" s="346"/>
-      <c r="G57" s="346"/>
-      <c r="H57" s="346"/>
-      <c r="I57" s="346"/>
-      <c r="J57" s="346"/>
-      <c r="K57" s="346"/>
-      <c r="L57" s="359"/>
+      <c r="D57" s="345"/>
+      <c r="E57" s="345"/>
+      <c r="F57" s="345"/>
+      <c r="G57" s="345"/>
+      <c r="H57" s="345"/>
+      <c r="I57" s="345"/>
+      <c r="J57" s="345"/>
+      <c r="K57" s="345"/>
+      <c r="L57" s="346"/>
     </row>
     <row r="58" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="164"/>
       <c r="B58" s="165" t="s">
         <v>263</v>
       </c>
-      <c r="C58" s="346" t="s">
+      <c r="C58" s="345" t="s">
         <v>264</v>
       </c>
-      <c r="D58" s="346"/>
-      <c r="E58" s="346"/>
-      <c r="F58" s="346"/>
-      <c r="G58" s="346"/>
-      <c r="H58" s="346"/>
-      <c r="I58" s="346"/>
-      <c r="J58" s="346"/>
-      <c r="K58" s="346"/>
-      <c r="L58" s="359"/>
+      <c r="D58" s="345"/>
+      <c r="E58" s="345"/>
+      <c r="F58" s="345"/>
+      <c r="G58" s="345"/>
+      <c r="H58" s="345"/>
+      <c r="I58" s="345"/>
+      <c r="J58" s="345"/>
+      <c r="K58" s="345"/>
+      <c r="L58" s="346"/>
     </row>
     <row r="59" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="164"/>
       <c r="B59" s="165" t="s">
         <v>324</v>
       </c>
-      <c r="C59" s="346" t="s">
+      <c r="C59" s="345" t="s">
         <v>325</v>
       </c>
-      <c r="D59" s="346"/>
-      <c r="E59" s="346"/>
-      <c r="F59" s="346"/>
-      <c r="G59" s="346"/>
-      <c r="H59" s="346"/>
-      <c r="I59" s="346"/>
-      <c r="J59" s="346"/>
-      <c r="K59" s="346"/>
-      <c r="L59" s="359"/>
+      <c r="D59" s="345"/>
+      <c r="E59" s="345"/>
+      <c r="F59" s="345"/>
+      <c r="G59" s="345"/>
+      <c r="H59" s="345"/>
+      <c r="I59" s="345"/>
+      <c r="J59" s="345"/>
+      <c r="K59" s="345"/>
+      <c r="L59" s="346"/>
     </row>
     <row r="60" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="164"/>
       <c r="B60" s="165" t="s">
         <v>98</v>
       </c>
-      <c r="C60" s="346" t="s">
+      <c r="C60" s="345" t="s">
         <v>99</v>
       </c>
-      <c r="D60" s="346"/>
-      <c r="E60" s="346"/>
-      <c r="F60" s="346"/>
-      <c r="G60" s="346"/>
-      <c r="H60" s="346"/>
-      <c r="I60" s="346"/>
-      <c r="J60" s="346"/>
-      <c r="K60" s="346"/>
-      <c r="L60" s="359"/>
+      <c r="D60" s="345"/>
+      <c r="E60" s="345"/>
+      <c r="F60" s="345"/>
+      <c r="G60" s="345"/>
+      <c r="H60" s="345"/>
+      <c r="I60" s="345"/>
+      <c r="J60" s="345"/>
+      <c r="K60" s="345"/>
+      <c r="L60" s="346"/>
     </row>
     <row r="61" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="164"/>
       <c r="B61" s="165" t="s">
         <v>198</v>
       </c>
-      <c r="C61" s="346" t="s">
+      <c r="C61" s="345" t="s">
         <v>199</v>
       </c>
-      <c r="D61" s="346"/>
-      <c r="E61" s="346"/>
-      <c r="F61" s="346"/>
-      <c r="G61" s="346"/>
-      <c r="H61" s="346"/>
-      <c r="I61" s="346"/>
-      <c r="J61" s="346"/>
-      <c r="K61" s="346"/>
-      <c r="L61" s="359"/>
+      <c r="D61" s="345"/>
+      <c r="E61" s="345"/>
+      <c r="F61" s="345"/>
+      <c r="G61" s="345"/>
+      <c r="H61" s="345"/>
+      <c r="I61" s="345"/>
+      <c r="J61" s="345"/>
+      <c r="K61" s="345"/>
+      <c r="L61" s="346"/>
     </row>
     <row r="62" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="164"/>
       <c r="B62" s="165" t="s">
         <v>163</v>
       </c>
-      <c r="C62" s="346" t="s">
+      <c r="C62" s="345" t="s">
         <v>463</v>
       </c>
-      <c r="D62" s="347"/>
-      <c r="E62" s="347"/>
-      <c r="F62" s="347"/>
-      <c r="G62" s="347"/>
-      <c r="H62" s="347"/>
-      <c r="I62" s="347"/>
-      <c r="J62" s="347"/>
-      <c r="K62" s="347"/>
-      <c r="L62" s="348"/>
+      <c r="D62" s="376"/>
+      <c r="E62" s="376"/>
+      <c r="F62" s="376"/>
+      <c r="G62" s="376"/>
+      <c r="H62" s="376"/>
+      <c r="I62" s="376"/>
+      <c r="J62" s="376"/>
+      <c r="K62" s="376"/>
+      <c r="L62" s="377"/>
     </row>
     <row r="63" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="164"/>
       <c r="B63" s="165" t="s">
         <v>390</v>
       </c>
-      <c r="C63" s="346" t="s">
+      <c r="C63" s="345" t="s">
         <v>391</v>
       </c>
-      <c r="D63" s="346"/>
-      <c r="E63" s="346"/>
-      <c r="F63" s="346"/>
-      <c r="G63" s="346"/>
-      <c r="H63" s="346"/>
-      <c r="I63" s="346"/>
-      <c r="J63" s="346"/>
-      <c r="K63" s="346"/>
-      <c r="L63" s="359"/>
+      <c r="D63" s="345"/>
+      <c r="E63" s="345"/>
+      <c r="F63" s="345"/>
+      <c r="G63" s="345"/>
+      <c r="H63" s="345"/>
+      <c r="I63" s="345"/>
+      <c r="J63" s="345"/>
+      <c r="K63" s="345"/>
+      <c r="L63" s="346"/>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="164"/>
@@ -17172,6 +17204,42 @@
     <row r="94" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="C62:L62"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B42:L42"/>
+    <mergeCell ref="C61:L61"/>
+    <mergeCell ref="C58:L58"/>
+    <mergeCell ref="B12:L12"/>
+    <mergeCell ref="B13:K13"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="C59:L59"/>
+    <mergeCell ref="B43:L43"/>
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B31:L31"/>
+    <mergeCell ref="B32:L32"/>
+    <mergeCell ref="B33:L33"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="B35:L35"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="B19:K19"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="C63:L63"/>
     <mergeCell ref="A47:L47"/>
     <mergeCell ref="A5:L5"/>
@@ -17188,42 +17256,6 @@
     <mergeCell ref="B8:L8"/>
     <mergeCell ref="B9:L9"/>
     <mergeCell ref="A11:L11"/>
-    <mergeCell ref="B14:L14"/>
-    <mergeCell ref="C59:L59"/>
-    <mergeCell ref="B43:L43"/>
-    <mergeCell ref="B30:L30"/>
-    <mergeCell ref="B31:L31"/>
-    <mergeCell ref="B32:L32"/>
-    <mergeCell ref="B33:L33"/>
-    <mergeCell ref="B34:L34"/>
-    <mergeCell ref="B35:L35"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="A37:L37"/>
-    <mergeCell ref="B38:L38"/>
-    <mergeCell ref="B39:L39"/>
-    <mergeCell ref="B12:L12"/>
-    <mergeCell ref="B13:K13"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A7:L7"/>
-    <mergeCell ref="B19:K19"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="C62:L62"/>
-    <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="A25:L25"/>
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B42:L42"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="C61:L61"/>
-    <mergeCell ref="C58:L58"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A70" r:id="rId1" xr:uid="{C9866D44-2827-49D7-B9C3-89CF23FACDC1}"/>
@@ -24562,62 +24594,62 @@
       <c r="G5" s="185" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="424" t="s">
+      <c r="I5" s="429" t="s">
         <v>420</v>
       </c>
-      <c r="J5" s="425"/>
-      <c r="K5" s="425"/>
-      <c r="L5" s="425"/>
-      <c r="M5" s="425"/>
-      <c r="N5" s="425"/>
-      <c r="O5" s="425"/>
-      <c r="P5" s="425"/>
-      <c r="Q5" s="425"/>
-      <c r="R5" s="425"/>
-      <c r="S5" s="425"/>
-      <c r="T5" s="425"/>
-      <c r="U5" s="425"/>
-      <c r="V5" s="425"/>
-      <c r="W5" s="426"/>
+      <c r="J5" s="430"/>
+      <c r="K5" s="430"/>
+      <c r="L5" s="430"/>
+      <c r="M5" s="430"/>
+      <c r="N5" s="430"/>
+      <c r="O5" s="430"/>
+      <c r="P5" s="430"/>
+      <c r="Q5" s="430"/>
+      <c r="R5" s="430"/>
+      <c r="S5" s="430"/>
+      <c r="T5" s="430"/>
+      <c r="U5" s="430"/>
+      <c r="V5" s="430"/>
+      <c r="W5" s="431"/>
       <c r="Y5" s="192"/>
       <c r="Z5" s="192"/>
       <c r="AA5" s="192"/>
       <c r="AB5" s="334"/>
     </row>
     <row r="6" spans="1:53" s="184" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B6" s="416" t="s">
+      <c r="B6" s="418" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="417"/>
-      <c r="D6" s="417"/>
-      <c r="E6" s="417"/>
-      <c r="F6" s="417"/>
-      <c r="G6" s="418"/>
-      <c r="I6" s="427" t="s">
+      <c r="C6" s="419"/>
+      <c r="D6" s="419"/>
+      <c r="E6" s="419"/>
+      <c r="F6" s="419"/>
+      <c r="G6" s="420"/>
+      <c r="I6" s="432" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="429" t="s">
+      <c r="J6" s="416" t="s">
         <v>406</v>
       </c>
-      <c r="K6" s="429" t="s">
+      <c r="K6" s="416" t="s">
         <v>405</v>
       </c>
-      <c r="L6" s="430" t="s">
+      <c r="L6" s="434" t="s">
         <v>215</v>
       </c>
-      <c r="M6" s="431"/>
-      <c r="N6" s="431"/>
-      <c r="O6" s="431"/>
-      <c r="P6" s="431"/>
-      <c r="Q6" s="432"/>
-      <c r="R6" s="433" t="s">
+      <c r="M6" s="435"/>
+      <c r="N6" s="435"/>
+      <c r="O6" s="435"/>
+      <c r="P6" s="435"/>
+      <c r="Q6" s="436"/>
+      <c r="R6" s="421" t="s">
         <v>216</v>
       </c>
-      <c r="S6" s="434"/>
-      <c r="T6" s="434"/>
-      <c r="U6" s="434"/>
-      <c r="V6" s="434"/>
-      <c r="W6" s="435"/>
+      <c r="S6" s="422"/>
+      <c r="T6" s="422"/>
+      <c r="U6" s="422"/>
+      <c r="V6" s="422"/>
+      <c r="W6" s="423"/>
       <c r="Y6" s="307"/>
       <c r="Z6" s="307"/>
       <c r="AA6" s="307"/>
@@ -24643,9 +24675,9 @@
         <f>SUM(C7:F7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="428"/>
-      <c r="J7" s="428"/>
-      <c r="K7" s="428"/>
+      <c r="I7" s="433"/>
+      <c r="J7" s="433"/>
+      <c r="K7" s="433"/>
       <c r="L7" s="186" t="s">
         <v>407</v>
       </c>
@@ -24849,14 +24881,14 @@
       <c r="AZ9" s="285"/>
     </row>
     <row r="10" spans="1:53" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="B10" s="419" t="s">
+      <c r="B10" s="424" t="s">
         <v>237</v>
       </c>
-      <c r="C10" s="419"/>
-      <c r="D10" s="419"/>
-      <c r="E10" s="419"/>
-      <c r="F10" s="419"/>
-      <c r="G10" s="419"/>
+      <c r="C10" s="424"/>
+      <c r="D10" s="424"/>
+      <c r="E10" s="424"/>
+      <c r="F10" s="424"/>
+      <c r="G10" s="424"/>
       <c r="I10" s="244" t="s">
         <v>231</v>
       </c>
@@ -25340,13 +25372,13 @@
       <c r="B16" s="193" t="s">
         <v>234</v>
       </c>
-      <c r="C16" s="420" t="s">
+      <c r="C16" s="425" t="s">
         <v>235</v>
       </c>
-      <c r="D16" s="421"/>
-      <c r="E16" s="421"/>
-      <c r="F16" s="421"/>
-      <c r="G16" s="422"/>
+      <c r="D16" s="426"/>
+      <c r="E16" s="426"/>
+      <c r="F16" s="426"/>
+      <c r="G16" s="427"/>
       <c r="I16" s="244" t="s">
         <v>401</v>
       </c>
@@ -25462,59 +25494,59 @@
     </row>
     <row r="18" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15"/>
     <row r="19" spans="2:58" s="192" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I19" s="423" t="s">
+      <c r="I19" s="428" t="s">
         <v>421</v>
       </c>
-      <c r="J19" s="423"/>
-      <c r="K19" s="423"/>
-      <c r="L19" s="423"/>
-      <c r="M19" s="423"/>
-      <c r="N19" s="423"/>
-      <c r="O19" s="423"/>
-      <c r="P19" s="423"/>
-      <c r="Q19" s="423"/>
-      <c r="R19" s="423"/>
-      <c r="S19" s="423"/>
-      <c r="T19" s="423"/>
-      <c r="U19" s="423"/>
+      <c r="J19" s="428"/>
+      <c r="K19" s="428"/>
+      <c r="L19" s="428"/>
+      <c r="M19" s="428"/>
+      <c r="N19" s="428"/>
+      <c r="O19" s="428"/>
+      <c r="P19" s="428"/>
+      <c r="Q19" s="428"/>
+      <c r="R19" s="428"/>
+      <c r="S19" s="428"/>
+      <c r="T19" s="428"/>
+      <c r="U19" s="428"/>
       <c r="Z19" s="250"/>
       <c r="AA19" s="250"/>
       <c r="AB19" s="250"/>
       <c r="AC19" s="250"/>
     </row>
     <row r="20" spans="2:58" s="192" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I20" s="429" t="s">
+      <c r="I20" s="416" t="s">
         <v>13</v>
       </c>
-      <c r="J20" s="429" t="s">
+      <c r="J20" s="416" t="s">
         <v>213</v>
       </c>
-      <c r="K20" s="429" t="s">
+      <c r="K20" s="416" t="s">
         <v>214</v>
       </c>
-      <c r="L20" s="416" t="s">
+      <c r="L20" s="418" t="s">
         <v>215</v>
       </c>
-      <c r="M20" s="417"/>
-      <c r="N20" s="417"/>
-      <c r="O20" s="417"/>
-      <c r="P20" s="418"/>
-      <c r="Q20" s="433" t="s">
+      <c r="M20" s="419"/>
+      <c r="N20" s="419"/>
+      <c r="O20" s="419"/>
+      <c r="P20" s="420"/>
+      <c r="Q20" s="421" t="s">
         <v>216</v>
       </c>
-      <c r="R20" s="434"/>
-      <c r="S20" s="434"/>
-      <c r="T20" s="434"/>
-      <c r="U20" s="435"/>
+      <c r="R20" s="422"/>
+      <c r="S20" s="422"/>
+      <c r="T20" s="422"/>
+      <c r="U20" s="423"/>
       <c r="Z20" s="254"/>
       <c r="AA20" s="254"/>
       <c r="AB20" s="254"/>
       <c r="AC20" s="254"/>
     </row>
     <row r="21" spans="2:58" s="192" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I21" s="436"/>
-      <c r="J21" s="436"/>
-      <c r="K21" s="436"/>
+      <c r="I21" s="417"/>
+      <c r="J21" s="417"/>
+      <c r="K21" s="417"/>
       <c r="L21" s="186" t="s">
         <v>218</v>
       </c>
@@ -26536,11 +26568,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:P20"/>
-    <mergeCell ref="Q20:U20"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="C16:G16"/>
@@ -26551,6 +26578,11 @@
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:Q6"/>
     <mergeCell ref="R6:W6"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:P20"/>
+    <mergeCell ref="Q20:U20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26883,16 +26915,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="437" t="e">
+      <c r="A1" s="438" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B1" s="437"/>
-      <c r="C1" s="437"/>
-      <c r="D1" s="437"/>
-      <c r="E1" s="437"/>
-      <c r="F1" s="437"/>
-      <c r="G1" s="437"/>
+      <c r="B1" s="438"/>
+      <c r="C1" s="438"/>
+      <c r="D1" s="438"/>
+      <c r="E1" s="438"/>
+      <c r="F1" s="438"/>
+      <c r="G1" s="438"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -27001,11 +27033,11 @@
         <v>40</v>
       </c>
       <c r="B10" s="112"/>
-      <c r="C10" s="438"/>
-      <c r="D10" s="438"/>
-      <c r="E10" s="438"/>
-      <c r="F10" s="438"/>
-      <c r="G10" s="438"/>
+      <c r="C10" s="437"/>
+      <c r="D10" s="437"/>
+      <c r="E10" s="437"/>
+      <c r="F10" s="437"/>
+      <c r="G10" s="437"/>
       <c r="N10" s="139"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -28268,6 +28300,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:G6"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="C9:G9"/>
@@ -28275,12 +28313,6 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N4" r:id="rId1" location="step-1-assign-parties-person-playing-and-strategies" xr:uid="{726B234F-7B54-4D33-A192-8F1604C6B04C}"/>

</xml_diff>

<commit_message>
Added current draft of dynamic storage plot
</commit_message>
<xml_diff>
--- a/LakeMeadWaterBankDivideInflow.xlsx
+++ b/LakeMeadWaterBankDivideInflow.xlsx
@@ -8,25 +8,101 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anabelle/Documents/LakeMeadDivideInflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5B5BEB-FED2-E04A-9F47-6BED2AEDF37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2133D94C-ACC9-0847-9CA7-B7D82E75B677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
+    <workbookView xWindow="-17120" yWindow="-24000" windowWidth="38400" windowHeight="24000" activeTab="3" xr2:uid="{5373AB19-D84C-490D-97DC-C516D358024A}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe-Directions" sheetId="62" r:id="rId1"/>
     <sheet name="Versions" sheetId="31" r:id="rId2"/>
     <sheet name="Master" sheetId="47" r:id="rId3"/>
-    <sheet name="DivideInflow" sheetId="61" r:id="rId4"/>
-    <sheet name="TribalWater" sheetId="63" r:id="rId5"/>
-    <sheet name="SplitInflowPlot" sheetId="59" r:id="rId6"/>
-    <sheet name="SplitInflowForPlot" sheetId="60" r:id="rId7"/>
-    <sheet name="MandatoryConservation" sheetId="41" r:id="rId8"/>
-    <sheet name="PowellReleaseTemperature" sheetId="43" r:id="rId9"/>
-    <sheet name="Mead-Elevation-Area" sheetId="10" r:id="rId10"/>
-    <sheet name="CellType" sheetId="54" r:id="rId11"/>
-    <sheet name="BasinConservationPrograms" sheetId="65" r:id="rId12"/>
-    <sheet name="LakeMeadInflowScenarios" sheetId="64" r:id="rId13"/>
+    <sheet name="DynamicStoragePlot" sheetId="67" r:id="rId4"/>
+    <sheet name="DivideInflow" sheetId="61" r:id="rId5"/>
+    <sheet name="TribalWater" sheetId="63" r:id="rId6"/>
+    <sheet name="SplitInflowPlot" sheetId="59" r:id="rId7"/>
+    <sheet name="SplitInflowForPlot" sheetId="60" r:id="rId8"/>
+    <sheet name="MandatoryConservation" sheetId="41" r:id="rId9"/>
+    <sheet name="PowellReleaseTemperature" sheetId="43" r:id="rId10"/>
+    <sheet name="Mead-Elevation-Area" sheetId="10" r:id="rId11"/>
+    <sheet name="CellType" sheetId="54" r:id="rId12"/>
+    <sheet name="BasinConservationPrograms" sheetId="65" r:id="rId13"/>
+    <sheet name="LakeMeadInflowScenarios" sheetId="64" r:id="rId14"/>
+    <sheet name="DynamicPlotData" sheetId="68" r:id="rId15"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.22" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.23" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.24" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.25" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.26" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.27" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.28" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.29" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.30" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.31" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.32" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.33" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.34" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.35" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.36" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.37" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.38" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.39" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.40" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.41" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.42" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.43" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.44" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.45" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.46" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.47" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.48" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.49" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.50" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.51" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.52" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.53" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.54" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.55" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.56" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.57" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.58" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.59" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.60" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.61" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.62" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.63" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.64" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.65" hidden="1">Master!$C$142:$G$142</definedName>
+    <definedName name="_xlchart.v1.66" hidden="1">Master!$C$143:$G$143</definedName>
+    <definedName name="_xlchart.v1.67" hidden="1">Master!$C$144:$G$144</definedName>
+    <definedName name="_xlchart.v1.68" hidden="1">Master!$C$145:$G$145</definedName>
+    <definedName name="_xlchart.v1.69" hidden="1">Master!$C$146:$G$146</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.70" hidden="1">Master!$C$147:$G$147</definedName>
+    <definedName name="_xlchart.v1.71" hidden="1">Master!$C$27:$G$27</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">DynamicPlotData!$B$2:$F$2</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Master!$C$142:$G$142</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -48,7 +124,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="485">
   <si>
     <t>Year 1</t>
   </si>
@@ -2328,6 +2404,18 @@
   </si>
   <si>
     <t>Protection Elevation [ft] without withdrawals</t>
+  </si>
+  <si>
+    <t>Chosen Protection Elevation</t>
+  </si>
+  <si>
+    <t>DCP Trigger</t>
+  </si>
+  <si>
+    <t>Min Power Pool</t>
+  </si>
+  <si>
+    <t>Final EIS Buffer Line</t>
   </si>
 </sst>
 </file>
@@ -3286,7 +3374,7 @@
     <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="456">
+  <cellXfs count="457">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4215,6 +4303,9 @@
     <xf numFmtId="0" fontId="36" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4955,16 +5046,16 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FFFBAE83"/>
-      <color rgb="FFFAA599"/>
-      <color rgb="FFFE976D"/>
-      <color rgb="FFFDA579"/>
-      <color rgb="FFF9B9B5"/>
-      <color rgb="FFFB9A99"/>
-      <color rgb="FFFC8F91"/>
-      <color rgb="FFF08D87"/>
-      <color rgb="FFFF948E"/>
-      <color rgb="FFFFB0AF"/>
+      <color rgb="FF529BE7"/>
+      <color rgb="FF3C82C0"/>
+      <color rgb="FF528CBF"/>
+      <color rgb="FF7AB5F2"/>
+      <color rgb="FF5CA7F1"/>
+      <color rgb="FF007DEF"/>
+      <color rgb="FF0077DB"/>
+      <color rgb="FF0086EC"/>
+      <color rgb="FF007AD6"/>
+      <color rgb="FF528EDC"/>
     </mruColors>
   </colors>
   <extLst>
@@ -4979,6 +5070,910 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.0901785917221303E-2"/>
+          <c:y val="3.4536042119895576E-2"/>
+          <c:w val="0.91173420288821727"/>
+          <c:h val="0.90589663262331543"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Reclamation Protect Zone</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln w="12700">
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="1"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Master!$C$27:$G$27</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Year 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Year 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Year 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Year 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Year 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Master!$C$142:$G$142</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C502-0346-B214-A35A0297EDD2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Tribal Nations</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0070C0"/>
+            </a:solidFill>
+            <a:ln w="12700">
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="1"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Master!$C$147:$G$147</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-C502-0346-B214-A35A0297EDD2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Mexico</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="3C82C0"/>
+            </a:solidFill>
+            <a:ln w="12700">
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="1"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Master!$C$146:$G$146</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-C502-0346-B214-A35A0297EDD2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Nevada</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="529BE7"/>
+            </a:solidFill>
+            <a:ln w="12700">
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="1"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Master!$C$27:$G$27</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Year 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Year 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Year 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Year 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Year 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Master!$C$145:$G$145</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-C502-0346-B214-A35A0297EDD2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Arizona</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7AB5F2"/>
+            </a:solidFill>
+            <a:ln w="12700">
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="1"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Master!$C$27:$G$27</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Year 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Year 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Year 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Year 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Year 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Master!$C$144:$G$144</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-C502-0346-B214-A35A0297EDD2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:v>California</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln w="12700">
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="1"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Master!$C$27:$G$27</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Year 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Year 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Year 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Year 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Year 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Master!$C$143:$G$143</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C502-0346-B214-A35A0297EDD2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="0"/>
+        <c:overlap val="100"/>
+        <c:axId val="1147498848"/>
+        <c:axId val="1147518256"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1147498848"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1500" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1147518256"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1147518256"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="7"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1500" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1500" b="1">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Lake</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1500" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> Mead Active Storage (maf)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" sz="1500" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:endParaRPr>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1500" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1147498848"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -6130,7 +7125,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -10377,7 +11372,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -14640,6 +15635,46 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -15200,7 +16235,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="276">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{CD5CBD06-5EA0-D143-9BD1-904F07A1EEEC}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/chartsheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{1C420103-4ACD-4AF8-BDB5-B91C302E6B07}">
   <sheetPr/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15413,7 +16977,40 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8665221" cy="6271327"/>
+    <xdr:ext cx="8667750" cy="6286500"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{798FB8B1-E190-278C-9E4F-96F9383B26C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="8681493" cy="6293134"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -15442,7 +17039,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
@@ -15498,7 +17095,7 @@
 </c:userShapes>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -15600,7 +17197,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -15996,20 +17593,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="376" t="s">
+      <c r="A1" s="377" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="376"/>
-      <c r="C1" s="376"/>
-      <c r="D1" s="376"/>
-      <c r="E1" s="376"/>
-      <c r="F1" s="376"/>
-      <c r="G1" s="376"/>
-      <c r="H1" s="376"/>
-      <c r="I1" s="376"/>
-      <c r="J1" s="376"/>
-      <c r="K1" s="376"/>
-      <c r="L1" s="376"/>
+      <c r="B1" s="377"/>
+      <c r="C1" s="377"/>
+      <c r="D1" s="377"/>
+      <c r="E1" s="377"/>
+      <c r="F1" s="377"/>
+      <c r="G1" s="377"/>
+      <c r="H1" s="377"/>
+      <c r="I1" s="377"/>
+      <c r="J1" s="377"/>
+      <c r="K1" s="377"/>
+      <c r="L1" s="377"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
@@ -16035,41 +17632,41 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:18" s="52" customFormat="1" ht="53.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="377" t="s">
+      <c r="A4" s="378" t="s">
         <v>296</v>
       </c>
-      <c r="B4" s="378"/>
-      <c r="C4" s="378"/>
-      <c r="D4" s="378"/>
-      <c r="E4" s="378"/>
-      <c r="F4" s="378"/>
-      <c r="G4" s="378"/>
-      <c r="H4" s="378"/>
-      <c r="I4" s="378"/>
-      <c r="J4" s="378"/>
-      <c r="K4" s="378"/>
-      <c r="L4" s="379"/>
-      <c r="N4" s="380"/>
-      <c r="O4" s="380"/>
-      <c r="P4" s="380"/>
-      <c r="Q4" s="380"/>
-      <c r="R4" s="380"/>
+      <c r="B4" s="379"/>
+      <c r="C4" s="379"/>
+      <c r="D4" s="379"/>
+      <c r="E4" s="379"/>
+      <c r="F4" s="379"/>
+      <c r="G4" s="379"/>
+      <c r="H4" s="379"/>
+      <c r="I4" s="379"/>
+      <c r="J4" s="379"/>
+      <c r="K4" s="379"/>
+      <c r="L4" s="380"/>
+      <c r="N4" s="381"/>
+      <c r="O4" s="381"/>
+      <c r="P4" s="381"/>
+      <c r="Q4" s="381"/>
+      <c r="R4" s="381"/>
     </row>
     <row r="5" spans="1:18" s="52" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="381" t="s">
+      <c r="A5" s="382" t="s">
         <v>280</v>
       </c>
-      <c r="B5" s="382"/>
-      <c r="C5" s="382"/>
-      <c r="D5" s="382"/>
-      <c r="E5" s="382"/>
-      <c r="F5" s="382"/>
-      <c r="G5" s="382"/>
-      <c r="H5" s="382"/>
-      <c r="I5" s="382"/>
-      <c r="J5" s="382"/>
-      <c r="K5" s="382"/>
-      <c r="L5" s="383"/>
+      <c r="B5" s="383"/>
+      <c r="C5" s="383"/>
+      <c r="D5" s="383"/>
+      <c r="E5" s="383"/>
+      <c r="F5" s="383"/>
+      <c r="G5" s="383"/>
+      <c r="H5" s="383"/>
+      <c r="I5" s="383"/>
+      <c r="J5" s="383"/>
+      <c r="K5" s="383"/>
+      <c r="L5" s="384"/>
       <c r="N5" s="110"/>
       <c r="O5" s="110"/>
       <c r="P5" s="110"/>
@@ -16077,20 +17674,20 @@
       <c r="R5" s="110"/>
     </row>
     <row r="6" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="381" t="s">
+      <c r="A6" s="382" t="s">
         <v>297</v>
       </c>
-      <c r="B6" s="382"/>
-      <c r="C6" s="382"/>
-      <c r="D6" s="382"/>
-      <c r="E6" s="382"/>
-      <c r="F6" s="382"/>
-      <c r="G6" s="382"/>
-      <c r="H6" s="382"/>
-      <c r="I6" s="382"/>
-      <c r="J6" s="382"/>
-      <c r="K6" s="382"/>
-      <c r="L6" s="383"/>
+      <c r="B6" s="383"/>
+      <c r="C6" s="383"/>
+      <c r="D6" s="383"/>
+      <c r="E6" s="383"/>
+      <c r="F6" s="383"/>
+      <c r="G6" s="383"/>
+      <c r="H6" s="383"/>
+      <c r="I6" s="383"/>
+      <c r="J6" s="383"/>
+      <c r="K6" s="383"/>
+      <c r="L6" s="384"/>
       <c r="N6" s="110"/>
       <c r="O6" s="110"/>
       <c r="P6" s="110"/>
@@ -16099,19 +17696,19 @@
     </row>
     <row r="7" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="214"/>
-      <c r="B7" s="382" t="s">
+      <c r="B7" s="383" t="s">
         <v>298</v>
       </c>
-      <c r="C7" s="382"/>
-      <c r="D7" s="382"/>
-      <c r="E7" s="382"/>
-      <c r="F7" s="382"/>
-      <c r="G7" s="382"/>
-      <c r="H7" s="382"/>
-      <c r="I7" s="382"/>
-      <c r="J7" s="382"/>
-      <c r="K7" s="382"/>
-      <c r="L7" s="383"/>
+      <c r="C7" s="383"/>
+      <c r="D7" s="383"/>
+      <c r="E7" s="383"/>
+      <c r="F7" s="383"/>
+      <c r="G7" s="383"/>
+      <c r="H7" s="383"/>
+      <c r="I7" s="383"/>
+      <c r="J7" s="383"/>
+      <c r="K7" s="383"/>
+      <c r="L7" s="384"/>
       <c r="N7" s="110"/>
       <c r="O7" s="110"/>
       <c r="P7" s="110"/>
@@ -16120,19 +17717,19 @@
     </row>
     <row r="8" spans="1:18" s="52" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="215"/>
-      <c r="B8" s="397" t="s">
+      <c r="B8" s="398" t="s">
         <v>299</v>
       </c>
-      <c r="C8" s="397"/>
-      <c r="D8" s="397"/>
-      <c r="E8" s="397"/>
-      <c r="F8" s="397"/>
-      <c r="G8" s="397"/>
-      <c r="H8" s="397"/>
-      <c r="I8" s="397"/>
-      <c r="J8" s="397"/>
-      <c r="K8" s="397"/>
-      <c r="L8" s="398"/>
+      <c r="C8" s="398"/>
+      <c r="D8" s="398"/>
+      <c r="E8" s="398"/>
+      <c r="F8" s="398"/>
+      <c r="G8" s="398"/>
+      <c r="H8" s="398"/>
+      <c r="I8" s="398"/>
+      <c r="J8" s="398"/>
+      <c r="K8" s="398"/>
+      <c r="L8" s="399"/>
       <c r="N8" s="110"/>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
@@ -16154,20 +17751,20 @@
       <c r="L9" s="110"/>
     </row>
     <row r="10" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="399" t="s">
+      <c r="A10" s="400" t="s">
         <v>334</v>
       </c>
-      <c r="B10" s="400"/>
-      <c r="C10" s="400"/>
-      <c r="D10" s="400"/>
-      <c r="E10" s="400"/>
-      <c r="F10" s="400"/>
-      <c r="G10" s="400"/>
-      <c r="H10" s="400"/>
-      <c r="I10" s="400"/>
-      <c r="J10" s="400"/>
-      <c r="K10" s="400"/>
-      <c r="L10" s="401"/>
+      <c r="B10" s="401"/>
+      <c r="C10" s="401"/>
+      <c r="D10" s="401"/>
+      <c r="E10" s="401"/>
+      <c r="F10" s="401"/>
+      <c r="G10" s="401"/>
+      <c r="H10" s="401"/>
+      <c r="I10" s="401"/>
+      <c r="J10" s="401"/>
+      <c r="K10" s="401"/>
+      <c r="L10" s="402"/>
     </row>
     <row r="11" spans="1:18" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="344"/>
@@ -16187,19 +17784,19 @@
       <c r="A12" s="344" t="s">
         <v>335</v>
       </c>
-      <c r="B12" s="402" t="s">
+      <c r="B12" s="403" t="s">
         <v>478</v>
       </c>
-      <c r="C12" s="402"/>
-      <c r="D12" s="402"/>
-      <c r="E12" s="402"/>
-      <c r="F12" s="402"/>
-      <c r="G12" s="402"/>
-      <c r="H12" s="402"/>
-      <c r="I12" s="402"/>
-      <c r="J12" s="402"/>
-      <c r="K12" s="402"/>
-      <c r="L12" s="403"/>
+      <c r="C12" s="403"/>
+      <c r="D12" s="403"/>
+      <c r="E12" s="403"/>
+      <c r="F12" s="403"/>
+      <c r="G12" s="403"/>
+      <c r="H12" s="403"/>
+      <c r="I12" s="403"/>
+      <c r="J12" s="403"/>
+      <c r="K12" s="403"/>
+      <c r="L12" s="404"/>
     </row>
     <row r="13" spans="1:18" s="57" customFormat="1" ht="231" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="344"/>
@@ -16219,19 +17816,19 @@
       <c r="A14" s="235" t="s">
         <v>336</v>
       </c>
-      <c r="B14" s="352" t="s">
+      <c r="B14" s="353" t="s">
         <v>338</v>
       </c>
-      <c r="C14" s="352"/>
-      <c r="D14" s="352"/>
-      <c r="E14" s="352"/>
-      <c r="F14" s="352"/>
-      <c r="G14" s="352"/>
-      <c r="H14" s="352"/>
-      <c r="I14" s="352"/>
-      <c r="J14" s="352"/>
-      <c r="K14" s="352"/>
-      <c r="L14" s="353"/>
+      <c r="C14" s="353"/>
+      <c r="D14" s="353"/>
+      <c r="E14" s="353"/>
+      <c r="F14" s="353"/>
+      <c r="G14" s="353"/>
+      <c r="H14" s="353"/>
+      <c r="I14" s="353"/>
+      <c r="J14" s="353"/>
+      <c r="K14" s="353"/>
+      <c r="L14" s="354"/>
     </row>
     <row r="15" spans="1:18" s="57" customFormat="1" ht="161.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="227"/>
@@ -16251,51 +17848,51 @@
       <c r="A16" s="235" t="s">
         <v>337</v>
       </c>
-      <c r="B16" s="352" t="s">
+      <c r="B16" s="353" t="s">
         <v>339</v>
       </c>
-      <c r="C16" s="352"/>
-      <c r="D16" s="352"/>
-      <c r="E16" s="352"/>
-      <c r="F16" s="352"/>
-      <c r="G16" s="352"/>
-      <c r="H16" s="352"/>
-      <c r="I16" s="352"/>
-      <c r="J16" s="352"/>
-      <c r="K16" s="352"/>
-      <c r="L16" s="353"/>
+      <c r="C16" s="353"/>
+      <c r="D16" s="353"/>
+      <c r="E16" s="353"/>
+      <c r="F16" s="353"/>
+      <c r="G16" s="353"/>
+      <c r="H16" s="353"/>
+      <c r="I16" s="353"/>
+      <c r="J16" s="353"/>
+      <c r="K16" s="353"/>
+      <c r="L16" s="354"/>
     </row>
     <row r="17" spans="1:14" s="57" customFormat="1" ht="90.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="227"/>
-      <c r="B17" s="354"/>
-      <c r="C17" s="354"/>
-      <c r="D17" s="354"/>
-      <c r="E17" s="354"/>
-      <c r="F17" s="354"/>
-      <c r="G17" s="354"/>
-      <c r="H17" s="354"/>
-      <c r="I17" s="354"/>
-      <c r="J17" s="354"/>
-      <c r="K17" s="354"/>
-      <c r="L17" s="355"/>
+      <c r="B17" s="355"/>
+      <c r="C17" s="355"/>
+      <c r="D17" s="355"/>
+      <c r="E17" s="355"/>
+      <c r="F17" s="355"/>
+      <c r="G17" s="355"/>
+      <c r="H17" s="355"/>
+      <c r="I17" s="355"/>
+      <c r="J17" s="355"/>
+      <c r="K17" s="355"/>
+      <c r="L17" s="356"/>
     </row>
     <row r="18" spans="1:14" s="56" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="235" t="s">
         <v>477</v>
       </c>
-      <c r="B18" s="352" t="s">
+      <c r="B18" s="353" t="s">
         <v>465</v>
       </c>
-      <c r="C18" s="352"/>
-      <c r="D18" s="352"/>
-      <c r="E18" s="352"/>
-      <c r="F18" s="352"/>
-      <c r="G18" s="352"/>
-      <c r="H18" s="352"/>
-      <c r="I18" s="352"/>
-      <c r="J18" s="352"/>
-      <c r="K18" s="352"/>
-      <c r="L18" s="353"/>
+      <c r="C18" s="353"/>
+      <c r="D18" s="353"/>
+      <c r="E18" s="353"/>
+      <c r="F18" s="353"/>
+      <c r="G18" s="353"/>
+      <c r="H18" s="353"/>
+      <c r="I18" s="353"/>
+      <c r="J18" s="353"/>
+      <c r="K18" s="353"/>
+      <c r="L18" s="354"/>
     </row>
     <row r="19" spans="1:14" s="57" customFormat="1" ht="269" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="227"/>
@@ -16312,12 +17909,12 @@
       <c r="L19" s="234"/>
     </row>
     <row r="20" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="350" t="s">
+      <c r="A20" s="351" t="s">
         <v>343</v>
       </c>
-      <c r="B20" s="351"/>
-      <c r="C20" s="351"/>
-      <c r="D20" s="351"/>
+      <c r="B20" s="352"/>
+      <c r="C20" s="352"/>
+      <c r="D20" s="352"/>
       <c r="E20" s="232" t="s">
         <v>344</v>
       </c>
@@ -16344,84 +17941,84 @@
       <c r="L21" s="110"/>
     </row>
     <row r="22" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="384" t="s">
+      <c r="A22" s="385" t="s">
         <v>165</v>
       </c>
-      <c r="B22" s="385"/>
-      <c r="C22" s="385"/>
-      <c r="D22" s="385"/>
-      <c r="E22" s="385"/>
-      <c r="F22" s="385"/>
-      <c r="G22" s="385"/>
-      <c r="H22" s="385"/>
-      <c r="I22" s="385"/>
-      <c r="J22" s="385"/>
-      <c r="K22" s="385"/>
-      <c r="L22" s="386"/>
+      <c r="B22" s="386"/>
+      <c r="C22" s="386"/>
+      <c r="D22" s="386"/>
+      <c r="E22" s="386"/>
+      <c r="F22" s="386"/>
+      <c r="G22" s="386"/>
+      <c r="H22" s="386"/>
+      <c r="I22" s="386"/>
+      <c r="J22" s="386"/>
+      <c r="K22" s="386"/>
+      <c r="L22" s="387"/>
     </row>
     <row r="23" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="387" t="s">
+      <c r="A23" s="388" t="s">
         <v>281</v>
       </c>
-      <c r="B23" s="388"/>
-      <c r="C23" s="388"/>
-      <c r="D23" s="388"/>
-      <c r="E23" s="388"/>
-      <c r="F23" s="388"/>
-      <c r="G23" s="388"/>
-      <c r="H23" s="388"/>
-      <c r="I23" s="388"/>
-      <c r="J23" s="388"/>
-      <c r="K23" s="388"/>
-      <c r="L23" s="389"/>
+      <c r="B23" s="389"/>
+      <c r="C23" s="389"/>
+      <c r="D23" s="389"/>
+      <c r="E23" s="389"/>
+      <c r="F23" s="389"/>
+      <c r="G23" s="389"/>
+      <c r="H23" s="389"/>
+      <c r="I23" s="389"/>
+      <c r="J23" s="389"/>
+      <c r="K23" s="389"/>
+      <c r="L23" s="390"/>
     </row>
     <row r="24" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="390" t="s">
+      <c r="A24" s="391" t="s">
         <v>282</v>
       </c>
-      <c r="B24" s="366"/>
-      <c r="C24" s="366"/>
-      <c r="D24" s="366"/>
-      <c r="E24" s="366"/>
-      <c r="F24" s="366"/>
-      <c r="G24" s="366"/>
-      <c r="H24" s="366"/>
-      <c r="I24" s="366"/>
-      <c r="J24" s="366"/>
-      <c r="K24" s="366"/>
-      <c r="L24" s="367"/>
+      <c r="B24" s="367"/>
+      <c r="C24" s="367"/>
+      <c r="D24" s="367"/>
+      <c r="E24" s="367"/>
+      <c r="F24" s="367"/>
+      <c r="G24" s="367"/>
+      <c r="H24" s="367"/>
+      <c r="I24" s="367"/>
+      <c r="J24" s="367"/>
+      <c r="K24" s="367"/>
+      <c r="L24" s="368"/>
     </row>
     <row r="25" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="390" t="s">
+      <c r="A25" s="391" t="s">
         <v>166</v>
       </c>
-      <c r="B25" s="366"/>
-      <c r="C25" s="366"/>
-      <c r="D25" s="366"/>
-      <c r="E25" s="366"/>
-      <c r="F25" s="366"/>
-      <c r="G25" s="366"/>
-      <c r="H25" s="366"/>
-      <c r="I25" s="366"/>
-      <c r="J25" s="366"/>
-      <c r="K25" s="366"/>
-      <c r="L25" s="367"/>
+      <c r="B25" s="367"/>
+      <c r="C25" s="367"/>
+      <c r="D25" s="367"/>
+      <c r="E25" s="367"/>
+      <c r="F25" s="367"/>
+      <c r="G25" s="367"/>
+      <c r="H25" s="367"/>
+      <c r="I25" s="367"/>
+      <c r="J25" s="367"/>
+      <c r="K25" s="367"/>
+      <c r="L25" s="368"/>
     </row>
     <row r="26" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="391" t="s">
+      <c r="A26" s="392" t="s">
         <v>283</v>
       </c>
-      <c r="B26" s="392"/>
-      <c r="C26" s="392"/>
-      <c r="D26" s="392"/>
-      <c r="E26" s="392"/>
-      <c r="F26" s="392"/>
-      <c r="G26" s="392"/>
-      <c r="H26" s="392"/>
-      <c r="I26" s="392"/>
-      <c r="J26" s="392"/>
-      <c r="K26" s="392"/>
-      <c r="L26" s="393"/>
+      <c r="B26" s="393"/>
+      <c r="C26" s="393"/>
+      <c r="D26" s="393"/>
+      <c r="E26" s="393"/>
+      <c r="F26" s="393"/>
+      <c r="G26" s="393"/>
+      <c r="H26" s="393"/>
+      <c r="I26" s="393"/>
+      <c r="J26" s="393"/>
+      <c r="K26" s="393"/>
+      <c r="L26" s="394"/>
     </row>
     <row r="27" spans="1:14" s="57" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="110"/>
@@ -16438,332 +18035,332 @@
       <c r="L27" s="110"/>
     </row>
     <row r="28" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="394" t="s">
+      <c r="A28" s="395" t="s">
         <v>279</v>
       </c>
-      <c r="B28" s="395"/>
-      <c r="C28" s="395"/>
-      <c r="D28" s="395"/>
-      <c r="E28" s="395"/>
-      <c r="F28" s="395"/>
-      <c r="G28" s="395"/>
-      <c r="H28" s="395"/>
-      <c r="I28" s="395"/>
-      <c r="J28" s="395"/>
-      <c r="K28" s="395"/>
-      <c r="L28" s="396"/>
+      <c r="B28" s="396"/>
+      <c r="C28" s="396"/>
+      <c r="D28" s="396"/>
+      <c r="E28" s="396"/>
+      <c r="F28" s="396"/>
+      <c r="G28" s="396"/>
+      <c r="H28" s="396"/>
+      <c r="I28" s="396"/>
+      <c r="J28" s="396"/>
+      <c r="K28" s="396"/>
+      <c r="L28" s="397"/>
       <c r="N28" s="1"/>
     </row>
     <row r="29" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="373" t="s">
+      <c r="A29" s="374" t="s">
         <v>175</v>
       </c>
-      <c r="B29" s="374"/>
-      <c r="C29" s="374"/>
-      <c r="D29" s="374"/>
-      <c r="E29" s="374"/>
-      <c r="F29" s="374"/>
-      <c r="G29" s="374"/>
-      <c r="H29" s="374"/>
-      <c r="I29" s="374"/>
-      <c r="J29" s="374"/>
-      <c r="K29" s="374"/>
-      <c r="L29" s="375"/>
+      <c r="B29" s="375"/>
+      <c r="C29" s="375"/>
+      <c r="D29" s="375"/>
+      <c r="E29" s="375"/>
+      <c r="F29" s="375"/>
+      <c r="G29" s="375"/>
+      <c r="H29" s="375"/>
+      <c r="I29" s="375"/>
+      <c r="J29" s="375"/>
+      <c r="K29" s="375"/>
+      <c r="L29" s="376"/>
       <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="209">
         <v>1</v>
       </c>
-      <c r="B30" s="359" t="s">
+      <c r="B30" s="360" t="s">
         <v>174</v>
       </c>
-      <c r="C30" s="359"/>
-      <c r="D30" s="359"/>
-      <c r="E30" s="359"/>
-      <c r="F30" s="359"/>
-      <c r="G30" s="359"/>
-      <c r="H30" s="359"/>
-      <c r="I30" s="359"/>
-      <c r="J30" s="359"/>
-      <c r="K30" s="359"/>
-      <c r="L30" s="360"/>
+      <c r="C30" s="360"/>
+      <c r="D30" s="360"/>
+      <c r="E30" s="360"/>
+      <c r="F30" s="360"/>
+      <c r="G30" s="360"/>
+      <c r="H30" s="360"/>
+      <c r="I30" s="360"/>
+      <c r="J30" s="360"/>
+      <c r="K30" s="360"/>
+      <c r="L30" s="361"/>
     </row>
     <row r="31" spans="1:14" s="57" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="209">
         <v>2</v>
       </c>
-      <c r="B31" s="359" t="s">
+      <c r="B31" s="360" t="s">
         <v>275</v>
       </c>
-      <c r="C31" s="359"/>
-      <c r="D31" s="359"/>
-      <c r="E31" s="359"/>
-      <c r="F31" s="359"/>
-      <c r="G31" s="359"/>
-      <c r="H31" s="359"/>
-      <c r="I31" s="359"/>
-      <c r="J31" s="359"/>
-      <c r="K31" s="359"/>
-      <c r="L31" s="360"/>
+      <c r="C31" s="360"/>
+      <c r="D31" s="360"/>
+      <c r="E31" s="360"/>
+      <c r="F31" s="360"/>
+      <c r="G31" s="360"/>
+      <c r="H31" s="360"/>
+      <c r="I31" s="360"/>
+      <c r="J31" s="360"/>
+      <c r="K31" s="360"/>
+      <c r="L31" s="361"/>
       <c r="N31" s="104"/>
     </row>
     <row r="32" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="209">
         <v>3</v>
       </c>
-      <c r="B32" s="359" t="s">
+      <c r="B32" s="360" t="s">
         <v>167</v>
       </c>
-      <c r="C32" s="359"/>
-      <c r="D32" s="359"/>
-      <c r="E32" s="359"/>
-      <c r="F32" s="359"/>
-      <c r="G32" s="359"/>
-      <c r="H32" s="359"/>
-      <c r="I32" s="359"/>
-      <c r="J32" s="359"/>
-      <c r="K32" s="359"/>
-      <c r="L32" s="360"/>
+      <c r="C32" s="360"/>
+      <c r="D32" s="360"/>
+      <c r="E32" s="360"/>
+      <c r="F32" s="360"/>
+      <c r="G32" s="360"/>
+      <c r="H32" s="360"/>
+      <c r="I32" s="360"/>
+      <c r="J32" s="360"/>
+      <c r="K32" s="360"/>
+      <c r="L32" s="361"/>
       <c r="N32" s="104"/>
     </row>
     <row r="33" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="209">
         <v>4</v>
       </c>
-      <c r="B33" s="359" t="s">
+      <c r="B33" s="360" t="s">
         <v>284</v>
       </c>
-      <c r="C33" s="359"/>
-      <c r="D33" s="359"/>
-      <c r="E33" s="359"/>
-      <c r="F33" s="359"/>
-      <c r="G33" s="359"/>
-      <c r="H33" s="359"/>
-      <c r="I33" s="359"/>
-      <c r="J33" s="359"/>
-      <c r="K33" s="359"/>
-      <c r="L33" s="360"/>
+      <c r="C33" s="360"/>
+      <c r="D33" s="360"/>
+      <c r="E33" s="360"/>
+      <c r="F33" s="360"/>
+      <c r="G33" s="360"/>
+      <c r="H33" s="360"/>
+      <c r="I33" s="360"/>
+      <c r="J33" s="360"/>
+      <c r="K33" s="360"/>
+      <c r="L33" s="361"/>
       <c r="N33" s="104"/>
     </row>
     <row r="34" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="209">
         <v>5</v>
       </c>
-      <c r="B34" s="359" t="s">
+      <c r="B34" s="360" t="s">
         <v>168</v>
       </c>
-      <c r="C34" s="359"/>
-      <c r="D34" s="359"/>
-      <c r="E34" s="359"/>
-      <c r="F34" s="359"/>
-      <c r="G34" s="359"/>
-      <c r="H34" s="359"/>
-      <c r="I34" s="359"/>
-      <c r="J34" s="359"/>
-      <c r="K34" s="359"/>
-      <c r="L34" s="360"/>
+      <c r="C34" s="360"/>
+      <c r="D34" s="360"/>
+      <c r="E34" s="360"/>
+      <c r="F34" s="360"/>
+      <c r="G34" s="360"/>
+      <c r="H34" s="360"/>
+      <c r="I34" s="360"/>
+      <c r="J34" s="360"/>
+      <c r="K34" s="360"/>
+      <c r="L34" s="361"/>
       <c r="N34" s="104"/>
     </row>
     <row r="35" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="209"/>
-      <c r="B35" s="359" t="s">
+      <c r="B35" s="360" t="s">
         <v>169</v>
       </c>
-      <c r="C35" s="359"/>
-      <c r="D35" s="359"/>
-      <c r="E35" s="359"/>
-      <c r="F35" s="359"/>
-      <c r="G35" s="359"/>
-      <c r="H35" s="359"/>
-      <c r="I35" s="359"/>
-      <c r="J35" s="359"/>
-      <c r="K35" s="359"/>
-      <c r="L35" s="360"/>
+      <c r="C35" s="360"/>
+      <c r="D35" s="360"/>
+      <c r="E35" s="360"/>
+      <c r="F35" s="360"/>
+      <c r="G35" s="360"/>
+      <c r="H35" s="360"/>
+      <c r="I35" s="360"/>
+      <c r="J35" s="360"/>
+      <c r="K35" s="360"/>
+      <c r="L35" s="361"/>
       <c r="N35" s="104"/>
     </row>
     <row r="36" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="209"/>
-      <c r="B36" s="359" t="s">
+      <c r="B36" s="360" t="s">
         <v>170</v>
       </c>
-      <c r="C36" s="359"/>
-      <c r="D36" s="359"/>
-      <c r="E36" s="359"/>
-      <c r="F36" s="359"/>
-      <c r="G36" s="359"/>
-      <c r="H36" s="359"/>
-      <c r="I36" s="359"/>
-      <c r="J36" s="359"/>
-      <c r="K36" s="359"/>
-      <c r="L36" s="360"/>
+      <c r="C36" s="360"/>
+      <c r="D36" s="360"/>
+      <c r="E36" s="360"/>
+      <c r="F36" s="360"/>
+      <c r="G36" s="360"/>
+      <c r="H36" s="360"/>
+      <c r="I36" s="360"/>
+      <c r="J36" s="360"/>
+      <c r="K36" s="360"/>
+      <c r="L36" s="361"/>
       <c r="N36" s="104"/>
     </row>
     <row r="37" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="368" t="s">
+      <c r="A37" s="369" t="s">
         <v>176</v>
       </c>
-      <c r="B37" s="369"/>
-      <c r="C37" s="369"/>
-      <c r="D37" s="369"/>
-      <c r="E37" s="369"/>
-      <c r="F37" s="369"/>
-      <c r="G37" s="369"/>
-      <c r="H37" s="369"/>
-      <c r="I37" s="369"/>
-      <c r="J37" s="369"/>
-      <c r="K37" s="369"/>
-      <c r="L37" s="370"/>
+      <c r="B37" s="370"/>
+      <c r="C37" s="370"/>
+      <c r="D37" s="370"/>
+      <c r="E37" s="370"/>
+      <c r="F37" s="370"/>
+      <c r="G37" s="370"/>
+      <c r="H37" s="370"/>
+      <c r="I37" s="370"/>
+      <c r="J37" s="370"/>
+      <c r="K37" s="370"/>
+      <c r="L37" s="371"/>
       <c r="N37" s="104"/>
     </row>
     <row r="38" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="209">
         <v>1</v>
       </c>
-      <c r="B38" s="359" t="s">
+      <c r="B38" s="360" t="s">
         <v>171</v>
       </c>
-      <c r="C38" s="359"/>
-      <c r="D38" s="359"/>
-      <c r="E38" s="359"/>
-      <c r="F38" s="359"/>
-      <c r="G38" s="359"/>
-      <c r="H38" s="359"/>
-      <c r="I38" s="359"/>
-      <c r="J38" s="359"/>
-      <c r="K38" s="359"/>
-      <c r="L38" s="360"/>
+      <c r="C38" s="360"/>
+      <c r="D38" s="360"/>
+      <c r="E38" s="360"/>
+      <c r="F38" s="360"/>
+      <c r="G38" s="360"/>
+      <c r="H38" s="360"/>
+      <c r="I38" s="360"/>
+      <c r="J38" s="360"/>
+      <c r="K38" s="360"/>
+      <c r="L38" s="361"/>
       <c r="N38" s="104"/>
     </row>
     <row r="39" spans="1:14" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="209"/>
-      <c r="B39" s="357" t="s">
+      <c r="B39" s="358" t="s">
         <v>426</v>
       </c>
-      <c r="C39" s="357"/>
-      <c r="D39" s="357"/>
-      <c r="E39" s="357"/>
-      <c r="F39" s="357"/>
-      <c r="G39" s="357"/>
-      <c r="H39" s="357"/>
-      <c r="I39" s="357"/>
-      <c r="J39" s="357"/>
-      <c r="K39" s="357"/>
-      <c r="L39" s="358"/>
+      <c r="C39" s="358"/>
+      <c r="D39" s="358"/>
+      <c r="E39" s="358"/>
+      <c r="F39" s="358"/>
+      <c r="G39" s="358"/>
+      <c r="H39" s="358"/>
+      <c r="I39" s="358"/>
+      <c r="J39" s="358"/>
+      <c r="K39" s="358"/>
+      <c r="L39" s="359"/>
       <c r="N39" s="104"/>
     </row>
     <row r="40" spans="1:14" s="57" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="209">
         <v>2</v>
       </c>
-      <c r="B40" s="359" t="s">
+      <c r="B40" s="360" t="s">
         <v>278</v>
       </c>
-      <c r="C40" s="359"/>
-      <c r="D40" s="359"/>
-      <c r="E40" s="359"/>
-      <c r="F40" s="359"/>
-      <c r="G40" s="359"/>
-      <c r="H40" s="359"/>
-      <c r="I40" s="359"/>
-      <c r="J40" s="359"/>
-      <c r="K40" s="359"/>
-      <c r="L40" s="360"/>
+      <c r="C40" s="360"/>
+      <c r="D40" s="360"/>
+      <c r="E40" s="360"/>
+      <c r="F40" s="360"/>
+      <c r="G40" s="360"/>
+      <c r="H40" s="360"/>
+      <c r="I40" s="360"/>
+      <c r="J40" s="360"/>
+      <c r="K40" s="360"/>
+      <c r="L40" s="361"/>
       <c r="N40" s="104"/>
     </row>
     <row r="41" spans="1:14" s="57" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="209">
         <v>3</v>
       </c>
-      <c r="B41" s="359" t="s">
+      <c r="B41" s="360" t="s">
         <v>475</v>
       </c>
-      <c r="C41" s="359"/>
-      <c r="D41" s="359"/>
-      <c r="E41" s="359"/>
-      <c r="F41" s="359"/>
-      <c r="G41" s="359"/>
-      <c r="H41" s="359"/>
-      <c r="I41" s="359"/>
-      <c r="J41" s="359"/>
-      <c r="K41" s="359"/>
-      <c r="L41" s="360"/>
+      <c r="C41" s="360"/>
+      <c r="D41" s="360"/>
+      <c r="E41" s="360"/>
+      <c r="F41" s="360"/>
+      <c r="G41" s="360"/>
+      <c r="H41" s="360"/>
+      <c r="I41" s="360"/>
+      <c r="J41" s="360"/>
+      <c r="K41" s="360"/>
+      <c r="L41" s="361"/>
       <c r="N41" s="104"/>
     </row>
     <row r="42" spans="1:14" s="57" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="209">
         <v>4</v>
       </c>
-      <c r="B42" s="359" t="s">
+      <c r="B42" s="360" t="s">
         <v>285</v>
       </c>
-      <c r="C42" s="359"/>
-      <c r="D42" s="359"/>
-      <c r="E42" s="359"/>
-      <c r="F42" s="359"/>
-      <c r="G42" s="359"/>
-      <c r="H42" s="359"/>
-      <c r="I42" s="359"/>
-      <c r="J42" s="359"/>
-      <c r="K42" s="359"/>
-      <c r="L42" s="360"/>
+      <c r="C42" s="360"/>
+      <c r="D42" s="360"/>
+      <c r="E42" s="360"/>
+      <c r="F42" s="360"/>
+      <c r="G42" s="360"/>
+      <c r="H42" s="360"/>
+      <c r="I42" s="360"/>
+      <c r="J42" s="360"/>
+      <c r="K42" s="360"/>
+      <c r="L42" s="361"/>
       <c r="N42" s="104"/>
     </row>
     <row r="43" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="209">
         <v>5</v>
       </c>
-      <c r="B43" s="357" t="s">
+      <c r="B43" s="358" t="s">
         <v>269</v>
       </c>
-      <c r="C43" s="357"/>
-      <c r="D43" s="357"/>
-      <c r="E43" s="357"/>
-      <c r="F43" s="357"/>
-      <c r="G43" s="357"/>
-      <c r="H43" s="357"/>
-      <c r="I43" s="357"/>
-      <c r="J43" s="357"/>
-      <c r="K43" s="357"/>
-      <c r="L43" s="358"/>
+      <c r="C43" s="358"/>
+      <c r="D43" s="358"/>
+      <c r="E43" s="358"/>
+      <c r="F43" s="358"/>
+      <c r="G43" s="358"/>
+      <c r="H43" s="358"/>
+      <c r="I43" s="358"/>
+      <c r="J43" s="358"/>
+      <c r="K43" s="358"/>
+      <c r="L43" s="359"/>
       <c r="N43" s="104"/>
     </row>
     <row r="44" spans="1:14" s="57" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="209">
         <v>6</v>
       </c>
-      <c r="B44" s="357" t="s">
+      <c r="B44" s="358" t="s">
         <v>476</v>
       </c>
-      <c r="C44" s="357"/>
-      <c r="D44" s="357"/>
-      <c r="E44" s="357"/>
-      <c r="F44" s="357"/>
-      <c r="G44" s="357"/>
-      <c r="H44" s="357"/>
-      <c r="I44" s="357"/>
-      <c r="J44" s="357"/>
-      <c r="K44" s="357"/>
-      <c r="L44" s="358"/>
+      <c r="C44" s="358"/>
+      <c r="D44" s="358"/>
+      <c r="E44" s="358"/>
+      <c r="F44" s="358"/>
+      <c r="G44" s="358"/>
+      <c r="H44" s="358"/>
+      <c r="I44" s="358"/>
+      <c r="J44" s="358"/>
+      <c r="K44" s="358"/>
+      <c r="L44" s="359"/>
       <c r="N44" s="104"/>
     </row>
     <row r="45" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="209">
         <v>7</v>
       </c>
-      <c r="B45" s="359" t="s">
+      <c r="B45" s="360" t="s">
         <v>270</v>
       </c>
-      <c r="C45" s="359"/>
-      <c r="D45" s="359"/>
-      <c r="E45" s="359"/>
-      <c r="F45" s="359"/>
-      <c r="G45" s="359"/>
-      <c r="H45" s="359"/>
-      <c r="I45" s="359"/>
-      <c r="J45" s="359"/>
-      <c r="K45" s="359"/>
-      <c r="L45" s="360"/>
+      <c r="C45" s="360"/>
+      <c r="D45" s="360"/>
+      <c r="E45" s="360"/>
+      <c r="F45" s="360"/>
+      <c r="G45" s="360"/>
+      <c r="H45" s="360"/>
+      <c r="I45" s="360"/>
+      <c r="J45" s="360"/>
+      <c r="K45" s="360"/>
+      <c r="L45" s="361"/>
     </row>
     <row r="46" spans="1:14" s="57" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="209"/>
@@ -16780,56 +18377,56 @@
       <c r="L46" s="211"/>
     </row>
     <row r="47" spans="1:14" s="57" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="368" t="s">
+      <c r="A47" s="369" t="s">
         <v>273</v>
       </c>
-      <c r="B47" s="369"/>
-      <c r="C47" s="369"/>
-      <c r="D47" s="369"/>
-      <c r="E47" s="369"/>
-      <c r="F47" s="369"/>
-      <c r="G47" s="369"/>
-      <c r="H47" s="369"/>
-      <c r="I47" s="369"/>
-      <c r="J47" s="369"/>
-      <c r="K47" s="369"/>
-      <c r="L47" s="370"/>
+      <c r="B47" s="370"/>
+      <c r="C47" s="370"/>
+      <c r="D47" s="370"/>
+      <c r="E47" s="370"/>
+      <c r="F47" s="370"/>
+      <c r="G47" s="370"/>
+      <c r="H47" s="370"/>
+      <c r="I47" s="370"/>
+      <c r="J47" s="370"/>
+      <c r="K47" s="370"/>
+      <c r="L47" s="371"/>
     </row>
     <row r="48" spans="1:14" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="212" t="s">
         <v>271</v>
       </c>
-      <c r="B48" s="359" t="s">
+      <c r="B48" s="360" t="s">
         <v>172</v>
       </c>
-      <c r="C48" s="359"/>
-      <c r="D48" s="359"/>
-      <c r="E48" s="359"/>
-      <c r="F48" s="359"/>
-      <c r="G48" s="359"/>
-      <c r="H48" s="359"/>
-      <c r="I48" s="359"/>
-      <c r="J48" s="359"/>
-      <c r="K48" s="359"/>
-      <c r="L48" s="360"/>
+      <c r="C48" s="360"/>
+      <c r="D48" s="360"/>
+      <c r="E48" s="360"/>
+      <c r="F48" s="360"/>
+      <c r="G48" s="360"/>
+      <c r="H48" s="360"/>
+      <c r="I48" s="360"/>
+      <c r="J48" s="360"/>
+      <c r="K48" s="360"/>
+      <c r="L48" s="361"/>
     </row>
     <row r="49" spans="1:12" s="57" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="213" t="s">
         <v>272</v>
       </c>
-      <c r="B49" s="361" t="s">
+      <c r="B49" s="362" t="s">
         <v>274</v>
       </c>
-      <c r="C49" s="361"/>
-      <c r="D49" s="361"/>
-      <c r="E49" s="361"/>
-      <c r="F49" s="361"/>
-      <c r="G49" s="361"/>
-      <c r="H49" s="361"/>
-      <c r="I49" s="361"/>
-      <c r="J49" s="361"/>
-      <c r="K49" s="361"/>
-      <c r="L49" s="362"/>
+      <c r="C49" s="362"/>
+      <c r="D49" s="362"/>
+      <c r="E49" s="362"/>
+      <c r="F49" s="362"/>
+      <c r="G49" s="362"/>
+      <c r="H49" s="362"/>
+      <c r="I49" s="362"/>
+      <c r="J49" s="362"/>
+      <c r="K49" s="362"/>
+      <c r="L49" s="363"/>
     </row>
     <row r="50" spans="1:12" s="57" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="157"/>
@@ -16846,20 +18443,20 @@
       <c r="L50" s="110"/>
     </row>
     <row r="51" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="363" t="s">
+      <c r="A51" s="364" t="s">
         <v>200</v>
       </c>
-      <c r="B51" s="364"/>
-      <c r="C51" s="364"/>
-      <c r="D51" s="364"/>
-      <c r="E51" s="364"/>
-      <c r="F51" s="364"/>
-      <c r="G51" s="364"/>
-      <c r="H51" s="364"/>
-      <c r="I51" s="364"/>
-      <c r="J51" s="364"/>
-      <c r="K51" s="364"/>
-      <c r="L51" s="365"/>
+      <c r="B51" s="365"/>
+      <c r="C51" s="365"/>
+      <c r="D51" s="365"/>
+      <c r="E51" s="365"/>
+      <c r="F51" s="365"/>
+      <c r="G51" s="365"/>
+      <c r="H51" s="365"/>
+      <c r="I51" s="365"/>
+      <c r="J51" s="365"/>
+      <c r="K51" s="365"/>
+      <c r="L51" s="366"/>
     </row>
     <row r="52" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="216" t="s">
@@ -16947,126 +18544,126 @@
       <c r="B57" s="165" t="s">
         <v>24</v>
       </c>
-      <c r="C57" s="366" t="s">
+      <c r="C57" s="367" t="s">
         <v>262</v>
       </c>
-      <c r="D57" s="366"/>
-      <c r="E57" s="366"/>
-      <c r="F57" s="366"/>
-      <c r="G57" s="366"/>
-      <c r="H57" s="366"/>
-      <c r="I57" s="366"/>
-      <c r="J57" s="366"/>
-      <c r="K57" s="366"/>
-      <c r="L57" s="367"/>
+      <c r="D57" s="367"/>
+      <c r="E57" s="367"/>
+      <c r="F57" s="367"/>
+      <c r="G57" s="367"/>
+      <c r="H57" s="367"/>
+      <c r="I57" s="367"/>
+      <c r="J57" s="367"/>
+      <c r="K57" s="367"/>
+      <c r="L57" s="368"/>
     </row>
     <row r="58" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="164"/>
       <c r="B58" s="165" t="s">
         <v>263</v>
       </c>
-      <c r="C58" s="366" t="s">
+      <c r="C58" s="367" t="s">
         <v>264</v>
       </c>
-      <c r="D58" s="366"/>
-      <c r="E58" s="366"/>
-      <c r="F58" s="366"/>
-      <c r="G58" s="366"/>
-      <c r="H58" s="366"/>
-      <c r="I58" s="366"/>
-      <c r="J58" s="366"/>
-      <c r="K58" s="366"/>
-      <c r="L58" s="367"/>
+      <c r="D58" s="367"/>
+      <c r="E58" s="367"/>
+      <c r="F58" s="367"/>
+      <c r="G58" s="367"/>
+      <c r="H58" s="367"/>
+      <c r="I58" s="367"/>
+      <c r="J58" s="367"/>
+      <c r="K58" s="367"/>
+      <c r="L58" s="368"/>
     </row>
     <row r="59" spans="1:12" s="56" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="164"/>
       <c r="B59" s="165" t="s">
         <v>327</v>
       </c>
-      <c r="C59" s="366" t="s">
+      <c r="C59" s="367" t="s">
         <v>328</v>
       </c>
-      <c r="D59" s="366"/>
-      <c r="E59" s="366"/>
-      <c r="F59" s="366"/>
-      <c r="G59" s="366"/>
-      <c r="H59" s="366"/>
-      <c r="I59" s="366"/>
-      <c r="J59" s="366"/>
-      <c r="K59" s="366"/>
-      <c r="L59" s="367"/>
+      <c r="D59" s="367"/>
+      <c r="E59" s="367"/>
+      <c r="F59" s="367"/>
+      <c r="G59" s="367"/>
+      <c r="H59" s="367"/>
+      <c r="I59" s="367"/>
+      <c r="J59" s="367"/>
+      <c r="K59" s="367"/>
+      <c r="L59" s="368"/>
     </row>
     <row r="60" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="164"/>
       <c r="B60" s="165" t="s">
         <v>98</v>
       </c>
-      <c r="C60" s="366" t="s">
+      <c r="C60" s="367" t="s">
         <v>99</v>
       </c>
-      <c r="D60" s="366"/>
-      <c r="E60" s="366"/>
-      <c r="F60" s="366"/>
-      <c r="G60" s="366"/>
-      <c r="H60" s="366"/>
-      <c r="I60" s="366"/>
-      <c r="J60" s="366"/>
-      <c r="K60" s="366"/>
-      <c r="L60" s="367"/>
+      <c r="D60" s="367"/>
+      <c r="E60" s="367"/>
+      <c r="F60" s="367"/>
+      <c r="G60" s="367"/>
+      <c r="H60" s="367"/>
+      <c r="I60" s="367"/>
+      <c r="J60" s="367"/>
+      <c r="K60" s="367"/>
+      <c r="L60" s="368"/>
     </row>
     <row r="61" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="164"/>
       <c r="B61" s="165" t="s">
         <v>198</v>
       </c>
-      <c r="C61" s="366" t="s">
+      <c r="C61" s="367" t="s">
         <v>199</v>
       </c>
-      <c r="D61" s="366"/>
-      <c r="E61" s="366"/>
-      <c r="F61" s="366"/>
-      <c r="G61" s="366"/>
-      <c r="H61" s="366"/>
-      <c r="I61" s="366"/>
-      <c r="J61" s="366"/>
-      <c r="K61" s="366"/>
-      <c r="L61" s="367"/>
+      <c r="D61" s="367"/>
+      <c r="E61" s="367"/>
+      <c r="F61" s="367"/>
+      <c r="G61" s="367"/>
+      <c r="H61" s="367"/>
+      <c r="I61" s="367"/>
+      <c r="J61" s="367"/>
+      <c r="K61" s="367"/>
+      <c r="L61" s="368"/>
     </row>
     <row r="62" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="164"/>
       <c r="B62" s="165" t="s">
         <v>163</v>
       </c>
-      <c r="C62" s="366" t="s">
+      <c r="C62" s="367" t="s">
         <v>466</v>
       </c>
-      <c r="D62" s="371"/>
-      <c r="E62" s="371"/>
-      <c r="F62" s="371"/>
-      <c r="G62" s="371"/>
-      <c r="H62" s="371"/>
-      <c r="I62" s="371"/>
-      <c r="J62" s="371"/>
-      <c r="K62" s="371"/>
-      <c r="L62" s="372"/>
+      <c r="D62" s="372"/>
+      <c r="E62" s="372"/>
+      <c r="F62" s="372"/>
+      <c r="G62" s="372"/>
+      <c r="H62" s="372"/>
+      <c r="I62" s="372"/>
+      <c r="J62" s="372"/>
+      <c r="K62" s="372"/>
+      <c r="L62" s="373"/>
     </row>
     <row r="63" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="164"/>
       <c r="B63" s="165" t="s">
         <v>393</v>
       </c>
-      <c r="C63" s="366" t="s">
+      <c r="C63" s="367" t="s">
         <v>394</v>
       </c>
-      <c r="D63" s="366"/>
-      <c r="E63" s="366"/>
-      <c r="F63" s="366"/>
-      <c r="G63" s="366"/>
-      <c r="H63" s="366"/>
-      <c r="I63" s="366"/>
-      <c r="J63" s="366"/>
-      <c r="K63" s="366"/>
-      <c r="L63" s="367"/>
+      <c r="D63" s="367"/>
+      <c r="E63" s="367"/>
+      <c r="F63" s="367"/>
+      <c r="G63" s="367"/>
+      <c r="H63" s="367"/>
+      <c r="I63" s="367"/>
+      <c r="J63" s="367"/>
+      <c r="K63" s="367"/>
+      <c r="L63" s="368"/>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="164"/>
@@ -17184,20 +18781,20 @@
       </c>
     </row>
     <row r="85" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="356" t="s">
+      <c r="A85" s="357" t="s">
         <v>397</v>
       </c>
-      <c r="B85" s="356"/>
-      <c r="C85" s="356"/>
-      <c r="D85" s="356"/>
-      <c r="E85" s="356"/>
-      <c r="F85" s="356"/>
-      <c r="G85" s="356"/>
-      <c r="H85" s="356"/>
-      <c r="I85" s="356"/>
-      <c r="J85" s="356"/>
-      <c r="K85" s="356"/>
-      <c r="L85" s="356"/>
+      <c r="B85" s="357"/>
+      <c r="C85" s="357"/>
+      <c r="D85" s="357"/>
+      <c r="E85" s="357"/>
+      <c r="F85" s="357"/>
+      <c r="G85" s="357"/>
+      <c r="H85" s="357"/>
+      <c r="I85" s="357"/>
+      <c r="J85" s="357"/>
+      <c r="K85" s="357"/>
+      <c r="L85" s="357"/>
     </row>
     <row r="90" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="91" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -17284,82 +18881,82 @@
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="448" t="s">
+      <c r="A3" s="449" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="448"/>
-      <c r="C3" s="448"/>
+      <c r="B3" s="449"/>
+      <c r="C3" s="449"/>
       <c r="D3" s="125" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="449" t="s">
+      <c r="A4" s="450" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="449"/>
-      <c r="C4" s="449"/>
+      <c r="B4" s="450"/>
+      <c r="C4" s="450"/>
       <c r="D4" s="172" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A5" s="453" t="s">
+      <c r="A5" s="454" t="s">
         <v>183</v>
       </c>
-      <c r="B5" s="450"/>
-      <c r="C5" s="450"/>
+      <c r="B5" s="451"/>
+      <c r="C5" s="451"/>
       <c r="D5" s="173" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="57.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="451" t="s">
+      <c r="A6" s="452" t="s">
         <v>184</v>
       </c>
-      <c r="B6" s="451"/>
-      <c r="C6" s="451"/>
+      <c r="B6" s="452"/>
+      <c r="C6" s="452"/>
       <c r="D6" s="174" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" s="452" t="s">
+      <c r="A7" s="453" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="452"/>
-      <c r="C7" s="452"/>
+      <c r="B7" s="453"/>
+      <c r="C7" s="453"/>
       <c r="D7" s="175" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="449" t="s">
+      <c r="A11" s="450" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="449"/>
-      <c r="C11" s="449"/>
+      <c r="B11" s="450"/>
+      <c r="C11" s="450"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="450" t="s">
+      <c r="A12" s="451" t="s">
         <v>113</v>
       </c>
-      <c r="B12" s="450"/>
-      <c r="C12" s="450"/>
+      <c r="B12" s="451"/>
+      <c r="C12" s="451"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="451" t="s">
+      <c r="A13" s="452" t="s">
         <v>114</v>
       </c>
-      <c r="B13" s="451"/>
-      <c r="C13" s="451"/>
+      <c r="B13" s="452"/>
+      <c r="C13" s="452"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="452" t="s">
+      <c r="A14" s="453" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="452"/>
-      <c r="C14" s="452"/>
+      <c r="B14" s="453"/>
+      <c r="C14" s="453"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -17620,28 +19217,28 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="454" t="s">
+      <c r="A2" s="455" t="s">
         <v>420</v>
       </c>
-      <c r="B2" s="455"/>
-      <c r="C2" s="455"/>
-      <c r="D2" s="455"/>
-      <c r="E2" s="455"/>
-      <c r="F2" s="455"/>
-      <c r="G2" s="455"/>
-      <c r="H2" s="455"/>
-      <c r="I2" s="455"/>
-      <c r="J2" s="455"/>
-      <c r="K2" s="455"/>
-      <c r="L2" s="455"/>
-      <c r="M2" s="455"/>
-      <c r="N2" s="455"/>
-      <c r="O2" s="455"/>
-      <c r="P2" s="455"/>
-      <c r="Q2" s="455"/>
-      <c r="R2" s="455"/>
-      <c r="S2" s="455"/>
-      <c r="T2" s="455"/>
+      <c r="B2" s="456"/>
+      <c r="C2" s="456"/>
+      <c r="D2" s="456"/>
+      <c r="E2" s="456"/>
+      <c r="F2" s="456"/>
+      <c r="G2" s="456"/>
+      <c r="H2" s="456"/>
+      <c r="I2" s="456"/>
+      <c r="J2" s="456"/>
+      <c r="K2" s="456"/>
+      <c r="L2" s="456"/>
+      <c r="M2" s="456"/>
+      <c r="N2" s="456"/>
+      <c r="O2" s="456"/>
+      <c r="P2" s="456"/>
+      <c r="Q2" s="456"/>
+      <c r="R2" s="456"/>
+      <c r="S2" s="456"/>
+      <c r="T2" s="456"/>
     </row>
     <row r="3" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:20" ht="32" x14ac:dyDescent="0.2">
@@ -18346,6 +19943,118 @@
   <mergeCells count="1">
     <mergeCell ref="A2:T2"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6EC9312-1D6A-C146-B06E-16E6A54035B4}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B1" s="101" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="101" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="101" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="101" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="101" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>481</v>
+      </c>
+      <c r="B2" s="95">
+        <f>Master!$C$20</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="95">
+        <f>Master!$C$20</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="95">
+        <f>Master!$C$20</f>
+        <v>0</v>
+      </c>
+      <c r="E2" s="95">
+        <f>Master!$C$20</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="95">
+        <f>Master!$C$20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>482</v>
+      </c>
+      <c r="B3" s="95">
+        <v>10.857008</v>
+      </c>
+      <c r="C3" s="95">
+        <v>10.857008</v>
+      </c>
+      <c r="D3" s="95">
+        <v>10.857008</v>
+      </c>
+      <c r="E3" s="95">
+        <v>10.857008</v>
+      </c>
+      <c r="F3" s="95">
+        <v>10.857008</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>483</v>
+      </c>
+      <c r="B4" s="95">
+        <v>2.2231700000000001</v>
+      </c>
+      <c r="C4" s="95">
+        <v>2.2231700000000001</v>
+      </c>
+      <c r="D4" s="95">
+        <v>2.2231700000000001</v>
+      </c>
+      <c r="E4" s="95">
+        <v>2.2231700000000001</v>
+      </c>
+      <c r="F4" s="95">
+        <v>2.2231700000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>484</v>
+      </c>
+      <c r="B5" s="95"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="95"/>
+      <c r="E5" s="95"/>
+      <c r="F5" s="95"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B6" s="95"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="95"/>
+      <c r="E6" s="95"/>
+      <c r="F6" s="95"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -19031,16 +20740,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="404" t="str">
+      <c r="A1" s="405" t="str">
         <f>'ReadMe-Directions'!A1</f>
         <v>Immersive Model for Lake Mead based on the Principle of Divide Reservoir Inflow</v>
       </c>
-      <c r="B1" s="404"/>
-      <c r="C1" s="404"/>
-      <c r="D1" s="404"/>
-      <c r="E1" s="404"/>
-      <c r="F1" s="404"/>
-      <c r="G1" s="404"/>
+      <c r="B1" s="405"/>
+      <c r="C1" s="405"/>
+      <c r="D1" s="405"/>
+      <c r="E1" s="405"/>
+      <c r="F1" s="405"/>
+      <c r="G1" s="405"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -19049,15 +20758,15 @@
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="412" t="s">
+      <c r="A3" s="413" t="s">
         <v>190</v>
       </c>
-      <c r="B3" s="412"/>
-      <c r="C3" s="412"/>
-      <c r="D3" s="412"/>
-      <c r="E3" s="412"/>
-      <c r="F3" s="412"/>
-      <c r="G3" s="412"/>
+      <c r="B3" s="413"/>
+      <c r="C3" s="413"/>
+      <c r="D3" s="413"/>
+      <c r="E3" s="413"/>
+      <c r="F3" s="413"/>
+      <c r="G3" s="413"/>
       <c r="H3" s="82"/>
       <c r="I3" s="82"/>
       <c r="J3" s="82"/>
@@ -19073,13 +20782,13 @@
       <c r="B4" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="413" t="s">
+      <c r="C4" s="414" t="s">
         <v>259</v>
       </c>
-      <c r="D4" s="414"/>
-      <c r="E4" s="414"/>
-      <c r="F4" s="414"/>
-      <c r="G4" s="415"/>
+      <c r="D4" s="415"/>
+      <c r="E4" s="415"/>
+      <c r="F4" s="415"/>
+      <c r="G4" s="416"/>
       <c r="N4" s="138" t="s">
         <v>329</v>
       </c>
@@ -19089,11 +20798,11 @@
         <v>238</v>
       </c>
       <c r="B5" s="111"/>
-      <c r="C5" s="416"/>
-      <c r="D5" s="411"/>
-      <c r="E5" s="411"/>
-      <c r="F5" s="411"/>
-      <c r="G5" s="411"/>
+      <c r="C5" s="417"/>
+      <c r="D5" s="412"/>
+      <c r="E5" s="412"/>
+      <c r="F5" s="412"/>
+      <c r="G5" s="412"/>
       <c r="N5" s="138"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -19101,11 +20810,11 @@
         <v>202</v>
       </c>
       <c r="B6" s="111"/>
-      <c r="C6" s="416"/>
-      <c r="D6" s="411"/>
-      <c r="E6" s="411"/>
-      <c r="F6" s="411"/>
-      <c r="G6" s="411"/>
+      <c r="C6" s="417"/>
+      <c r="D6" s="412"/>
+      <c r="E6" s="412"/>
+      <c r="F6" s="412"/>
+      <c r="G6" s="412"/>
       <c r="N6" s="139"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -19113,11 +20822,11 @@
         <v>203</v>
       </c>
       <c r="B7" s="111"/>
-      <c r="C7" s="416"/>
-      <c r="D7" s="411"/>
-      <c r="E7" s="411"/>
-      <c r="F7" s="411"/>
-      <c r="G7" s="411"/>
+      <c r="C7" s="417"/>
+      <c r="D7" s="412"/>
+      <c r="E7" s="412"/>
+      <c r="F7" s="412"/>
+      <c r="G7" s="412"/>
       <c r="N7" s="139"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -19125,11 +20834,11 @@
         <v>204</v>
       </c>
       <c r="B8" s="88"/>
-      <c r="C8" s="411"/>
-      <c r="D8" s="411"/>
-      <c r="E8" s="411"/>
-      <c r="F8" s="411"/>
-      <c r="G8" s="411"/>
+      <c r="C8" s="412"/>
+      <c r="D8" s="412"/>
+      <c r="E8" s="412"/>
+      <c r="F8" s="412"/>
+      <c r="G8" s="412"/>
       <c r="N8" s="139"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -19137,11 +20846,11 @@
         <v>18</v>
       </c>
       <c r="B9" s="88"/>
-      <c r="C9" s="417"/>
-      <c r="D9" s="417"/>
-      <c r="E9" s="417"/>
-      <c r="F9" s="417"/>
-      <c r="G9" s="417"/>
+      <c r="C9" s="418"/>
+      <c r="D9" s="418"/>
+      <c r="E9" s="418"/>
+      <c r="F9" s="418"/>
+      <c r="G9" s="418"/>
       <c r="N9" s="139"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -19149,11 +20858,11 @@
         <v>277</v>
       </c>
       <c r="B10" s="88"/>
-      <c r="C10" s="411"/>
-      <c r="D10" s="411"/>
-      <c r="E10" s="411"/>
-      <c r="F10" s="411"/>
-      <c r="G10" s="411"/>
+      <c r="C10" s="412"/>
+      <c r="D10" s="412"/>
+      <c r="E10" s="412"/>
+      <c r="F10" s="412"/>
+      <c r="G10" s="412"/>
       <c r="N10" s="139"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -19166,36 +20875,36 @@
       <c r="A12" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B12" s="418" t="s">
+      <c r="B12" s="419" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="419"/>
-      <c r="D12" s="420"/>
+      <c r="C12" s="420"/>
+      <c r="D12" s="421"/>
       <c r="N12" s="138" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B13" s="421" t="s">
+      <c r="B13" s="422" t="s">
         <v>189</v>
       </c>
-      <c r="C13" s="422"/>
-      <c r="D13" s="423"/>
+      <c r="C13" s="423"/>
+      <c r="D13" s="424"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B14" s="405" t="s">
+      <c r="B14" s="406" t="s">
         <v>184</v>
       </c>
-      <c r="C14" s="406"/>
-      <c r="D14" s="407"/>
+      <c r="C14" s="407"/>
+      <c r="D14" s="408"/>
       <c r="N14" s="139"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B15" s="408" t="s">
+      <c r="B15" s="409" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="409"/>
-      <c r="D15" s="410"/>
+      <c r="C15" s="410"/>
+      <c r="D15" s="411"/>
       <c r="N15" s="139"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
@@ -20538,7 +22247,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N54" s="140"/>
-      <c r="P54" s="79"/>
+      <c r="P54" s="350"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" t="str">
@@ -20579,7 +22288,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N55" s="140"/>
-      <c r="P55" s="79"/>
+      <c r="P55" s="350"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="str">
@@ -24637,62 +26346,62 @@
       <c r="G5" s="185" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="437" t="s">
+      <c r="I5" s="438" t="s">
         <v>423</v>
       </c>
-      <c r="J5" s="438"/>
-      <c r="K5" s="438"/>
-      <c r="L5" s="438"/>
-      <c r="M5" s="438"/>
-      <c r="N5" s="438"/>
-      <c r="O5" s="438"/>
-      <c r="P5" s="438"/>
-      <c r="Q5" s="438"/>
-      <c r="R5" s="438"/>
-      <c r="S5" s="438"/>
-      <c r="T5" s="438"/>
-      <c r="U5" s="438"/>
-      <c r="V5" s="438"/>
-      <c r="W5" s="439"/>
+      <c r="J5" s="439"/>
+      <c r="K5" s="439"/>
+      <c r="L5" s="439"/>
+      <c r="M5" s="439"/>
+      <c r="N5" s="439"/>
+      <c r="O5" s="439"/>
+      <c r="P5" s="439"/>
+      <c r="Q5" s="439"/>
+      <c r="R5" s="439"/>
+      <c r="S5" s="439"/>
+      <c r="T5" s="439"/>
+      <c r="U5" s="439"/>
+      <c r="V5" s="439"/>
+      <c r="W5" s="440"/>
       <c r="Y5" s="192"/>
       <c r="Z5" s="192"/>
       <c r="AA5" s="192"/>
       <c r="AB5" s="334"/>
     </row>
     <row r="6" spans="1:53" s="184" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B6" s="426" t="s">
+      <c r="B6" s="427" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="427"/>
-      <c r="D6" s="427"/>
-      <c r="E6" s="427"/>
-      <c r="F6" s="427"/>
-      <c r="G6" s="428"/>
-      <c r="I6" s="440" t="s">
+      <c r="C6" s="428"/>
+      <c r="D6" s="428"/>
+      <c r="E6" s="428"/>
+      <c r="F6" s="428"/>
+      <c r="G6" s="429"/>
+      <c r="I6" s="441" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="424" t="s">
+      <c r="J6" s="425" t="s">
         <v>409</v>
       </c>
-      <c r="K6" s="424" t="s">
+      <c r="K6" s="425" t="s">
         <v>408</v>
       </c>
-      <c r="L6" s="442" t="s">
+      <c r="L6" s="443" t="s">
         <v>215</v>
       </c>
-      <c r="M6" s="443"/>
-      <c r="N6" s="443"/>
-      <c r="O6" s="443"/>
-      <c r="P6" s="443"/>
-      <c r="Q6" s="444"/>
-      <c r="R6" s="429" t="s">
+      <c r="M6" s="444"/>
+      <c r="N6" s="444"/>
+      <c r="O6" s="444"/>
+      <c r="P6" s="444"/>
+      <c r="Q6" s="445"/>
+      <c r="R6" s="430" t="s">
         <v>216</v>
       </c>
-      <c r="S6" s="430"/>
-      <c r="T6" s="430"/>
-      <c r="U6" s="430"/>
-      <c r="V6" s="430"/>
-      <c r="W6" s="431"/>
+      <c r="S6" s="431"/>
+      <c r="T6" s="431"/>
+      <c r="U6" s="431"/>
+      <c r="V6" s="431"/>
+      <c r="W6" s="432"/>
       <c r="Y6" s="307"/>
       <c r="Z6" s="307"/>
       <c r="AA6" s="307"/>
@@ -24718,9 +26427,9 @@
         <f>SUM(C7:F7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="441"/>
-      <c r="J7" s="441"/>
-      <c r="K7" s="441"/>
+      <c r="I7" s="442"/>
+      <c r="J7" s="442"/>
+      <c r="K7" s="442"/>
       <c r="L7" s="186" t="s">
         <v>410</v>
       </c>
@@ -24924,14 +26633,14 @@
       <c r="AZ9" s="285"/>
     </row>
     <row r="10" spans="1:53" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="B10" s="432" t="s">
+      <c r="B10" s="433" t="s">
         <v>237</v>
       </c>
-      <c r="C10" s="432"/>
-      <c r="D10" s="432"/>
-      <c r="E10" s="432"/>
-      <c r="F10" s="432"/>
-      <c r="G10" s="432"/>
+      <c r="C10" s="433"/>
+      <c r="D10" s="433"/>
+      <c r="E10" s="433"/>
+      <c r="F10" s="433"/>
+      <c r="G10" s="433"/>
       <c r="I10" s="244" t="s">
         <v>231</v>
       </c>
@@ -25415,13 +27124,13 @@
       <c r="B16" s="193" t="s">
         <v>234</v>
       </c>
-      <c r="C16" s="433" t="s">
+      <c r="C16" s="434" t="s">
         <v>235</v>
       </c>
-      <c r="D16" s="434"/>
-      <c r="E16" s="434"/>
-      <c r="F16" s="434"/>
-      <c r="G16" s="435"/>
+      <c r="D16" s="435"/>
+      <c r="E16" s="435"/>
+      <c r="F16" s="435"/>
+      <c r="G16" s="436"/>
       <c r="I16" s="244" t="s">
         <v>404</v>
       </c>
@@ -25537,59 +27246,59 @@
     </row>
     <row r="18" spans="2:58" s="192" customFormat="1" ht="14" x14ac:dyDescent="0.15"/>
     <row r="19" spans="2:58" s="192" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I19" s="436" t="s">
+      <c r="I19" s="437" t="s">
         <v>424</v>
       </c>
-      <c r="J19" s="436"/>
-      <c r="K19" s="436"/>
-      <c r="L19" s="436"/>
-      <c r="M19" s="436"/>
-      <c r="N19" s="436"/>
-      <c r="O19" s="436"/>
-      <c r="P19" s="436"/>
-      <c r="Q19" s="436"/>
-      <c r="R19" s="436"/>
-      <c r="S19" s="436"/>
-      <c r="T19" s="436"/>
-      <c r="U19" s="436"/>
+      <c r="J19" s="437"/>
+      <c r="K19" s="437"/>
+      <c r="L19" s="437"/>
+      <c r="M19" s="437"/>
+      <c r="N19" s="437"/>
+      <c r="O19" s="437"/>
+      <c r="P19" s="437"/>
+      <c r="Q19" s="437"/>
+      <c r="R19" s="437"/>
+      <c r="S19" s="437"/>
+      <c r="T19" s="437"/>
+      <c r="U19" s="437"/>
       <c r="Z19" s="250"/>
       <c r="AA19" s="250"/>
       <c r="AB19" s="250"/>
       <c r="AC19" s="250"/>
     </row>
     <row r="20" spans="2:58" s="192" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I20" s="424" t="s">
+      <c r="I20" s="425" t="s">
         <v>13</v>
       </c>
-      <c r="J20" s="424" t="s">
+      <c r="J20" s="425" t="s">
         <v>213</v>
       </c>
-      <c r="K20" s="424" t="s">
+      <c r="K20" s="425" t="s">
         <v>214</v>
       </c>
-      <c r="L20" s="426" t="s">
+      <c r="L20" s="427" t="s">
         <v>215</v>
       </c>
-      <c r="M20" s="427"/>
-      <c r="N20" s="427"/>
-      <c r="O20" s="427"/>
-      <c r="P20" s="428"/>
-      <c r="Q20" s="429" t="s">
+      <c r="M20" s="428"/>
+      <c r="N20" s="428"/>
+      <c r="O20" s="428"/>
+      <c r="P20" s="429"/>
+      <c r="Q20" s="430" t="s">
         <v>216</v>
       </c>
-      <c r="R20" s="430"/>
-      <c r="S20" s="430"/>
-      <c r="T20" s="430"/>
-      <c r="U20" s="431"/>
+      <c r="R20" s="431"/>
+      <c r="S20" s="431"/>
+      <c r="T20" s="431"/>
+      <c r="U20" s="432"/>
       <c r="Z20" s="254"/>
       <c r="AA20" s="254"/>
       <c r="AB20" s="254"/>
       <c r="AC20" s="254"/>
     </row>
     <row r="21" spans="2:58" s="192" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I21" s="425"/>
-      <c r="J21" s="425"/>
-      <c r="K21" s="425"/>
+      <c r="I21" s="426"/>
+      <c r="J21" s="426"/>
+      <c r="K21" s="426"/>
       <c r="L21" s="186" t="s">
         <v>218</v>
       </c>
@@ -26958,16 +28667,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="446" t="e">
+      <c r="A1" s="447" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B1" s="446"/>
-      <c r="C1" s="446"/>
-      <c r="D1" s="446"/>
-      <c r="E1" s="446"/>
-      <c r="F1" s="446"/>
-      <c r="G1" s="446"/>
+      <c r="B1" s="447"/>
+      <c r="C1" s="447"/>
+      <c r="D1" s="447"/>
+      <c r="E1" s="447"/>
+      <c r="F1" s="447"/>
+      <c r="G1" s="447"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -26976,15 +28685,15 @@
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="412" t="s">
+      <c r="A3" s="413" t="s">
         <v>177</v>
       </c>
-      <c r="B3" s="412"/>
-      <c r="C3" s="412"/>
-      <c r="D3" s="412"/>
-      <c r="E3" s="412"/>
-      <c r="F3" s="412"/>
-      <c r="G3" s="412"/>
+      <c r="B3" s="413"/>
+      <c r="C3" s="413"/>
+      <c r="D3" s="413"/>
+      <c r="E3" s="413"/>
+      <c r="F3" s="413"/>
+      <c r="G3" s="413"/>
       <c r="H3" s="82"/>
       <c r="I3" s="82"/>
       <c r="J3" s="82"/>
@@ -27000,13 +28709,13 @@
       <c r="B4" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="413" t="s">
+      <c r="C4" s="414" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="414"/>
-      <c r="E4" s="414"/>
-      <c r="F4" s="414"/>
-      <c r="G4" s="415"/>
+      <c r="D4" s="415"/>
+      <c r="E4" s="415"/>
+      <c r="F4" s="415"/>
+      <c r="G4" s="416"/>
       <c r="N4" s="136" t="s">
         <v>128</v>
       </c>
@@ -27016,11 +28725,11 @@
         <v>16</v>
       </c>
       <c r="B5" s="111"/>
-      <c r="C5" s="416"/>
-      <c r="D5" s="411"/>
-      <c r="E5" s="411"/>
-      <c r="F5" s="411"/>
-      <c r="G5" s="411"/>
+      <c r="C5" s="417"/>
+      <c r="D5" s="412"/>
+      <c r="E5" s="412"/>
+      <c r="F5" s="412"/>
+      <c r="G5" s="412"/>
       <c r="N5" s="139"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -27028,11 +28737,11 @@
         <v>17</v>
       </c>
       <c r="B6" s="111"/>
-      <c r="C6" s="416"/>
-      <c r="D6" s="411"/>
-      <c r="E6" s="411"/>
-      <c r="F6" s="411"/>
-      <c r="G6" s="411"/>
+      <c r="C6" s="417"/>
+      <c r="D6" s="412"/>
+      <c r="E6" s="412"/>
+      <c r="F6" s="412"/>
+      <c r="G6" s="412"/>
       <c r="N6" s="139"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -27040,11 +28749,11 @@
         <v>18</v>
       </c>
       <c r="B7" s="111"/>
-      <c r="C7" s="416"/>
-      <c r="D7" s="411"/>
-      <c r="E7" s="411"/>
-      <c r="F7" s="411"/>
-      <c r="G7" s="411"/>
+      <c r="C7" s="417"/>
+      <c r="D7" s="412"/>
+      <c r="E7" s="412"/>
+      <c r="F7" s="412"/>
+      <c r="G7" s="412"/>
       <c r="N7" s="139"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -27052,11 +28761,11 @@
         <v>39</v>
       </c>
       <c r="B8" s="88"/>
-      <c r="C8" s="411"/>
-      <c r="D8" s="411"/>
-      <c r="E8" s="411"/>
-      <c r="F8" s="411"/>
-      <c r="G8" s="411"/>
+      <c r="C8" s="412"/>
+      <c r="D8" s="412"/>
+      <c r="E8" s="412"/>
+      <c r="F8" s="412"/>
+      <c r="G8" s="412"/>
       <c r="N8" s="139"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -27064,11 +28773,11 @@
         <v>162</v>
       </c>
       <c r="B9" s="88"/>
-      <c r="C9" s="417"/>
-      <c r="D9" s="417"/>
-      <c r="E9" s="417"/>
-      <c r="F9" s="417"/>
-      <c r="G9" s="417"/>
+      <c r="C9" s="418"/>
+      <c r="D9" s="418"/>
+      <c r="E9" s="418"/>
+      <c r="F9" s="418"/>
+      <c r="G9" s="418"/>
       <c r="N9" s="139"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -27076,11 +28785,11 @@
         <v>40</v>
       </c>
       <c r="B10" s="112"/>
-      <c r="C10" s="445"/>
-      <c r="D10" s="445"/>
-      <c r="E10" s="445"/>
-      <c r="F10" s="445"/>
-      <c r="G10" s="445"/>
+      <c r="C10" s="446"/>
+      <c r="D10" s="446"/>
+      <c r="E10" s="446"/>
+      <c r="F10" s="446"/>
+      <c r="G10" s="446"/>
       <c r="N10" s="139"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -27093,37 +28802,37 @@
       <c r="A12" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B12" s="418" t="s">
+      <c r="B12" s="419" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="419"/>
-      <c r="D12" s="420"/>
+      <c r="C12" s="420"/>
+      <c r="D12" s="421"/>
       <c r="N12" s="138" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B13" s="421" t="s">
+      <c r="B13" s="422" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="422"/>
-      <c r="D13" s="423"/>
+      <c r="C13" s="423"/>
+      <c r="D13" s="424"/>
       <c r="N13" s="139"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B14" s="405" t="s">
+      <c r="B14" s="406" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="406"/>
-      <c r="D14" s="407"/>
+      <c r="C14" s="407"/>
+      <c r="D14" s="408"/>
       <c r="N14" s="139"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B15" s="408" t="s">
+      <c r="B15" s="409" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="409"/>
-      <c r="D15" s="410"/>
+      <c r="C15" s="410"/>
+      <c r="D15" s="411"/>
       <c r="N15" s="139"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
@@ -28410,26 +30119,26 @@
       </c>
     </row>
     <row r="3" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D3" s="447" t="s">
+      <c r="D3" s="448" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="447"/>
-      <c r="F3" s="447" t="s">
+      <c r="E3" s="448"/>
+      <c r="F3" s="448" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="447"/>
-      <c r="H3" s="447"/>
-      <c r="I3" s="447" t="s">
+      <c r="G3" s="448"/>
+      <c r="H3" s="448"/>
+      <c r="I3" s="448" t="s">
         <v>61</v>
       </c>
-      <c r="J3" s="447"/>
-      <c r="K3" s="447"/>
+      <c r="J3" s="448"/>
+      <c r="K3" s="448"/>
       <c r="L3" s="131"/>
-      <c r="M3" s="447" t="s">
+      <c r="M3" s="448" t="s">
         <v>18</v>
       </c>
-      <c r="N3" s="447"/>
-      <c r="O3" s="447"/>
+      <c r="N3" s="448"/>
+      <c r="O3" s="448"/>
     </row>
     <row r="4" spans="1:16" s="45" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="44" t="s">

</xml_diff>